<commit_message>
Count the bar before a window over changes in its warm-up
relative_change and rolling_money_flow_gain_share take their first change off the bar
before their window, so a window of n of them is finite from its (n + 1)-th bar while the
warm-up counted n — one bar short of what the first decision reads, and published so for
relative_change10 and centered_rolling_money_flow_gain_share14. Their records now carry
warmup_offset_bars, term_warmup_bars adds it, and features_status.json, regenerated by the
stage, publishes 11 and 15; WARMUP_TOP_TIMEFRAME_BARS, and with it every artifact of the
chain, is unchanged.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -13996,7 +13996,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SERIES_KERNELS` and `INDICATORS` at the end of `indicators.py`, `OPERATORS` and `NORMALISERS` in `catalogue.py`, each `{token: {"kernel": …}}` even where a record holds one fact; an indicator's record holding its `parameter_word`, its `warmup_multiple`, its fixed `inputs` and its bounded `output_range` where it has them, and its `historical_aliases`, its kernel the function named for the token; `term_name()`, `term_warmup_bars()`, `catalogue.term_values()` and `status.term_block()` reading the record, and no invariant in a second table, a constant or a branch on one token.</t>
+          <t xml:space="preserve">`SERIES_KERNELS` and `INDICATORS` at the end of `indicators.py`, `OPERATORS` and `NORMALISERS` in `catalogue.py`, each `{token: {"kernel": …}}` even where a record holds one fact; an indicator's record holding its `parameter_word`, its `warmup_multiple`, its `warmup_offset_bars` for a window over changes, its fixed `inputs` and its bounded `output_range` where it has them, and its `historical_aliases`, its kernel the function named for the token; `term_name()`, `term_warmup_bars()`, `catalogue.term_values()` and `status.term_block()` reading the record, and no invariant in a second table, a constant or a branch on one token.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -14514,7 +14514,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">`WARMUP_TOP_TIMEFRAME_BARS` the maximum of `definition_warmup_bars()` over `FEATURE_CATALOGUE` — each term's `warmup_multiple` times its parameter — and `WARMUP_END_MS` the research start plus that many bars of the top timeframe; the catalogue's first decision row at or after `WARMUP_END_MS`, every catalogued value finite from there, asserted by `catalogue.build_catalogue`; both in the contract, and in `catalogue.warmup` of `features_status.json` the end as a UTC time.</t>
+          <t xml:space="preserve">`WARMUP_TOP_TIMEFRAME_BARS` the maximum of `definition_warmup_bars()` over `FEATURE_CATALOGUE` — each term's `warmup_multiple` times its parameter, plus its `warmup_offset_bars` where the window is one of changes — and `WARMUP_END_MS` the research start plus that many bars of the top timeframe; the catalogue's first decision row at or after `WARMUP_END_MS`, every catalogued value finite from there, asserted by `catalogue.build_catalogue`; both in the contract, and in `catalogue.warmup` of `features_status.json` the end as a UTC time.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">

</xml_diff>

<commit_message>
Render the name register into module_skills/skill_glossary.md
The register is a Skill of the canon like the others, so it lies among
module_skills/skill_*.md: skill_places lists the canon's two places and no exception,
and the files matrix heads its column skill_glossary. Every reference follows the
file — the contract, the orientations, the terminals' docstrings, the five equal copies
of tui.py and eleven cells of the sheet — and so does the line status.py writes at the
foot of <TICKER>_README.md, which moves the tracked BTC_README.md by that line alone.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -151,7 +151,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The name and its register row in `module_skills/skills_sheet.xlsx` in one commit, `module_skills/glossary.md` synced from it; no second name for a concept the register already holds.</t>
+          <t xml:space="preserve">The name and its register row in `module_skills/skills_sheet.xlsx` in one commit, `module_skills/skill_glossary.md` synced from it; no second name for a concept the register already holds.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every `skill_*.md` and `module_skills/glossary.md` is rendered from the sheet by `make skills-sync`, carries the marker on its first line, is never edited by hand, and is the only kind of document the crawler sends as context.</t>
+          <t xml:space="preserve">Every `skill_*.md` and `module_skills/skill_glossary.md` is rendered from the sheet by `make skills-sync`, carries the marker on its first line, is never edited by hand, and is the only kind of document the crawler sends as context.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1606,7 +1606,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/glossary.md</t>
+          <t xml:space="preserve">module_skills/skill_glossary.md</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1643,7 +1643,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/glossary.md</t>
+          <t xml:space="preserve">module_skills/skill_glossary.md</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">`partition_dir()`, `schema_json()`, `artifact_dir()` and the descriptors over them — `ohlcv_1m_canonical_parquet()`, `bars_parquet()`, `parameters_json()` and the rest — called at the point of use, and no store path assembled there; a descriptor another module needs carried as a copy registered in `module_skills/glossary.md` § Twice by extraction.</t>
+          <t xml:space="preserve">`partition_dir()`, `schema_json()`, `artifact_dir()` and the descriptors over them — `ohlcv_1m_canonical_parquet()`, `bars_parquet()`, `parameters_json()` and the rest — called at the point of use, and no store path assembled there; a descriptor another module needs carried as a copy registered in `module_skills/skill_glossary.md` § Twice by extraction.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t xml:space="preserve">gum run over `subprocess` in `tui.py` alone, which imports the standard library and its own `config` for `OUTPUT_PLAIN`; every header, placeholder and line of content a caller's argument, the words of `tui.py` itself being the block labels and the line naming the columns left out; no Rich, Textual or curses and no escape code written by Python; one `tui.py`, byte for byte, in every terminal, registered as twice by extraction in `module_skills/glossary.md`.</t>
+          <t xml:space="preserve">gum run over `subprocess` in `tui.py` alone, which imports the standard library and its own `config` for `OUTPUT_PLAIN`; every header, placeholder and line of content a caller's argument, the words of `tui.py` itself being the block labels and the line naming the columns left out; no Rich, Textual or curses and no escape code written by Python; one `tui.py`, byte for byte, in every terminal, registered as twice by extraction in `module_skills/skill_glossary.md`.</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3703,7 +3703,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Header words the register's UI labels as `module_skills/glossary.md` spells them, the terminal's own words lower case; `#` counting from 1 in the order the file holds; a fact such as `command  &lt;command line&gt;` printed as a line; the rows handed to `gum table --print` as CSV from Python's `csv` on its standard input, `TERM=dumb` in its environment so that no row is bold, and no `--widths`, colour flag or padding by Python.</t>
+          <t xml:space="preserve">Header words the register's UI labels as `module_skills/skill_glossary.md` spells them, the terminal's own words lower case; `#` counting from 1 in the order the file holds; a fact such as `command  &lt;command line&gt;` printed as a line; the rows handed to `gum table --print` as CSV from Python's `csv` on its standard input, `TERM=dumb` in its environment so that no row is bold, and no `--widths`, colour flag or padding by Python.</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -11962,7 +11962,7 @@
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t xml:space="preserve">every `skill_*.md` and `module_skills/glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
+          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
@@ -12094,7 +12094,7 @@
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
+          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
@@ -16928,7 +16928,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/index.html`, `README.md`, `module_monitoring/README_module_monitoring.md`, `module_skills/glossary.md`</t>
+          <t xml:space="preserve">`module_monitoring/index.html`, `README.md`, `module_monitoring/README_module_monitoring.md`, `module_skills/skill_glossary.md`</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -17412,7 +17412,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/glossary.md</t>
+          <t xml:space="preserve">module_skills/skill_glossary.md</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -17636,7 +17636,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">glossary</t>
+          <t xml:space="preserve">skill_glossary</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>

<commit_message>
Spell the timeframe placeholder <timeframe> and the sub-module's <subject>
One concept, one placeholder: the forty <tf> of the partition paths — twenty-seven in the
contract, the READMEs, the methodology and the partition_dir() docstring of its four
equal copies, thirteen in the sheet's cells — become <timeframe>, the word the feature
grammar and the raw store already use, and the one sub_module_<domain> becomes the
sub_module_<subject> of the grammar row. The two path listings the longer word pushed
out of line are aligned again, and the docstring is wrapped.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -3190,7 +3190,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Serialised schema — a family name, a feature id, an artifact key — keeps the compact token, being a contract with the files on disk, and so does the raw store `store/raw_1m/`, the one raw child of `store/`; a partition `timeframe=&lt;tf&gt;/` of a family carries the compact token as its value and a Parquet file inside it carries no slot; a partition of the `catalogue` family carries no timeframe in its columns.</t>
+          <t xml:space="preserve">Serialised schema — a family name, a feature id, an artifact key — keeps the compact token, being a contract with the files on disk, and so does the raw store `store/raw_1m/`, the one raw child of `store/`; a partition `timeframe=&lt;timeframe&gt;/` of a family carries the compact token as its value and a Parquet file inside it carries no slot; a partition of the `catalogue` family carries no timeframe in its columns.</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ohlcv_1m_binance`, `ohlcv_1m_bybit`, `ohlcv_1m_canonical`, `bars`, `catalogue`, `labels`, `oos_predictions` under `STORE_ASSETS_ARTIFACTS_DIR`; `hpo_trials`, `score_trials` under `STORE_TRIALS_DIR`; `&lt;family&gt;/ticker=&lt;TICKER&gt;/[timeframe=&lt;tf&gt;/]&lt;family&gt;.parquet` or `.jsonl`; `partition_dir()` in every `config.py` that writes or reads one; DuckDB the engine, in memory</t>
+          <t xml:space="preserve">`ohlcv_1m_binance`, `ohlcv_1m_bybit`, `ohlcv_1m_canonical`, `bars`, `catalogue`, `labels`, `oos_predictions` under `STORE_ASSETS_ARTIFACTS_DIR`; `hpo_trials`, `score_trials` under `STORE_TRIALS_DIR`; `&lt;family&gt;/ticker=&lt;TICKER&gt;/[timeframe=&lt;timeframe&gt;/]&lt;family&gt;.parquet` or `.jsonl`; `partition_dir()` in every `config.py` that writes or reads one; DuckDB the engine, in memory</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -8919,7 +8919,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ticker=&lt;TICKER&gt;/`, `timeframe=&lt;tf&gt;/` — Hive's `key=value`, the value the ticker in capitals and the compact timeframe token; `partition_dir()`</t>
+          <t xml:space="preserve">`ticker=&lt;TICKER&gt;/`, `timeframe=&lt;timeframe&gt;/` — Hive's `key=value`, the value the ticker in capitals and the compact timeframe token; `partition_dir()`</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -10723,7 +10723,7 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/bars.py` writes `bars/ticker=&lt;TICKER&gt;/timeframe=&lt;tf&gt;/bars.parquet` and the family's `schema.json`; `bars_parquet()`</t>
+          <t xml:space="preserve">`module_features/bars.py` writes `bars/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/bars.parquet` and the family's `schema.json`; `bars_parquet()`</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -10745,7 +10745,7 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/catalogue.py` writes `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;tf&gt;/catalogue.parquet` and the family's `schema.json` from `catalogue_schema()`, the columns of the union of its partitions in catalogue order; `catalogue_parquet()` — in `module_ml/config.py` the same name over the contract's `parquet_by_timeframe`</t>
+          <t xml:space="preserve">`module_features/catalogue.py` writes `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet` and the family's `schema.json` from `catalogue_schema()`, the columns of the union of its partitions in catalogue order; `catalogue_parquet()` — in `module_ml/config.py` the same name over the contract's `parquet_by_timeframe`</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -10767,7 +10767,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/labels.py` writes `labels/ticker=&lt;TICKER&gt;/timeframe=&lt;tf&gt;/labels.parquet` and the family's `schema.json`; `labels_parquet()`</t>
+          <t xml:space="preserve">`module_ml/labels.py` writes `labels/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/labels.parquet` and the family's `schema.json`; `labels_parquet()`</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -10789,7 +10789,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/train.py` writes `oos_predictions/ticker=&lt;TICKER&gt;/timeframe=&lt;tf&gt;/oos_predictions.parquet` and the family's `schema.json`; `oos_predictions_parquet()`</t>
+          <t xml:space="preserve">`module_ml/train.py` writes `oos_predictions/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/oos_predictions.parquet` and the family's `schema.json`; `oos_predictions_parquet()`</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -10860,7 +10860,7 @@
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature layer's contract the ML layer reads instead of the feature configuration: `decision_timeframe`, `timeframes` (each `timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe` — each value a path relative to the artifacts store, `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;tf&gt;/catalogue.parquet`; untracked</t>
+          <t xml:space="preserve">the feature layer's contract the ML layer reads instead of the feature configuration: `decision_timeframe`, `timeframes` (each `timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe` — each value a path relative to the artifacts store, `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet`; untracked</t>
         </is>
       </c>
     </row>
@@ -11248,7 +11248,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;tf&gt;/` carries it)</t>
+          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
         </is>
       </c>
     </row>
@@ -14144,7 +14144,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_id(definition_name, timeframe)` = `&lt;definition&gt;_&lt;timeframe&gt;` over `[&lt;normaliser&gt;_]&lt;term&gt;{_&lt;operator&gt;_&lt;term&gt;}`, the column of X and the key of an importance; a partition's column the definition's name alone, its partition carrying the timeframe; never `trend_&lt;tf&gt;`, `momentum_&lt;…&gt;`, a ticker, an hour count or a second timeframe inside an id.</t>
+          <t xml:space="preserve">`feature_id(definition_name, timeframe)` = `&lt;definition&gt;_&lt;timeframe&gt;` over `[&lt;normaliser&gt;_]&lt;term&gt;{_&lt;operator&gt;_&lt;term&gt;}`, the column of X and the key of an importance; a partition's column the definition's name alone, its partition carrying the timeframe; never `trend_&lt;timeframe&gt;`, `momentum_&lt;…&gt;`, a ticker, an hour count or a second timeframe inside an id.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -14255,7 +14255,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">`bars/ticker=&lt;TICKER&gt;/timeframe=&lt;tf&gt;/bars.parquet` and `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;tf&gt;/catalogue.parquet` in the artifacts store for every timeframe of `HIERARCHY_TIMEFRAMES`, each family's `schema.json` beside its partitions — the bars' read off a written partition, the catalogue's from the register (`catalogue_schema()`), the union of its partitions' columns; a catalogue partition holding `decision_ts` and the definitions `catalogue_columns(&lt;tf&gt;)` offers; never a bars table in a database, a Parquet outside a family or a timeframe inside a column name.</t>
+          <t xml:space="preserve">`bars/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/bars.parquet` and `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet` in the artifacts store for every timeframe of `HIERARCHY_TIMEFRAMES`, each family's `schema.json` beside its partitions — the bars' read off a written partition, the catalogue's from the register (`catalogue_schema()`), the union of its partitions' columns; a catalogue partition holding `decision_ts` and the definitions `catalogue_columns(&lt;timeframe&gt;)` offers; never a bars table in a database, a Parquet outside a family or a timeframe inside a column name.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">

</xml_diff>

<commit_message>
Hold a hand's search action to one ticker, hand the tmux twin its project, write each step once
The promotion, the reset and the detached search checked ASSET for presence alone, and the
reset put it unquoted into rm -rf: ASSET='BTC *' would have removed the contents of the
tree's root. one_asset — one ticker of TICKERS, or make stops before a line of the recipe
runs — replaces the three copies of the check. The tmux session takes the tmux server's
environment, not the shell's, so the twin's command line carries COMPOSE_PROJECT_NAME
where it is set, and the session is named behind it. Each of the search's two steps has
one command, serpentine_turn and serpentine_score over the new stage and each macros, read
by its own target and by the loop; make -n prints what it printed before. The target
grammar names <module>-<process> and its actions in general, the search's targets its
examples, and the register takes the new names.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TICKER_LIST` — `ASSET` if set, else `TICKERS` — feeding `fanout`; no service environment carrying `ASSET`; `build_ticker_parser()` declaring `--tickers` required; no stage module reading `ASSET`.</t>
+          <t xml:space="preserve">`TICKER_LIST` — `ASSET` if set, else `TICKERS` — the list `each` and `fanout` go over; `one_asset` stopping make before a line of the recipe runs where the promotion, the reset or the detached search is given anything but one ticker of `TICKERS`; no service environment carrying `ASSET`; `build_ticker_parser()` declaring `--tickers` required; no stage module reading `ASSET`.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -585,17 +585,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">The compose project is named `liora` in the file, so a container is `liora-&lt;service&gt;-1` on every host; two checkouts on one host share the name and run one at a time, unless `COMPOSE_PROJECT_NAME` overrides it at invocation.</t>
+          <t xml:space="preserve">The compose project is named `liora` in the file, so a container is `liora-&lt;service&gt;-1` on every host; two checkouts on one host share the name and run one at a time, unless `COMPOSE_PROJECT_NAME` overrides it at invocation — and the detached serpentine search, whose tmux session takes the tmux server's environment, is handed the override.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">`docker-compose.yml`</t>
+          <t xml:space="preserve">`docker-compose.yml`, `Makefile`</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">`name: liora` at the top of the file; containers `liora-&lt;service&gt;-1` and the network `liora_default`; no project name derived from the checkout's directory, none per ticker.</t>
+          <t xml:space="preserve">`name: liora` at the top of the file; containers `liora-&lt;service&gt;-1` and the network `liora_default`; no project name derived from the checkout's directory, none per ticker; `tmux-features-serpentine-search` carrying `COMPOSE_PROJECT_NAME`, where it is set, on its session's command line, and `SERPENTINE_SEARCH_SESSION` putting it before the session's name.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">`docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers …` through the `run`, `fanout` and `basket` macros — the chain's stages, the serpentine search's turn and `ml-score`, and the promotion; no `docker compose exec`; `record.py` measuring a stage from outside and knowing no container.</t>
+          <t xml:space="preserve">`docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers …` through the `run` and `stage` macros, fanned out by `each` and `fanout` or run once by `basket` — the chain's stages, the serpentine search's turn and `ml-score`, and the promotion; no `docker compose exec`; `record.py` measuring a stage from outside and knowing no container.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">`fanout` — `TICKER_LIST` into `xargs -P &lt;width&gt;`, one `run` with `--tickers &lt;TICKER&gt;` each, `data-ingest` at width 1 and every other per-asset stage at `$(JOBS)`; `basket` — one `run` with `--tickers $(TICKERS_CSV)`: the three status stages, and the download as one container per venue, a venue's rate limit being budgeted per process.</t>
+          <t xml:space="preserve">`fanout` — `each`, `TICKER_LIST` into `xargs -P &lt;width&gt;`, one `stage` with `--tickers &lt;TICKER&gt;` each, `data-ingest` at width 1 and every other per-asset stage at `$(JOBS)`; `basket` — one `stage` with `--tickers $(TICKERS_CSV)`: the three status stages, and the download as one container per venue, a venue's rate limit being budgeted per process.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/`: `serpentine_search.py`, `coordinate_barrier.py`, `coordinate_feature_set.py`, `promote.py`; `make features-serpentine-search` — per asset a turn, then `ml-score` and a turn again while the turn leaves a question — and its detached twin `tmux-features-serpentine-search` in the tmux session `SERPENTINE_SEARCH_SESSION`, one asset per session</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/`: `serpentine_search.py`, `coordinate_barrier.py`, `coordinate_feature_set.py`, `promote.py`; `make features-serpentine-search` — per asset a turn, then `ml-score` and a turn again while the turn leaves a question, the Makefile's `serpentine_turn` and `serpentine_score`, the one command of each step — and its detached twin `tmux-features-serpentine-search` in the tmux session `SERPENTINE_SEARCH_SESSION`, one asset per session, behind `COMPOSE_PROJECT_NAME` where it is set</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -9017,7 +9017,7 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TICKERS` in the `Makefile`, the basket's one list; `TICKER_LIST`, the `fanout` macro's list, which `ASSET` narrows; `TICKERS_CSV`, the basket as one `--tickers` argument of a basket-wide stage, which `ASSET` never narrows</t>
+          <t xml:space="preserve">`TICKERS` in the `Makefile`, the basket's one list; `TICKER_LIST`, the list the `each` macro goes over, which `ASSET` narrows; `one_asset`, the one ticker of `TICKERS` a hand's action on the serpentine search names; `TICKERS_CSV`, the basket as one `--tickers` argument of a basket-wide stage, which `ASSET` never narrows</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -11447,7 +11447,7 @@
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t xml:space="preserve">the `fanout` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` once per ticker of `TICKER_LIST`, `JOBS` at a time</t>
+          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
@@ -11469,7 +11469,7 @@
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `fanout` and `basket` macros of the `Makefile`</t>
+          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
@@ -17366,7 +17366,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The runtime contract every module runs inside: the one image, the three runners and the one resident `docker-compose.yml` writes under two anchors, the stores each service mounts and how a container addresses them, and the Makefile's `run`, `fanout` and `basket` macros that run a stage in a one-off container for one asset or for the whole basket. It also governs the host user, the init process, the one memory ceiling, the compose project's name and the host port the Makefile measures.</t>
+          <t xml:space="preserve">The runtime contract every module runs inside: the one image, the three runners and the one resident `docker-compose.yml` writes under two anchors, the stores each service mounts and how a container addresses them, and the Makefile's `run`, `stage`, `each`, `fanout` and `basket` macros that run a stage in a one-off container for one asset or for the whole basket. It also governs the host user, the init process, the one memory ceiling, the compose project's name and the host port the Makefile measures.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Promote the one proposal a search holds, and refuse in one line when it holds none
proposals_block() returns the champion alone or nothing, yet the promotion took a rank —
PROPOSAL=<n> on the make line, --proposal in promote.py, a choice from a list of at most
one on the features terminal — and ended in a KeyError when the search proposed nothing.
The rank is gone from all three: promote.py copies the one proposal, or refuses in one
line before it writes anything, and the terminal's plan shows the proposal's trial and
what it moves straight away, one step fewer. § Values names the refusal beside the stages'
others; the sheet, the READMEs and the methodology follow.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -4110,7 +4110,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t xml:space="preserve">A `gum choose` headed `&lt;verb&gt; …?` — `&lt;target&gt;?`, `draft &lt;file&gt;?`, `promote proposal &lt;n&gt; of &lt;TICKER&gt;?`; `back` asking the action's forms again from the first, every default preselected, so that an action with its defaults is one Enter per form and one on the gate; a list of data carrying neither, Esc its cancel; the menu ending on `quit`; no option `exit` or `run`.</t>
+          <t xml:space="preserve">A `gum choose` headed `&lt;verb&gt; …?` — `&lt;target&gt;?`, `draft &lt;file&gt;?`, `promote the proposal of &lt;TICKER&gt;?`; `back` asking the action's forms again from the first, every default preselected, so that an action with its defaults is one Enter per form and one on the gate; a list of data carrying neither, Esc its cancel; the menu ending on `quit`; no option `exit` or `run`.</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -7447,7 +7447,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py`, `make features-serpentine-search-promote ASSET=&lt;TICKER&gt; PROPOSAL=&lt;n&gt;`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py`, `make features-serpentine-search-promote ASSET=&lt;TICKER&gt;`</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -7462,7 +7462,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t xml:space="preserve">apply, activate, deploy; a promotion of the whole basket; a counter or a rank in the file — git holds the history</t>
+          <t xml:space="preserve">apply, activate, deploy; a promotion of the whole basket; a counter or a rank in the file — git holds the history; a rank on the make line or the command line, a search holding one proposal at most</t>
         </is>
       </c>
     </row>
@@ -10147,7 +10147,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one call of make — a terminal starts a target through it and no other way, its lines uncaptured; it takes its arguments open, `_make(*arguments)`, so a menu target with its asset and the promotion with its proposal pass through one signature</t>
+          <t xml:space="preserve">the one call of make — a terminal starts a target through it and no other way, its lines uncaptured; it takes its arguments open, `_make(*arguments)`, so a target alone and a target with its asset — the promotion's among them — pass through one signature</t>
         </is>
       </c>
     </row>
@@ -10399,7 +10399,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal's own actions, the serpentine search's: draft the profile, read the recorded serpentine search, promote a proposal</t>
+          <t xml:space="preserve">the features terminal's own actions, the serpentine search's: draft the profile, read the recorded serpentine search, promote the proposal</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -10426,12 +10426,12 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t xml:space="preserve">the steps table: the steps of one of the features terminal's actions in order, above the step it asks — each answered DONE with its choice, the one asked CURRENT, the rest PENDING</t>
+          <t xml:space="preserve">the steps table: the steps of the features terminal's draft in order, above the step it asks — each answered DONE with its choice, the one asked CURRENT, the rest PENDING</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_step_rows()`, `_step_answer()`, `DRAFT_STEPS`, `PROMOTE_STEPS` in `module_features/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">`_step_rows()`, `_step_answer()`, `DRAFT_STEPS` in `module_features/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -10480,7 +10480,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t xml:space="preserve">the target the features terminal opens its own screen for — the promotion, whose proposal's number no bare run can answer</t>
+          <t xml:space="preserve">the target the features terminal opens its own screen for — the promotion, whose plan shows the one state it promotes</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -14879,12 +14879,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `Makefile`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_features/sub_module_terminal/terminal.py`, `Makefile`</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json` and `&lt;TICKER&gt;_barriers.json` written by `promote.py` alone, for the proposal `make features-serpentine-search-promote ASSET=&lt;TICKER&gt; PROPOSAL=&lt;n&gt;` names, then `ml-all` for that asset; never the proposal's `best_params`; the active state promoted again writing nothing; a converged serpentine search writing neither file.</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json` and `&lt;TICKER&gt;_barriers.json` written by `promote.py` alone, from the one proposal of the asset's search, by `make features-serpentine-search-promote ASSET=&lt;TICKER&gt;`, then `ml-all` for that asset; no rank and no choice among proposals, a search holding one at most; a search that proposes none refused in one line, before either file is written; never the proposal's `best_params`; the active state promoted again writing nothing; a converged serpentine search writing neither file.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">

</xml_diff>

<commit_message>
State once, by dependency, what a change asks of a serpentine search
The frozen-inputs rule stood in two rows of the sheet and four places of the prose, with
two paths: a change of a field the search records restarted it by itself, any other went
through make all and a reset. The window and SEED are among the recorded fields, so the
documented path skipped make all for them, and the search restarted on the bars, the
catalogue, the labels and the parameters of the old window. One row,
SERPENTINE-SEARCH-ONE-SEARCH-IS-ONE-EXPERIMENT, orders by dependency: a change of anything
the chain reads goes through make all ASSET=<TICKER>, the reset and a new search, in that
order; a change of the profile or of the beam width alone needs the next turn. README.md,
both orientations and both methodologies cite the row and restate none of it.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -14795,22 +14795,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-INPUTS-DECIDE-RESUME</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-ONE-SEARCH-IS-ONE-EXPERIMENT</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">A rerun compares its recorded `inputs` by equality: equal resumes at the round boundary, different starts again with a fresh state and ledger; `inputs_current` is false, never an error, when they differ or the asset has no profile.</t>
+          <t xml:space="preserve">A serpentine search is one experiment, and a change reaches it through what depends on it: after a change of anything the chain reads — the data inside the research window, or a CONFIGURABLES record of the chain, the window, the seed and the warm-up among them — `make all ASSET=&lt;TICKER&gt;` recomputes the asset's chain, `make features-serpentine-search-reset ASSET=&lt;TICKER&gt;` removes its search, and a new search starts, in that order; a change of the profile or of the beam width alone needs the next turn and nothing else, the turn starting afresh by itself. No line scored before a change is read as a cache hit after it.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_features/status.py`</t>
+          <t xml:space="preserve">`Makefile`, `module_features/sub_module_serpentine_search/**/*.py`, `module_features/status.py`</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_search_inputs()` — the research window with the seed and the warm-up, `best_params`, the catalogue's columns, the asset's active columns and barriers, the profile and the beam width — recorded in the state file; a turn whose `inputs` differ removing the ledger, the request and the response before its first question; `serpentine_search_block()` publishing `inputs_current` as a boolean, raising nothing on a missing profile and publishing no proposal while it is false.</t>
+          <t xml:space="preserve">`build_search_inputs()` — the research window with the seed and the warm-up, `best_params`, the catalogue's columns, the asset's active columns and barriers, the profile and the beam width — recorded in the state file and compared by equality at every turn: equal resumes at the round boundary, different removes the ledger, the request and the response before the first question; `serpentine_search_block()` publishing `inputs_current` as a boolean, raising nothing on a missing profile and publishing no proposal while it is false; `features-serpentine-search-reset`, `ASSET=` one ticker of `TICKERS`, removing `&lt;TICKER&gt;_serpentine_search.json`, `&lt;TICKER&gt;_serpentine_search_trials.jsonl`, `&lt;TICKER&gt;_score_request.json`, `&lt;TICKER&gt;_score_response.json` and the asset's partition `score_trials/ticker=&lt;TICKER&gt;/` of the trials store, keeping the profile, the promoted state, the chain's files and `hpo_trials`, and running no stage.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -14832,22 +14832,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-A-CHANGE-OUTSIDE-THE-INPUTS-NEEDS-A-RESET</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-PROMOTION-IS-A-HAND</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">A change the `inputs` do not record — the canonical data inside the research window, the catalogue's values, a CONFIGURABLES record of `module_ml` — is invisible to a turn, so it is followed by `make all ASSET=&lt;TICKER&gt;` and then `make features-serpentine-search-reset ASSET=&lt;TICKER&gt;` before a new serpentine search starts, and no line scored before it is read as a cache hit after it.</t>
+          <t xml:space="preserve">A proposal becomes an asset's feature set and barrier geometry by a hand's act alone, never because the serpentine search finished; the promotion copies the proposal's columns and geometry, and the asset's ML chain then tunes it anew.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">`Makefile`, `module_features/sub_module_serpentine_search/**/*.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_features/sub_module_terminal/terminal.py`, `Makefile`</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">`features-serpentine-search-reset`, `ASSET=` required, removing `&lt;TICKER&gt;_serpentine_search.json`, `&lt;TICKER&gt;_serpentine_search_trials.jsonl`, `&lt;TICKER&gt;_score_request.json`, `&lt;TICKER&gt;_score_response.json` and the asset's partition `score_trials/ticker=&lt;TICKER&gt;/` of the trials store, keeping the profile, the promoted state, the chain's files and `hpo_trials`, and running no stage.</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json` and `&lt;TICKER&gt;_barriers.json` written by `promote.py` alone, from the one proposal of the asset's search, by `make features-serpentine-search-promote ASSET=&lt;TICKER&gt;`, then `ml-all` for that asset; no rank and no choice among proposals, a search holding one at most; a search that proposes none refused in one line, before either file is written; never the proposal's `best_params`; the active state promoted again writing nothing; a converged serpentine search writing neither file.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -14864,27 +14864,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Workflow</t>
+          <t xml:space="preserve">FileLayout</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-PROMOTION-IS-A-HAND</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-ITS-RECORD-IS-TRACKED</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">A proposal becomes an asset's feature set and barrier geometry by a hand's act alone, never because the serpentine search finished; the promotion copies the proposal's columns and geometry, and the asset's ML chain then tunes it anew.</t>
+          <t xml:space="preserve">The record of an asset's serpentine search — its state file, its ledger and its profile — and the state a promotion wrote are tracked files of the asset's folder; the question, the answer and the asset's `score_trials` partition are transient and never tracked.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_features/sub_module_terminal/terminal.py`, `Makefile`</t>
+          <t xml:space="preserve">`.gitignore`, `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json` and `&lt;TICKER&gt;_barriers.json` written by `promote.py` alone, from the one proposal of the asset's search, by `make features-serpentine-search-promote ASSET=&lt;TICKER&gt;`, then `ml-all` for that asset; no rank and no choice among proposals, a search holding one at most; a search that proposes none refused in one line, before either file is written; never the proposal's `best_params`; the active state promoted again writing nothing; a converged serpentine search writing neither file.</t>
+          <t xml:space="preserve">`.gitignore` admitting `store/assets_artifacts/ticker=*/*_serpentine_search.json`, `*_serpentine_search_trials.jsonl`, `*_serpentine_search_profile.json`, `*_feature_set.json` and `*_barriers.json` among the files of the asset's folder, leaving `*_score_request.json` and `*_score_response.json` ignored, and ignoring the trials store whole; each of these files built by a descriptor of the sub-module's `config.py` under `artifact_dir()`.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -14901,27 +14901,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">FileLayout</t>
+          <t xml:space="preserve">Determinism</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-ITS-RECORD-IS-TRACKED</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-A-STATE-IS-KEYED-BY-ITS-CANONICAL-TEXT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">The record of an asset's serpentine search — its state file, its ledger and its profile — and the state a promotion wrote are tracked files of the asset's folder; the question, the answer and the asset's `score_trials` partition are transient and never tracked.</t>
+          <t xml:space="preserve">A state — its columns per timeframe, its barrier coordinates and its hyper-parameter point — is keyed by its own canonical JSON text, so two states are equal exactly or not at all, a state read back off disk keys as the one that wrote it, and a state already in the ledger is looked up, never scored again.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.gitignore`, `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_ml/score.py`</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.gitignore` admitting `store/assets_artifacts/ticker=*/*_serpentine_search.json`, `*_serpentine_search_trials.jsonl`, `*_serpentine_search_profile.json`, `*_feature_set.json` and `*_barriers.json` among the files of the asset's folder, leaving `*_score_request.json` and `*_score_response.json` ignored, and ignoring the trials store whole; each of these files built by a descriptor of the sub-module's `config.py` under `artifact_dir()`.</t>
+          <t xml:space="preserve">`state_key()` over `theta()` — `json.dumps(state, sort_keys=True, separators=(",", ":"))` — twice by extraction with `module_ml/score.py`; every barrier value through `BARRIER_COORDINATE_CASTS` and a float carried as JSON writes it; `index_by_state` the one lookup, with no tolerance and no rounding in a comparison of states.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -14938,27 +14938,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Determinism</t>
+          <t xml:space="preserve">Methodology</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-A-STATE-IS-KEYED-BY-ITS-CANONICAL-TEXT</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-HPO-ENDS-THE-ROUND</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">A state — its columns per timeframe, its barrier coordinates and its hyper-parameter point — is keyed by its own canonical JSON text, so two states are equal exactly or not at all, a state read back off disk keys as the one that wrote it, and a state already in the ledger is looked up, never scored again.</t>
+          <t xml:space="preserve">The hyper-parameter family is the last family of a round, so a study is never left for a later turn to recover.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_ml/score.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">`state_key()` over `theta()` — `json.dumps(state, sort_keys=True, separators=(",", ":"))` — twice by extraction with `module_ml/score.py`; every barrier value through `BARRIER_COORDINATE_CASTS` and a float carried as JSON writes it; `index_by_state` the one lookup, with no tolerance and no rounding in a comparison of states.</t>
+          <t xml:space="preserve">`ROUND_SCHEDULE` ending with the `hpo` loop's `study` family, and the turn that reads its response ending the round; a schedule that moves it is a new decision, not a setting.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -14980,12 +14980,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-HPO-ENDS-THE-ROUND</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-A-MOVE-CLEARS-THE-NOISE-OF-ITS-PASS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">The hyper-parameter family is the last family of a round, so a study is never left for a later turn to recover.</t>
+          <t xml:space="preserve">A child clears the gate only where its threshold constraint is met, its fold measure beats its parent's strictly on every validation fold and its path CAGR beats the parent's by more than k(n) times the asset's noise sigma, n the candidates of its pass — for every family, a move that shrinks the state included; a calibration run, whose profile has no sigma, clears a child strictly better on the path CAGR and on every fold, and a move that shrinks the state where it is no worse on either. k(n) is where the best of n candidates carrying independent normal noise of one size would beat an equal parent at `GATE_THRESHOLD_FALSE_EXCEEDANCE_RATE`: a heuristic margin, not a test at that rate.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -14995,7 +14995,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ROUND_SCHEDULE` ending with the `hpo` loop's `study` family, and the turn that reads its response ending the round; a schedule that moves it is a new decision, not a setting.</t>
+          <t xml:space="preserve">`is_gate_cleared()` with the pass's `gate_threshold()`: n `len(candidates_of())` — every state the family offers from the beam, cache hits included — or, for the hpo family, the points its studies drew, `trial_count_drawn` summed; a row whose `entry_edge_threshold_constraint_met` is false refused before any comparison; `SELECTION_FOLD_MEASURE` compared fold by fold; without sigma `&gt;` for `forward` and `&gt;=` for `backward`; the barrier and hpo loops labelling every move `forward`; `gate_threshold_multiple()` by quadrature and bisection on fixed constants, one n one k on every machine.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -15017,22 +15017,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-A-MOVE-CLEARS-THE-NOISE-OF-ITS-PASS</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-THE-BEAM-KEEPS-ITS-PARENTS</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">A child clears the gate only where its threshold constraint is met, its fold measure beats its parent's strictly on every validation fold and its path CAGR beats the parent's by more than k(n) times the asset's noise sigma, n the candidates of its pass — for every family, a move that shrinks the state included; a calibration run, whose profile has no sigma, clears a child strictly better on the path CAGR and on every fold, and a move that shrinks the state where it is no worse on either. k(n) is where the best of n candidates carrying independent normal noise of one size would beat an equal parent at `GATE_THRESHOLD_FALSE_EXCEEDANCE_RATE`: a heuristic margin, not a test at that rate.</t>
+          <t xml:space="preserve">Each family leaves the beam the best distinct states, at most `SERPENTINE_SEARCH_BEAM_WIDTH`, among the children that cleared the gate and the parents they came from, ranked by the chained validation path's CAGR, then its Calmar ratio, then its profit factor, then the fewer columns, then the earlier trial; so the champion, the beam's leader moved once at the round's end, never ranks worse than it did.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">`is_gate_cleared()` with the pass's `gate_threshold()`: n `len(candidates_of())` — every state the family offers from the beam, cache hits included — or, for the hpo family, the points its studies drew, `trial_count_drawn` summed; a row whose `entry_edge_threshold_constraint_met` is false refused before any comparison; `SELECTION_FOLD_MEASURE` compared fold by fold; without sigma `&gt;` for `forward` and `&gt;=` for `backward`; the barrier and hpo loops labelling every move `forward`; `gate_threshold_multiple()` by quadrature and bisection on fixed constants, one n one k on every machine.</t>
+          <t xml:space="preserve">`top_beam(children + beam)` after every family, the indices made distinct before the width applies, ordered by `ranking_key()` over `state_objective()` — a path without a losing trade counting as the highest profit factor — then `column_count()` ascending, then the trial index; `champion_trial_index` set to `beam[0]` with the counters at the round's end, trial 1, the start, the champion until a family keeps a move.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -15054,12 +15054,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-THE-BEAM-KEEPS-ITS-PARENTS</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-CONVERGED-MEANS-NO-FAMILY-MOVED-THE-BEAM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Each family leaves the beam the best distinct states, at most `SERPENTINE_SEARCH_BEAM_WIDTH`, among the children that cleared the gate and the parents they came from, ranked by the chained validation path's CAGR, then its Calmar ratio, then its profit factor, then the fewer columns, then the earlier trial; so the champion, the beam's leader moved once at the round's end, never ranks worse than it did.</t>
+          <t xml:space="preserve">The serpentine search is over after a round in which no family of the executed schedule changed the beam: a fixed point of its own schedule, gate and beam, not an optimum — a neighbour better by less than the margin or not on every fold was refused, and a child that cleared the gate but ranked below a full beam was not kept.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -15069,7 +15069,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">`top_beam(children + beam)` after every family, the indices made distinct before the width applies, ordered by `ranking_key()` over `state_objective()` — a path without a losing trade counting as the highest profit factor — then `column_count()` ascending, then the trial index; `champion_trial_index` set to `beam[0]` with the counters at the round's end, trial 1, the start, the champion until a family keeps a move.</t>
+          <t xml:space="preserve">`search_converged = not round_accepted`, `round_accepted` set only where `top_beam()` returned another beam than the one its family started from; a loop the profile's `loops` leave out no part of the executed schedule; a converged state described as the end of this schedule, never as an optimum of the objective.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -15091,22 +15091,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-CONVERGED-MEANS-NO-FAMILY-MOVED-THE-BEAM</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-ONLY-A-CHAMPION-ABOVE-THE-NOISE-IS-PROPOSED</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">The serpentine search is over after a round in which no family of the executed schedule changed the beam: a fixed point of its own schedule, gate and beam, not an optimum — a neighbour better by less than the margin or not on every fold was refused, and a child that cleared the gate but ranked below a full beam was not kept.</t>
+          <t xml:space="preserve">The one proposal is the champion, and only when its threshold constraint is met, it is not the state the serpentine search started from, no validation fold scores it below that start and its path CAGR beats the start's by more than k(N) times the asset's noise sigma, N the sum of `trial_count_by_loop`; a calibration run proposes nothing.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_features/status.py`</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">`search_converged = not round_accepted`, `round_accepted` set only where `top_beam()` returned another beam than the one its family started from; a loop the profile's `loops` leave out no part of the executed schedule; a converged state described as the end of this schedule, never as an optimum of the objective.</t>
+          <t xml:space="preserve">`proposals_block()` at every round boundary returning the champion as proposal 1 under those conditions — the fold condition `&gt;=` on `SELECTION_FOLD_MEASURE` — and an empty list otherwise, and always without a noise sigma; the snapshot publishing the proposals only while `inputs_current` holds.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -15128,22 +15128,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-ONLY-A-CHAMPION-ABOVE-THE-NOISE-IS-PROPOSED</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-A-DRAWN-POINT-IS-COUNTED-ONCE</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">The one proposal is the champion, and only when its threshold constraint is met, it is not the state the serpentine search started from, no validation fold scores it below that start and its path CAGR beats the start's by more than k(N) times the asset's noise sigma, N the sum of `trial_count_by_loop`; a calibration run proposes nothing.</t>
+          <t xml:space="preserve">`trial_count_by_loop`, whose sum is the N of the proposal, counts per loop the ledger's lines after the start and the points the studies drew that did not become lines, so a study's candidate, itself a drawn point, is counted once, as its line; it is written at a round boundary alone and rebuilt from the ledger on resume, so a resumed turn counts what an unbroken one would.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_features/status.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_features/status.py`</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">`proposals_block()` at every round boundary returning the champion as proposal 1 under those conditions — the fold condition `&gt;=` on `SELECTION_FOLD_MEASURE` — and an empty list otherwise, and always without a noise sigma; the snapshot publishing the proposals only while `inputs_current` holds.</t>
+          <t xml:space="preserve">At a round's end the ledger's lines by loop, the start's excluded, plus every round's draws less the lines that round's studies left; at a turn's start the draws still to count rebuilt as the recorded count less the lines of the rounds it covers; `status.serpentine_search_block()` copying `trial_count_by_loop`, never recounting it.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -15165,62 +15165,25 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-A-DRAWN-POINT-IS-COUNTED-ONCE</t>
+          <t xml:space="preserve">SERPENTINE-SEARCH-THE-NOISE-SIGMA-IS-DRAFTED</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">`trial_count_by_loop`, whose sum is the N of the proposal, counts per loop the ledger's lines after the start and the points the studies drew that did not become lines, so a study's candidate, itself a drawn point, is counted once, as its line; it is written at a round boundary alone and rebuilt from the ledger on resume, so a resumed turn counts what an unbroken one would.</t>
+          <t xml:space="preserve">The asset's noise sigma is a number of its profile and so of the serpentine search's inputs: absent on the asset's first searches, the calibration runs, and set by a hand from a decision — estimated by `path_cagr_noise_standard_deviation()` off the ledgers of the asset's calibration searches, never recomputed by a serpentine search.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_features/status.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_features/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">At a round's end the ledger's lines by loop, the start's excluded, plus every round's draws less the lines that round's studies left; at a turn's start the draws still to count rebuilt as the recorded count less the lines of the rounds it covers; `status.serpentine_search_block()` copying `trial_count_by_loop`, never recounting it.</t>
+          <t xml:space="preserve">`path_cagr_noise_standard_deviation` in `&lt;TICKER&gt;_serpentine_search_profile.json`, `null` or a number, read by the turn and carried unchanged by the features terminal's draft; a calibration run's last turn printing the estimate of its own ledger — the median absolute deviation of the path-CAGR differences between each line and its parent, both meeting the threshold constraint and the child fitted on its own, times `NOISE_MEDIAN_ABSOLUTE_DEVIATION_SCALE` over the square root of two.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">none</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">module_features/sub_module_serpentine_search/skill_serpentine_search.md</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Methodology</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SERPENTINE-SEARCH-THE-NOISE-SIGMA-IS-DRAFTED</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The asset's noise sigma is a number of its profile and so of the serpentine search's inputs: absent on the asset's first searches, the calibration runs, and set by a hand from a decision — estimated by `path_cagr_noise_standard_deviation()` off the ledgers of the asset's calibration searches, never recomputed by a serpentine search.</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/**/*.py`, `module_features/sub_module_terminal/terminal.py`</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`path_cagr_noise_standard_deviation` in `&lt;TICKER&gt;_serpentine_search_profile.json`, `null` or a number, read by the turn and carried unchanged by the features terminal's draft; a calibration run's last turn printing the estimate of its own ledger — the median absolute deviation of the path-CAGR differences between each line and its parent, both meeting the threshold constraint and the child fitted on its own, times `NOISE_MEDIAN_ABSOLUTE_DEVIATION_SCALE` over the square root of two.</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
         <is>
           <t xml:space="preserve">none</t>
         </is>

</xml_diff>

<commit_message>
Orient every sub-module by its own README_sub_module_<subject>.md
Five sub-modules had an orientation beside their code and two a section of their
module's, so where a sub-module is explained could not be told from its name. The
serpentine search's part of README_module_features.md moves to
sub_module_serpentine_search/README_sub_module_serpentine_search.md, and the canon
terminal's section of module_skills/README.md to
module_skills/sub_module_terminal/README_sub_module_terminal.md — moved, not rewritten —
each leaving a pointer behind. The grammar row loses "or a section of its module's",
§ The default choice its exception for the canon's terminal, the files matrix marks the
two files as it marks their siblings, and the neutral skills_status.json holds 95 files.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -1335,7 +1335,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">One `README.md` at the root; in each module one `README_module_&lt;name&gt;.md`, its name read off the module's directory, with its § Design rationale; a sub-module oriented by its own `README_sub_module_&lt;subject&gt;.md` or by a section of its module's; none holding or restating a rule, a methodology or the crawler's internals, and no bare `README.md` inside a module.</t>
+          <t xml:space="preserve">One `README.md` at the root; in each module one `README_module_&lt;name&gt;.md`, its name read off the module's directory, with its § Design rationale; every sub-module oriented by its own `README_sub_module_&lt;subject&gt;.md`, beside its code; none holding or restating a rule, a methodology or the crawler's internals, and no bare `README.md` inside a module.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -9078,7 +9078,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module: a nesting inside the module, or the canon, that owns it — its own `config.py`, an action module with `main()` for each action of a hand, `tui.py` where it draws a terminal, its orientation beside it or in its module's; no part in the chain's dataflow, a hand's research outside the chain at most, whose promotion writes files the chain reads</t>
+          <t xml:space="preserve">a sub-module: a nesting inside the module, or the canon, that owns it — its own `config.py`, an action module with `main()` for each action of a hand, `tui.py` where it draws a terminal, its orientation `README_sub_module_&lt;subject&gt;.md` beside it; no part in the chain's dataflow, a hand's research outside the chain at most, whose promotion writes files the chain reads</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -12292,12 +12292,12 @@
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`</t>
+          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill</t>
+          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
         </is>
       </c>
     </row>
@@ -18149,35 +18149,15 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_features/sub_module_serpentine_search/*.py</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
+          <t xml:space="preserve">module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18186,15 +18166,35 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_features/sub_module_terminal/README_sub_module_terminal.md</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
+          <t xml:space="preserve">module_features/sub_module_serpentine_search/*.py</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18203,20 +18203,15 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_features/sub_module_terminal/*.py</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
+          <t xml:space="preserve">module_features/sub_module_terminal/README_sub_module_terminal.md</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18225,10 +18220,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_features/sub_module_terminal/config.py</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
+          <t xml:space="preserve">module_features/sub_module_terminal/*.py</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18237,15 +18242,10 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_features/sub_module_terminal/terminal.py</t>
+          <t xml:space="preserve">module_features/sub_module_terminal/config.py</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18254,10 +18254,15 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_features/sub_module_terminal/tui.py</t>
+          <t xml:space="preserve">module_features/sub_module_terminal/terminal.py</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18266,20 +18271,10 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_ml/README_module_ml.md</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
+          <t xml:space="preserve">module_features/sub_module_terminal/tui.py</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18288,10 +18283,10 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_ml/*.py</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
+          <t xml:space="preserve">module_ml/README_module_ml.md</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18302,21 +18297,6 @@
         </is>
       </c>
       <c r="G46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="P46" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18325,10 +18305,35 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_ml/score.py</t>
-        </is>
-      </c>
-      <c r="O47" t="inlineStr">
+          <t xml:space="preserve">module_ml/*.py</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18337,15 +18342,10 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_ml/sub_module_terminal/README_sub_module_terminal.md</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
+          <t xml:space="preserve">module_ml/score.py</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18354,20 +18354,15 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_ml/sub_module_terminal/*.py</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
+          <t xml:space="preserve">module_ml/sub_module_terminal/README_sub_module_terminal.md</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18376,10 +18371,20 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_ml/sub_module_terminal/config.py</t>
-        </is>
-      </c>
-      <c r="K50" t="inlineStr">
+          <t xml:space="preserve">module_ml/sub_module_terminal/*.py</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18388,7 +18393,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_ml/sub_module_terminal/terminal.py</t>
+          <t xml:space="preserve">module_ml/sub_module_terminal/config.py</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -18400,7 +18405,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_ml/sub_module_terminal/tui.py</t>
+          <t xml:space="preserve">module_ml/sub_module_terminal/terminal.py</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -18412,20 +18417,10 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/README_module_monitoring.md</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
+          <t xml:space="preserve">module_ml/sub_module_terminal/tui.py</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18434,30 +18429,20 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/*.py</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
+          <t xml:space="preserve">module_monitoring/README_module_monitoring.md</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="Q54" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18466,10 +18451,25 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/*.js</t>
+          <t xml:space="preserve">module_monitoring/*.py</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18483,7 +18483,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/*.html</t>
+          <t xml:space="preserve">module_monitoring/*.js</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -18500,7 +18500,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/*.css</t>
+          <t xml:space="preserve">module_monitoring/*.html</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -18517,15 +18517,15 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/sub_module_terminal/README_sub_module_terminal.md</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
+          <t xml:space="preserve">module_monitoring/*.css</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="Q58" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18534,20 +18534,15 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/sub_module_terminal/*.py</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
+          <t xml:space="preserve">module_monitoring/sub_module_terminal/README_sub_module_terminal.md</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18556,10 +18551,20 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/sub_module_terminal/config.py</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
+          <t xml:space="preserve">module_monitoring/sub_module_terminal/*.py</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18568,7 +18573,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/sub_module_terminal/terminal.py</t>
+          <t xml:space="preserve">module_monitoring/sub_module_terminal/config.py</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -18580,7 +18585,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_monitoring/sub_module_terminal/tui.py</t>
+          <t xml:space="preserve">module_monitoring/sub_module_terminal/terminal.py</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -18592,20 +18597,10 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/README.md</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
+          <t xml:space="preserve">module_monitoring/sub_module_terminal/tui.py</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18614,10 +18609,10 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/*.py</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
+          <t xml:space="preserve">module_skills/README.md</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18627,7 +18622,7 @@
           <t xml:space="preserve">X</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="G64" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18636,15 +18631,20 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sheet.py</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
+          <t xml:space="preserve">module_skills/*.py</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="F65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18653,10 +18653,15 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sync.py</t>
+          <t xml:space="preserve">module_skills/sheet.py</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18665,15 +18670,10 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md</t>
+          <t xml:space="preserve">module_skills/sync.py</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18682,20 +18682,15 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/*.py</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
+          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18704,10 +18699,20 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/config.py</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
+          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/*.py</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18716,17 +18721,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/crawl.py</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
+          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/config.py</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -18738,10 +18733,15 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/status.py</t>
+          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/crawl.py</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18755,15 +18755,10 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/crawlers_mission.md</t>
+          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/status.py</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18777,7 +18772,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/vendors_for_crawling.toml</t>
+          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/crawlers_mission.md</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -18794,20 +18794,15 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_terminal/*.py</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
+          <t xml:space="preserve">module_skills/sub_module_scalability_crawler/vendors_for_crawling.toml</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t xml:space="preserve">X</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
+      <c r="L74" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18816,10 +18811,15 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_terminal/config.py</t>
-        </is>
-      </c>
-      <c r="K75" t="inlineStr">
+          <t xml:space="preserve">module_skills/sub_module_terminal/README_sub_module_terminal.md</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18828,10 +18828,20 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">module_skills/sub_module_terminal/terminal.py</t>
-        </is>
-      </c>
-      <c r="K76" t="inlineStr">
+          <t xml:space="preserve">module_skills/sub_module_terminal/*.py</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>
@@ -18840,10 +18850,34 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t xml:space="preserve">module_skills/sub_module_terminal/config.py</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">module_skills/sub_module_terminal/terminal.py</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t xml:space="preserve">module_skills/sub_module_terminal/tui.py</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr">
+      <c r="K79" t="inlineStr">
         <is>
           <t xml:space="preserve">X</t>
         </is>

</xml_diff>

<commit_message>
Seed a search study by its round, and walk Y again only when the label's geometry moves
Every study of the serpentine search drew with SEED, so each round's study of a parent
that stayed in the beam repeated the same trials, and the round's own study repeated the
chain's startup points on the same X and Y. The chain's study keeps SEED; a search study
takes SEED plus its round, so a surviving parent draws new points, and the search ends on
a round in which no family moved the beam — the end of its schedule, no longer a fixed
point. The docstring that said the parent's own point stops after one fold now says why
it can never be offered. score.xy_for_state compared all four barrier coordinates, so a
move of the trade's exit alone walked Y down the 1m path again for the same labels; it
compares the label's two coordinates, as fit_identity already does, and no byte changes.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -1702,7 +1702,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">The serpentine search is over after a round in which no family of the executed schedule changed the beam: a fixed point of its own schedule, gate and beam, not an optimum — a neighbour better on the path but not on every fold was refused, and a child that cleared the gate but ranked below a full beam was not kept.</t>
+          <t xml:space="preserve">The serpentine search is over after a round in which no family of the executed schedule changed the beam: the end of its own schedule and gate, not an optimum and not a fixed point, a study of the next round drawing new points — a neighbour better on the path but not on every fold was refused, and a child that cleared the gate but ranked below a full beam was not kept.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">`hpo.search_hyperparameters()` creating a fresh seeded study with no enqueued trial and reading no parameters file; a best point equal to the parent's own offered as no move.</t>
+          <t xml:space="preserve">`hpo.search_hyperparameters()` creating a fresh seeded study with no enqueued trial and reading no parameters file; the parent's own point never offered, no threshold beating the parent on every fold at it.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">One fixed seed, the record `SEED`, in every study's sampler and every fit, and every study optimised with `n_jobs=1`.</t>
+          <t xml:space="preserve">The record `SEED` in every fit and in the chain's study, `SEED` plus the round in a study of the serpentine search, and every study optimised with `n_jobs=1`.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">One one-off container per asset — the Makefile's `fanout` and the serpentine search's loop — the processes side by side, each under the same `SEED` and the same caps.</t>
+          <t xml:space="preserve">One one-off container per asset — the Makefile's `fanout` and the serpentine search's loop — the processes side by side, each under the same seeds and the same caps.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -11286,7 +11286,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t xml:space="preserve">the convergence — a round in which no family of the executed schedule changed the beam, after which the serpentine search is over: a fixed point of its own schedule and gate, not an optimum</t>
+          <t xml:space="preserve">the convergence — a round in which no family of the executed schedule changed the beam, after which the serpentine search is over: the end of its own schedule and gate, not an optimum</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -17346,7 +17346,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two runs of the same experiment give the same bits — for the same code, the same frozen input window and the same execution environment, never a byte-identical rebuild of that environment at an arbitrary future date: thread caps at one, one fixed seed, pinned orders and a sort before every write, and speed only from processes side by side. *The repository shows the destination, not the road*: bit parity is the proof, and no test suite stands in for it.</t>
+          <t xml:space="preserve">Two runs of the same experiment give the same bits — for the same code, the same frozen input window and the same execution environment, never a byte-identical rebuild of that environment at an arbitrary future date: thread caps at one, fixed seeds, pinned orders and a sort before every write, and speed only from processes side by side. *The repository shows the destination, not the road*: bit parity is the proof, and no test suite stands in for it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Promote the proposal's whole state, and start the chain's study from its point
The promotion writes <TICKER>_hyperparameter_point.json beside the feature set and
the barriers, and calls a state unchanged only when its columns, its geometry and
its point are all the active ones. ml-hpo enqueues the promoted point as its
study's first trial: on the promoted state's own X and Y, with the same fits and
the same threshold rule, that trial scores the proposal's path CAGR, so the point
the chain keeps is worth at least that. A hyper-parameter move of the search is no
longer lost at the promotion. The rule that no study is handed a starting point
names this one exception; the README of an asset lists the third file of a hand's
stage.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">A proposal becomes an asset's feature set and barrier geometry by a hand's act alone, never because the serpentine search finished; the promotion copies the proposal's columns and geometry, and the asset's ML chain then tunes it anew.</t>
+          <t xml:space="preserve">A proposal becomes an asset's state — its feature set, its barrier geometry and its hyper-parameter point — by a hand's act alone, never because the serpentine search finished; the promotion copies the whole state, and the asset's ML chain then tunes it anew from its point.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json` and `&lt;TICKER&gt;_barriers.json` written by `promote.py` alone, from the one proposal of the asset's search, by `make features-serpentine-search-promote ASSET=&lt;TICKER&gt;`, then `ml-all` for that asset; no rank and no choice among proposals, a search holding one at most; a search that proposes none refused in one line, before either file is written; never the proposal's `best_params`; the active state promoted again writing nothing; a converged serpentine search writing neither file.</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json`, `&lt;TICKER&gt;_barriers.json` and `&lt;TICKER&gt;_hyperparameter_point.json` written by `promote.py` alone, from the one proposal of the asset's search, by `make features-serpentine-search-promote ASSET=&lt;TICKER&gt;`, then `ml-all` for that asset, whose study takes the promoted point as its first trial; no rank and no choice among proposals, a search holding one at most; a search that proposes none refused in one line, before any file is written; the active state — its columns, its geometry and the point of `&lt;TICKER&gt;_parameters.json` — promoted again writing nothing; a converged serpentine search writing none of the three.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.gitignore` admitting `store/assets_artifacts/ticker=*/*_serpentine_search.json`, `*_serpentine_search_trials.jsonl`, `*_serpentine_search_profile.json`, `*_feature_set.json` and `*_barriers.json` among the files of the asset's folder, leaving `*_score_request.json` and `*_score_response.json` ignored, and ignoring the trials store whole; each of these files built by a descriptor of the sub-module's `config.py` under `artifact_dir()`.</t>
+          <t xml:space="preserve">`.gitignore` admitting `store/assets_artifacts/ticker=*/*_serpentine_search.json`, `*_serpentine_search_trials.jsonl`, `*_serpentine_search_profile.json`, `*_feature_set.json`, `*_barriers.json` and `*_hyperparameter_point.json` among the files of the asset's folder, leaving `*_score_request.json` and `*_score_response.json` ignored, and ignoring the trials store whole; each of these files built by a descriptor of the sub-module's `config.py` under `artifact_dir()`.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2533,12 +2533,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">`hpo.search_hyperparameters()` creating a fresh seeded study with no enqueued trial and reading no parameters file; the parent's own point never offered, no threshold beating the parent on every fold at it.</t>
+          <t xml:space="preserve">`hpo.search_hyperparameters()` creating a fresh seeded study, enqueuing no trial but the `first_point` it is handed, and reading no parameters file; the parent's own point never offered, no threshold beating the parent on every fold at it.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t xml:space="preserve">none</t>
+          <t xml:space="preserve">The chain's study of an asset a hand has promoted: `hpo.main()` hands it the `best_params` of `&lt;TICKER&gt;_hyperparameter_point.json` as its first trial — a drafted file, so `&lt;TICKER&gt;_parameters.json` still never depends on its own last value.</t>
         </is>
       </c>
     </row>
@@ -10853,7 +10853,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t xml:space="preserve">HPO — the search for model hyper-parameters, and the stage that runs it: a function of X, Y and the frozen constants, drawing no point to start from</t>
+          <t xml:space="preserve">HPO — the search for model hyper-parameters, and the stage that runs it: a function of X, Y, the frozen constants and the point a hand promoted, its first trial when there is one</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -11318,7 +11318,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion — a hand's copy of one proposal's columns and barrier geometry into the asset's own state, followed by its ML chain, which tunes it again: its realised result differs from the search's, and the same proposal twice changes nothing</t>
+          <t xml:space="preserve">the promotion — a hand's copy of one proposal's whole state — its columns, its barrier geometry and its hyper-parameter point — into the asset's own, followed by its ML chain, whose study starts from that point, so the point it keeps is worth at least the proposal's path CAGR; the same proposal twice changes nothing</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -11328,7 +11328,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json` with `columns_by_timeframe` and `&lt;TICKER&gt;_barriers.json` with the four of `BARRIER_COORDINATE_NAMES`, and nothing else</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json` with `columns_by_timeframe`, `&lt;TICKER&gt;_barriers.json` with the four of `BARRIER_COORDINATE_NAMES` and `&lt;TICKER&gt;_hyperparameter_point.json` with `best_params`, and nothing else</t>
         </is>
       </c>
       <c r="E217" t="inlineStr">
@@ -11338,7 +11338,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t xml:space="preserve">apply, activate, deploy; a promotion of the whole basket; a counter or a rank in the file — git holds the history; a rank on the make line or the command line, a search holding one proposal at most</t>
+          <t xml:space="preserve">apply, activate, deploy; a promotion of the whole basket; a counter or a rank in the file — git holds the history; a rank on the make line or the command line, a search holding one proposal at most; a part of the state left behind</t>
         </is>
       </c>
     </row>
@@ -12854,7 +12854,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t xml:space="preserve">its tracked remnant: `&lt;TICKER&gt;_README.md`, `&lt;TICKER&gt;_parameters.json` and, once written, `&lt;TICKER&gt;_serpentine_search_profile.json`, `&lt;TICKER&gt;_serpentine_search.json`, `&lt;TICKER&gt;_serpentine_search_trials.jsonl`, `&lt;TICKER&gt;_feature_set.json`, `&lt;TICKER&gt;_barriers.json`; every other file the chain rebuilds</t>
+          <t xml:space="preserve">its tracked remnant: `&lt;TICKER&gt;_README.md`, `&lt;TICKER&gt;_parameters.json` and, once written, `&lt;TICKER&gt;_serpentine_search_profile.json`, `&lt;TICKER&gt;_serpentine_search.json`, `&lt;TICKER&gt;_serpentine_search_trials.jsonl`, `&lt;TICKER&gt;_feature_set.json`, `&lt;TICKER&gt;_barriers.json`, `&lt;TICKER&gt;_hyperparameter_point.json`; every other file the chain rebuilds</t>
         </is>
       </c>
     </row>
@@ -13815,7 +13815,7 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_set_json()`, `barriers_json()` — equal by value</t>
+          <t xml:space="preserve">`feature_set_json()`, `barriers_json()`, `hyperparameter_point_json()` — equal by value</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion writes the two, the ML chain and the serpentine search read them, and the features terminal names them on its promotion screen; the writer and the reader of a boundary must name one artifact, and the terminal cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the promotion writes the three, the ML chain reads them and the serpentine search the first two, and the features terminal names them on its promotion screen; the writer and the reader of a boundary must name one artifact, and the terminal cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -14687,7 +14687,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/status.py` writes it, `asset_readme_md()`; its file list `file_manifest()`, the two files of `HAND_STAGE_FILE_DESCRIPTORS` listed with no size</t>
+          <t xml:space="preserve">`module_ml/status.py` writes it, `asset_readme_md()`; its file list `file_manifest()`, the three files of `HAND_STAGE_FILE_DESCRIPTORS` listed with no size</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -14770,17 +14770,17 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_model_evaluation.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_hyperparameter_point.json`</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/train.py` writes it; `model_evaluation_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `hyperparameter_point_json()`; `hpo.main()` in `module_ml/hpo.py` reads it</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`validation` — a `fold_&lt;id&gt;` per fold of `VALIDATION_FOLD_IDS` — and `final_holdout`, each `prior_logloss`, `model_logloss`, `relative_logloss_skill`, `scored_row_count`; `validation_importance`, a `fold_&lt;id&gt;` per validation fold, each `gain_importance` and `mean_abs_shap_importance` per column; `feature_columns`; `class_counts`, `labels`, `segments`; untracked</t>
+          <t xml:space="preserve">`best_params` — the promoted hyper-parameter point, a hand's choice: the first trial of the chain's study, and nothing else; absent, the study draws every point; tracked once promoted, like the feature set and the geometry beside it</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_parameters.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_model_evaluation.json`</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/hpo.py` writes it; `parameters_json()`</t>
+          <t xml:space="preserve">`module_ml/train.py` writes it; `model_evaluation_json()`</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`hyperparameter_search_result` (`best_params`, `best_cagr_validation_path`, `trial_count`); tracked</t>
+          <t xml:space="preserve">`validation` — a `fold_&lt;id&gt;` per fold of `VALIDATION_FOLD_IDS` — and `final_holdout`, each `prior_logloss`, `model_logloss`, `relative_logloss_skill`, `scored_row_count`; `validation_importance`, a `fold_&lt;id&gt;` per validation fold, each `gain_importance` and `mean_abs_shap_importance` per column; `feature_columns`; `class_counts`, `labels`, `segments`; untracked</t>
         </is>
       </c>
     </row>
@@ -14814,27 +14814,17 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_score_request.json`: the serpentine search's question</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_parameters.json`</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_request_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by a turn, `features-serpentine-turn`, read by `module_ml.score`, `ml-score`; the one file the loop of `features-serpentine-search` tests, running `ml-score` and a turn again while it exists</t>
-        </is>
-      </c>
-      <c r="D355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`kind` (`score` or `hpo`), `round`, `states`</t>
-        </is>
-      </c>
-      <c r="F355" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a key beside these three; a request the evaluator writes; a second file the loop tests</t>
+          <t xml:space="preserve">`module_ml/hpo.py` writes it; `parameters_json()`</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t xml:space="preserve">what one family pass asks to be scored: the kind of scoring, the round it runs in, and the states — a state of its own for `score`, a beam parent's scored row for `hpo`; untracked</t>
+          <t xml:space="preserve">`hyperparameter_search_result` (`best_params`, `best_cagr_validation_path`, `trial_count`); tracked</t>
         </is>
       </c>
     </row>
@@ -14846,27 +14836,27 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_score_response.json`: the serpentine search's answer</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_score_request.json`: the serpentine search's question</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_response_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by `module_ml.score` alone</t>
+          <t xml:space="preserve">`score_request_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by a turn, `features-serpentine-turn`, read by `module_ml.score`, `ml-score`; the one file the loop of `features-serpentine-search` tests, running `ml-score` and a turn again while it exists</t>
         </is>
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`kind`, `round`, `results`; a `score` result the row of one scored state of the serpentine search, an `hpo` result `state_key`, `trial_count_drawn` and `candidate`</t>
+          <t xml:space="preserve">`kind` (`score` or `hpo`), `round`, `states`</t>
         </is>
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t xml:space="preserve">a key beside these three; a result out of the order the request named; a response written before every state has one</t>
+          <t xml:space="preserve">a key beside these three; a request the evaluator writes; a second file the loop tests</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t xml:space="preserve">what the states of one request are worth, in the order the request named them; `candidate` a scored row or `null`, and `null` is an answer; untracked</t>
+          <t xml:space="preserve">what one family pass asks to be scored: the kind of scoring, the round it runs in, and the states — a state of its own for `score`, a beam parent's scored row for `hpo`; untracked</t>
         </is>
       </c>
     </row>
@@ -14878,17 +14868,27 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_score_response.json`: the serpentine search's answer</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_json()`</t>
+          <t xml:space="preserve">`score_response_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by `module_ml.score` alone</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`kind`, `round`, `results`; a `score` result the row of one scored state of the serpentine search, an `hpo` result `state_key`, `trial_count_drawn` and `candidate`</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a key beside these three; a result out of the order the request named; a response written before every state has one</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs`, `beam`, `champion_trial_index`, `round_count`, `search_converged`, `path` (each `round`, `loop`, `family`, `trial_index`, `beam`, `move`), `proposals` (each `proposal`, `trial_index`), `trial_count_by_loop` — where the search stands at a round boundary, naming trials by index and carrying none of their columns; tracked once a search has run</t>
+          <t xml:space="preserve">what the states of one request are worth, in the order the request named them; `candidate` a scored row or `null`, and `null` is an answer; untracked</t>
         </is>
       </c>
     </row>
@@ -14900,17 +14900,17 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search.json`</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hand, in the file or through the features terminal's draft; `serpentine_search_profile_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_json()`</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`columns_admitted_by_timeframe`, `start_columns_by_timeframe` (`null` = the asset's own set), `grid_by_coordinate` (one list per coordinate, in the order it is searched), `loops` (a subset of `SERPENTINE_SEARCH_ROUND_LOOPS`), `path_cagr_noise_standard_deviation` (the asset's noise sigma, `null` on the calibration run) — what a hand asks the serpentine search to look at; drafted, never derived, and tracked</t>
+          <t xml:space="preserve">`inputs`, `beam`, `champion_trial_index`, `round_count`, `search_converged`, `path` (each `round`, `loop`, `family`, `trial_index`, `beam`, `move`), `proposals` (each `proposal`, `trial_index`), `trial_count_by_loop` — where the search stands at a round boundary, naming trials by index and carrying none of their columns; tracked once a search has run</t>
         </is>
       </c>
     </row>
@@ -14922,17 +14922,17 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_trials.jsonl`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_trials_jsonl()`</t>
+          <t xml:space="preserve">a hand, in the file or through the features terminal's draft; `serpentine_search_profile_json()`</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t xml:space="preserve">one scored state of the serpentine search a line, appended and never rewritten; `trial_index` = the line number, counted from one; tracked once a search has run</t>
+          <t xml:space="preserve">`columns_admitted_by_timeframe`, `start_columns_by_timeframe` (`null` = the asset's own set), `grid_by_coordinate` (one list per coordinate, in the order it is searched), `loops` (a subset of `SERPENTINE_SEARCH_ROUND_LOOPS`), `path_cagr_noise_standard_deviation` (the asset's noise sigma, `null` on the calibration run) — what a hand asks the serpentine search to look at; drafted, never derived, and tracked</t>
         </is>
       </c>
     </row>
@@ -14944,49 +14944,39 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_strategy_evaluation.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_trials.jsonl`</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/strategy.py` writes it; `strategy_evaluation_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_trials_jsonl()`</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `cleared_point_count`, `median_cagr_over_cleared`, `max_cagr_over_cleared`, `selection_score_cagr_validation_path`, `execution_cost_rate_per_trade_side`; per fold `sharpe`, `cagr`, `max_drawdown`, `calmar`, `profit_factor`, `trade_count`, `hit_rate`, `average_trade_return`, `exposure`, `exit_counts`, `final_equity`; `validation_path` over the validation folds; the final holdout's `equity_curve`; untracked</t>
+          <t xml:space="preserve">one scored state of the serpentine search a line, appended and never rewritten; `trial_index` = the line number, counted from one; tracked once a search has run</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Features</t>
+          <t xml:space="preserve">Artifacts</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t xml:space="preserve">a series of one timeframe's bars, with no parameter</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_strategy_evaluation.json`</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`open`, `high`, `low`, `close`, `volume` — a bar column — and the series with a kernel: `logarithmic_volume`, `true_range`, `cumulative_signed_volume`; `SERIES_KERNELS`, `module_features/indicators.py`</t>
-        </is>
-      </c>
-      <c r="D361" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`inputs` of a term</t>
-        </is>
-      </c>
-      <c r="E361" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the series token</t>
-        </is>
-      </c>
-      <c r="F361" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a series with a parameter; `log_volume`</t>
+          <t xml:space="preserve">`module_ml/strategy.py` writes it; `strategy_evaluation_json()`</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `cleared_point_count`, `median_cagr_over_cleared`, `max_cagr_over_cleared`, `selection_score_cagr_validation_path`, `execution_cost_rate_per_trade_side`; per fold `sharpe`, `cagr`, `max_drawdown`, `calmar`, `profit_factor`, `trade_count`, `hit_rate`, `average_trade_return`, `exposure`, `exit_counts`, `final_equity`; `validation_path` over the validation folds; the final holdout's `equity_curve`; untracked</t>
         </is>
       </c>
     </row>
@@ -14998,32 +14988,27 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t xml:space="preserve">an indicator — one computation with exactly one integer parameter, named by its token, its invariants one record of the register beside its kernel, the popular names it answers to among them</t>
+          <t xml:space="preserve">a series of one timeframe's bars, with no parameter</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t xml:space="preserve">`exponential_smoothing&lt;n&gt;`, `rolling_mean&lt;n&gt;`, `recursive_mean&lt;n&gt;`, `recursive_mean_gain_share&lt;n&gt;`, `rolling_standard_score&lt;n&gt;`, `rolling_range_position&lt;n&gt;`, `rolling_standard_deviation&lt;n&gt;`, `relative_change&lt;n&gt;`, `recursive_mean_upward_movement_share&lt;n&gt;`, `recursive_mean_directional_movement_imbalance&lt;n&gt;`, `rolling_volume_weighted_mean&lt;n&gt;`, `rolling_volume_weighted_close_location&lt;n&gt;`, `rolling_money_flow_gain_share&lt;n&gt;`; `INDICATORS` — `kernel`, `parameter_word`, `warmup_multiple`, `inputs`, `output_range`, `historical_aliases` of a record, `module_features/indicators.py`</t>
+          <t xml:space="preserve">`open`, `high`, `low`, `close`, `volume` — a bar column — and the series with a kernel: `logarithmic_volume`, `true_range`, `cumulative_signed_volume`; `SERIES_KERNELS`, `module_features/indicators.py`</t>
         </is>
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t xml:space="preserve">`indicator`, `parameter_word`, `parameter_bars`, `output_range`, `historical_aliases` of a term</t>
+          <t xml:space="preserve">`inputs` of a term</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t xml:space="preserve">the token with its parameter, `&lt;PARAMETER_WORD&gt; &lt;n&gt; bars of &lt;inputs&gt;` beside it and `output &lt;low&gt;–&lt;high&gt;` when the indicator is bounded (the catalogue table's terms)</t>
+          <t xml:space="preserve">the series token</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t xml:space="preserve">`rsi_14`, `sma_200`, `bb20`; a table of indicator facts in `config.py` beside the register; `kernel` for anything but the function a record computes with; the abbreviations these tokens replaced: `ema`, `sma`, `rsi`, `atr`, `zscore`, `rolling_zscore`, `wilder_smoothing`, `range_position`</t>
-        </is>
-      </c>
-      <c r="I362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
+          <t xml:space="preserve">a series with a parameter; `log_volume`</t>
         </is>
       </c>
     </row>
@@ -15035,27 +15020,32 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t xml:space="preserve">a term — a series or an indicator inside a feature definition</t>
+          <t xml:space="preserve">an indicator — one computation with exactly one integer parameter, named by its token, its invariants one record of the register beside its kernel, the popular names it answers to among them</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`("&lt;indicator&gt;", &lt;parameter_bars&gt;)` on the default series close, `("&lt;series&gt;", "&lt;indicator&gt;", &lt;parameter_bars&gt;)` on another series, `("&lt;series&gt;",)` a bare series; `term_name()`</t>
+          <t xml:space="preserve">`exponential_smoothing&lt;n&gt;`, `rolling_mean&lt;n&gt;`, `recursive_mean&lt;n&gt;`, `recursive_mean_gain_share&lt;n&gt;`, `rolling_standard_score&lt;n&gt;`, `rolling_range_position&lt;n&gt;`, `rolling_standard_deviation&lt;n&gt;`, `relative_change&lt;n&gt;`, `recursive_mean_upward_movement_share&lt;n&gt;`, `recursive_mean_directional_movement_imbalance&lt;n&gt;`, `rolling_volume_weighted_mean&lt;n&gt;`, `rolling_volume_weighted_close_location&lt;n&gt;`, `rolling_money_flow_gain_share&lt;n&gt;`; `INDICATORS` — `kernel`, `parameter_word`, `warmup_multiple`, `inputs`, `output_range`, `historical_aliases` of a record, `module_features/indicators.py`</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`terms`</t>
+          <t xml:space="preserve">`indicator`, `parameter_word`, `parameter_bars`, `output_range`, `historical_aliases` of a term</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">terms</t>
+          <t xml:space="preserve">the token with its parameter, `&lt;PARAMETER_WORD&gt; &lt;n&gt; bars of &lt;inputs&gt;` beside it and `output &lt;low&gt;–&lt;high&gt;` when the indicator is bounded (the catalogue table's terms)</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">atom</t>
+          <t xml:space="preserve">`rsi_14`, `sma_200`, `bb20`; a table of indicator facts in `config.py` beside the register; `kernel` for anything but the function a record computes with; the abbreviations these tokens replaced: `ema`, `sma`, `rsi`, `atr`, `zscore`, `rolling_zscore`, `wilder_smoothing`, `range_position`</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
         </is>
       </c>
     </row>
@@ -15067,32 +15057,27 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t xml:space="preserve">a feature definition — terms of one timeframe composed by the operators, with an optional normaliser; the timeframe-less half of a feature, carrying the tier it belongs to and the popular names that denote the whole of it</t>
+          <t xml:space="preserve">a term — a series or an indicator inside a feature definition</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t xml:space="preserve">one record of `FEATURE_CATALOGUE`; `feature_definition_name()`; `OPERATORS` = {`minus`, `over`} and `NORMALISERS` = {`centered`}, one record per token beside its kernel in `module_features/catalogue.py`</t>
+          <t xml:space="preserve">`("&lt;indicator&gt;", &lt;parameter_bars&gt;)` on the default series close, `("&lt;series&gt;", "&lt;indicator&gt;", &lt;parameter_bars&gt;)` on another series, `("&lt;series&gt;",)` a bare series; `term_name()`</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_definition`, `tier` = `CORE` / `EXTENDED` / `COMPOSITE`, `historical_aliases`</t>
+          <t xml:space="preserve">`terms`</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">definition (the catalogue table)</t>
+          <t xml:space="preserve">terms</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t xml:space="preserve">molecule, family, feature family, indicator (for a composite); `trend`, `momentum`, `volatility`, `structure`, `activity` — a category, not a computation; a popular name as the key, the column or a second name beside the canonical one; a tier written anywhere but the record; `centred` — the normaliser token keeps its American spelling, a column and a key on disk</t>
-        </is>
-      </c>
-      <c r="I364" t="inlineStr">
-        <is>
-          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
+          <t xml:space="preserve">atom</t>
         </is>
       </c>
     </row>
@@ -15104,27 +15089,32 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t xml:space="preserve">a feature — a definition aligned to the decision grid on one timeframe; the column of X and the key of an importance</t>
+          <t xml:space="preserve">a feature definition — terms of one timeframe composed by the operators, with an optional normaliser; the timeframe-less half of a feature, carrying the tier it belongs to and the popular names that denote the whole of it</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_id()` = `&lt;definition&gt;_&lt;timeframe&gt;`</t>
+          <t xml:space="preserve">one record of `FEATURE_CATALOGUE`; `feature_definition_name()`; `OPERATORS` = {`minus`, `over`} and `NORMALISERS` = {`centered`}, one record per token beside its kernel in `module_features/catalogue.py`</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_columns`, the keys of an importance</t>
+          <t xml:space="preserve">`feature_definition`, `tier` = `CORE` / `EXTENDED` / `COMPOSITE`, `historical_aliases`</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature id — `column &lt;timeframe&gt;` in the FEATURE SET frame</t>
+          <t xml:space="preserve">definition (the catalogue table)</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
+          <t xml:space="preserve">molecule, family, feature family, indicator (for a composite); `trend`, `momentum`, `volatility`, `structure`, `activity` — a category, not a computation; a popular name as the key, the column or a second name beside the canonical one; a tier written anywhere but the record; `centred` — the normaliser token keeps its American spelling, a column and a key on disk</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
         </is>
       </c>
     </row>
@@ -15136,27 +15126,27 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature catalogue — every definition the repository can compute, with the timeframes it is offered on; drafted, like the rest of `config.py`</t>
+          <t xml:space="preserve">a feature — a definition aligned to the decision grid on one timeframe; the column of X and the key of an importance</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t xml:space="preserve">`FEATURE_CATALOGUE`, `catalogue_columns()`, `CATALOGUE_COLUMNS`; the stage `features-catalogue`, `module_features/catalogue.py`</t>
+          <t xml:space="preserve">`feature_id()` = `&lt;definition&gt;_&lt;timeframe&gt;`</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue` (of `features_status.json`); `&lt;TICKER&gt;_catalogue.json`; the family `catalogue`</t>
+          <t xml:space="preserve">`feature_columns`, the keys of an importance</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t xml:space="preserve">CATALOGUE</t>
+          <t xml:space="preserve">the feature id — `column &lt;timeframe&gt;` in the FEATURE SET frame</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t xml:space="preserve">palette, feature list, feature store</t>
+          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
         </is>
       </c>
     </row>
@@ -15168,22 +15158,27 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature layer's contract, per asset — what the ML layer reads instead of this module's configuration</t>
+          <t xml:space="preserve">the feature catalogue — every definition the repository can compute, with the timeframes it is offered on; drafted, like the rest of `config.py`</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue_contract()`, `catalogue_json()` in `module_features/config.py`; the descriptor's copy in `module_ml/config.py`; `load_catalogue()` in `module_ml/dataset.py`, `cat`</t>
+          <t xml:space="preserve">`FEATURE_CATALOGUE`, `catalogue_columns()`, `CATALOGUE_COLUMNS`; the stage `features-catalogue`, `module_features/catalogue.py`</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`: `decision_timeframe`, `timeframes` (`timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe`</t>
+          <t xml:space="preserve">`catalogue` (of `features_status.json`); `&lt;TICKER&gt;_catalogue.json`; the family `catalogue`</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CATALOGUE</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t xml:space="preserve">an import of `module_features` from `module_ml`; a token or a slot parsed in the ML layer; a second read of the file inside one stage; a path built from the slot grammar outside `module_features`; a parquet named in the contract by anything but its path relative to the artifact store</t>
+          <t xml:space="preserve">palette, feature list, feature store</t>
         </is>
       </c>
     </row>
@@ -15195,27 +15190,22 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t xml:space="preserve">the effective history — what a parameter covers on a timeframe, `bars × timeframe`, the quantity the nesting rule compares</t>
+          <t xml:space="preserve">the feature layer's contract, per asset — what the ML layer reads instead of this module's configuration</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t xml:space="preserve">`definition_effective_history_hours()`</t>
+          <t xml:space="preserve">`catalogue_contract()`, `catalogue_json()` in `module_features/config.py`; the descriptor's copy in `module_ml/config.py`; `load_catalogue()` in `module_ml/dataset.py`, `cat`</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t xml:space="preserve">`effective_history_hours_by_timeframe`; `lower_longest_effective_history_hours`, `upper_shortest_effective_history_hours` of `nesting`</t>
-        </is>
-      </c>
-      <c r="E368" t="inlineStr">
-        <is>
-          <t xml:space="preserve">effective history</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`: `decision_timeframe`, `timeframes` (`timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe`</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t xml:space="preserve">history (bare — a recursion has no window), span (the parameter word of an exponential smoothing), lookback hours</t>
+          <t xml:space="preserve">an import of `module_features` from `module_ml`; a token or a slot parsed in the ML layer; a second read of the file inside one stage; a path built from the slot grammar outside `module_features`; a parquet named in the contract by anything but its path relative to the artifact store</t>
         </is>
       </c>
     </row>
@@ -15227,22 +15217,27 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t xml:space="preserve">the Bollinger %b reading — the trade's %b(20, 2σ), `rolling_standard_score20` / 4 + 0.5, an affine map a tree model is invariant to, so no %b column exists</t>
+          <t xml:space="preserve">the effective history — what a parameter covers on a timeframe, `bars × timeframe`, the quantity the nesting rule compares</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`definition_effective_history_hours()`</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`effective_history_hours_by_timeframe`; `lower_longest_effective_history_hours`, `upper_shortest_effective_history_hours` of `nesting`</t>
         </is>
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t xml:space="preserve">— (no page shows it; Bollinger %b in the definitions table of `methodology_features.md`)</t>
+          <t xml:space="preserve">effective history</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t xml:space="preserve">`bb20`, `%b` as a column, `z / 2 + 0.5`; `zscore20`</t>
-        </is>
-      </c>
-      <c r="I369" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bollinger (technical analysis)</t>
+          <t xml:space="preserve">history (bare — a recursion has no window), span (the parameter word of an exponential smoothing), lookback hours</t>
         </is>
       </c>
     </row>
@@ -15254,27 +15249,22 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t xml:space="preserve">the definitions an asset's model sees until a promotion — the frozen experiment's default definitions on every timeframe of the register, in the order it stacks them</t>
-        </is>
-      </c>
-      <c r="C370" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME`; `definition_in_default_set` of a record</t>
-        </is>
-      </c>
-      <c r="D370" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`definition_in_default_set`; `default_columns_by_timeframe` of the contract</t>
+          <t xml:space="preserve">the Bollinger %b reading — the trade's %b(20, 2σ), `rolling_standard_score20` / 4 + 0.5, an affine map a tree model is invariant to, so no %b column exists</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t xml:space="preserve">default set</t>
+          <t xml:space="preserve">— (no page shows it; Bollinger %b in the definitions table of `methodology_features.md`)</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t xml:space="preserve">the frozen fifteen (as a name)</t>
+          <t xml:space="preserve">`bb20`, `%b` as a column, `z / 2 + 0.5`; `zscore20`</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bollinger (technical analysis)</t>
         </is>
       </c>
     </row>
@@ -15286,49 +15276,59 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t xml:space="preserve">the definition the strategy hierarchy reads on every timeframe, set or no set</t>
+          <t xml:space="preserve">the definitions an asset's model sees until a promotion — the frozen experiment's default definitions on every timeframe of the register, in the order it stacks them</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TREND_GATE_FEATURE_DEFINITION` in `module_ml/config.py` — the name of the catalogue's first definition, owned by the strategy that reads it; the gate's timeframe is the top of the contract's hierarchy, `trend_gate_timeframe(cat)`</t>
+          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME`; `definition_in_default_set` of a record</t>
         </is>
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t xml:space="preserve">`trend_gate_feature`</t>
+          <t xml:space="preserve">`definition_in_default_set`; `default_columns_by_timeframe` of the contract</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t xml:space="preserve">gate (the asset's STRATEGY frame)</t>
+          <t xml:space="preserve">default set</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TREND_FAMILY`; a column literal in `asset.js`; a second copy of the name in the feature layer, which reads nothing of it</t>
+          <t xml:space="preserve">the frozen fifteen (as a name)</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset containers</t>
+          <t xml:space="preserve">Features</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t xml:space="preserve">an asset container: a runner's one-off for one asset, exiting with its stage</t>
+          <t xml:space="preserve">the definition the strategy hierarchy reads on every timeframe, set or no set</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
+          <t xml:space="preserve">`TREND_GATE_FEATURE_DEFINITION` in `module_ml/config.py` — the name of the catalogue's first definition, owned by the strategy that reads it; the gate's timeframe is the top of the contract's hierarchy, `trend_gate_timeframe(cat)`</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`trend_gate_feature`</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gate (the asset's STRATEGY frame)</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t xml:space="preserve">a compose service per asset; a resident per asset; a `restart:` policy; a published port</t>
+          <t xml:space="preserve">`TREND_FAMILY`; a column literal in `asset.js`; a second copy of the name in the feature layer, which reads nothing of it</t>
         </is>
       </c>
     </row>
@@ -15340,17 +15340,17 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t xml:space="preserve">a runner: a compose service that is a role and a one-off — no command of its own; the run supplies one and the container exits with the stage</t>
+          <t xml:space="preserve">an asset container: a runner's one-off for one asset, exiting with its stage</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
+          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t xml:space="preserve">`pipeline`, one runner for every module; a stage run by `exec` inside a resident; a runner with a `command:`</t>
+          <t xml:space="preserve">a compose service per asset; a resident per asset; a `restart:` policy; a published port</t>
         </is>
       </c>
     </row>
@@ -15362,17 +15362,17 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t xml:space="preserve">a service's mounts: the tree at `/app` and the stores it touches at `/store/&lt;content&gt;`, read-only where it only reads</t>
+          <t xml:space="preserve">a runner: a compose service that is a role and a one-off — no command of its own; the run supplies one and the container exits with the stage</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.:/app` and `./store/&lt;content&gt;:/store/&lt;content&gt;` in each service's `volumes:` of `docker-compose.yml`, respelled whole because a service's key replaces the anchor's</t>
+          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t xml:space="preserve">`/app/store/&lt;content&gt;` as an address; a mount of a store the service does not touch; a named volume</t>
+          <t xml:space="preserve">`pipeline`, one runner for every module; a stage run by `exec` inside a resident; a runner with a `command:`</t>
         </is>
       </c>
     </row>
@@ -15384,17 +15384,17 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t xml:space="preserve">the memory ceiling of the one runner that needs it — HPO and XGBoost allocate above `DUCKDB_MEMORY_LIMIT`</t>
+          <t xml:space="preserve">a service's mounts: the tree at `/app` and the stores it touches at `/store/&lt;content&gt;`, read-only where it only reads</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t xml:space="preserve">`deploy.resources.limits.memory` of the `ml` runner alone</t>
+          <t xml:space="preserve">`.:/app` and `./store/&lt;content&gt;:/store/&lt;content&gt;` in each service's `volumes:` of `docker-compose.yml`, respelled whole because a service's key replaces the anchor's</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t xml:space="preserve">`mem_limit` beside it, a CPU quota, a reservation; a ceiling on the anchor, so on the dashboard too</t>
+          <t xml:space="preserve">`/app/store/&lt;content&gt;` as an address; a mount of a store the service does not touch; a named volume</t>
         </is>
       </c>
     </row>
@@ -15406,17 +15406,17 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t xml:space="preserve">the thread cap: every computation's threads pinned to one — OpenMP's by the compose anchor's environment, beside the store contract, DuckDB's and XGBoost's in the code</t>
+          <t xml:space="preserve">the memory ceiling of the one runner that needs it — HPO and XGBoost allocate above `DUCKDB_MEMORY_LIMIT`</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OMP_NUM_THREADS` in the `x-store-environment` anchor of `docker-compose.yml`; `SET threads=1` on every DuckDB connection; `nthread` of the booster's parameters in `module_ml/config.py`</t>
+          <t xml:space="preserve">`deploy.resources.limits.memory` of the `ml` runner alone</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t xml:space="preserve">a thread count read from a stage's command line; a cap set per service</t>
+          <t xml:space="preserve">`mem_limit` beside it, a CPU quota, a reservation; a ceiling on the anchor, so on the dashboard too</t>
         </is>
       </c>
     </row>
@@ -15428,17 +15428,17 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t xml:space="preserve">the dashboard's command: the server, on the container's internal port</t>
+          <t xml:space="preserve">the thread cap: every computation's threads pinned to one — OpenMP's by the compose anchor's environment, beside the store contract, DuckDB's and XGBoost's in the code</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command: python -m module_monitoring.serve` of `dashboard`; `CONTAINER_PORT` and `BIND_ADDRESS` in `module_monitoring/config.py`</t>
+          <t xml:space="preserve">`OMP_NUM_THREADS` in the `x-store-environment` anchor of `docker-compose.yml`; `SET threads=1` on every DuckDB connection; `nthread` of the booster's parameters in `module_ml/config.py`</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t xml:space="preserve">a port or a bind address read from the environment or the command line; `PORT` inside a container</t>
+          <t xml:space="preserve">a thread count read from a stage's command line; a cap set per service</t>
         </is>
       </c>
     </row>
@@ -15450,22 +15450,17 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t xml:space="preserve">the host port: the host side of the dashboard's mapping, measured at invocation and never written down — and the page's address, the one `make on` prints</t>
+          <t xml:space="preserve">the dashboard's command: the server, on the container's internal port</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t xml:space="preserve">`PORT` of the `Makefile` — the port the dashboard already publishes, else the first free one upward from the internal port's number; `PORT=n` overrides; the `ports:` of `dashboard`, published on `127.0.0.1`</t>
-        </is>
-      </c>
-      <c r="E378" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`dashboard at http://127.0.0.1:&lt;port&gt;/`</t>
+          <t xml:space="preserve">`command: python -m module_monitoring.serve` of `dashboard`; `CONTAINER_PORT` and `BIND_ADDRESS` in `module_monitoring/config.py`</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t xml:space="preserve">the internal port's number as the page's address in a document, a command or a comment; a second variable for it; `PORT` inside a container; a measurement outside the `Makefile`</t>
+          <t xml:space="preserve">a port or a bind address read from the environment or the command line; `PORT` inside a container</t>
         </is>
       </c>
     </row>
@@ -15477,17 +15472,22 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t xml:space="preserve">the compose project: the one fixed name every container, network and volume of this project carries on every host</t>
+          <t xml:space="preserve">the host port: the host side of the dashboard's mapping, measured at invocation and never written down — and the page's address, the one `make on` prints</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t xml:space="preserve">`name: liora` in `docker-compose.yml` — the resident `liora-dashboard-1`</t>
+          <t xml:space="preserve">`PORT` of the `Makefile` — the port the dashboard already publishes, else the first free one upward from the internal port's number; `PORT=n` overrides; the `ports:` of `dashboard`, published on `127.0.0.1`</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`dashboard at http://127.0.0.1:&lt;port&gt;/`</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t xml:space="preserve">a name derived from the checkout's directory; a project per ticker; two checkouts of the project up at once on one host — they share the name: run one, or set `COMPOSE_PROJECT_NAME`</t>
+          <t xml:space="preserve">the internal port's number as the page's address in a document, a command or a comment; a second variable for it; `PORT` inside a container; a measurement outside the `Makefile`</t>
         </is>
       </c>
     </row>
@@ -15499,17 +15499,17 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t xml:space="preserve">how long a container lives: one-off — a `run --rm` process that exits with its stage — or resident — a server that stays up</t>
+          <t xml:space="preserve">the compose project: the one fixed name every container, network and volume of this project carries on every host</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run --rm -T`, the `run` macro of the `Makefile`, for a one-off; `up -d dashboard` of `make on` for the one resident</t>
+          <t xml:space="preserve">`name: liora` in `docker-compose.yml` — the resident `liora-dashboard-1`</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t xml:space="preserve">one-shot, ephemeral, daemon, long-running; `task` or `job` for the one-off; a stage run in a resident</t>
+          <t xml:space="preserve">a name derived from the checkout's directory; a project per ticker; two checkouts of the project up at once on one host — they share the name: run one, or set `COMPOSE_PROJECT_NAME`</t>
         </is>
       </c>
     </row>
@@ -15521,49 +15521,39 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t xml:space="preserve">the presentation switch: the dashboard up with the page's address printed and opened, or every container of this project down, in one word</t>
+          <t xml:space="preserve">how long a container lives: one-off — a `run --rm` process that exits with its stage — or resident — a server that stays up</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make on`, `make off` — the two bare lifecycle targets a presenter types</t>
+          <t xml:space="preserve">`run --rm -T`, the `run` macro of the `Makefile`, for a one-off; `up -d dashboard` of `make on` for the one resident</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t xml:space="preserve">`start` / `stop`, bare `up` / `down` (compose's), `run`, a second switch pair; a switch that runs a stage</t>
+          <t xml:space="preserve">one-shot, ephemeral, daemon, long-running; `task` or `job` for the one-off; a stage run in a resident</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run record</t>
+          <t xml:space="preserve">Asset containers</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t xml:space="preserve">one recorded run of the chain — the execution name, read forward</t>
+          <t xml:space="preserve">the presentation switch: the dashboard up with the page's address printed and opened, or every container of this project down, in one word</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run_id`; `RUN_ID` of the `Makefile`, `&lt;YYYYMMDDTHHMMSS&gt;Z_&lt;short commit&gt;` — the UTC time, then git's short commit — so it sorts by time and names the code that ran</t>
-        </is>
-      </c>
-      <c r="D382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`run_id`</t>
-        </is>
-      </c>
-      <c r="E382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">run</t>
+          <t xml:space="preserve">`make on`, `make off` — the two bare lifecycle targets a presenter types</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t xml:space="preserve">build, job, a content hash; a generated run id bound to no project name; a run id inside an artifact or a ledger</t>
+          <t xml:space="preserve">`start` / `stop`, bare `up` / `down` (compose's), `run`, a second switch pair; a switch that runs a stage</t>
         </is>
       </c>
     </row>
@@ -15575,27 +15565,27 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
+          <t xml:space="preserve">one recorded run of the chain — the execution name, read forward</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t xml:space="preserve">the target name; `RECORDED_STAGES` in the `Makefile` — `DATA_STAGES`, `FEATURES_STAGES`, `ML_STAGES` in order; `make all-record`</t>
+          <t xml:space="preserve">`run_id`; `RUN_ID` of the `Makefile`, `&lt;YYYYMMDDTHHMMSS&gt;Z_&lt;short commit&gt;` — the UTC time, then git's short commit — so it sorts by time and names the code that ran</t>
         </is>
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t xml:space="preserve">`stage` — the file name `&lt;stage&gt;.json`</t>
+          <t xml:space="preserve">`run_id`</t>
         </is>
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t xml:space="preserve">stage</t>
+          <t xml:space="preserve">run</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
+          <t xml:space="preserve">build, job, a content hash; a generated run id bound to no project name; a run id inside an artifact or a ledger</t>
         </is>
       </c>
     </row>
@@ -15607,22 +15597,27 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t xml:space="preserve">the command the recorder ran</t>
+          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command` — the make command line, joined by spaces</t>
+          <t xml:space="preserve">the target name; `RECORDED_STAGES` in the `Makefile` — `DATA_STAGES`, `FEATURES_STAGES`, `ML_STAGES` in order; `make all-record`</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command`</t>
+          <t xml:space="preserve">`stage` — the file name `&lt;stage&gt;.json`</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stage</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage's own command line; anything a stage says about itself</t>
+          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
         </is>
       </c>
     </row>
@@ -15634,27 +15629,22 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t xml:space="preserve">the exit code: how the stage ended; `all-record` stops at the first stage that exits non-zero and keeps its record</t>
+          <t xml:space="preserve">the command the recorder ran</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t xml:space="preserve">the command's exit code, `record.py`'s own</t>
+          <t xml:space="preserve">`command` — the make command line, joined by spaces</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t xml:space="preserve">`exit_code`</t>
-        </is>
-      </c>
-      <c r="E385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">exit</t>
+          <t xml:space="preserve">`command`</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t xml:space="preserve">status, ok</t>
+          <t xml:space="preserve">a stage's own command line; anything a stage says about itself</t>
         </is>
       </c>
     </row>
@@ -15666,27 +15656,27 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stage timing: when the stage ran, and for how long</t>
+          <t xml:space="preserve">the exit code: how the stage ended; `all-record` stops at the first stage that exits non-zero and keeps its record</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t xml:space="preserve">`main()` in `record.py` — the UTC clock before and after the command, the monotonic clock for the duration</t>
+          <t xml:space="preserve">the command's exit code, `record.py`'s own</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t xml:space="preserve">`started_at_utc`, `ended_at_utc`, `duration_seconds`</t>
+          <t xml:space="preserve">`exit_code`</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t xml:space="preserve">start; time; start / end and total time in the run's header</t>
+          <t xml:space="preserve">exit</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t xml:space="preserve">wall, elapsed</t>
+          <t xml:space="preserve">status, ok</t>
         </is>
       </c>
     </row>
@@ -15698,27 +15688,27 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store diff: what the stage did to the stores — every file added, changed (size or mtime moved) or removed, by store and path</t>
+          <t xml:space="preserve">the stage timing: when the stage ran, and for how long</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the four stores of `STORES` — every store but the trials store</t>
+          <t xml:space="preserve">`main()` in `record.py` — the UTC clock before and after the command, the monotonic clock for the duration</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t xml:space="preserve">`store_diff` with `added`, `changed` — each `store`, `path`, `size_bytes`, `mtime_ns` — and `removed` — each `store`, `path`</t>
+          <t xml:space="preserve">`started_at_utc`, `ended_at_utc`, `duration_seconds`</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t xml:space="preserve">added / changed / removed; bytes written; the STORES frame</t>
+          <t xml:space="preserve">start; time; start / end and total time in the run's header</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t xml:space="preserve">output, artifacts, a stage → artifact map; a trial ledger read by the recorder</t>
+          <t xml:space="preserve">wall, elapsed</t>
         </is>
       </c>
     </row>
@@ -15730,17 +15720,27 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t xml:space="preserve">the basket one run covered — not in the record: the recorder knows no basket</t>
+          <t xml:space="preserve">the store diff: what the stage did to the stores — every file added, changed (size or mtime moved) or removed, by store and path</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t xml:space="preserve">the launcher's `TICKERS`, which the make target the recorder wraps carries into every stage command</t>
+          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the four stores of `STORES` — every store but the trials store</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`store_diff` with `added`, `changed` — each `store`, `path`, `size_bytes`, `mtime_ns` — and `removed` — each `store`, `path`</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added / changed / removed; bytes written; the STORES frame</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ticker`, the first of the basket standing for it; one record per asset</t>
+          <t xml:space="preserve">output, artifacts, a stage → artifact map; a trial ledger read by the recorder</t>
         </is>
       </c>
     </row>
@@ -15752,27 +15752,17 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run index: every run with a record, newest first, each with its records — the one file the page reads to find a run</t>
+          <t xml:space="preserve">the basket one run covered — not in the record: the recorder knows no basket</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_run_index()` in `record.py`, written again after every record from the store's listing, as `store/run_records/index.json`</t>
-        </is>
-      </c>
-      <c r="D389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`generated_at_utc`; `runs[]`, each `run_id` and `records` — the record files, relative to the run's directory, in path order</t>
-        </is>
-      </c>
-      <c r="E389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`&lt;n&gt; recorded run(s) · showing &lt;run_id&gt; · &lt;n&gt; records`</t>
+          <t xml:space="preserve">the launcher's `TICKERS`, which the make target the recorder wraps carries into every stage command</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t xml:space="preserve">a run list per asset; a listing by the page; a route that lists the store; an index written by a stage</t>
+          <t xml:space="preserve">`ticker`, the first of the basket standing for it; one record per asset</t>
         </is>
       </c>
     </row>
@@ -15784,22 +15774,27 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stage records of one run, in the order the stages started — each read by the page at the relative path the index lists</t>
+          <t xml:space="preserve">the run index: every run with a record, newest first, each with its records — the one file the page reads to find a run</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t xml:space="preserve">`runs[].records` of the index; `fetchRunRecord()` in `module_monitoring/run.js`, which sorts them by `started_at_utc`</t>
+          <t xml:space="preserve">`build_run_index()` in `record.py`, written again after every record from the store's listing, as `store/run_records/index.json`</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`generated_at_utc`; `runs[]`, each `run_id` and `records` — the record files, relative to the run's directory, in path order</t>
         </is>
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAGES — stage, asset, start, time, exit, added, changed, removed, bytes written</t>
+          <t xml:space="preserve">`&lt;n&gt; recorded run(s) · showing &lt;run_id&gt; · &lt;n&gt; records`</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t xml:space="preserve">a record per asset of a basket stage; an envelope built by a server</t>
+          <t xml:space="preserve">a run list per asset; a listing by the page; a route that lists the store; an index written by a stage</t>
         </is>
       </c>
     </row>
@@ -15811,39 +15806,44 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, written whole after the stage's second listing so it never appears in its own difference; untracked</t>
+          <t xml:space="preserve">the stage records of one run, in the order the stages started — each read by the page at the relative path the index lists</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STORE_RUN_RECORDS_DIR`, `store/run_records/&lt;run_id&gt;/&lt;stage&gt;.json`; `write_json()` in `record.py`, beside its place, then moved onto it</t>
+          <t xml:space="preserve">`runs[].records` of the index; `fetchRunRecord()` in `module_monitoring/run.js`, which sorts them by `started_at_utc`</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STAGES — stage, asset, start, time, exit, added, changed, removed, bytes written</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `runtime/` folder under an asset; one run record per asset; a run record tracked</t>
+          <t xml:space="preserve">a record per asset of a basket stage; an envelope built by a server</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentation ownership</t>
+          <t xml:space="preserve">Run record</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generated document: one the sync renders from the sheet and a hand never edits, its first line the marker, its rules cited by `rule_id`</t>
+          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, written whole after the stage's second listing so it never appears in its own difference; untracked</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
+          <t xml:space="preserve">`STORE_RUN_RECORDS_DIR`, `store/run_records/&lt;run_id&gt;/&lt;stage&gt;.json`; `write_json()` in `record.py`, beside its place, then moved onto it</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Skill edited in its file; a Skill cited by a numbered or titled section — a rule is cited by its `rule_id`; a hand-written `skill_*.md`</t>
+          <t xml:space="preserve">a `runtime/` folder under an asset; one run record per asset; a run record tracked</t>
         </is>
       </c>
     </row>
@@ -15855,17 +15855,17 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hand-written document: one a hand keeps and the sync never touches, no marker on its first line</t>
+          <t xml:space="preserve">a generated document: one the sync renders from the sheet and a hand never edits, its first line the marker, its rules cited by `rule_id`</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md`, `CLAUDE.md`, `README.md`, `module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`, `module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`, every `README_sub_module_&lt;subject&gt;.md`, `module_skills/README.md`, `module_skills/sub_module_scalability_crawler/crawlers_mission.md`</t>
+          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule kept only there; a second copy of a rule</t>
+          <t xml:space="preserve">a Skill edited in its file; a Skill cited by a numbered or titled section — a rule is cited by its `rule_id`; a hand-written `skill_*.md`</t>
         </is>
       </c>
     </row>
@@ -15877,17 +15877,17 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t xml:space="preserve">a normative document describing one module's own responsibility</t>
+          <t xml:space="preserve">a hand-written document: one a hand keeps and the sync never touches, no marker on its first line</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_&lt;domain&gt;`</t>
+          <t xml:space="preserve">`AGENTS.md`, `CLAUDE.md`, `README.md`, `module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`, `module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`, every `README_sub_module_&lt;subject&gt;.md`, `module_skills/README.md`, `module_skills/sub_module_scalability_crawler/crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">a module's rule kept in `module_skills/`; a per-module `docs/` or `doc/` folder</t>
+          <t xml:space="preserve">a rule kept only there; a second copy of a rule</t>
         </is>
       </c>
     </row>
@@ -15899,17 +15899,17 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t xml:space="preserve">a normative document that crosses modules or governs the project — the canon's</t>
+          <t xml:space="preserve">a normative document describing one module's own responsibility</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_skills`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_&lt;domain&gt;`</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t xml:space="preserve">a cross-cutting rule filed under one module; an edit to a copy</t>
+          <t xml:space="preserve">a module's rule kept in `module_skills/`; a per-module `docs/` or `doc/` folder</t>
         </is>
       </c>
     </row>
@@ -15921,17 +15921,17 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module skill: the normative document about one sub-module alone, kept beside its code as `skill_&lt;subject&gt;.md` — the serpentine search's and the crawler's; a terminal has none of its own, `module_skills/skill_tui_designer.md` holding what the terminals share</t>
+          <t xml:space="preserve">a normative document that crosses modules or governs the project — the canon's</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_&lt;subject&gt;/skill_&lt;subject&gt;.md`, rendered from its owner's tab</t>
+          <t xml:space="preserve">`module_skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_skills`</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module's own rule among `module_skills/skill_*.md` or in its module's `skills/`; a rule two sub-modules obey kept beside one of them; a `skill_&lt;module&gt;_terminal.md`; a `skills/` folder for one document</t>
+          <t xml:space="preserve">a cross-cutting rule filed under one module; an edit to a copy</t>
         </is>
       </c>
     </row>
@@ -15943,17 +15943,17 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t xml:space="preserve">the directory holding one module's own documents: its Skills and its methodology</t>
+          <t xml:space="preserve">a sub-module skill: the normative document about one sub-module alone, kept beside its code as `skill_&lt;subject&gt;.md` — the serpentine search's and the crawler's; a terminal has none of its own, `module_skills/skill_tui_designer.md` holding what the terminals share</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/`</t>
+          <t xml:space="preserve">`sub_module_&lt;subject&gt;/skill_&lt;subject&gt;.md`, rendered from its owner's tab</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skill/`, `module_&lt;domain&gt;/documentation/`</t>
+          <t xml:space="preserve">a sub-module's own rule among `module_skills/skill_*.md` or in its module's `skills/`; a rule two sub-modules obey kept beside one of them; a `skill_&lt;module&gt;_terminal.md`; a `skills/` folder for one document</t>
         </is>
       </c>
     </row>
@@ -15965,17 +15965,17 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t xml:space="preserve">the name register: one concept, one name, in code, artifacts and interface, and the copies no module may import across — rendered from the glossary table of the sheet with the register's own rules</t>
+          <t xml:space="preserve">the directory holding one module's own documents: its Skills and its methodology</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/`</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">a register edited by hand; a second register; a name entering the tree in a commit that does not add its row</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skill/`, `module_&lt;domain&gt;/documentation/`</t>
         </is>
       </c>
     </row>
@@ -15987,17 +15987,17 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sheet: the one source of every Skill and of the register — a tab per owner, each with its rule table; the glossary and the `rule_type_id` list; the skill register and the files matrix</t>
+          <t xml:space="preserve">the name register: one concept, one name, in code, artifacts and interface, and the copies no module may import across — rendered from the glossary table of the sheet with the register's own rules</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skills_sheet.xlsx`, `SKILLS_SHEET_PATH`; `load_sheet()` in `module_skills/sheet.py`; `RULE_HEADER`, `SKILL_REGISTER_HEADER`, `GLOSSARY_HEADER`, `RULE_TYPE_ID_HEADER`, `FILES_MATRIX_HEADER` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Skill edited in its file; a second workbook; a CSV or JSON beside it; a sheet written by code</t>
+          <t xml:space="preserve">a register edited by hand; a second register; a name entering the tree in a commit that does not add its row</t>
         </is>
       </c>
     </row>
@@ -16009,17 +16009,17 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t xml:space="preserve">the skill register: a row per generated Skill — the tab that holds its rules, its `skill_path` and its summary</t>
+          <t xml:space="preserve">the sheet: the one source of every Skill and of the register — a tab per owner, each with its rule table; the glossary and the `rule_type_id` list; the skill register and the files matrix</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILL_REGISTER_HEADER` in `module_skills/config.py`; `Skill` in `module_skills/sheet.py`</t>
+          <t xml:space="preserve">`module_skills/skills_sheet.xlsx`, `SKILLS_SHEET_PATH`; `load_sheet()` in `module_skills/sheet.py`; `RULE_HEADER`, `SKILL_REGISTER_HEADER`, `GLOSSARY_HEADER`, `RULE_TYPE_ID_HEADER`, `FILES_MATRIX_HEADER` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t xml:space="preserve">document register, `DOCUMENT_REGISTER_HEADER`; a Skill without a register row; a summary in a rule row; an owner read off the files matrix</t>
+          <t xml:space="preserve">a Skill edited in its file; a second workbook; a CSV or JSON beside it; a sheet written by code</t>
         </is>
       </c>
     </row>
@@ -16031,17 +16031,17 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sync: every Skill and the register rendered from the sheet beside what each governs, and every generated file the sheet no longer names deleted</t>
+          <t xml:space="preserve">the skill register: a row per generated Skill — the tab that holds its rules, its `skill_path` and its summary</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make skills-sync`; `main()`, `to_markdown()`, `build_documents()`, `write_text()`, `delete_stale()` in `module_skills/sync.py`; `GENERATED_MARKER`</t>
+          <t xml:space="preserve">`SKILL_REGISTER_HEADER` in `module_skills/config.py`; `Skill` in `module_skills/sheet.py`</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t xml:space="preserve">distribute, generate, export; a stamp; a comparison of copies; a Markdown edited by hand; a sync that reads the sheet twice; a document without the marker deleted</t>
+          <t xml:space="preserve">document register, `DOCUMENT_REGISTER_HEADER`; a Skill without a register row; a summary in a rule row; an owner read off the files matrix</t>
         </is>
       </c>
     </row>
@@ -16053,17 +16053,17 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t xml:space="preserve">the table of every configurable: every CONFIGURABLES record of the controlled `config.py` files, read as literals, on stdout</t>
+          <t xml:space="preserve">the sync: every Skill and the register rendered from the sheet beside what each governs, and every generated file the sheet no longer names deleted</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make skills-configurables`; `main()`, `load_records()`, `to_cell()` in `module_skills/configurables.py`</t>
+          <t xml:space="preserve">`make skills-sync`; `main()`, `to_markdown()`, `build_documents()`, `write_text()`, `delete_stale()` in `module_skills/sync.py`; `GENERATED_MARKER`</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t xml:space="preserve">a file the table is written into; an import of the module whose records it reads; a record the table carries and no `config.py` holds</t>
+          <t xml:space="preserve">distribute, generate, export; a stamp; a comparison of copies; a Markdown edited by hand; a sync that reads the sheet twice; a document without the marker deleted</t>
         </is>
       </c>
     </row>
@@ -16075,17 +16075,17 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t xml:space="preserve">the contract: what every change answers to, read in full before a session's first edit</t>
+          <t xml:space="preserve">the table of every configurable: every CONFIGURABLES record of the controlled `config.py` files, read as literals, on stdout</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md` at the root</t>
+          <t xml:space="preserve">`make skills-configurables`; `main()`, `load_records()`, `to_cell()` in `module_skills/configurables.py`</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second contract; a per-module `AGENTS.md`</t>
+          <t xml:space="preserve">a file the table is written into; an import of the module whose records it reads; a record the table carries and no `config.py` holds</t>
         </is>
       </c>
     </row>
@@ -16097,17 +16097,17 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
+          <t xml:space="preserve">the contract: what every change answers to, read in full before a session's first edit</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t xml:space="preserve">`CLAUDE.md` at the root</t>
+          <t xml:space="preserve">`AGENTS.md` at the root</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule written in it; a per-module `CLAUDE.md`; `CLAUDE.local.md` or `.claude/` inside the tree</t>
+          <t xml:space="preserve">a second contract; a per-module `AGENTS.md`</t>
         </is>
       </c>
     </row>
@@ -16119,17 +16119,17 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t xml:space="preserve">the project's front door: what the project is, how to run it and where its Skills are</t>
+          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README.md` at the root</t>
+          <t xml:space="preserve">`CLAUDE.md` at the root</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule restated in it; a front door that restates a Skill or a decision table</t>
+          <t xml:space="preserve">a rule written in it; a per-module `CLAUDE.md`; `CLAUDE.local.md` or `.claude/` inside the tree</t>
         </is>
       </c>
     </row>
@@ -16141,17 +16141,17 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t xml:space="preserve">one module's reader-facing front door, its orientation</t>
+          <t xml:space="preserve">the project's front door: what the project is, how to run it and where its Skills are</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`README.md` at the root</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/README.md`; an orientation that restates a Skill or a decision table</t>
+          <t xml:space="preserve">a rule restated in it; a front door that restates a Skill or a decision table</t>
         </is>
       </c>
     </row>
@@ -16163,17 +16163,17 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module's orientation, beside its code</t>
+          <t xml:space="preserve">one module's reader-facing front door, its orientation</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/README.md`; an orientation that restates a Skill or a decision table</t>
         </is>
       </c>
     </row>
@@ -16185,17 +16185,17 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t xml:space="preserve">the design rationale: the section of a module's orientation that says, per object, analogous pair or the module's documents, why here, why beside these, why this boundary and which mapping row it answers to — the fourth the test of the first three</t>
+          <t xml:space="preserve">a sub-module's orientation, beside its code</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t xml:space="preserve">`## Design rationale` of each `README_module_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t xml:space="preserve">a decision table; a rule restated; an object with no row or two; ADR, decision record, decision log, `docs/`</t>
+          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
         </is>
       </c>
     </row>
@@ -16207,17 +16207,17 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t xml:space="preserve">a methodology document: reference material for a human — the equations, the derivations and the citations of one module</t>
+          <t xml:space="preserve">the design rationale: the section of a module's orientation that says, per object, analogous pair or the module's documents, why here, why beside these, why this boundary and which mapping row it answers to — the fourth the test of the first three</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`## Design rationale` of each `README_module_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t xml:space="preserve">a row of the files matrix; a document the crawler sends; a rule stated only there</t>
+          <t xml:space="preserve">a decision table; a rule restated; an object with no row or two; ADR, decision record, decision log, `docs/`</t>
         </is>
       </c>
     </row>
@@ -16229,44 +16229,39 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t xml:space="preserve">the canon's index: every Skill by its path, and the canon's prose that is no rule, the mapping table among it</t>
+          <t xml:space="preserve">a methodology document: reference material for a human — the equations, the derivations and the citations of one module</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/README.md`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t xml:space="preserve">a collection of copies; an index that restates a rule it links to</t>
+          <t xml:space="preserve">a row of the files matrix; a document the crawler sends; a rule stated only there</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-AWS direction</t>
+          <t xml:space="preserve">Documentation ownership</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stance: a local academic architecture whose boundaries would survive a move onto standard cloud primitives, with no cloud used and none planned</t>
+          <t xml:space="preserve">the canon's index: every Skill by its path, and the canon's prose that is no rule, the mapping table among it</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_pre_aws_solution.md` — `pre_aws` its stem, the one tracked name that carries the word; no identifier</t>
+          <t xml:space="preserve">`module_skills/README.md`</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t xml:space="preserve">cloud-ready, AWS-ready, cloud-native; a migration plan, a deployment guide; `pre-aws` or `PreAWS` in prose</t>
-        </is>
-      </c>
-      <c r="I411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pre-AWS — before Amazon Web Services (AWS), the cloud the mapping reads forward to</t>
+          <t xml:space="preserve">a collection of copies; an index that restates a rule it links to</t>
         </is>
       </c>
     </row>
@@ -16278,22 +16273,22 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t xml:space="preserve">compute: a process that reads a store, writes a store and exits, owning no asset state between invocations</t>
+          <t xml:space="preserve">the stance: a local academic architecture whose boundaries would survive a move onto standard cloud primitives, with no cloud used and none planned</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t xml:space="preserve">every stage's `main()`, `python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;`; the one-off container that runs it</t>
+          <t xml:space="preserve">`module_skills/skill_pre_aws_solution.md` — `pre_aws` its stem, the one tracked name that carries the word; no identifier</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t xml:space="preserve">a container as the home of an asset's state; a resident as a requirement of a stage; an in-process cache between stages; `worker`, `processor`</t>
+          <t xml:space="preserve">cloud-ready, AWS-ready, cloud-native; a migration plan, a deployment guide; `pre-aws` or `PreAWS` in prose</t>
         </is>
       </c>
       <c r="I412" t="inlineStr">
         <is>
-          <t xml:space="preserve">a task — one run of the one task definition on the container instance every asset's runs share (Amazon ECS on Amazon EC2)</t>
+          <t xml:space="preserve">Pre-AWS — before Amazon Web Services (AWS), the cloud the mapping reads forward to</t>
         </is>
       </c>
     </row>
@@ -16305,22 +16300,22 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t xml:space="preserve">the rebuild condition: whether an asset's artifacts must be rebuilt from its canonical series, answered without launching anything; its freshness half is unwritten, its names reserved — `has_new_market_data()`, `requires_canonical_rebuild()`, `requires_feature_rebuild()`, `requires_model_rebuild()`</t>
+          <t xml:space="preserve">compute: a process that reads a store, writes a store and exits, owning no asset state between invocations</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t xml:space="preserve">`is_artifact_set_complete()` in `module_ml/config.py`, its completeness half; the rerun table of `module_ml/skills/methodology_ml.md`, read by a human</t>
+          <t xml:space="preserve">every stage's `main()`, `python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;`; the one-off container that runs it</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t xml:space="preserve">a scheduler, a watcher, an event bus; a function that both detects new data and trains; `should_run()`, `check_update()`, `trigger()`</t>
+          <t xml:space="preserve">a container as the home of an asset's state; a resident as a requirement of a stage; an in-process cache between stages; `worker`, `processor`</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t xml:space="preserve">a choice state between two states of the machine (AWS Step Functions)</t>
+          <t xml:space="preserve">a task — one run of the one task definition on the container instance every asset's runs share (Amazon ECS on Amazon EC2)</t>
         </is>
       </c>
     </row>
@@ -16332,17 +16327,22 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mapping table: what this repository has, the responsibility, the same responsibility elsewhere and the move, row by row — the one table that sets a cloud proper noun beside a local object; its third column is the elsewhere column</t>
+          <t xml:space="preserve">the rebuild condition: whether an asset's artifacts must be rebuilt from its canonical series, answered without launching anything; its freshness half is unwritten, its names reserved — `has_new_market_data()`, `requires_canonical_rebuild()`, `requires_feature_rebuild()`, `requires_model_rebuild()`</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/README.md`, its hand-written home</t>
+          <t xml:space="preserve">`is_artifact_set_complete()` in `module_ml/config.py`, its completeness half; the rerun table of `module_ml/skills/methodology_ml.md`, read by a human</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t xml:space="preserve">an adapter, a cloud configuration file; a cloud proper noun in an identifier, a key, a path, a make target, a compose service or an environment variable; a path of the elsewhere column read as a proposal for a local directory</t>
+          <t xml:space="preserve">a scheduler, a watcher, an event bus; a function that both detects new data and trains; `should_run()`, `check_update()`, `trigger()`</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a choice state between two states of the machine (AWS Step Functions)</t>
         </is>
       </c>
     </row>
@@ -16354,17 +16354,17 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t xml:space="preserve">a seat: the standard primitive a local object would sit on elsewhere, named in the mapping table's words — spoken in the stance's skill and in the mapping table, and in no other Skill</t>
+          <t xml:space="preserve">the mapping table: what this repository has, the responsibility, the same responsibility elsewhere and the move, row by row — the one table that sets a cloud proper noun beside a local object; its third column is the elsewhere column</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`module_skills/README.md`, its hand-written home</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t xml:space="preserve">a seat paragraph in any other Skill; two seats for one object; a seat in an identifier, a key or a path; `target`, `cloud note`, `mapping section`</t>
-        </is>
-      </c>
-      <c r="I415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the image registry (Amazon ECR), the container service (Amazon ECS), the container instance (Amazon EC2), the block volume (Amazon EBS), object storage (Amazon S3), the state machine (AWS Step Functions), the schedule (Amazon EventBridge Scheduler)</t>
+          <t xml:space="preserve">an adapter, a cloud configuration file; a cloud proper noun in an identifier, a key, a path, a make target, a compose service or an environment variable; a path of the elsewhere column read as a proposal for a local directory</t>
         </is>
       </c>
     </row>
@@ -16376,17 +16376,17 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t xml:space="preserve">the resource role: the name a cloud resource would carry, `&lt;project&gt;-&lt;environment&gt;-&lt;resource-role&gt;` — the role a seat's name or the task a row of the mapping table names, lower case with `-` between its words, the project `liora`</t>
-        </is>
-      </c>
-      <c r="C416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`name: liora` and `liora-1m-pipeline` in `docker-compose.yml` — the names of that shape the tree holds, with no environment token</t>
+          <t xml:space="preserve">a seat: the standard primitive a local object would sit on elsewhere, named in the mapping table's words — spoken in the stance's skill and in the mapping table, and in no other Skill</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second list of roles; a role no seat or row names; `dev` or `prod` in a tracked name; a ticker in a resource name; an environment token on the image</t>
+          <t xml:space="preserve">a seat paragraph in any other Skill; two seats for one object; a seat in an identifier, a key or a path; `target`, `cloud note`, `mapping section`</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the image registry (Amazon ECR), the container service (Amazon ECS), the container instance (Amazon EC2), the block volume (Amazon EBS), object storage (Amazon S3), the state machine (AWS Step Functions), the schedule (Amazon EventBridge Scheduler)</t>
         </is>
       </c>
     </row>
@@ -16398,17 +16398,17 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state name: the one-line name a stage would carry as a state of the machine, one per stage, and PublishStores, the copy after a run, which no stage answers to; *Publish* in a state name means write the object where its readers read it</t>
+          <t xml:space="preserve">the resource role: the name a cloud resource would carry, `&lt;project&gt;-&lt;environment&gt;-&lt;resource-role&gt;` — the role a seat's name or the task a row of the mapping table names, lower case with `-` between its words, the project `liora`</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`name: liora` and `liora-1m-pipeline` in `docker-compose.yml` — the names of that shape the tree holds, with no environment token</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state registered one by one; a state name with *and* in it; *publish* as *make public*</t>
-        </is>
-      </c>
-      <c r="I417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a state of AWS Step Functions</t>
+          <t xml:space="preserve">a second list of roles; a role no seat or row names; `dev` or `prod` in a tracked name; a ticker in a resource name; an environment token on the image</t>
         </is>
       </c>
     </row>
@@ -16420,17 +16420,17 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t xml:space="preserve">an instance: one Linux virtual machine elsewhere, the host containers run on — the task host every asset's runs share, with the store volume beside it, and the strategy host</t>
+          <t xml:space="preserve">a state name: the one-line name a stage would carry as a state of the machine, one per stage, and PublishStores, the copy after a run, which no stage answers to; *Publish* in a state name means write the object where its readers read it</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t xml:space="preserve">`instance` or `host` for a container; a host per asset; node</t>
+          <t xml:space="preserve">a state registered one by one; a state name with *and* in it; *publish* as *make public*</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
         <is>
-          <t xml:space="preserve">a container instance (Amazon EC2)</t>
+          <t xml:space="preserve">a state of AWS Step Functions</t>
         </is>
       </c>
     </row>
@@ -16442,22 +16442,17 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store volume: the task host's durable disk — the five stores at `/store/&lt;content&gt;`, each at the path its `STORE_*_DIR` names; the home of state, never the copy</t>
-        </is>
-      </c>
-      <c r="C419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the `./store/&lt;content&gt;` mounts of `docker-compose.yml`, read forward as `&lt;volume&gt;/&lt;content&gt;:/store/&lt;content&gt;`</t>
+          <t xml:space="preserve">an instance: one Linux virtual machine elsewhere, the host containers run on — the task host every asset's runs share, with the store volume beside it, and the strategy host</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset volume; a volume per asset; the volume as the copy; `data_volume`; a shared network filesystem (Amazon EFS)</t>
+          <t xml:space="preserve">`instance` or `host` for a container; a host per asset; node</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t xml:space="preserve">a block volume (Amazon EBS)</t>
+          <t xml:space="preserve">a container instance (Amazon EC2)</t>
         </is>
       </c>
     </row>
@@ -16469,17 +16464,22 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t xml:space="preserve">the copy: the whole files a state after the last stage of a run would copy from the store volume to object storage — never a stage's own write, never mid-run; absent here, described</t>
+          <t xml:space="preserve">the store volume: the task host's durable disk — the five stores at `/store/&lt;content&gt;`, each at the path its `STORE_*_DIR` names; the home of state, never the copy</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the `./store/&lt;content&gt;` mounts of `docker-compose.yml`, read forward as `&lt;volume&gt;/&lt;content&gt;:/store/&lt;content&gt;`</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage writing to object storage; a stage reading the copy; `s3://` in a path constant; an adapter for the copy</t>
+          <t xml:space="preserve">asset volume; a volume per asset; the volume as the copy; `data_volume`; a shared network filesystem (Amazon EFS)</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t xml:space="preserve">object storage (Amazon S3), written by PublishStores</t>
+          <t xml:space="preserve">a block volume (Amazon EBS)</t>
         </is>
       </c>
     </row>
@@ -16491,12 +16491,17 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t xml:space="preserve">the ladder: the three phases in which the runtime elsewhere would become true, each named for what it changes — *the lift*, *the idiom*, *the image carries the code*; all elsewhere, built nowhere here</t>
+          <t xml:space="preserve">the copy: the whole files a state after the last stage of a run would copy from the store volume to object storage — never a stage's own write, never mid-run; absent here, described</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t xml:space="preserve">a letter or a number for a phase; a phase as a branch or an environment; `dev` / `prod`; a phase built here; rung</t>
+          <t xml:space="preserve">a stage writing to object storage; a stage reading the copy; `s3://` in a path constant; an adapter for the copy</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">object storage (Amazon S3), written by PublishStores</t>
         </is>
       </c>
     </row>
@@ -16508,17 +16513,12 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion threshold: a second concurrent writer of one partition, or a reader that needs one transaction across families — the one condition under which a managed database replaces the table families</t>
+          <t xml:space="preserve">the ladder: the three phases in which the runtime elsewhere would become true, each named for what it changes — *the lift*, *the idiom*, *the image carries the code*; all elsewhere, built nowhere here</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t xml:space="preserve">a database process for one writer; a threshold in rows or bytes</t>
-        </is>
-      </c>
-      <c r="I422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a managed database (Amazon RDS)</t>
+          <t xml:space="preserve">a letter or a number for a phase; a phase as a branch or an environment; `dev` / `prod`; a phase built here; rung</t>
         </is>
       </c>
     </row>
@@ -16530,22 +16530,17 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t xml:space="preserve">the active version: the one version of an asset's artifacts a reader reads, chosen where the reader is; the version is the execution name</t>
-        </is>
-      </c>
-      <c r="C423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`run_id`</t>
+          <t xml:space="preserve">the promotion threshold: a second concurrent writer of one partition, or a reader that needs one transaction across families — the one condition under which a managed database replaces the table families</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t xml:space="preserve">latest, current, prod; a mark inside a file; a version inside an artifact</t>
+          <t xml:space="preserve">a database process for one writer; a threshold in rows or bytes</t>
         </is>
       </c>
       <c r="I423" t="inlineStr">
         <is>
-          <t xml:space="preserve">the version prefix `assets_artifacts/&lt;run_id&gt;/` of the copy (Amazon S3)</t>
+          <t xml:space="preserve">a managed database (Amazon RDS)</t>
         </is>
       </c>
     </row>
@@ -16557,22 +16552,22 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t xml:space="preserve">the tunnel: how a reader reaches the page on a host that is not theirs — a local forward onto the loopback port `make on` printed there</t>
+          <t xml:space="preserve">the active version: the one version of an asset's artifacts a reader reads, chosen where the reader is; the version is the execution name</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ssh -N -L` of `README.md` § Quickstart</t>
+          <t xml:space="preserve">`run_id`</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t xml:space="preserve">a public port; a load balancer</t>
+          <t xml:space="preserve">latest, current, prod; a mark inside a file; a version inside an artifact</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">a port-forward, the elsewhere column's word</t>
+          <t xml:space="preserve">the version prefix `assets_artifacts/&lt;run_id&gt;/` of the copy (Amazon S3)</t>
         </is>
       </c>
     </row>
@@ -16584,12 +16579,22 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t xml:space="preserve">read forward: a local object read as the same responsibility elsewhere — the mapping table's third column — with nothing moved</t>
+          <t xml:space="preserve">the tunnel: how a reader reaches the page on a host that is not theirs — a local forward onto the loopback port `make on` printed there</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`ssh -N -L` of `README.md` § Quickstart</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t xml:space="preserve">migrated, ported, deployed, in production</t>
+          <t xml:space="preserve">a public port; a load balancer</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a port-forward, the elsewhere column's word</t>
         </is>
       </c>
     </row>
@@ -16601,12 +16606,12 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t xml:space="preserve">the move: what a local thing's seat elsewhere costs it — a rename, one edit, or absent here, described; the mapping table's fourth column</t>
+          <t xml:space="preserve">read forward: a local object read as the same responsibility elsewhere — the mapping table's third column — with nothing moved</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t xml:space="preserve">migration, deployment, a plan, a roadmap</t>
+          <t xml:space="preserve">migrated, ported, deployed, in production</t>
         </is>
       </c>
     </row>
@@ -16618,44 +16623,34 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t xml:space="preserve">an absent object: a primitive, a state of the machine or a Skill that nothing local answers to and a document describes — a sentence ending, or a verdict reading, *absent here — described*</t>
-        </is>
-      </c>
-      <c r="C427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`AGENTS.md` § Skills absent here, described, for the Skills</t>
+          <t xml:space="preserve">the move: what a local thing's seat elsewhere costs it — a rename, one edit, or absent here, described; the mapping table's fourth column</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t xml:space="preserve">planned, a debt marker, future, ghost, placeholder, missing</t>
+          <t xml:space="preserve">migration, deployment, a plan, a roadmap</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t xml:space="preserve">The page</t>
+          <t xml:space="preserve">Pre-AWS direction</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page: one static page of plain HTML, CSS and JavaScript that reads every datum by a relative path and writes nothing</t>
+          <t xml:space="preserve">an absent object: a primitive, a state of the machine or a Skill that nothing local answers to and a document describes — a sentence ending, or a verdict reading, *absent here — described*</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/index.html`, `style.css` and its scripts `page.js`, `data.js`, `asset.js`, `features.js`, `ml.js`, `run.js`, `scalability.js`</t>
-        </is>
-      </c>
-      <c r="E428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1m crypto research pipeline — status</t>
+          <t xml:space="preserve">`AGENTS.md` § Skills absent here, described, for the Skills</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t xml:space="preserve">a framework or a build step; a second page beside it; a datum computed by the server; an absolute path</t>
+          <t xml:space="preserve">planned, a debt marker, future, ghost, placeholder, missing</t>
         </is>
       </c>
     </row>
@@ -16667,17 +16662,22 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page's reads: where the page takes its data from, by relative path</t>
+          <t xml:space="preserve">the page: one static page of plain HTML, CSS and JavaScript that reads every datum by a relative path and writes nothing</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t xml:space="preserve">`status/data_status.json`, `status/features_status.json`, `status/ml_status.json`, `status/skills_status.json`; `run_records/index.json`, then each record of a run at `run_records/&lt;run_id&gt;/` and the path the index lists</t>
+          <t xml:space="preserve">`module_monitoring/index.html`, `style.css` and its scripts `page.js`, `data.js`, `asset.js`, `features.js`, `ml.js`, `run.js`, `scalability.js`</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1m crypto research pipeline — status</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t xml:space="preserve">an absolute path; a route per snapshot; a directory listing; a store the page reads beside these two</t>
+          <t xml:space="preserve">a framework or a build step; a second page beside it; a datum computed by the server; an absolute path</t>
         </is>
       </c>
     </row>
@@ -16689,22 +16689,17 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three prefixes: what the dashboard's server answers — the page's own files at `/`, the status store under `/status/`, the run-records store under `/run_records/`; every other path 404, and no directory listed</t>
+          <t xml:space="preserve">the page's reads: where the page takes its data from, by relative path</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/serve.py` — `DashboardHandler`, `translate_path()`, `main()`; `STORE_DIR_BY_ROUTE_PREFIX` in `module_monitoring/config.py`, `/status/` onto `STORE_STATUS_DIR` and `/run_records/` onto `STORE_RUN_RECORDS_DIR`; `MODULE_MONITORING_DIR`, `PAGE_FILE_SUFFIXES`, `PAGE_INDEX_FILE_NAME` for the page's own files</t>
+          <t xml:space="preserve">`status/data_status.json`, `status/features_status.json`, `status/ml_status.json`, `status/skills_status.json`; `run_records/index.json`, then each record of a run at `run_records/&lt;run_id&gt;/` and the path the index lists</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t xml:space="preserve">a route per snapshot; a directory listed; a path outside the three prefixes answered; a server that computes, writes or proxies; `dashboard.py`, `proxy.py`, `server.py` beside `serve.py`</t>
-        </is>
-      </c>
-      <c r="I430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`http.server`</t>
+          <t xml:space="preserve">an absolute path; a route per snapshot; a directory listing; a store the page reads beside these two</t>
         </is>
       </c>
     </row>
@@ -16716,17 +16711,22 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t xml:space="preserve">the toolkit the page loads before its own sections</t>
+          <t xml:space="preserve">the three prefixes: what the dashboard's server answers — the page's own files at `/`, the status store under `/status/`, the run-records store under `/run_records/`; every other path 404, and no directory listed</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t xml:space="preserve">`page.js`</t>
+          <t xml:space="preserve">`module_monitoring/serve.py` — `DashboardHandler`, `translate_path()`, `main()`; `STORE_DIR_BY_ROUTE_PREFIX` in `module_monitoring/config.py`, `/status/` onto `STORE_STATUS_DIR` and `/run_records/` onto `STORE_RUN_RECORDS_DIR`; `MODULE_MONITORING_DIR`, `PAGE_FILE_SUFFIXES`, `PAGE_INDEX_FILE_NAME` for the page's own files</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t xml:space="preserve">`utils.js`, `common.js`, `shared.js`, `lib.js`; a page-specific element written from it; a second page beside the status page</t>
+          <t xml:space="preserve">a route per snapshot; a directory listed; a path outside the three prefixes answered; a server that computes, writes or proxies; `dashboard.py`, `proxy.py`, `server.py` beside `serve.py`</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`http.server`</t>
         </is>
       </c>
     </row>
@@ -16738,17 +16738,17 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one selector component of the page — the top tabs, the ML Assets views, the asset rows — each group wired by its `data-key`</t>
+          <t xml:space="preserve">the toolkit the page loads before its own sections</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.pills`, `.pill`, `.pill--active`, `initPills()`, `PILL_HOOKS` in `page.js`; `data-pills` on a group, `data-panel` on its panels</t>
+          <t xml:space="preserve">`page.js`</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second selector component</t>
+          <t xml:space="preserve">`utils.js`, `common.js`, `shared.js`, `lib.js`; a page-specific element written from it; a second page beside the status page</t>
         </is>
       </c>
     </row>
@@ -16760,44 +16760,44 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page's navigation: the seven tabs, the five views of the ML Assets tab, and one row per asset</t>
+          <t xml:space="preserve">the one selector component of the page — the top tabs, the ML Assets views, the asset rows — each group wired by its `data-key`</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t xml:space="preserve">the groups of `data-pills` in `module_monitoring/index.html` — `tab`: `pipeline`, `quality`, `features`, `ml`, `asset`, `scalability`, `lifecycle`; `mlview`: `labels`, `classification`, `strategy`, `search`, `feature-set`; `asset`, filled from the snapshot</t>
-        </is>
-      </c>
-      <c r="E433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pipeline; Data Quality; Features; ML Research; ML Assets; Scalability; Lifecycle — Labels &amp; data; Classification; Strategy; HPO; Feature set</t>
+          <t xml:space="preserve">`.pills`, `.pill`, `.pill--active`, `initPills()`, `PILL_HOOKS` in `page.js`; `data-pills` on a group, `data-panel` on its panels</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t xml:space="preserve">a menu, a sidebar or a second navigation; a tab named for a tool</t>
+          <t xml:space="preserve">a second selector component</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scalability crawler</t>
+          <t xml:space="preserve">The page</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t xml:space="preserve">the crawler: the canon's sub-module that reads each controlled file against the Skills marked for it with the one active vendor, and writes a report per file and its snapshot; it asks nothing, goes on past a failed file and gates nothing</t>
+          <t xml:space="preserve">the page's navigation: the seven tabs, the five views of the ML Assets tab, and one row per asset</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_scalability_crawler`; `make skills-crawl`, after `make skills-sync`; `main()` in `crawl.py`</t>
+          <t xml:space="preserve">the groups of `data-pills` in `module_monitoring/index.html` — `tab`: `pipeline`, `quality`, `features`, `ml`, `asset`, `scalability`, `lifecycle`; `mlview`: `labels`, `classification`, `strategy`, `search`, `feature-set`; `asset`, filled from the snapshot</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pipeline; Data Quality; Features; ML Research; ML Assets; Scalability; Lifecycle — Labels &amp; data; Classification; Strategy; HPO; Feature set</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t xml:space="preserve">a linter, a check, a gate, a CI step; a web crawler, walking sites or services to gather what they hold; conformance, review — names that tell a reader nothing; a TUI of its own, `make skills-terminal` being the canon's terminal</t>
+          <t xml:space="preserve">a menu, a sidebar or a second navigation; a tab named for a tool</t>
         </is>
       </c>
     </row>
@@ -16809,22 +16809,17 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t xml:space="preserve">the files matrix: a row per path — a file or a glob — a column per Skill headed by its stem, an `X` where that Skill is sent with the file; the crawler's whole contract</t>
+          <t xml:space="preserve">the crawler: the canon's sub-module that reads each controlled file against the Skills marked for it with the one active vendor, and writes a report per file and its snapshot; it asks nothing, goes on past a failed file and gates nothing</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t xml:space="preserve">the table of the sheet headed by `FILES_MATRIX_HEADER` in `module_skills/config.py`; `Mark` in `module_skills/sheet.py`</t>
-        </is>
-      </c>
-      <c r="E435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">path; the Skill's stem; `X`</t>
+          <t xml:space="preserve">`sub_module_scalability_crawler`; `make skills-crawl`, after `make skills-sync`; `main()` in `crawl.py`</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column per rule; a mark a crawl writes; a mark derived from `scope`; a generated file, a report or the snapshot as a target; a second row for one path; a precedence between rows; a Markdown table kept beside the crawler</t>
+          <t xml:space="preserve">a linter, a check, a gate, a CI step; a web crawler, walking sites or services to gather what they hold; conformance, review — names that tell a reader nothing; a TUI of its own, `make skills-terminal` being the canon's terminal</t>
         </is>
       </c>
     </row>
@@ -16836,22 +16831,22 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t xml:space="preserve">a mark: `X` under a Skill's column in a row of the files matrix, sending that Skill with every file the row reaches; two rows that reach one file join their marks</t>
+          <t xml:space="preserve">the files matrix: a row per path — a file or a glob — a column per Skill headed by its stem, an `X` where that Skill is sent with the file; the crawler's whole contract</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILL_MARK` in `module_skills/config.py`</t>
+          <t xml:space="preserve">the table of the sheet headed by `FILES_MATRIX_HEADER` in `module_skills/config.py`; `Mark` in `module_skills/sheet.py`</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t xml:space="preserve">`X`; marked; unmarked</t>
+          <t xml:space="preserve">path; the Skill's stem; `X`</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t xml:space="preserve">assign, tag, tick, check, enable; `x`, `✓` or `yes` in a cell; a mark a crawl writes; a mark derived from `scope`; a row that marks no Skill</t>
+          <t xml:space="preserve">a column per rule; a mark a crawl writes; a mark derived from `scope`; a generated file, a report or the snapshot as a target; a second row for one path; a precedence between rows; a Markdown table kept beside the crawler</t>
         </is>
       </c>
     </row>
@@ -16863,22 +16858,22 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t xml:space="preserve">a controlled file: a file a row of the files matrix reaches, read against the Skills marked for it; its key is its path from the root of the tree</t>
+          <t xml:space="preserve">a mark: `X` under a Skill's column in a row of the files matrix, sending that Skill with every file the row reaches; two rows that reach one file join their marks</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ControlledFile`, `build_controlled_files()` in `crawl.py`</t>
+          <t xml:space="preserve">`SKILL_MARK` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">`X`; marked; unmarked</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t xml:space="preserve">listed file; a file the crawler finds by itself; a file read from the working directory; a rendered Skill or the snapshot as a controlled file</t>
+          <t xml:space="preserve">assign, tag, tick, check, enable; `x`, `✓` or `yes` in a cell; a mark a crawl writes; a mark derived from `scope`; a row that marks no Skill</t>
         </is>
       </c>
     </row>
@@ -16890,17 +16885,22 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t xml:space="preserve">the context: the documents sent with a file — the Skills its row of the files matrix marks, each whole as `make skills-sync` rendered it</t>
+          <t xml:space="preserve">a controlled file: a file a row of the files matrix reaches, read against the Skills marked for it; its key is its path from the root of the tree</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_skill_texts()`, `build_message()` in `crawl.py`</t>
+          <t xml:space="preserve">`ControlledFile`, `build_controlled_files()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule filtered out by its `scope` before it is sent; a Skill not marked; the contract; an orientation; a methodology; a list of rules kept per module</t>
+          <t xml:space="preserve">listed file; a file the crawler finds by itself; a file read from the working directory; a rendered Skill or the snapshot as a controlled file</t>
         </is>
       </c>
     </row>
@@ -16912,17 +16912,17 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t xml:space="preserve">a file's message: the Skills marked for it, then the file with every line after its number, then the mission</t>
+          <t xml:space="preserve">the context: the documents sent with a file — the Skills its row of the files matrix marks, each whole as `make skills-sync` rendered it</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_message()` in `crawl.py`; `crawlers_mission.md`</t>
+          <t xml:space="preserve">`load_skill_texts()`, `build_message()` in `crawl.py`</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t xml:space="preserve">a list of unmarked Skills; an orientation; a commit; a measure of the message; a line number the agent has to count</t>
+          <t xml:space="preserve">a rule filtered out by its `scope` before it is sent; a Skill not marked; the contract; an orientation; a methodology; a list of rules kept per module</t>
         </is>
       </c>
     </row>
@@ -16934,17 +16934,17 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mission: what the agent reports of one file, and how — kept by hand</t>
+          <t xml:space="preserve">a file's message: the Skills marked for it, then the file with every line after its number, then the mission</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t xml:space="preserve">`crawlers_mission.md`, `CRAWLERS_MISSION_MD_PATH`</t>
+          <t xml:space="preserve">`build_message()` in `crawl.py`; `crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule restated in it; a work order or a plan</t>
+          <t xml:space="preserve">a list of unmarked Skills; an orientation; a commit; a measure of the message; a line number the agent has to count</t>
         </is>
       </c>
     </row>
@@ -16956,17 +16956,17 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sub-module's folder and the root of the tree: where the crawler's own files are read, and where a controlled file and a Skill lie and the vendor runs</t>
+          <t xml:space="preserve">the mission: what the agent reports of one file, and how — kept by hand</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SUB_MODULE_DIR` in the crawler's `config.py`; `TREE_ROOT_DIR` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`crawlers_mission.md`, `CRAWLERS_MISSION_MD_PATH`</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t xml:space="preserve">a host path; a controlled file read from the working directory</t>
+          <t xml:space="preserve">a rule restated in it; a work order or a plan</t>
         </is>
       </c>
     </row>
@@ -16978,22 +16978,17 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t xml:space="preserve">a vendor: an agent's command line the crawl sends each controlled file to — one table of `vendors_for_crawling.toml`, exactly one `active`, its `argv` the whole command line, run without a shell, the message on its stdin and the answer its stdout</t>
+          <t xml:space="preserve">the sub-module's folder and the root of the tree: where the crawler's own files are read, and where a controlled file and a Skill lie and the vendor runs</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t xml:space="preserve">`vendors_for_crawling.toml` with `active`, `argv`; `VENDORS_FOR_CRAWLING_TOML_PATH`, `load_vendor()`, `AGENT_TIMEOUT_SECONDS`</t>
-        </is>
-      </c>
-      <c r="E442" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vendor</t>
+          <t xml:space="preserve">`SUB_MODULE_DIR` in the crawler's `config.py`; `TREE_ROOT_DIR` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t xml:space="preserve">an API key; a vendor named in the code; a form for its model, effort or permissions; a vendor chosen on a screen; two active vendors; every vendor run in turn</t>
+          <t xml:space="preserve">a host path; a controlled file read from the working directory</t>
         </is>
       </c>
     </row>
@@ -17005,27 +17000,22 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t xml:space="preserve">a report: the one current file per controlled file — the file's key, the vendor and the time, then the answer as it came; reset by every crawl, never tracked</t>
+          <t xml:space="preserve">a vendor: an agent's command line the crawl sends each controlled file to — one table of `vendors_for_crawling.toml`, exactly one `active`, its `argv` the whole command line, run without a shell, the message on its stdin and the answer its stdout</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t xml:space="preserve">`REPORTS_DIR`, `report_path()` in the crawler's `config.py` — `store/status/reports_after_crawled_files/&lt;path&gt;.report.md`; `write_atomically()` in `status.py`</t>
-        </is>
-      </c>
-      <c r="D443" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`report`</t>
+          <t xml:space="preserve">`vendors_for_crawling.toml` with `active`, `argv`; `VENDORS_FOR_CRAWLING_TOML_PATH`, `load_vendor()`, `AGENT_TIMEOUT_SECONDS`</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">vendor</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t xml:space="preserve">a history of entries; an append; a report in the sub-module's folder; a commit in its first line; a report tracked</t>
+          <t xml:space="preserve">an API key; a vendor named in the code; a form for its model, effort or permissions; a vendor chosen on a screen; two active vendors; every vendor run in turn</t>
         </is>
       </c>
     </row>
@@ -17037,17 +17027,27 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t xml:space="preserve">a finding: one line of a report, `rule_id | file:line | problem | correction`; `OK` the answer of a file that departs from nothing</t>
+          <t xml:space="preserve">a report: the one current file per controlled file — the file's key, the vendor and the time, then the answer as it came; reset by every crawl, never tracked</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t xml:space="preserve">`crawlers_mission.md`</t>
+          <t xml:space="preserve">`REPORTS_DIR`, `report_path()` in the crawler's `config.py` — `store/status/reports_after_crawled_files/&lt;path&gt;.report.md`; `write_atomically()` in `status.py`</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`report`</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">report</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t xml:space="preserve">a finding without a `rule_id`; a rule that was not sent; a table; `conformant` as a line</t>
+          <t xml:space="preserve">a history of entries; an append; a report in the sub-module's folder; a commit in its first line; a report tracked</t>
         </is>
       </c>
     </row>
@@ -17059,27 +17059,17 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t xml:space="preserve">a controlled file's state: where its crawl stands — `pending` before, `running` while the vendor works, `done` once its report is written, `failed` otherwise, `interrupted` where Ctrl-C ended it</t>
+          <t xml:space="preserve">a finding: one line of a report, `rule_id | file:line | problem | correction`; `OK` the answer of a file that departs from nothing</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t xml:space="preserve">`row()` in `status.py`; `main()` in `crawl.py`</t>
-        </is>
-      </c>
-      <c r="D445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`state`</t>
-        </is>
-      </c>
-      <c r="E445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pending; running; done; failed; interrupted</t>
+          <t xml:space="preserve">`crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t xml:space="preserve">`done` read as conformant — it says the report was written; a change of state left out of the snapshot</t>
+          <t xml:space="preserve">a finding without a `rule_id`; a rule that was not sent; a table; `conformant` as a line</t>
         </is>
       </c>
     </row>
@@ -17091,22 +17081,27 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t xml:space="preserve">the crawl's progress: one line per controlled file after its result, then one closing line; the reason a file failed one line on stderr</t>
+          <t xml:space="preserve">a controlled file's state: where its crawl stands — `pending` before, `running` while the vendor works, `done` once its report is written, `failed` otherwise, `interrupted` where Ctrl-C ended it</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t xml:space="preserve">`main()` in `crawl.py`</t>
+          <t xml:space="preserve">`row()` in `status.py`; `main()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`state`</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;current&gt;/&lt;total&gt; | &lt;controlled file&gt; | &lt;vendor&gt; | &lt;state&gt;`; `&lt;processed&gt;/&lt;total&gt; | crawl | &lt;vendor&gt; | done`, `failed` or `interrupted`</t>
+          <t xml:space="preserve">pending; running; done; failed; interrupted</t>
         </is>
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t xml:space="preserve">a spinner, a progress bar, a percentage; an answer summarised on the screen — the report holds it; a results table</t>
+          <t xml:space="preserve">`done` read as conformant — it says the report was written; a change of state left out of the snapshot</t>
         </is>
       </c>
     </row>
@@ -17118,17 +17113,22 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t xml:space="preserve">the refusals and the exits: a state the crawler cannot read ends it in one named line before anything is reset; a file the vendor fails is `failed` and the crawl goes on — 0 every file done, 1 a refusal or a failed file, 130 Ctrl-C</t>
+          <t xml:space="preserve">the crawl's progress: one line per controlled file after its result, then one closing line; the reason a file failed one line on stderr</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SystemExit` in `module_skills/sheet.py`, `module_skills/sync.py` and the crawler's `crawl.py`</t>
+          <t xml:space="preserve">`main()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`&lt;current&gt;/&lt;total&gt; | &lt;controlled file&gt; | &lt;vendor&gt; | &lt;state&gt;`; `&lt;processed&gt;/&lt;total&gt; | crawl | &lt;vendor&gt; | done`, `failed` or `interrupted`</t>
         </is>
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t xml:space="preserve">a traceback for an expected failure; exit 0 after a failure; a crawl that stops at the first failed file</t>
+          <t xml:space="preserve">a spinner, a progress bar, a percentage; an answer summarised on the screen — the report holds it; a results table</t>
         </is>
       </c>
     </row>
@@ -17140,27 +17140,17 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t xml:space="preserve">the snapshot: `skills_status.json`, the current state of every controlled file, sorted by path and rewritten whole at every change; tracked in its neutral state, every controlled file `pending` with no report</t>
+          <t xml:space="preserve">the refusals and the exits: a state the crawler cannot read ends it in one named line before anything is reset; a file the vendor fails is `failed` and the crawl goes on — 0 every file done, 1 a refusal or a failed file, 130 Ctrl-C</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILLS_STATUS_JSON_PATH` in the crawler's `config.py`; `row()`, `write_skills_status()`, `write_atomically()` in `status.py`</t>
-        </is>
-      </c>
-      <c r="D448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`files`, each `path`, `state`, `vendor`, `finished_at_utc`, `report`</t>
-        </is>
-      </c>
-      <c r="E448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">file; state; vendor; finished_at_utc; report</t>
+          <t xml:space="preserve">`SystemExit` in `module_skills/sheet.py`, `module_skills/sync.py` and the crawler's `crawl.py`</t>
         </is>
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t xml:space="preserve">a count of crawls; an age; a clock but `finished_at_utc`; a snapshot that reads itself back; a partial file</t>
+          <t xml:space="preserve">a traceback for an expected failure; exit 0 after a failure; a crawl that stops at the first failed file</t>
         </is>
       </c>
     </row>
@@ -17172,104 +17162,136 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
+          <t xml:space="preserve">the snapshot: `skills_status.json`, the current state of every controlled file, sorted by path and rewritten whole at every change; tracked in its neutral state, every controlled file `pending` with no report</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`SKILLS_STATUS_JSON_PATH` in the crawler's `config.py`; `row()`, `write_skills_status()`, `write_atomically()` in `status.py`</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`files`, each `path`, `state`, `vendor`, `finished_at_utc`, `report`</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">file; state; vendor; finished_at_utc; report</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a count of crawls; an age; a clock but `finished_at_utc`; a snapshot that reads itself back; a partial file</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scalability crawler</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
           <t xml:space="preserve">the page's view of the reports</t>
         </is>
       </c>
-      <c r="C449" t="inlineStr">
+      <c r="C450" t="inlineStr">
         <is>
           <t xml:space="preserve">`scalability.js` — `SKILLS_STATUS`, `renderCrawlState()`</t>
         </is>
       </c>
-      <c r="E449" t="inlineStr">
+      <c r="E450" t="inlineStr">
         <is>
           <t xml:space="preserve">Scalability — CRAWL STATE</t>
         </is>
       </c>
-      <c r="F449" t="inlineStr">
+      <c r="F450" t="inlineStr">
         <is>
           <t xml:space="preserve">a tab named for a tool; scale for a larger basket, which is `ASSET=&lt;TICKER&gt;`</t>
-        </is>
-      </c>
-    </row>
-    <row r="451">
-      <c r="A451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rule_type_id</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t xml:space="preserve">Architecture</t>
+          <t xml:space="preserve">rule_type_id</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t xml:space="preserve">Naming</t>
+          <t xml:space="preserve">Architecture</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conformities</t>
+          <t xml:space="preserve">Naming</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t xml:space="preserve">Workflow</t>
+          <t xml:space="preserve">Conformities</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t xml:space="preserve">FileLayout</t>
+          <t xml:space="preserve">Workflow</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t xml:space="preserve">UI_TUI</t>
+          <t xml:space="preserve">FileLayout</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scalability</t>
+          <t xml:space="preserve">UI_TUI</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t xml:space="preserve">Complexity</t>
+          <t xml:space="preserve">Scalability</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t xml:space="preserve">Determinism</t>
+          <t xml:space="preserve">Complexity</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t xml:space="preserve">Performance</t>
+          <t xml:space="preserve">Determinism</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
         <is>
           <t xml:space="preserve">Methodology</t>
         </is>

</xml_diff>

<commit_message>
Remove the copies and parts nothing reads, and give the active set one reader
Gone: module_data's BYTES_PER_KIBIBYTE, the search's derived
SERPENTINE_SEARCH_ROUND_LOOPS, gum_filter(), the CRAWLING, NOT CRAWLED and
FAILED states and gum_input's value in the five tui.py, score's rebuild flag and
the REBUILD_* constants, and the crawler's second atomic writer — it writes
through sync.write_text(). The search reads the asset's state with the verb its
layer asks for: load_feature_columns(), registered as the ML dataset's twin,
load_barrier_coordinates() and load_best_params(). An unknown kind of scoring is
refused in one line. The CONFIGURABLES headers name their registered copies, and
the HPO block drops its postponed clause.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -1120,7 +1120,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME` read off the records and published as `default_columns_by_timeframe` in `&lt;TICKER&gt;_catalogue.json`; `active_columns()` returning it where the asset has no promoted file, else the file's columns in catalogue order; a flag turned `True` a change of the frozen experiment for every asset without a promoted set, never a setting of one asset.</t>
+          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME` read off the records and published as `default_columns_by_timeframe` in `&lt;TICKER&gt;_catalogue.json`; `load_feature_columns()` returning it where the asset has no promoted file, else the file's columns in catalogue order; a flag turned `True` a change of the frozen experiment for every asset without a promoted set, never a setting of one asset.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -7172,7 +7172,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t xml:space="preserve">`gum_&lt;subcommand&gt;` — `gum_table()`, `gum_style()`, `gum_choose()`, `gum_filter()`, `gum_input()` — and `_gum()`, the one private call that runs a prompt and returns its answer; never `render_`, `show_`, `print_` or `draw_`.</t>
+          <t xml:space="preserve">`gum_&lt;subcommand&gt;` — `gum_table()`, `gum_style()`, `gum_choose()`, `gum_input()` — and `_gum()`, the one private call that runs a prompt and returns its answer; never `render_`, `show_`, `print_` or `draw_`.</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -7421,7 +7421,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Each role on a screen takes one instrument: a block for the context and the outcome, a printed table for rows read, a choice for every decision, a filter for a value of a set too long to list, an input for a line no list can offer, and a printed line for one fact.</t>
+          <t xml:space="preserve">Each role on a screen takes one instrument: a block for the context and the outcome, a printed table for rows read, a choice for every decision, an input for a line no list can offer, and a printed line for one fact.</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t xml:space="preserve">`gum style` in a rounded border for the header block, the `DONE` block and the failure, never a banner, a block inside a block or a block around a table; `gum table --print`, never the interactive table; `gum choose` for the menu, the asset, each form and every gate, never `gum confirm`; `gum filter` without `--no-strict`, its placeholder the caller's; `gum input` only for what no list of the tree holds, the assets a direct call did not name; Python's `print` for a fact beside a table, the `CURRENT` line of a command, `WARN` and `CANCELLED`; never `gum spin`.</t>
+          <t xml:space="preserve">`gum style` in a rounded border for the header block, the `DONE` block and the failure, never a banner, a block inside a block or a block around a table; `gum table --print`, never the interactive table; `gum choose` for the menu, the asset, each form and every gate, never `gum confirm`; `gum input` only for what no list of the tree holds, the assets a direct call did not name; Python's `print` for a fact beside a table, the `CURRENT` line of a command, `WARN` and `CANCELLED`; never `gum spin`.</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every state drawn by `state_label()` from a key of `STATE_SYMBOLS`: `DONE` an action carried out or a step answered, `CURRENT` what is asked or started now, `PENDING` a step still to come, `WARN` what an action will overwrite, `CANCELLED` Esc, `cancel`, `quit` or Ctrl-C with nothing more written, `FAILED` one item not carried out, `ERROR` the failure that ends the run; never a colour or a symbol without its word, a coloured row, or `running`, `ok` or `success` as a state of the screen — a state a file holds, the crawl snapshot's among them, is a value shown as the file holds it.</t>
+          <t xml:space="preserve">Every state drawn by `state_label()` from a key of `STATE_SYMBOLS`: `DONE` an action carried out or a step answered, `CURRENT` what is asked or started now, `PENDING` a step still to come, `WARN` what an action will overwrite, `CANCELLED` Esc, `cancel`, `quit` or Ctrl-C with nothing more written, `ERROR` the failure that ends the run; never a colour or a symbol without its word, a coloured row, or `running`, `ok` or `success` as a state of the screen — a state a file holds, the crawl snapshot's among them, is a value shown as the file holds it.</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -13133,12 +13133,12 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/config.py`, `module_ml/config.py`; the browser's own in `module_monitoring/page.js`</t>
+          <t xml:space="preserve">`module_ml/config.py`; the browser's own in `module_monitoring/page.js`</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t xml:space="preserve">a unit, like the unit constants: the data and ML modules and the page each size a file, and none of them imports another</t>
+          <t xml:space="preserve">a unit, like the unit constants: the ML module and the page each size a file, and neither imports the other</t>
         </is>
       </c>
     </row>
@@ -13815,17 +13815,17 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_set_json()`, `barriers_json()`, `hyperparameter_point_json()` — equal by value</t>
+          <t xml:space="preserve">`load_feature_columns()` — equal by value</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`, `module_features/sub_module_terminal/config.py`, each over its own `artifact_dir()` or its module's</t>
+          <t xml:space="preserve">`module_ml/dataset.py`; `module_features/sub_module_serpentine_search/serpentine_search.py`</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion writes the three, the ML chain reads them and the serpentine search the first two, and the features terminal names them on its promotion screen; the writer and the reader of a boundary must name one artifact, and the terminal cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the asset's feature set — the promoted file's columns in catalogue order, else the default set — is read by the chain that fits it and by the search that starts from it, and neither module imports the other</t>
         </is>
       </c>
     </row>
@@ -13837,17 +13837,17 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t xml:space="preserve">`theta()`, `state_key()` — identical</t>
+          <t xml:space="preserve">`feature_set_json()`, `barriers_json()`, `hyperparameter_point_json()` — equal by value</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_ml/score.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`, `module_features/sub_module_terminal/config.py`, each over its own `artifact_dir()` or its module's</t>
         </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t xml:space="preserve">the serpentine search keys a state to know whether it has scored it, and the module that scores names the parent of a study by the same key: one differing separator and every answer would look like the answer to another question</t>
+          <t xml:space="preserve">the promotion writes the three, the ML chain reads them and the serpentine search the first two, and the features terminal names them on its promotion screen; the writer and the reader of a boundary must name one artifact, and the terminal cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13859,7 +13859,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t xml:space="preserve">`KIND_SCORE`, `KIND_HYPERPARAMETER` — identical</t>
+          <t xml:space="preserve">`theta()`, `state_key()` — identical</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -13869,7 +13869,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t xml:space="preserve">the two kinds of question: one side writes the word into a request and the other branches on it, so one word apart and every question would be answered as the other kind or refused</t>
+          <t xml:space="preserve">the serpentine search keys a state to know whether it has scored it, and the module that scores names the parent of a study by the same key: one differing separator and every answer would look like the answer to another question</t>
         </is>
       </c>
     </row>
@@ -13881,17 +13881,17 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t xml:space="preserve">`serpentine_search_json()`, `serpentine_search_trials_jsonl()`, `serpentine_search_profile_json()` — equal by value</t>
+          <t xml:space="preserve">`KIND_SCORE`, `KIND_HYPERPARAMETER` — identical</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, over its module's `artifact_dir()`; `module_features/sub_module_terminal/config.py`, over its own</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_ml/score.py`</t>
         </is>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal reads the state and the ledger and writes the profile on the host's `python3`, and the sub-module's `config.py` imports the module's, which imports numpy</t>
+          <t xml:space="preserve">the two kinds of question: one side writes the word into a request and the other branches on it, so one word apart and every question would be answered as the other kind or refused</t>
         </is>
       </c>
     </row>
@@ -13903,17 +13903,17 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SERPENTINE_SEARCH_ROUND_LOOPS` — equal by value</t>
+          <t xml:space="preserve">`serpentine_search_json()`, `serpentine_search_trials_jsonl()`, `serpentine_search_profile_json()` — equal by value</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, derived from `ROUND_SCHEDULE`; `module_features/sub_module_terminal/config.py`, written out</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, over its module's `artifact_dir()`; `module_features/sub_module_terminal/config.py`, over its own</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t xml:space="preserve">the loops a round runs, in its order: the features terminal offers them to a draft, and it cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the features terminal reads the state and the ledger and writes the profile on the host's `python3`, and the sub-module's `config.py` imports the module's, which imports numpy</t>
         </is>
       </c>
     </row>
@@ -13925,17 +13925,17 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`, `PROMOTE_TARGET` — equal by value</t>
+          <t xml:space="preserve">`SERPENTINE_SEARCH_ROUND_LOOPS` — equal by value to the loops of `ROUND_SCHEDULE`</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONFIGURABLES records of `module_features/sub_module_serpentine_search/config.py`; constants of `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_terminal/config.py`, written out; `ROUND_SCHEDULE` in `module_features/sub_module_serpentine_search/config.py`, its loops in their order</t>
         </is>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal offers the grid to a draft and opens its own screen for the promotion's target on the host's `python3`, and cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the loops a round runs, in its order: the features terminal offers them to a draft, and it cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13947,17 +13947,17 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t xml:space="preserve">`tui.py`, the whole file — the gum layer of every terminal</t>
+          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`, `PROMOTE_TARGET` — equal by value</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical to the byte in `module_data/sub_module_terminal/tui.py`, `module_features/sub_module_terminal/tui.py`, `module_ml/sub_module_terminal/tui.py`, `module_monitoring/sub_module_terminal/tui.py`, `module_skills/sub_module_terminal/tui.py`</t>
+          <t xml:space="preserve">CONFIGURABLES records of `module_features/sub_module_serpentine_search/config.py`; constants of `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t xml:space="preserve">one module speaks gum in each, and a package for what the terminals share would make every module import `module_skills` (`AGENTS.md` D02). It holds no sentence about a screen's content — a placeholder, a header and a state's words are the caller's; its own words are the block labels and the line naming the columns a narrow terminal leaves out — so each owner holds the file as its own local adapter</t>
+          <t xml:space="preserve">the features terminal offers the grid to a draft and opens its own screen for the promotion's target on the host's `python3`, and cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13969,17 +13969,17 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OUTPUT_PLAIN` and the three conditions it reads — `NO_COLOR`, `TERM`, `sys.stdout.isatty()`</t>
+          <t xml:space="preserve">`tui.py`, the whole file — the gum layer of every terminal</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/config.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`, `module_skills/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">identical to the byte in `module_data/sub_module_terminal/tui.py`, `module_features/sub_module_terminal/tui.py`, `module_ml/sub_module_terminal/tui.py`, `module_monitoring/sub_module_terminal/tui.py`, `module_skills/sub_module_terminal/tui.py`</t>
         </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t xml:space="preserve">plain output follows the environment and is never a flag; each `tui.py` reads its own sub-module's `config.py`, and no module imports another</t>
+          <t xml:space="preserve">one module speaks gum in each, and a package for what the terminals share would make every module import `module_skills` (`AGENTS.md` D02). It holds no sentence about a screen's content — a placeholder, a header and a state's words are the caller's; its own words are the block labels and the line naming the columns a narrow terminal leaves out — so each owner holds the file as its own local adapter</t>
         </is>
       </c>
     </row>
@@ -13991,17 +13991,17 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t xml:space="preserve">the screen helpers `_option_rows()`, `_cancelled_exit_code()`, `_failure_exit_code()`</t>
+          <t xml:space="preserve">`OUTPUT_PLAIN` and the three conditions it reads — `NO_COLOR`, `TERM`, `sys.stdout.isatty()`</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`, `module_monitoring/sub_module_terminal/terminal.py`, `module_skills/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/config.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`, `module_skills/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t xml:space="preserve">every terminal uses the same outcome and option conventions, and no terminal imports another module's code; a terminal that asks more than two forms keeps its own step helpers, in its own words</t>
+          <t xml:space="preserve">plain output follows the environment and is never a flag; each `tui.py` reads its own sub-module's `config.py`, and no module imports another</t>
         </is>
       </c>
     </row>
@@ -14013,7 +14013,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_make()`</t>
+          <t xml:space="preserve">the screen helpers `_option_rows()`, `_cancelled_exit_code()`, `_failure_exit_code()`</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -14023,7 +14023,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one call of make — a terminal starts a target through it and no other way, its lines uncaptured; it takes its arguments open, `_make(*arguments)`, so a target alone and a target with its asset — the promotion's among them — pass through one signature</t>
+          <t xml:space="preserve">every terminal uses the same outcome and option conventions, and no terminal imports another module's code; a terminal that asks more than two forms keeps its own step helpers, in its own words</t>
         </is>
       </c>
     </row>
@@ -14035,7 +14035,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()`</t>
+          <t xml:space="preserve">`_make()`</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -14045,7 +14045,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one reading of make — the menu is the Makefile's own targets, read from `make help` and filtered by the terminal's `MENU_TARGET_PATTERN`, so a terminal keeps no second list of them and a target gains its option by carrying a `##`</t>
+          <t xml:space="preserve">the one call of make — a terminal starts a target through it and no other way, its lines uncaptured; it takes its arguments open, `_make(*arguments)`, so a target alone and a target with its asset — the promotion's among them — pass through one signature</t>
         </is>
       </c>
     </row>
@@ -14057,7 +14057,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_target()`</t>
+          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()`</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -14067,7 +14067,7 @@
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t xml:space="preserve">one plan, one gate and one call for every target a menu offers; each owner holds its own local adapter with the same signature</t>
+          <t xml:space="preserve">the one reading of make — the menu is the Makefile's own targets, read from `make help` and filtered by the terminal's `MENU_TARGET_PATTERN`, so a terminal keeps no second list of them and a target gains its option by carrying a `##`</t>
         </is>
       </c>
     </row>
@@ -14079,17 +14079,17 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_tickers()`</t>
+          <t xml:space="preserve">`_write_target()`</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`, `module_monitoring/sub_module_terminal/terminal.py`, `module_skills/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three terminals whose module takes an asset read the assets `--tickers` names and ask for them only when a direct run named none; no module defines a basket of its own, and no terminal imports another module's code</t>
+          <t xml:space="preserve">one plan, one gate and one call for every target a menu offers; each owner holds its own local adapter with the same signature</t>
         </is>
       </c>
     </row>
@@ -14101,7 +14101,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_present()`</t>
+          <t xml:space="preserve">`_tickers()`</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -14111,34 +14111,29 @@
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three terminals whose module keeps an asset's files answer whether one stands in the same word, and a terminal reads another module's files through none of that module's code</t>
+          <t xml:space="preserve">the three terminals whose module takes an asset read the assets `--tickers` names and ask for them only when a direct run named none; no module defines a basket of its own, and no terminal imports another module's code</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t xml:space="preserve">Terminals</t>
+          <t xml:space="preserve">Twice by extraction</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t xml:space="preserve">a module's terminal: the sub-module that shows what the module's stores hold — per asset where the module takes one — and starts one of the module's own targets through `make`; outside an action it creates no domain state, and it gates nothing</t>
+          <t xml:space="preserve">`_present()`</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_terminal` — `module_data/sub_module_terminal/`, `module_features/sub_module_terminal/`, `module_ml/sub_module_terminal/`, `module_monitoring/sub_module_terminal/` and the canon's `module_skills/sub_module_terminal/`, each `terminal.py` with `main()`, `config.py` and `tui.py`</t>
-        </is>
-      </c>
-      <c r="E327" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Data terminal; Features terminal; ML terminal; Monitoring terminal; Skills terminal</t>
-        </is>
-      </c>
-      <c r="F327" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a cockpit, a console, a dashboard; a second terminal in one module; a TUI that computes, schedules or gates; `&lt;module&gt;-tui`, `&lt;module&gt;-menu`; the crawler drawing a terminal of its own</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the three terminals whose module keeps an asset's files answer whether one stands in the same word, and a terminal reads another module's files through none of that module's code</t>
         </is>
       </c>
     </row>
@@ -14150,17 +14145,22 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t xml:space="preserve">a terminal's entry: the one make target that opens it, run by `python3` on the host and never in a container; it carries no `##`, so it is no option of any menu</t>
+          <t xml:space="preserve">a module's terminal: the sub-module that shows what the module's stores hold — per asset where the module takes one — and starts one of the module's own targets through `make`; outside an action it creates no domain state, and it gates nothing</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make data-terminal`, `make features-terminal`, `make ml-terminal`, `make monitoring-terminal`, `make skills-terminal`; the three whose module takes an asset given `--tickers` from `ASSET` or `TICKERS_CSV`</t>
+          <t xml:space="preserve">`sub_module_terminal` — `module_data/sub_module_terminal/`, `module_features/sub_module_terminal/`, `module_ml/sub_module_terminal/`, `module_monitoring/sub_module_terminal/` and the canon's `module_skills/sub_module_terminal/`, each `terminal.py` with `main()`, `config.py` and `tui.py`</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data terminal; Features terminal; ML terminal; Monitoring terminal; Skills terminal</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `##` on an entry; a `tmux-` twin of a terminal; `make tui`; a terminal started in a runner</t>
+          <t xml:space="preserve">a cockpit, a console, a dashboard; a second terminal in one module; a TUI that computes, schedules or gates; `&lt;module&gt;-tui`, `&lt;module&gt;-menu`; the crawler drawing a terminal of its own</t>
         </is>
       </c>
     </row>
@@ -14172,17 +14172,17 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t xml:space="preserve">a terminal's sources: what a terminal reads</t>
+          <t xml:space="preserve">a terminal's entry: the one make target that opens it, run by `python3` on the host and never in a container; it carries no `##`, so it is no option of any menu</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t xml:space="preserve">its own module's `config.py` where that is standard library — the data terminal's, with `lean.py`, and the ML terminal's; the features terminal its own `config.py`'s copies, `module_features/config.py` importing numpy; the monitoring terminal the snapshots through `STORE_STATUS_DIR` and `SNAPSHOT_FILE_NAMES` of its own `config.py`; the skills terminal the canon's `config.py` and, through the crawler's `config.py`, `vendors_for_crawling.toml` and the snapshot; every terminal `make help`</t>
+          <t xml:space="preserve">`make data-terminal`, `make features-terminal`, `make ml-terminal`, `make monitoring-terminal`, `make skills-terminal`; the three whose module takes an asset given `--tickers` from `ASSET` or `TICKERS_CSV`</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t xml:space="preserve">a snapshot read for freshness; duckdb; a store literal; another module's code; a third-party package</t>
+          <t xml:space="preserve">a `##` on an entry; a `tmux-` twin of a terminal; `make tui`; a terminal started in a runner</t>
         </is>
       </c>
     </row>
@@ -14194,22 +14194,17 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t xml:space="preserve">the menu: the options a terminal offers — one per target of the one Makefile that carries a `##` and whose name gives it to the terminal's module, then the terminal's own actions, `quit` last</t>
+          <t xml:space="preserve">a terminal's sources: what a terminal reads</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()` in each `terminal.py`; `MENU_TARGET_PATTERN` in each terminal's `config.py`; `_write_target()`</t>
-        </is>
-      </c>
-      <c r="E330" t="inlineStr">
-        <is>
-          <t xml:space="preserve">action</t>
+          <t xml:space="preserve">its own module's `config.py` where that is standard library — the data terminal's, with `lean.py`, and the ML terminal's; the features terminal its own `config.py`'s copies, `module_features/config.py` importing numpy; the monitoring terminal the snapshots through `STORE_STATUS_DIR` and `SNAPSHOT_FILE_NAMES` of its own `config.py`; the skills terminal the canon's `config.py` and, through the crawler's `config.py`, `vendors_for_crawling.toml` and the snapshot; every terminal `make help`</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second list of the targets in the program that opens the menu; a menu written out by hand; a target offered in a second terminal; the terminal's own entry among its options; `MODULE_TOKEN`, `STAGES`, `WRITES_BY_STAGE`, a target map; a grouping or a sorting of the targets; `run`, `exit`</t>
+          <t xml:space="preserve">a snapshot read for freshness; duckdb; a store literal; another module's code; a third-party package</t>
         </is>
       </c>
     </row>
@@ -14221,22 +14216,22 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset choice: the assets a run is about — the ones `--tickers` named, typed only when a direct run named none — then the one asset an action is for, one answered without asking</t>
+          <t xml:space="preserve">the menu: the options a terminal offers — one per target of the one Makefile that carries a `##` and whose name gives it to the terminal's module, then the terminal's own actions, `quit` last</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_tickers()` and its `gum_input` headed `asset`; `gum_choose` headed `asset` over those assets</t>
+          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()` in each `terminal.py`; `MENU_TARGET_PATTERN` in each terminal's `config.py`; `_write_target()`</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset</t>
+          <t xml:space="preserve">action</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t xml:space="preserve">a ticker typed where the launcher already named the set; a basket the terminal defines; a list of assets read from a store to fill it; a default basket in a module</t>
+          <t xml:space="preserve">a second list of the targets in the program that opens the menu; a menu written out by hand; a target offered in a second terminal; the terminal's own entry among its options; `MODULE_TOKEN`, `STAGES`, `WRITES_BY_STAGE`, a target map; a grouping or a sorting of the targets; `run`, `exit`</t>
         </is>
       </c>
     </row>
@@ -14248,22 +14243,22 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t xml:space="preserve">the plan and its gate: the choices, the `command` line verbatim and the target's purpose, then the question that runs or cancels</t>
+          <t xml:space="preserve">the asset choice: the assets a run is about — the ones `--tickers` named, typed only when a direct run named none — then the one asset an action is for, one answered without asking</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_target()`; the `command` line; `_make()`</t>
+          <t xml:space="preserve">`_tickers()` and its `gum_input` headed `asset`; `gum_choose` headed `asset` over those assets</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t xml:space="preserve">`target`, `purpose` and each variable as `parameter` and `value`; `command make &lt;target&gt; ASSET=&lt;TICKER&gt;`; `&lt;target&gt;?` with the target and `cancel`</t>
+          <t xml:space="preserve">asset</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage run before the gate; a gate that refuses what a hand confirms; `run`</t>
+          <t xml:space="preserve">a ticker typed where the launcher already named the set; a basket the terminal defines; a list of assets read from a store to fill it; a default basket in a module</t>
         </is>
       </c>
     </row>
@@ -14275,22 +14270,22 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal's own actions, the serpentine search's: draft the profile, read the recorded serpentine search, promote the proposal</t>
+          <t xml:space="preserve">the plan and its gate: the choices, the `command` line verbatim and the target's purpose, then the question that runs or cancels</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_search_profile()`, `_recorded_search_tables()`, `_write_promoted_proposal()` in `module_features/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">`_write_target()`; the `command` line; `_make()`</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t xml:space="preserve">draft; recorded search; `features-serpentine-search-promote`</t>
+          <t xml:space="preserve">`target`, `purpose` and each variable as `parameter` and `value`; `command make &lt;target&gt; ASSET=&lt;TICKER&gt;`; `&lt;target&gt;?` with the target and `cancel`</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t xml:space="preserve">`status` for the recorded search — the word is a stage's; a start of the serpentine search of its own — the search is the menu's `features-serpentine-search` or its `tmux-` twin; holdout, which the ML chain a promotion is followed by computes; a second menu after the action</t>
+          <t xml:space="preserve">a stage run before the gate; a gate that refuses what a hand confirms; `run`</t>
         </is>
       </c>
     </row>
@@ -14302,22 +14297,22 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t xml:space="preserve">the steps table: the steps of the features terminal's draft in order, above the step it asks — each answered DONE with its choice, the one asked CURRENT, the rest PENDING</t>
+          <t xml:space="preserve">the features terminal's own actions, the serpentine search's: draft the profile, read the recorded serpentine search, promote the proposal</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_step_rows()`, `_step_answer()`, `DRAFT_STEPS` in `module_features/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">`_write_search_profile()`, `_recorded_search_tables()`, `_write_promoted_proposal()` in `module_features/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t xml:space="preserve">step; state; choice; select now</t>
+          <t xml:space="preserve">draft; recorded search; `features-serpentine-search-promote`</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t xml:space="preserve">workflow, wizard, stepper; the steps of two actions; a step asked when its one option answers it</t>
+          <t xml:space="preserve">`status` for the recorded search — the word is a stage's; a start of the serpentine search of its own — the search is the menu's `features-serpentine-search` or its `tmux-` twin; holdout, which the ML chain a promotion is followed by computes; a second menu after the action</t>
         </is>
       </c>
     </row>
@@ -14329,22 +14324,22 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one file a terminal writes</t>
+          <t xml:space="preserve">the steps table: the steps of the features terminal's draft in order, above the step it asks — each answered DONE with its choice, the one asked CURRENT, the rest PENDING</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t xml:space="preserve">`write_json()`, `serpentine_search_profile_json()` in `module_features/sub_module_terminal/config.py` — the features terminal's draft</t>
-        </is>
-      </c>
-      <c r="D335" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
+          <t xml:space="preserve">`_step_rows()`, `_step_answer()`, `DRAFT_STEPS` in `module_features/sub_module_terminal/terminal.py`</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t xml:space="preserve">step; state; choice; select now</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second file; a file in the sub-module's own folder</t>
+          <t xml:space="preserve">workflow, wizard, stepper; the steps of two actions; a step asked when its one option answers it</t>
         </is>
       </c>
     </row>
@@ -14356,22 +14351,22 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t xml:space="preserve">the target the features terminal opens its own screen for — the promotion, whose plan shows the one state it promotes</t>
+          <t xml:space="preserve">the one file a terminal writes</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t xml:space="preserve">`PROMOTE_TARGET` in `module_features/sub_module_terminal/config.py`</t>
-        </is>
-      </c>
-      <c r="E336" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the menu's `features-serpentine-search-promote`</t>
+          <t xml:space="preserve">`write_json()`, `serpentine_search_profile_json()` in `module_features/sub_module_terminal/config.py` — the features terminal's draft</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second named target; the module's stages listed beside it; a name for a target that runs bare</t>
+          <t xml:space="preserve">a second file; a file in the sub-module's own folder</t>
         </is>
       </c>
     </row>
@@ -14383,22 +14378,22 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t xml:space="preserve">the profile state: where the asset's profile stands against the serpentine search recorded under it — the one comparison the features terminal makes, on parsed objects and not on bytes</t>
+          <t xml:space="preserve">the target the features terminal opens its own screen for — the promotion, whose plan shows the one state it promotes</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_profile_state()`</t>
+          <t xml:space="preserve">`PROMOTE_TARGET` in `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t xml:space="preserve">`not drafted` / `no search` / `matches the search` / `differs from the search`</t>
+          <t xml:space="preserve">the menu's `features-serpentine-search-promote`</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs_current`, which folds the parameters, the catalogue and the asset's own state and stays the page's</t>
+          <t xml:space="preserve">a second named target; the module's stages listed beside it; a name for a target that runs bare</t>
         </is>
       </c>
     </row>
@@ -14410,27 +14405,22 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t xml:space="preserve">the coordinate grid: what each coordinate is searched over, one preset, so a grid is a decision of the file and not of a form</t>
+          <t xml:space="preserve">the profile state: where the asset's profile stands against the serpentine search recorded under it — the one comparison the features terminal makes, on parsed objects and not on bytes</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`</t>
-        </is>
-      </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`grid_by_coordinate`</t>
+          <t xml:space="preserve">`_profile_state()`</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t xml:space="preserve">grid; points</t>
+          <t xml:space="preserve">`not drafted` / `no search` / `matches the search` / `differs from the search`</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t xml:space="preserve">a grid typed into a prompt; a point the terminal offers outside the preset</t>
+          <t xml:space="preserve">`inputs_current`, which folds the parameters, the catalogue and the asset's own state and stays the page's</t>
         </is>
       </c>
     </row>
@@ -14442,22 +14432,27 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t xml:space="preserve">gum: the terminal instrument the TUI speaks — `gum table --print`, `gum style`, `gum choose`, `gum filter`, `gum input`; gum 2, a binary of the host</t>
+          <t xml:space="preserve">the coordinate grid: what each coordinate is searched over, one preset, so a grid is a decision of the file and not of a form</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t xml:space="preserve">`gum`, over `subprocess` in `tui.py` alone: `gum_table()`, `gum_style()`, `gum_choose()`, `gum_filter()`, `gum_input()`, `_gum()`</t>
+          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`grid_by_coordinate`</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid; points</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Python dependency, Rich among them; a chooser, a table or a colour written over curses or escape codes; a gum configuration in the tree; `gum spin`, `gum confirm`; `gum input` for a value the tree already holds, which is a selection and belongs to `gum choose`; gum's own pink and purple</t>
-        </is>
-      </c>
-      <c r="I339" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gum</t>
+          <t xml:space="preserve">a grid typed into a prompt; a point the terminal offers outside the preset</t>
         </is>
       </c>
     </row>
@@ -14469,22 +14464,22 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t xml:space="preserve">plain output: the screens without colour, symbol or border, chosen by the environment alone — `NO_COLOR` set and not empty, `TERM=dumb`, or standard output not a terminal</t>
+          <t xml:space="preserve">gum: the terminal instrument the TUI speaks — `gum table --print`, `gum style`, `gum choose`, `gum input`; gum 2, a binary of the host</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OUTPUT_PLAIN` in each terminal's `config.py`, read by its `tui.py`</t>
-        </is>
-      </c>
-      <c r="E340" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`[&lt;word&gt;]`</t>
+          <t xml:space="preserve">`gum`, over `subprocess` in `tui.py` alone: `gum_table()`, `gum_style()`, `gum_choose()`, `gum_input()`, `_gum()`</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t xml:space="preserve">a flag, `--no-color`, `--simple`, `--a11y`; a theme or a gum configuration in the tree; a meaning a colour alone carries</t>
+          <t xml:space="preserve">a Python dependency, Rich among them; a chooser, a table or a colour written over curses or escape codes; a gum configuration in the tree; `gum spin`, `gum confirm`; `gum input` for a value the tree already holds, which is a selection and belongs to `gum choose`; gum's own pink and purple</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gum</t>
         </is>
       </c>
     </row>
@@ -14496,22 +14491,22 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state word: the closed list of words that say how a step, a file or an action stands — its symbol and colour beside it in normal output, the word in brackets in plain output</t>
+          <t xml:space="preserve">plain output: the screens without colour, symbol or border, chosen by the environment alone — `NO_COLOR` set and not empty, `TERM=dumb`, or standard output not a terminal</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STATE_SYMBOLS`, `STATE_COLOURS`, `state_label()` in `tui.py`</t>
+          <t xml:space="preserve">`OUTPUT_PLAIN` in each terminal's `config.py`, read by its `tui.py`</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t xml:space="preserve">DONE; CURRENT; PENDING; CANCELLED; WARN; FAILED; ERROR — and CRAWLING, NOT CRAWLED, which `STATE_SYMBOLS` still holds and no screen draws since the crawler has no screen</t>
+          <t xml:space="preserve">`[&lt;word&gt;]`</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t xml:space="preserve">a colour or a symbol without its word; a coloured row; `ok`, `success` as a state word</t>
+          <t xml:space="preserve">a flag, `--no-color`, `--simple`, `--a11y`; a theme or a gum configuration in the tree; a meaning a colour alone carries</t>
         </is>
       </c>
     </row>
@@ -14523,44 +14518,49 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t xml:space="preserve">the failure block and the exits: a failure on stderr as what failed, where, why and what next, the run's last block — 0 an action done or cancelled, 1 a failure, 2 an unknown argument, 130 Ctrl-C</t>
+          <t xml:space="preserve">a state word: the closed list of words that say how a step, a file or an action stands — its symbol and colour beside it in normal output, the word in brackets in plain output</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t xml:space="preserve">`error_lines()`, `INTERRUPTED_EXIT_CODE` in `tui.py`; `_failure_exit_code()`, `_cancelled_exit_code()` in each `terminal.py`</t>
+          <t xml:space="preserve">`STATE_SYMBOLS`, `STATE_COLOURS`, `state_label()` in `tui.py`</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t xml:space="preserve">where; why; next; `nothing written`</t>
+          <t xml:space="preserve">DONE; CURRENT; PENDING; CANCELLED; WARN; ERROR</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t xml:space="preserve">a traceback for an expected failure; a failure on stdout; exit 0 after a failure</t>
+          <t xml:space="preserve">a colour or a symbol without its word; a coloured row; `ok`, `success` as a state word</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artifacts</t>
+          <t xml:space="preserve">Terminals</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `ohlcv_1m_binance`, `ohlcv_1m_bybit`: one venue's minutes as printed, one partition per asset</t>
+          <t xml:space="preserve">the failure block and the exits: a failure on stderr as what failed, where, why and what next, the run's last block — 0 an action done or cancelled, 1 a failure, 2 an unknown argument, 130 Ctrl-C</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_&lt;venue&gt;/ticker=&lt;TICKER&gt;/ohlcv_1m_&lt;venue&gt;.parquet` and the family's `schema.json`; `venue_parquet()` in `module_data/config.py`</t>
-        </is>
-      </c>
-      <c r="G343" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume` — the venue's rows, ordered by every column, so a duplicate minute keeps one order; untracked</t>
+          <t xml:space="preserve">`error_lines()`, `INTERRUPTED_EXIT_CODE` in `tui.py`; `_failure_exit_code()`, `_cancelled_exit_code()` in each `terminal.py`</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t xml:space="preserve">where; why; next; `nothing written`</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a traceback for an expected failure; a failure on stdout; exit 0 after a failure</t>
         </is>
       </c>
     </row>
@@ -14572,17 +14572,17 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `ohlcv_1m_canonical`: the canonical 1m series, one partition per asset</t>
+          <t xml:space="preserve">the family `ohlcv_1m_binance`, `ohlcv_1m_bybit`: one venue's minutes as printed, one partition per asset</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_canonical/ticker=&lt;TICKER&gt;/ohlcv_1m_canonical.parquet` and the family's `schema.json`; `ohlcv_1m_canonical_parquet()`</t>
+          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_&lt;venue&gt;/ticker=&lt;TICKER&gt;/ohlcv_1m_&lt;venue&gt;.parquet` and the family's `schema.json`; `venue_parquet()` in `module_data/config.py`</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `source`, `zero_volume`, `binance_valid`, `bybit_valid`, `rel_divergence` — the full grid of the window, ordered by `timestamp_ms`; untracked</t>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume` — the venue's rows, ordered by every column, so a duplicate minute keeps one order; untracked</t>
         </is>
       </c>
     </row>
@@ -14594,17 +14594,17 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `bars`: the bars of every timeframe of the timeframe register, one partition per asset and timeframe</t>
+          <t xml:space="preserve">the family `ohlcv_1m_canonical`: the canonical 1m series, one partition per asset</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/bars.py` writes `bars/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/bars.parquet` and the family's `schema.json`; `bars_parquet()`</t>
+          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_canonical/ticker=&lt;TICKER&gt;/ohlcv_1m_canonical.parquet` and the family's `schema.json`; `ohlcv_1m_canonical_parquet()`</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `ffill_bars`, `zero_volume_bars` inside the research window, ordered by `timestamp_ms`; untracked</t>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `source`, `zero_volume`, `binance_valid`, `bybit_valid`, `rel_divergence` — the full grid of the window, ordered by `timestamp_ms`; untracked</t>
         </is>
       </c>
     </row>
@@ -14616,17 +14616,17 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `catalogue`: every catalogued column on the decision grid, one partition per asset and timeframe; a partition may omit a column the feature catalogue does not offer on its timeframe, never rename one or change its type</t>
+          <t xml:space="preserve">the family `bars`: the bars of every timeframe of the timeframe register, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/catalogue.py` writes `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet` and the family's `schema.json` from `catalogue_schema()`, the columns of the union of its partitions in catalogue order; `catalogue_parquet()` — in `module_ml/config.py` the same name over the contract's `parquet_by_timeframe`</t>
+          <t xml:space="preserve">`module_features/bars.py` writes `bars/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/bars.parquet` and the family's `schema.json`; `bars_parquet()`</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts` and every definition offered on the partition's timeframe, on the decision grid; untracked</t>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `ffill_bars`, `zero_volume_bars` inside the research window, ordered by `timestamp_ms`; untracked</t>
         </is>
       </c>
     </row>
@@ -14638,17 +14638,17 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `labels`: Y on the decision timeframe, one partition per asset and timeframe</t>
+          <t xml:space="preserve">the family `catalogue`: every catalogued column on the decision grid, one partition per asset and timeframe; a partition may omit a column the feature catalogue does not offer on its timeframe, never rename one or change its type</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/labels.py` writes `labels/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/labels.parquet` and the family's `schema.json`; `labels_parquet()`</t>
+          <t xml:space="preserve">`module_features/catalogue.py` writes `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet` and the family's `schema.json` from `catalogue_schema()`, the columns of the union of its partitions in catalogue order; `catalogue_parquet()` — in `module_ml/config.py` the same name over the contract's `parquet_by_timeframe`</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts`, `entry_ts`, `y`, `event_end_ts`, `entry_observable`, `label_valid`, `event_resolution`, `entry_price`, `upper_barrier`, `lower_barrier`, `exit_reference_price`; an ambiguous event carries `y = 0` with `label_valid = false`, so `y` is never read without `label_valid`; untracked</t>
+          <t xml:space="preserve">`decision_ts` and every definition offered on the partition's timeframe, on the decision grid; untracked</t>
         </is>
       </c>
     </row>
@@ -14660,17 +14660,17 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `oos_predictions`: the out-of-sample class probabilities, one partition per asset and timeframe</t>
+          <t xml:space="preserve">the family `labels`: Y on the decision timeframe, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/train.py` writes `oos_predictions/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/oos_predictions.parquet` and the family's `schema.json`; `oos_predictions_parquet()`</t>
+          <t xml:space="preserve">`module_ml/labels.py` writes `labels/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/labels.parquet` and the family's `schema.json`; `labels_parquet()`</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts`, `oos_fold_id`, `p_short`, `p_neutral`, `p_long` — the full window of every validation fold and of the final holdout; metrics score only the supervised subset; untracked</t>
+          <t xml:space="preserve">`decision_ts`, `entry_ts`, `y`, `event_end_ts`, `entry_observable`, `label_valid`, `event_resolution`, `entry_price`, `upper_barrier`, `lower_barrier`, `exit_reference_price`; an ambiguous event carries `y = 0` with `label_valid = false`, so `y` is never read without `label_valid`; untracked</t>
         </is>
       </c>
     </row>
@@ -14682,17 +14682,17 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_README.md`</t>
+          <t xml:space="preserve">the family `oos_predictions`: the out-of-sample class probabilities, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/status.py` writes it, `asset_readme_md()`; its file list `file_manifest()`, the three files of `HAND_STAGE_FILE_DESCRIPTORS` listed with no size</t>
+          <t xml:space="preserve">`module_ml/train.py` writes `oos_predictions/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/oos_predictions.parquet` and the family's `schema.json`; `oos_predictions_parquet()`</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t xml:space="preserve">what the folder holds and what came out of it; no timestamp; tracked</t>
+          <t xml:space="preserve">`decision_ts`, `oos_fold_id`, `p_short`, `p_neutral`, `p_long` — the full window of every validation fold and of the final holdout; metrics score only the supervised subset; untracked</t>
         </is>
       </c>
     </row>
@@ -14704,17 +14704,17 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_barriers.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_README.md`</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `barriers_json()`; `load_barriers()` in `module_ml/dataset.py` reads it</t>
+          <t xml:space="preserve">`module_ml/status.py` writes it, `asset_readme_md()`; its file list `file_manifest()`, the three files of `HAND_STAGE_FILE_DESCRIPTORS` listed with no size</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t xml:space="preserve">`label_barrier_true_range_multiplier`, `label_horizon`, `take_profit_true_range_multiplier`, `stop_loss_true_range_multiplier` — the asset's promoted barrier geometry, a hand's choice; absent, `START_BY_COORDINATE_DEFAULT` of `module_ml/config.py` is the asset's; tracked once promoted, like the feature set beside it</t>
+          <t xml:space="preserve">what the folder holds and what came out of it; no timestamp; tracked</t>
         </is>
       </c>
     </row>
@@ -14726,17 +14726,17 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_barriers.json`</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/catalogue.py` writes it from `catalogue_contract()`; `catalogue_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `barriers_json()`; `load_barriers()` in `module_ml/dataset.py` reads it</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature layer's contract the ML layer reads instead of the feature configuration: `decision_timeframe`, `timeframes` (each `timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe` — each value a path relative to the artifacts store, `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet`; untracked</t>
+          <t xml:space="preserve">`label_barrier_true_range_multiplier`, `label_horizon`, `take_profit_true_range_multiplier`, `stop_loss_true_range_multiplier` — the asset's promoted barrier geometry, a hand's choice; absent, `START_BY_COORDINATE_DEFAULT` of `module_ml/config.py` is the asset's; tracked once promoted, like the feature set beside it</t>
         </is>
       </c>
     </row>
@@ -14748,17 +14748,17 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `feature_set_json()`</t>
+          <t xml:space="preserve">`module_features/catalogue.py` writes it from `catalogue_contract()`; `catalogue_json()`</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t xml:space="preserve">`columns_by_timeframe` — the promoted feature set, a hand's choice, and nothing else; absent, the default set is the asset's; tracked once promoted, like the parameters it conditions</t>
+          <t xml:space="preserve">the feature layer's contract the ML layer reads instead of the feature configuration: `decision_timeframe`, `timeframes` (each `timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe` — each value a path relative to the artifacts store, `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet`; untracked</t>
         </is>
       </c>
     </row>
@@ -14770,17 +14770,17 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_hyperparameter_point.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json`</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `hyperparameter_point_json()`; `hpo.main()` in `module_ml/hpo.py` reads it</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `feature_set_json()`</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`best_params` — the promoted hyper-parameter point, a hand's choice: the first trial of the chain's study, and nothing else; absent, the study draws every point; tracked once promoted, like the feature set and the geometry beside it</t>
+          <t xml:space="preserve">`columns_by_timeframe` — the promoted feature set, a hand's choice, and nothing else; absent, the default set is the asset's; tracked once promoted, like the parameters it conditions</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_model_evaluation.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_hyperparameter_point.json`</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/train.py` writes it; `model_evaluation_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `hyperparameter_point_json()`; `hpo.main()` in `module_ml/hpo.py` reads it</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`validation` — a `fold_&lt;id&gt;` per fold of `VALIDATION_FOLD_IDS` — and `final_holdout`, each `prior_logloss`, `model_logloss`, `relative_logloss_skill`, `scored_row_count`; `validation_importance`, a `fold_&lt;id&gt;` per validation fold, each `gain_importance` and `mean_abs_shap_importance` per column; `feature_columns`; `class_counts`, `labels`, `segments`; untracked</t>
+          <t xml:space="preserve">`best_params` — the promoted hyper-parameter point, a hand's choice: the first trial of the chain's study, and nothing else; absent, the study draws every point; tracked once promoted, like the feature set and the geometry beside it</t>
         </is>
       </c>
     </row>
@@ -14814,17 +14814,17 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_parameters.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_model_evaluation.json`</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/hpo.py` writes it; `parameters_json()`</t>
+          <t xml:space="preserve">`module_ml/train.py` writes it; `model_evaluation_json()`</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`hyperparameter_search_result` (`best_params`, `best_cagr_validation_path`, `trial_count`); tracked</t>
+          <t xml:space="preserve">`validation` — a `fold_&lt;id&gt;` per fold of `VALIDATION_FOLD_IDS` — and `final_holdout`, each `prior_logloss`, `model_logloss`, `relative_logloss_skill`, `scored_row_count`; `validation_importance`, a `fold_&lt;id&gt;` per validation fold, each `gain_importance` and `mean_abs_shap_importance` per column; `feature_columns`; `class_counts`, `labels`, `segments`; untracked</t>
         </is>
       </c>
     </row>
@@ -14836,27 +14836,17 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_score_request.json`: the serpentine search's question</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_parameters.json`</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_request_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by a turn, `features-serpentine-turn`, read by `module_ml.score`, `ml-score`; the one file the loop of `features-serpentine-search` tests, running `ml-score` and a turn again while it exists</t>
-        </is>
-      </c>
-      <c r="D356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`kind` (`score` or `hpo`), `round`, `states`</t>
-        </is>
-      </c>
-      <c r="F356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a key beside these three; a request the evaluator writes; a second file the loop tests</t>
+          <t xml:space="preserve">`module_ml/hpo.py` writes it; `parameters_json()`</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t xml:space="preserve">what one family pass asks to be scored: the kind of scoring, the round it runs in, and the states — a state of its own for `score`, a beam parent's scored row for `hpo`; untracked</t>
+          <t xml:space="preserve">`hyperparameter_search_result` (`best_params`, `best_cagr_validation_path`, `trial_count`); tracked</t>
         </is>
       </c>
     </row>
@@ -14868,27 +14858,27 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_score_response.json`: the serpentine search's answer</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_score_request.json`: the serpentine search's question</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_response_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by `module_ml.score` alone</t>
+          <t xml:space="preserve">`score_request_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by a turn, `features-serpentine-turn`, read by `module_ml.score`, `ml-score`; the one file the loop of `features-serpentine-search` tests, running `ml-score` and a turn again while it exists</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`kind`, `round`, `results`; a `score` result the row of one scored state of the serpentine search, an `hpo` result `state_key`, `trial_count_drawn` and `candidate`</t>
+          <t xml:space="preserve">`kind` (`score` or `hpo`), `round`, `states`</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">a key beside these three; a result out of the order the request named; a response written before every state has one</t>
+          <t xml:space="preserve">a key beside these three; a request the evaluator writes; a second file the loop tests</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t xml:space="preserve">what the states of one request are worth, in the order the request named them; `candidate` a scored row or `null`, and `null` is an answer; untracked</t>
+          <t xml:space="preserve">what one family pass asks to be scored: the kind of scoring, the round it runs in, and the states — a state of its own for `score`, a beam parent's scored row for `hpo`; untracked</t>
         </is>
       </c>
     </row>
@@ -14900,17 +14890,27 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_score_response.json`: the serpentine search's answer</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_json()`</t>
+          <t xml:space="preserve">`score_response_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by `module_ml.score` alone</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`kind`, `round`, `results`; a `score` result the row of one scored state of the serpentine search, an `hpo` result `state_key`, `trial_count_drawn` and `candidate`</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a key beside these three; a result out of the order the request named; a response written before every state has one</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs`, `beam`, `champion_trial_index`, `round_count`, `search_converged`, `path` (each `round`, `loop`, `family`, `trial_index`, `beam`, `move`), `proposals` (each `proposal`, `trial_index`), `trial_count_by_loop` — where the search stands at a round boundary, naming trials by index and carrying none of their columns; tracked once a search has run</t>
+          <t xml:space="preserve">what the states of one request are worth, in the order the request named them; `candidate` a scored row or `null`, and `null` is an answer; untracked</t>
         </is>
       </c>
     </row>
@@ -14922,17 +14922,17 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search.json`</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hand, in the file or through the features terminal's draft; `serpentine_search_profile_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_json()`</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`columns_admitted_by_timeframe`, `start_columns_by_timeframe` (`null` = the asset's own set), `grid_by_coordinate` (one list per coordinate, in the order it is searched), `loops` (a subset of `SERPENTINE_SEARCH_ROUND_LOOPS`), `path_cagr_noise_standard_deviation` (the asset's noise sigma, `null` on the calibration run) — what a hand asks the serpentine search to look at; drafted, never derived, and tracked</t>
+          <t xml:space="preserve">`inputs`, `beam`, `champion_trial_index`, `round_count`, `search_converged`, `path` (each `round`, `loop`, `family`, `trial_index`, `beam`, `move`), `proposals` (each `proposal`, `trial_index`), `trial_count_by_loop` — where the search stands at a round boundary, naming trials by index and carrying none of their columns; tracked once a search has run</t>
         </is>
       </c>
     </row>
@@ -14944,17 +14944,17 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_trials.jsonl`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_trials_jsonl()`</t>
+          <t xml:space="preserve">a hand, in the file or through the features terminal's draft; `serpentine_search_profile_json()`</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t xml:space="preserve">one scored state of the serpentine search a line, appended and never rewritten; `trial_index` = the line number, counted from one; tracked once a search has run</t>
+          <t xml:space="preserve">`columns_admitted_by_timeframe`, `start_columns_by_timeframe` (`null` = the asset's own set), `grid_by_coordinate` (one list per coordinate, in the order it is searched), `loops` (a subset of `SERPENTINE_SEARCH_ROUND_LOOPS`), `path_cagr_noise_standard_deviation` (the asset's noise sigma, `null` on the calibration run) — what a hand asks the serpentine search to look at; drafted, never derived, and tracked</t>
         </is>
       </c>
     </row>
@@ -14966,49 +14966,39 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_strategy_evaluation.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_trials.jsonl`</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/strategy.py` writes it; `strategy_evaluation_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_trials_jsonl()`</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `cleared_point_count`, `median_cagr_over_cleared`, `max_cagr_over_cleared`, `selection_score_cagr_validation_path`, `execution_cost_rate_per_trade_side`; per fold `sharpe`, `cagr`, `max_drawdown`, `calmar`, `profit_factor`, `trade_count`, `hit_rate`, `average_trade_return`, `exposure`, `exit_counts`, `final_equity`; `validation_path` over the validation folds; the final holdout's `equity_curve`; untracked</t>
+          <t xml:space="preserve">one scored state of the serpentine search a line, appended and never rewritten; `trial_index` = the line number, counted from one; tracked once a search has run</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Features</t>
+          <t xml:space="preserve">Artifacts</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t xml:space="preserve">a series of one timeframe's bars, with no parameter</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_strategy_evaluation.json`</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t xml:space="preserve">`open`, `high`, `low`, `close`, `volume` — a bar column — and the series with a kernel: `logarithmic_volume`, `true_range`, `cumulative_signed_volume`; `SERIES_KERNELS`, `module_features/indicators.py`</t>
-        </is>
-      </c>
-      <c r="D362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`inputs` of a term</t>
-        </is>
-      </c>
-      <c r="E362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the series token</t>
-        </is>
-      </c>
-      <c r="F362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a series with a parameter; `log_volume`</t>
+          <t xml:space="preserve">`module_ml/strategy.py` writes it; `strategy_evaluation_json()`</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `cleared_point_count`, `median_cagr_over_cleared`, `max_cagr_over_cleared`, `selection_score_cagr_validation_path`, `execution_cost_rate_per_trade_side`; per fold `sharpe`, `cagr`, `max_drawdown`, `calmar`, `profit_factor`, `trade_count`, `hit_rate`, `average_trade_return`, `exposure`, `exit_counts`, `final_equity`; `validation_path` over the validation folds; the final holdout's `equity_curve`; untracked</t>
         </is>
       </c>
     </row>
@@ -15020,32 +15010,27 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t xml:space="preserve">an indicator — one computation with exactly one integer parameter, named by its token, its invariants one record of the register beside its kernel, the popular names it answers to among them</t>
+          <t xml:space="preserve">a series of one timeframe's bars, with no parameter</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`exponential_smoothing&lt;n&gt;`, `rolling_mean&lt;n&gt;`, `recursive_mean&lt;n&gt;`, `recursive_mean_gain_share&lt;n&gt;`, `rolling_standard_score&lt;n&gt;`, `rolling_range_position&lt;n&gt;`, `rolling_standard_deviation&lt;n&gt;`, `relative_change&lt;n&gt;`, `recursive_mean_upward_movement_share&lt;n&gt;`, `recursive_mean_directional_movement_imbalance&lt;n&gt;`, `rolling_volume_weighted_mean&lt;n&gt;`, `rolling_volume_weighted_close_location&lt;n&gt;`, `rolling_money_flow_gain_share&lt;n&gt;`; `INDICATORS` — `kernel`, `parameter_word`, `warmup_multiple`, `inputs`, `output_range`, `historical_aliases` of a record, `module_features/indicators.py`</t>
+          <t xml:space="preserve">`open`, `high`, `low`, `close`, `volume` — a bar column — and the series with a kernel: `logarithmic_volume`, `true_range`, `cumulative_signed_volume`; `SERIES_KERNELS`, `module_features/indicators.py`</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`indicator`, `parameter_word`, `parameter_bars`, `output_range`, `historical_aliases` of a term</t>
+          <t xml:space="preserve">`inputs` of a term</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">the token with its parameter, `&lt;PARAMETER_WORD&gt; &lt;n&gt; bars of &lt;inputs&gt;` beside it and `output &lt;low&gt;–&lt;high&gt;` when the indicator is bounded (the catalogue table's terms)</t>
+          <t xml:space="preserve">the series token</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`rsi_14`, `sma_200`, `bb20`; a table of indicator facts in `config.py` beside the register; `kernel` for anything but the function a record computes with; the abbreviations these tokens replaced: `ema`, `sma`, `rsi`, `atr`, `zscore`, `rolling_zscore`, `wilder_smoothing`, `range_position`</t>
-        </is>
-      </c>
-      <c r="I363" t="inlineStr">
-        <is>
-          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
+          <t xml:space="preserve">a series with a parameter; `log_volume`</t>
         </is>
       </c>
     </row>
@@ -15057,27 +15042,32 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t xml:space="preserve">a term — a series or an indicator inside a feature definition</t>
+          <t xml:space="preserve">an indicator — one computation with exactly one integer parameter, named by its token, its invariants one record of the register beside its kernel, the popular names it answers to among them</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t xml:space="preserve">`("&lt;indicator&gt;", &lt;parameter_bars&gt;)` on the default series close, `("&lt;series&gt;", "&lt;indicator&gt;", &lt;parameter_bars&gt;)` on another series, `("&lt;series&gt;",)` a bare series; `term_name()`</t>
+          <t xml:space="preserve">`exponential_smoothing&lt;n&gt;`, `rolling_mean&lt;n&gt;`, `recursive_mean&lt;n&gt;`, `recursive_mean_gain_share&lt;n&gt;`, `rolling_standard_score&lt;n&gt;`, `rolling_range_position&lt;n&gt;`, `rolling_standard_deviation&lt;n&gt;`, `relative_change&lt;n&gt;`, `recursive_mean_upward_movement_share&lt;n&gt;`, `recursive_mean_directional_movement_imbalance&lt;n&gt;`, `rolling_volume_weighted_mean&lt;n&gt;`, `rolling_volume_weighted_close_location&lt;n&gt;`, `rolling_money_flow_gain_share&lt;n&gt;`; `INDICATORS` — `kernel`, `parameter_word`, `warmup_multiple`, `inputs`, `output_range`, `historical_aliases` of a record, `module_features/indicators.py`</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t xml:space="preserve">`terms`</t>
+          <t xml:space="preserve">`indicator`, `parameter_word`, `parameter_bars`, `output_range`, `historical_aliases` of a term</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">terms</t>
+          <t xml:space="preserve">the token with its parameter, `&lt;PARAMETER_WORD&gt; &lt;n&gt; bars of &lt;inputs&gt;` beside it and `output &lt;low&gt;–&lt;high&gt;` when the indicator is bounded (the catalogue table's terms)</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t xml:space="preserve">atom</t>
+          <t xml:space="preserve">`rsi_14`, `sma_200`, `bb20`; a table of indicator facts in `config.py` beside the register; `kernel` for anything but the function a record computes with; the abbreviations these tokens replaced: `ema`, `sma`, `rsi`, `atr`, `zscore`, `rolling_zscore`, `wilder_smoothing`, `range_position`</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
         </is>
       </c>
     </row>
@@ -15089,32 +15079,27 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t xml:space="preserve">a feature definition — terms of one timeframe composed by the operators, with an optional normaliser; the timeframe-less half of a feature, carrying the tier it belongs to and the popular names that denote the whole of it</t>
+          <t xml:space="preserve">a term — a series or an indicator inside a feature definition</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t xml:space="preserve">one record of `FEATURE_CATALOGUE`; `feature_definition_name()`; `OPERATORS` = {`minus`, `over`} and `NORMALISERS` = {`centered`}, one record per token beside its kernel in `module_features/catalogue.py`</t>
+          <t xml:space="preserve">`("&lt;indicator&gt;", &lt;parameter_bars&gt;)` on the default series close, `("&lt;series&gt;", "&lt;indicator&gt;", &lt;parameter_bars&gt;)` on another series, `("&lt;series&gt;",)` a bare series; `term_name()`</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_definition`, `tier` = `CORE` / `EXTENDED` / `COMPOSITE`, `historical_aliases`</t>
+          <t xml:space="preserve">`terms`</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t xml:space="preserve">definition (the catalogue table)</t>
+          <t xml:space="preserve">terms</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t xml:space="preserve">molecule, family, feature family, indicator (for a composite); `trend`, `momentum`, `volatility`, `structure`, `activity` — a category, not a computation; a popular name as the key, the column or a second name beside the canonical one; a tier written anywhere but the record; `centred` — the normaliser token keeps its American spelling, a column and a key on disk</t>
-        </is>
-      </c>
-      <c r="I365" t="inlineStr">
-        <is>
-          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
+          <t xml:space="preserve">atom</t>
         </is>
       </c>
     </row>
@@ -15126,27 +15111,32 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t xml:space="preserve">a feature — a definition aligned to the decision grid on one timeframe; the column of X and the key of an importance</t>
+          <t xml:space="preserve">a feature definition — terms of one timeframe composed by the operators, with an optional normaliser; the timeframe-less half of a feature, carrying the tier it belongs to and the popular names that denote the whole of it</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_id()` = `&lt;definition&gt;_&lt;timeframe&gt;`</t>
+          <t xml:space="preserve">one record of `FEATURE_CATALOGUE`; `feature_definition_name()`; `OPERATORS` = {`minus`, `over`} and `NORMALISERS` = {`centered`}, one record per token beside its kernel in `module_features/catalogue.py`</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_columns`, the keys of an importance</t>
+          <t xml:space="preserve">`feature_definition`, `tier` = `CORE` / `EXTENDED` / `COMPOSITE`, `historical_aliases`</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature id — `column &lt;timeframe&gt;` in the FEATURE SET frame</t>
+          <t xml:space="preserve">definition (the catalogue table)</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
+          <t xml:space="preserve">molecule, family, feature family, indicator (for a composite); `trend`, `momentum`, `volatility`, `structure`, `activity` — a category, not a computation; a popular name as the key, the column or a second name beside the canonical one; a tier written anywhere but the record; `centred` — the normaliser token keeps its American spelling, a column and a key on disk</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
         </is>
       </c>
     </row>
@@ -15158,27 +15148,27 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature catalogue — every definition the repository can compute, with the timeframes it is offered on; drafted, like the rest of `config.py`</t>
+          <t xml:space="preserve">a feature — a definition aligned to the decision grid on one timeframe; the column of X and the key of an importance</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t xml:space="preserve">`FEATURE_CATALOGUE`, `catalogue_columns()`, `CATALOGUE_COLUMNS`; the stage `features-catalogue`, `module_features/catalogue.py`</t>
+          <t xml:space="preserve">`feature_id()` = `&lt;definition&gt;_&lt;timeframe&gt;`</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue` (of `features_status.json`); `&lt;TICKER&gt;_catalogue.json`; the family `catalogue`</t>
+          <t xml:space="preserve">`feature_columns`, the keys of an importance</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t xml:space="preserve">CATALOGUE</t>
+          <t xml:space="preserve">the feature id — `column &lt;timeframe&gt;` in the FEATURE SET frame</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t xml:space="preserve">palette, feature list, feature store</t>
+          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
         </is>
       </c>
     </row>
@@ -15190,22 +15180,27 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature layer's contract, per asset — what the ML layer reads instead of this module's configuration</t>
+          <t xml:space="preserve">the feature catalogue — every definition the repository can compute, with the timeframes it is offered on; drafted, like the rest of `config.py`</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue_contract()`, `catalogue_json()` in `module_features/config.py`; the descriptor's copy in `module_ml/config.py`; `load_catalogue()` in `module_ml/dataset.py`, `cat`</t>
+          <t xml:space="preserve">`FEATURE_CATALOGUE`, `catalogue_columns()`, `CATALOGUE_COLUMNS`; the stage `features-catalogue`, `module_features/catalogue.py`</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`: `decision_timeframe`, `timeframes` (`timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe`</t>
+          <t xml:space="preserve">`catalogue` (of `features_status.json`); `&lt;TICKER&gt;_catalogue.json`; the family `catalogue`</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CATALOGUE</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t xml:space="preserve">an import of `module_features` from `module_ml`; a token or a slot parsed in the ML layer; a second read of the file inside one stage; a path built from the slot grammar outside `module_features`; a parquet named in the contract by anything but its path relative to the artifact store</t>
+          <t xml:space="preserve">palette, feature list, feature store</t>
         </is>
       </c>
     </row>
@@ -15217,27 +15212,22 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t xml:space="preserve">the effective history — what a parameter covers on a timeframe, `bars × timeframe`, the quantity the nesting rule compares</t>
+          <t xml:space="preserve">the feature layer's contract, per asset — what the ML layer reads instead of this module's configuration</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t xml:space="preserve">`definition_effective_history_hours()`</t>
+          <t xml:space="preserve">`catalogue_contract()`, `catalogue_json()` in `module_features/config.py`; the descriptor's copy in `module_ml/config.py`; `load_catalogue()` in `module_ml/dataset.py`, `cat`</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t xml:space="preserve">`effective_history_hours_by_timeframe`; `lower_longest_effective_history_hours`, `upper_shortest_effective_history_hours` of `nesting`</t>
-        </is>
-      </c>
-      <c r="E369" t="inlineStr">
-        <is>
-          <t xml:space="preserve">effective history</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`: `decision_timeframe`, `timeframes` (`timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe`</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t xml:space="preserve">history (bare — a recursion has no window), span (the parameter word of an exponential smoothing), lookback hours</t>
+          <t xml:space="preserve">an import of `module_features` from `module_ml`; a token or a slot parsed in the ML layer; a second read of the file inside one stage; a path built from the slot grammar outside `module_features`; a parquet named in the contract by anything but its path relative to the artifact store</t>
         </is>
       </c>
     </row>
@@ -15249,22 +15239,27 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t xml:space="preserve">the Bollinger %b reading — the trade's %b(20, 2σ), `rolling_standard_score20` / 4 + 0.5, an affine map a tree model is invariant to, so no %b column exists</t>
+          <t xml:space="preserve">the effective history — what a parameter covers on a timeframe, `bars × timeframe`, the quantity the nesting rule compares</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`definition_effective_history_hours()`</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`effective_history_hours_by_timeframe`; `lower_longest_effective_history_hours`, `upper_shortest_effective_history_hours` of `nesting`</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t xml:space="preserve">— (no page shows it; Bollinger %b in the definitions table of `methodology_features.md`)</t>
+          <t xml:space="preserve">effective history</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t xml:space="preserve">`bb20`, `%b` as a column, `z / 2 + 0.5`; `zscore20`</t>
-        </is>
-      </c>
-      <c r="I370" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bollinger (technical analysis)</t>
+          <t xml:space="preserve">history (bare — a recursion has no window), span (the parameter word of an exponential smoothing), lookback hours</t>
         </is>
       </c>
     </row>
@@ -15276,27 +15271,22 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t xml:space="preserve">the definitions an asset's model sees until a promotion — the frozen experiment's default definitions on every timeframe of the register, in the order it stacks them</t>
-        </is>
-      </c>
-      <c r="C371" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME`; `definition_in_default_set` of a record</t>
-        </is>
-      </c>
-      <c r="D371" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`definition_in_default_set`; `default_columns_by_timeframe` of the contract</t>
+          <t xml:space="preserve">the Bollinger %b reading — the trade's %b(20, 2σ), `rolling_standard_score20` / 4 + 0.5, an affine map a tree model is invariant to, so no %b column exists</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t xml:space="preserve">default set</t>
+          <t xml:space="preserve">— (no page shows it; Bollinger %b in the definitions table of `methodology_features.md`)</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t xml:space="preserve">the frozen fifteen (as a name)</t>
+          <t xml:space="preserve">`bb20`, `%b` as a column, `z / 2 + 0.5`; `zscore20`</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bollinger (technical analysis)</t>
         </is>
       </c>
     </row>
@@ -15308,49 +15298,59 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t xml:space="preserve">the definition the strategy hierarchy reads on every timeframe, set or no set</t>
+          <t xml:space="preserve">the definitions an asset's model sees until a promotion — the frozen experiment's default definitions on every timeframe of the register, in the order it stacks them</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TREND_GATE_FEATURE_DEFINITION` in `module_ml/config.py` — the name of the catalogue's first definition, owned by the strategy that reads it; the gate's timeframe is the top of the contract's hierarchy, `trend_gate_timeframe(cat)`</t>
+          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME`; `definition_in_default_set` of a record</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t xml:space="preserve">`trend_gate_feature`</t>
+          <t xml:space="preserve">`definition_in_default_set`; `default_columns_by_timeframe` of the contract</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t xml:space="preserve">gate (the asset's STRATEGY frame)</t>
+          <t xml:space="preserve">default set</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TREND_FAMILY`; a column literal in `asset.js`; a second copy of the name in the feature layer, which reads nothing of it</t>
+          <t xml:space="preserve">the frozen fifteen (as a name)</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset containers</t>
+          <t xml:space="preserve">Features</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t xml:space="preserve">an asset container: a runner's one-off for one asset, exiting with its stage</t>
+          <t xml:space="preserve">the definition the strategy hierarchy reads on every timeframe, set or no set</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
+          <t xml:space="preserve">`TREND_GATE_FEATURE_DEFINITION` in `module_ml/config.py` — the name of the catalogue's first definition, owned by the strategy that reads it; the gate's timeframe is the top of the contract's hierarchy, `trend_gate_timeframe(cat)`</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`trend_gate_feature`</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gate (the asset's STRATEGY frame)</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t xml:space="preserve">a compose service per asset; a resident per asset; a `restart:` policy; a published port</t>
+          <t xml:space="preserve">`TREND_FAMILY`; a column literal in `asset.js`; a second copy of the name in the feature layer, which reads nothing of it</t>
         </is>
       </c>
     </row>
@@ -15362,17 +15362,17 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t xml:space="preserve">a runner: a compose service that is a role and a one-off — no command of its own; the run supplies one and the container exits with the stage</t>
+          <t xml:space="preserve">an asset container: a runner's one-off for one asset, exiting with its stage</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
+          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t xml:space="preserve">`pipeline`, one runner for every module; a stage run by `exec` inside a resident; a runner with a `command:`</t>
+          <t xml:space="preserve">a compose service per asset; a resident per asset; a `restart:` policy; a published port</t>
         </is>
       </c>
     </row>
@@ -15384,17 +15384,17 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t xml:space="preserve">a service's mounts: the tree at `/app` and the stores it touches at `/store/&lt;content&gt;`, read-only where it only reads</t>
+          <t xml:space="preserve">a runner: a compose service that is a role and a one-off — no command of its own; the run supplies one and the container exits with the stage</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.:/app` and `./store/&lt;content&gt;:/store/&lt;content&gt;` in each service's `volumes:` of `docker-compose.yml`, respelled whole because a service's key replaces the anchor's</t>
+          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t xml:space="preserve">`/app/store/&lt;content&gt;` as an address; a mount of a store the service does not touch; a named volume</t>
+          <t xml:space="preserve">`pipeline`, one runner for every module; a stage run by `exec` inside a resident; a runner with a `command:`</t>
         </is>
       </c>
     </row>
@@ -15406,17 +15406,17 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t xml:space="preserve">the memory ceiling of the one runner that needs it — HPO and XGBoost allocate above `DUCKDB_MEMORY_LIMIT`</t>
+          <t xml:space="preserve">a service's mounts: the tree at `/app` and the stores it touches at `/store/&lt;content&gt;`, read-only where it only reads</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t xml:space="preserve">`deploy.resources.limits.memory` of the `ml` runner alone</t>
+          <t xml:space="preserve">`.:/app` and `./store/&lt;content&gt;:/store/&lt;content&gt;` in each service's `volumes:` of `docker-compose.yml`, respelled whole because a service's key replaces the anchor's</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t xml:space="preserve">`mem_limit` beside it, a CPU quota, a reservation; a ceiling on the anchor, so on the dashboard too</t>
+          <t xml:space="preserve">`/app/store/&lt;content&gt;` as an address; a mount of a store the service does not touch; a named volume</t>
         </is>
       </c>
     </row>
@@ -15428,17 +15428,17 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t xml:space="preserve">the thread cap: every computation's threads pinned to one — OpenMP's by the compose anchor's environment, beside the store contract, DuckDB's and XGBoost's in the code</t>
+          <t xml:space="preserve">the memory ceiling of the one runner that needs it — HPO and XGBoost allocate above `DUCKDB_MEMORY_LIMIT`</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OMP_NUM_THREADS` in the `x-store-environment` anchor of `docker-compose.yml`; `SET threads=1` on every DuckDB connection; `nthread` of the booster's parameters in `module_ml/config.py`</t>
+          <t xml:space="preserve">`deploy.resources.limits.memory` of the `ml` runner alone</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t xml:space="preserve">a thread count read from a stage's command line; a cap set per service</t>
+          <t xml:space="preserve">`mem_limit` beside it, a CPU quota, a reservation; a ceiling on the anchor, so on the dashboard too</t>
         </is>
       </c>
     </row>
@@ -15450,17 +15450,17 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t xml:space="preserve">the dashboard's command: the server, on the container's internal port</t>
+          <t xml:space="preserve">the thread cap: every computation's threads pinned to one — OpenMP's by the compose anchor's environment, beside the store contract, DuckDB's and XGBoost's in the code</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command: python -m module_monitoring.serve` of `dashboard`; `CONTAINER_PORT` and `BIND_ADDRESS` in `module_monitoring/config.py`</t>
+          <t xml:space="preserve">`OMP_NUM_THREADS` in the `x-store-environment` anchor of `docker-compose.yml`; `SET threads=1` on every DuckDB connection; `nthread` of the booster's parameters in `module_ml/config.py`</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t xml:space="preserve">a port or a bind address read from the environment or the command line; `PORT` inside a container</t>
+          <t xml:space="preserve">a thread count read from a stage's command line; a cap set per service</t>
         </is>
       </c>
     </row>
@@ -15472,22 +15472,17 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t xml:space="preserve">the host port: the host side of the dashboard's mapping, measured at invocation and never written down — and the page's address, the one `make on` prints</t>
+          <t xml:space="preserve">the dashboard's command: the server, on the container's internal port</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t xml:space="preserve">`PORT` of the `Makefile` — the port the dashboard already publishes, else the first free one upward from the internal port's number; `PORT=n` overrides; the `ports:` of `dashboard`, published on `127.0.0.1`</t>
-        </is>
-      </c>
-      <c r="E379" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`dashboard at http://127.0.0.1:&lt;port&gt;/`</t>
+          <t xml:space="preserve">`command: python -m module_monitoring.serve` of `dashboard`; `CONTAINER_PORT` and `BIND_ADDRESS` in `module_monitoring/config.py`</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t xml:space="preserve">the internal port's number as the page's address in a document, a command or a comment; a second variable for it; `PORT` inside a container; a measurement outside the `Makefile`</t>
+          <t xml:space="preserve">a port or a bind address read from the environment or the command line; `PORT` inside a container</t>
         </is>
       </c>
     </row>
@@ -15499,17 +15494,22 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t xml:space="preserve">the compose project: the one fixed name every container, network and volume of this project carries on every host</t>
+          <t xml:space="preserve">the host port: the host side of the dashboard's mapping, measured at invocation and never written down — and the page's address, the one `make on` prints</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t xml:space="preserve">`name: liora` in `docker-compose.yml` — the resident `liora-dashboard-1`</t>
+          <t xml:space="preserve">`PORT` of the `Makefile` — the port the dashboard already publishes, else the first free one upward from the internal port's number; `PORT=n` overrides; the `ports:` of `dashboard`, published on `127.0.0.1`</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`dashboard at http://127.0.0.1:&lt;port&gt;/`</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t xml:space="preserve">a name derived from the checkout's directory; a project per ticker; two checkouts of the project up at once on one host — they share the name: run one, or set `COMPOSE_PROJECT_NAME`</t>
+          <t xml:space="preserve">the internal port's number as the page's address in a document, a command or a comment; a second variable for it; `PORT` inside a container; a measurement outside the `Makefile`</t>
         </is>
       </c>
     </row>
@@ -15521,17 +15521,17 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t xml:space="preserve">how long a container lives: one-off — a `run --rm` process that exits with its stage — or resident — a server that stays up</t>
+          <t xml:space="preserve">the compose project: the one fixed name every container, network and volume of this project carries on every host</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run --rm -T`, the `run` macro of the `Makefile`, for a one-off; `up -d dashboard` of `make on` for the one resident</t>
+          <t xml:space="preserve">`name: liora` in `docker-compose.yml` — the resident `liora-dashboard-1`</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t xml:space="preserve">one-shot, ephemeral, daemon, long-running; `task` or `job` for the one-off; a stage run in a resident</t>
+          <t xml:space="preserve">a name derived from the checkout's directory; a project per ticker; two checkouts of the project up at once on one host — they share the name: run one, or set `COMPOSE_PROJECT_NAME`</t>
         </is>
       </c>
     </row>
@@ -15543,49 +15543,39 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t xml:space="preserve">the presentation switch: the dashboard up with the page's address printed and opened, or every container of this project down, in one word</t>
+          <t xml:space="preserve">how long a container lives: one-off — a `run --rm` process that exits with its stage — or resident — a server that stays up</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make on`, `make off` — the two bare lifecycle targets a presenter types</t>
+          <t xml:space="preserve">`run --rm -T`, the `run` macro of the `Makefile`, for a one-off; `up -d dashboard` of `make on` for the one resident</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t xml:space="preserve">`start` / `stop`, bare `up` / `down` (compose's), `run`, a second switch pair; a switch that runs a stage</t>
+          <t xml:space="preserve">one-shot, ephemeral, daemon, long-running; `task` or `job` for the one-off; a stage run in a resident</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run record</t>
+          <t xml:space="preserve">Asset containers</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t xml:space="preserve">one recorded run of the chain — the execution name, read forward</t>
+          <t xml:space="preserve">the presentation switch: the dashboard up with the page's address printed and opened, or every container of this project down, in one word</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run_id`; `RUN_ID` of the `Makefile`, `&lt;YYYYMMDDTHHMMSS&gt;Z_&lt;short commit&gt;` — the UTC time, then git's short commit — so it sorts by time and names the code that ran</t>
-        </is>
-      </c>
-      <c r="D383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`run_id`</t>
-        </is>
-      </c>
-      <c r="E383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">run</t>
+          <t xml:space="preserve">`make on`, `make off` — the two bare lifecycle targets a presenter types</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t xml:space="preserve">build, job, a content hash; a generated run id bound to no project name; a run id inside an artifact or a ledger</t>
+          <t xml:space="preserve">`start` / `stop`, bare `up` / `down` (compose's), `run`, a second switch pair; a switch that runs a stage</t>
         </is>
       </c>
     </row>
@@ -15597,27 +15587,27 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
+          <t xml:space="preserve">one recorded run of the chain — the execution name, read forward</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t xml:space="preserve">the target name; `RECORDED_STAGES` in the `Makefile` — `DATA_STAGES`, `FEATURES_STAGES`, `ML_STAGES` in order; `make all-record`</t>
+          <t xml:space="preserve">`run_id`; `RUN_ID` of the `Makefile`, `&lt;YYYYMMDDTHHMMSS&gt;Z_&lt;short commit&gt;` — the UTC time, then git's short commit — so it sorts by time and names the code that ran</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t xml:space="preserve">`stage` — the file name `&lt;stage&gt;.json`</t>
+          <t xml:space="preserve">`run_id`</t>
         </is>
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t xml:space="preserve">stage</t>
+          <t xml:space="preserve">run</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
+          <t xml:space="preserve">build, job, a content hash; a generated run id bound to no project name; a run id inside an artifact or a ledger</t>
         </is>
       </c>
     </row>
@@ -15629,22 +15619,27 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t xml:space="preserve">the command the recorder ran</t>
+          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command` — the make command line, joined by spaces</t>
+          <t xml:space="preserve">the target name; `RECORDED_STAGES` in the `Makefile` — `DATA_STAGES`, `FEATURES_STAGES`, `ML_STAGES` in order; `make all-record`</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command`</t>
+          <t xml:space="preserve">`stage` — the file name `&lt;stage&gt;.json`</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stage</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage's own command line; anything a stage says about itself</t>
+          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
         </is>
       </c>
     </row>
@@ -15656,27 +15651,22 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t xml:space="preserve">the exit code: how the stage ended; `all-record` stops at the first stage that exits non-zero and keeps its record</t>
+          <t xml:space="preserve">the command the recorder ran</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t xml:space="preserve">the command's exit code, `record.py`'s own</t>
+          <t xml:space="preserve">`command` — the make command line, joined by spaces</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t xml:space="preserve">`exit_code`</t>
-        </is>
-      </c>
-      <c r="E386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">exit</t>
+          <t xml:space="preserve">`command`</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t xml:space="preserve">status, ok</t>
+          <t xml:space="preserve">a stage's own command line; anything a stage says about itself</t>
         </is>
       </c>
     </row>
@@ -15688,27 +15678,27 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stage timing: when the stage ran, and for how long</t>
+          <t xml:space="preserve">the exit code: how the stage ended; `all-record` stops at the first stage that exits non-zero and keeps its record</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t xml:space="preserve">`main()` in `record.py` — the UTC clock before and after the command, the monotonic clock for the duration</t>
+          <t xml:space="preserve">the command's exit code, `record.py`'s own</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t xml:space="preserve">`started_at_utc`, `ended_at_utc`, `duration_seconds`</t>
+          <t xml:space="preserve">`exit_code`</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t xml:space="preserve">start; time; start / end and total time in the run's header</t>
+          <t xml:space="preserve">exit</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t xml:space="preserve">wall, elapsed</t>
+          <t xml:space="preserve">status, ok</t>
         </is>
       </c>
     </row>
@@ -15720,27 +15710,27 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store diff: what the stage did to the stores — every file added, changed (size or mtime moved) or removed, by store and path</t>
+          <t xml:space="preserve">the stage timing: when the stage ran, and for how long</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the four stores of `STORES` — every store but the trials store</t>
+          <t xml:space="preserve">`main()` in `record.py` — the UTC clock before and after the command, the monotonic clock for the duration</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t xml:space="preserve">`store_diff` with `added`, `changed` — each `store`, `path`, `size_bytes`, `mtime_ns` — and `removed` — each `store`, `path`</t>
+          <t xml:space="preserve">`started_at_utc`, `ended_at_utc`, `duration_seconds`</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t xml:space="preserve">added / changed / removed; bytes written; the STORES frame</t>
+          <t xml:space="preserve">start; time; start / end and total time in the run's header</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t xml:space="preserve">output, artifacts, a stage → artifact map; a trial ledger read by the recorder</t>
+          <t xml:space="preserve">wall, elapsed</t>
         </is>
       </c>
     </row>
@@ -15752,17 +15742,27 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t xml:space="preserve">the basket one run covered — not in the record: the recorder knows no basket</t>
+          <t xml:space="preserve">the store diff: what the stage did to the stores — every file added, changed (size or mtime moved) or removed, by store and path</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t xml:space="preserve">the launcher's `TICKERS`, which the make target the recorder wraps carries into every stage command</t>
+          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the four stores of `STORES` — every store but the trials store</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`store_diff` with `added`, `changed` — each `store`, `path`, `size_bytes`, `mtime_ns` — and `removed` — each `store`, `path`</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added / changed / removed; bytes written; the STORES frame</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ticker`, the first of the basket standing for it; one record per asset</t>
+          <t xml:space="preserve">output, artifacts, a stage → artifact map; a trial ledger read by the recorder</t>
         </is>
       </c>
     </row>
@@ -15774,27 +15774,17 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run index: every run with a record, newest first, each with its records — the one file the page reads to find a run</t>
+          <t xml:space="preserve">the basket one run covered — not in the record: the recorder knows no basket</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_run_index()` in `record.py`, written again after every record from the store's listing, as `store/run_records/index.json`</t>
-        </is>
-      </c>
-      <c r="D390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`generated_at_utc`; `runs[]`, each `run_id` and `records` — the record files, relative to the run's directory, in path order</t>
-        </is>
-      </c>
-      <c r="E390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`&lt;n&gt; recorded run(s) · showing &lt;run_id&gt; · &lt;n&gt; records`</t>
+          <t xml:space="preserve">the launcher's `TICKERS`, which the make target the recorder wraps carries into every stage command</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t xml:space="preserve">a run list per asset; a listing by the page; a route that lists the store; an index written by a stage</t>
+          <t xml:space="preserve">`ticker`, the first of the basket standing for it; one record per asset</t>
         </is>
       </c>
     </row>
@@ -15806,22 +15796,27 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stage records of one run, in the order the stages started — each read by the page at the relative path the index lists</t>
+          <t xml:space="preserve">the run index: every run with a record, newest first, each with its records — the one file the page reads to find a run</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t xml:space="preserve">`runs[].records` of the index; `fetchRunRecord()` in `module_monitoring/run.js`, which sorts them by `started_at_utc`</t>
+          <t xml:space="preserve">`build_run_index()` in `record.py`, written again after every record from the store's listing, as `store/run_records/index.json`</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`generated_at_utc`; `runs[]`, each `run_id` and `records` — the record files, relative to the run's directory, in path order</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAGES — stage, asset, start, time, exit, added, changed, removed, bytes written</t>
+          <t xml:space="preserve">`&lt;n&gt; recorded run(s) · showing &lt;run_id&gt; · &lt;n&gt; records`</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t xml:space="preserve">a record per asset of a basket stage; an envelope built by a server</t>
+          <t xml:space="preserve">a run list per asset; a listing by the page; a route that lists the store; an index written by a stage</t>
         </is>
       </c>
     </row>
@@ -15833,39 +15828,44 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, written whole after the stage's second listing so it never appears in its own difference; untracked</t>
+          <t xml:space="preserve">the stage records of one run, in the order the stages started — each read by the page at the relative path the index lists</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STORE_RUN_RECORDS_DIR`, `store/run_records/&lt;run_id&gt;/&lt;stage&gt;.json`; `write_json()` in `record.py`, beside its place, then moved onto it</t>
+          <t xml:space="preserve">`runs[].records` of the index; `fetchRunRecord()` in `module_monitoring/run.js`, which sorts them by `started_at_utc`</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STAGES — stage, asset, start, time, exit, added, changed, removed, bytes written</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `runtime/` folder under an asset; one run record per asset; a run record tracked</t>
+          <t xml:space="preserve">a record per asset of a basket stage; an envelope built by a server</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentation ownership</t>
+          <t xml:space="preserve">Run record</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generated document: one the sync renders from the sheet and a hand never edits, its first line the marker, its rules cited by `rule_id`</t>
+          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, written whole after the stage's second listing so it never appears in its own difference; untracked</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
+          <t xml:space="preserve">`STORE_RUN_RECORDS_DIR`, `store/run_records/&lt;run_id&gt;/&lt;stage&gt;.json`; `write_json()` in `record.py`, beside its place, then moved onto it</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Skill edited in its file; a Skill cited by a numbered or titled section — a rule is cited by its `rule_id`; a hand-written `skill_*.md`</t>
+          <t xml:space="preserve">a `runtime/` folder under an asset; one run record per asset; a run record tracked</t>
         </is>
       </c>
     </row>
@@ -15877,17 +15877,17 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hand-written document: one a hand keeps and the sync never touches, no marker on its first line</t>
+          <t xml:space="preserve">a generated document: one the sync renders from the sheet and a hand never edits, its first line the marker, its rules cited by `rule_id`</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md`, `CLAUDE.md`, `README.md`, `module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`, `module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`, every `README_sub_module_&lt;subject&gt;.md`, `module_skills/README.md`, `module_skills/sub_module_scalability_crawler/crawlers_mission.md`</t>
+          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule kept only there; a second copy of a rule</t>
+          <t xml:space="preserve">a Skill edited in its file; a Skill cited by a numbered or titled section — a rule is cited by its `rule_id`; a hand-written `skill_*.md`</t>
         </is>
       </c>
     </row>
@@ -15899,17 +15899,17 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t xml:space="preserve">a normative document describing one module's own responsibility</t>
+          <t xml:space="preserve">a hand-written document: one a hand keeps and the sync never touches, no marker on its first line</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_&lt;domain&gt;`</t>
+          <t xml:space="preserve">`AGENTS.md`, `CLAUDE.md`, `README.md`, `module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`, `module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`, every `README_sub_module_&lt;subject&gt;.md`, `module_skills/README.md`, `module_skills/sub_module_scalability_crawler/crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t xml:space="preserve">a module's rule kept in `module_skills/`; a per-module `docs/` or `doc/` folder</t>
+          <t xml:space="preserve">a rule kept only there; a second copy of a rule</t>
         </is>
       </c>
     </row>
@@ -15921,17 +15921,17 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t xml:space="preserve">a normative document that crosses modules or governs the project — the canon's</t>
+          <t xml:space="preserve">a normative document describing one module's own responsibility</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_skills`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_&lt;domain&gt;`</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t xml:space="preserve">a cross-cutting rule filed under one module; an edit to a copy</t>
+          <t xml:space="preserve">a module's rule kept in `module_skills/`; a per-module `docs/` or `doc/` folder</t>
         </is>
       </c>
     </row>
@@ -15943,17 +15943,17 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module skill: the normative document about one sub-module alone, kept beside its code as `skill_&lt;subject&gt;.md` — the serpentine search's and the crawler's; a terminal has none of its own, `module_skills/skill_tui_designer.md` holding what the terminals share</t>
+          <t xml:space="preserve">a normative document that crosses modules or governs the project — the canon's</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_&lt;subject&gt;/skill_&lt;subject&gt;.md`, rendered from its owner's tab</t>
+          <t xml:space="preserve">`module_skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_skills`</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module's own rule among `module_skills/skill_*.md` or in its module's `skills/`; a rule two sub-modules obey kept beside one of them; a `skill_&lt;module&gt;_terminal.md`; a `skills/` folder for one document</t>
+          <t xml:space="preserve">a cross-cutting rule filed under one module; an edit to a copy</t>
         </is>
       </c>
     </row>
@@ -15965,17 +15965,17 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t xml:space="preserve">the directory holding one module's own documents: its Skills and its methodology</t>
+          <t xml:space="preserve">a sub-module skill: the normative document about one sub-module alone, kept beside its code as `skill_&lt;subject&gt;.md` — the serpentine search's and the crawler's; a terminal has none of its own, `module_skills/skill_tui_designer.md` holding what the terminals share</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/`</t>
+          <t xml:space="preserve">`sub_module_&lt;subject&gt;/skill_&lt;subject&gt;.md`, rendered from its owner's tab</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skill/`, `module_&lt;domain&gt;/documentation/`</t>
+          <t xml:space="preserve">a sub-module's own rule among `module_skills/skill_*.md` or in its module's `skills/`; a rule two sub-modules obey kept beside one of them; a `skill_&lt;module&gt;_terminal.md`; a `skills/` folder for one document</t>
         </is>
       </c>
     </row>
@@ -15987,17 +15987,17 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t xml:space="preserve">the name register: one concept, one name, in code, artifacts and interface, and the copies no module may import across — rendered from the glossary table of the sheet with the register's own rules</t>
+          <t xml:space="preserve">the directory holding one module's own documents: its Skills and its methodology</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/`</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t xml:space="preserve">a register edited by hand; a second register; a name entering the tree in a commit that does not add its row</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skill/`, `module_&lt;domain&gt;/documentation/`</t>
         </is>
       </c>
     </row>
@@ -16009,17 +16009,17 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sheet: the one source of every Skill and of the register — a tab per owner, each with its rule table; the glossary and the `rule_type_id` list; the skill register and the files matrix</t>
+          <t xml:space="preserve">the name register: one concept, one name, in code, artifacts and interface, and the copies no module may import across — rendered from the glossary table of the sheet with the register's own rules</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skills_sheet.xlsx`, `SKILLS_SHEET_PATH`; `load_sheet()` in `module_skills/sheet.py`; `RULE_HEADER`, `SKILL_REGISTER_HEADER`, `GLOSSARY_HEADER`, `RULE_TYPE_ID_HEADER`, `FILES_MATRIX_HEADER` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Skill edited in its file; a second workbook; a CSV or JSON beside it; a sheet written by code</t>
+          <t xml:space="preserve">a register edited by hand; a second register; a name entering the tree in a commit that does not add its row</t>
         </is>
       </c>
     </row>
@@ -16031,17 +16031,17 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t xml:space="preserve">the skill register: a row per generated Skill — the tab that holds its rules, its `skill_path` and its summary</t>
+          <t xml:space="preserve">the sheet: the one source of every Skill and of the register — a tab per owner, each with its rule table; the glossary and the `rule_type_id` list; the skill register and the files matrix</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILL_REGISTER_HEADER` in `module_skills/config.py`; `Skill` in `module_skills/sheet.py`</t>
+          <t xml:space="preserve">`module_skills/skills_sheet.xlsx`, `SKILLS_SHEET_PATH`; `load_sheet()` in `module_skills/sheet.py`; `RULE_HEADER`, `SKILL_REGISTER_HEADER`, `GLOSSARY_HEADER`, `RULE_TYPE_ID_HEADER`, `FILES_MATRIX_HEADER` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t xml:space="preserve">document register, `DOCUMENT_REGISTER_HEADER`; a Skill without a register row; a summary in a rule row; an owner read off the files matrix</t>
+          <t xml:space="preserve">a Skill edited in its file; a second workbook; a CSV or JSON beside it; a sheet written by code</t>
         </is>
       </c>
     </row>
@@ -16053,17 +16053,17 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sync: every Skill and the register rendered from the sheet beside what each governs, and every generated file the sheet no longer names deleted</t>
+          <t xml:space="preserve">the skill register: a row per generated Skill — the tab that holds its rules, its `skill_path` and its summary</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make skills-sync`; `main()`, `to_markdown()`, `build_documents()`, `write_text()`, `delete_stale()` in `module_skills/sync.py`; `GENERATED_MARKER`</t>
+          <t xml:space="preserve">`SKILL_REGISTER_HEADER` in `module_skills/config.py`; `Skill` in `module_skills/sheet.py`</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t xml:space="preserve">distribute, generate, export; a stamp; a comparison of copies; a Markdown edited by hand; a sync that reads the sheet twice; a document without the marker deleted</t>
+          <t xml:space="preserve">document register, `DOCUMENT_REGISTER_HEADER`; a Skill without a register row; a summary in a rule row; an owner read off the files matrix</t>
         </is>
       </c>
     </row>
@@ -16075,17 +16075,17 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t xml:space="preserve">the table of every configurable: every CONFIGURABLES record of the controlled `config.py` files, read as literals, on stdout</t>
+          <t xml:space="preserve">the sync: every Skill and the register rendered from the sheet beside what each governs, and every generated file the sheet no longer names deleted</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make skills-configurables`; `main()`, `load_records()`, `to_cell()` in `module_skills/configurables.py`</t>
+          <t xml:space="preserve">`make skills-sync`; `main()`, `to_markdown()`, `build_documents()`, `write_text()`, `delete_stale()` in `module_skills/sync.py`; `GENERATED_MARKER`</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">a file the table is written into; an import of the module whose records it reads; a record the table carries and no `config.py` holds</t>
+          <t xml:space="preserve">distribute, generate, export; a stamp; a comparison of copies; a Markdown edited by hand; a sync that reads the sheet twice; a document without the marker deleted</t>
         </is>
       </c>
     </row>
@@ -16097,17 +16097,17 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t xml:space="preserve">the contract: what every change answers to, read in full before a session's first edit</t>
+          <t xml:space="preserve">the table of every configurable: every CONFIGURABLES record of the controlled `config.py` files, read as literals, on stdout</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md` at the root</t>
+          <t xml:space="preserve">`make skills-configurables`; `main()`, `load_records()`, `to_cell()` in `module_skills/configurables.py`</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second contract; a per-module `AGENTS.md`</t>
+          <t xml:space="preserve">a file the table is written into; an import of the module whose records it reads; a record the table carries and no `config.py` holds</t>
         </is>
       </c>
     </row>
@@ -16119,17 +16119,17 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
+          <t xml:space="preserve">the contract: what every change answers to, read in full before a session's first edit</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t xml:space="preserve">`CLAUDE.md` at the root</t>
+          <t xml:space="preserve">`AGENTS.md` at the root</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule written in it; a per-module `CLAUDE.md`; `CLAUDE.local.md` or `.claude/` inside the tree</t>
+          <t xml:space="preserve">a second contract; a per-module `AGENTS.md`</t>
         </is>
       </c>
     </row>
@@ -16141,17 +16141,17 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t xml:space="preserve">the project's front door: what the project is, how to run it and where its Skills are</t>
+          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README.md` at the root</t>
+          <t xml:space="preserve">`CLAUDE.md` at the root</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule restated in it; a front door that restates a Skill or a decision table</t>
+          <t xml:space="preserve">a rule written in it; a per-module `CLAUDE.md`; `CLAUDE.local.md` or `.claude/` inside the tree</t>
         </is>
       </c>
     </row>
@@ -16163,17 +16163,17 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t xml:space="preserve">one module's reader-facing front door, its orientation</t>
+          <t xml:space="preserve">the project's front door: what the project is, how to run it and where its Skills are</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`README.md` at the root</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/README.md`; an orientation that restates a Skill or a decision table</t>
+          <t xml:space="preserve">a rule restated in it; a front door that restates a Skill or a decision table</t>
         </is>
       </c>
     </row>
@@ -16185,17 +16185,17 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module's orientation, beside its code</t>
+          <t xml:space="preserve">one module's reader-facing front door, its orientation</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/README.md`; an orientation that restates a Skill or a decision table</t>
         </is>
       </c>
     </row>
@@ -16207,17 +16207,17 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t xml:space="preserve">the design rationale: the section of a module's orientation that says, per object, analogous pair or the module's documents, why here, why beside these, why this boundary and which mapping row it answers to — the fourth the test of the first three</t>
+          <t xml:space="preserve">a sub-module's orientation, beside its code</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t xml:space="preserve">`## Design rationale` of each `README_module_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t xml:space="preserve">a decision table; a rule restated; an object with no row or two; ADR, decision record, decision log, `docs/`</t>
+          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
         </is>
       </c>
     </row>
@@ -16229,17 +16229,17 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t xml:space="preserve">a methodology document: reference material for a human — the equations, the derivations and the citations of one module</t>
+          <t xml:space="preserve">the design rationale: the section of a module's orientation that says, per object, analogous pair or the module's documents, why here, why beside these, why this boundary and which mapping row it answers to — the fourth the test of the first three</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`## Design rationale` of each `README_module_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t xml:space="preserve">a row of the files matrix; a document the crawler sends; a rule stated only there</t>
+          <t xml:space="preserve">a decision table; a rule restated; an object with no row or two; ADR, decision record, decision log, `docs/`</t>
         </is>
       </c>
     </row>
@@ -16251,44 +16251,39 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t xml:space="preserve">the canon's index: every Skill by its path, and the canon's prose that is no rule, the mapping table among it</t>
+          <t xml:space="preserve">a methodology document: reference material for a human — the equations, the derivations and the citations of one module</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/README.md`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t xml:space="preserve">a collection of copies; an index that restates a rule it links to</t>
+          <t xml:space="preserve">a row of the files matrix; a document the crawler sends; a rule stated only there</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-AWS direction</t>
+          <t xml:space="preserve">Documentation ownership</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stance: a local academic architecture whose boundaries would survive a move onto standard cloud primitives, with no cloud used and none planned</t>
+          <t xml:space="preserve">the canon's index: every Skill by its path, and the canon's prose that is no rule, the mapping table among it</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_pre_aws_solution.md` — `pre_aws` its stem, the one tracked name that carries the word; no identifier</t>
+          <t xml:space="preserve">`module_skills/README.md`</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t xml:space="preserve">cloud-ready, AWS-ready, cloud-native; a migration plan, a deployment guide; `pre-aws` or `PreAWS` in prose</t>
-        </is>
-      </c>
-      <c r="I412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pre-AWS — before Amazon Web Services (AWS), the cloud the mapping reads forward to</t>
+          <t xml:space="preserve">a collection of copies; an index that restates a rule it links to</t>
         </is>
       </c>
     </row>
@@ -16300,22 +16295,22 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t xml:space="preserve">compute: a process that reads a store, writes a store and exits, owning no asset state between invocations</t>
+          <t xml:space="preserve">the stance: a local academic architecture whose boundaries would survive a move onto standard cloud primitives, with no cloud used and none planned</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t xml:space="preserve">every stage's `main()`, `python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;`; the one-off container that runs it</t>
+          <t xml:space="preserve">`module_skills/skill_pre_aws_solution.md` — `pre_aws` its stem, the one tracked name that carries the word; no identifier</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t xml:space="preserve">a container as the home of an asset's state; a resident as a requirement of a stage; an in-process cache between stages; `worker`, `processor`</t>
+          <t xml:space="preserve">cloud-ready, AWS-ready, cloud-native; a migration plan, a deployment guide; `pre-aws` or `PreAWS` in prose</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t xml:space="preserve">a task — one run of the one task definition on the container instance every asset's runs share (Amazon ECS on Amazon EC2)</t>
+          <t xml:space="preserve">Pre-AWS — before Amazon Web Services (AWS), the cloud the mapping reads forward to</t>
         </is>
       </c>
     </row>
@@ -16327,22 +16322,22 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t xml:space="preserve">the rebuild condition: whether an asset's artifacts must be rebuilt from its canonical series, answered without launching anything; its freshness half is unwritten, its names reserved — `has_new_market_data()`, `requires_canonical_rebuild()`, `requires_feature_rebuild()`, `requires_model_rebuild()`</t>
+          <t xml:space="preserve">compute: a process that reads a store, writes a store and exits, owning no asset state between invocations</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t xml:space="preserve">`is_artifact_set_complete()` in `module_ml/config.py`, its completeness half; the rerun table of `module_ml/skills/methodology_ml.md`, read by a human</t>
+          <t xml:space="preserve">every stage's `main()`, `python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;`; the one-off container that runs it</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t xml:space="preserve">a scheduler, a watcher, an event bus; a function that both detects new data and trains; `should_run()`, `check_update()`, `trigger()`</t>
+          <t xml:space="preserve">a container as the home of an asset's state; a resident as a requirement of a stage; an in-process cache between stages; `worker`, `processor`</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">a choice state between two states of the machine (AWS Step Functions)</t>
+          <t xml:space="preserve">a task — one run of the one task definition on the container instance every asset's runs share (Amazon ECS on Amazon EC2)</t>
         </is>
       </c>
     </row>
@@ -16354,17 +16349,22 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mapping table: what this repository has, the responsibility, the same responsibility elsewhere and the move, row by row — the one table that sets a cloud proper noun beside a local object; its third column is the elsewhere column</t>
+          <t xml:space="preserve">the rebuild condition: whether an asset's artifacts must be rebuilt from its canonical series, answered without launching anything; its freshness half is unwritten, its names reserved — `has_new_market_data()`, `requires_canonical_rebuild()`, `requires_feature_rebuild()`, `requires_model_rebuild()`</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/README.md`, its hand-written home</t>
+          <t xml:space="preserve">`is_artifact_set_complete()` in `module_ml/config.py`, its completeness half; the rerun table of `module_ml/skills/methodology_ml.md`, read by a human</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t xml:space="preserve">an adapter, a cloud configuration file; a cloud proper noun in an identifier, a key, a path, a make target, a compose service or an environment variable; a path of the elsewhere column read as a proposal for a local directory</t>
+          <t xml:space="preserve">a scheduler, a watcher, an event bus; a function that both detects new data and trains; `should_run()`, `check_update()`, `trigger()`</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a choice state between two states of the machine (AWS Step Functions)</t>
         </is>
       </c>
     </row>
@@ -16376,17 +16376,17 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t xml:space="preserve">a seat: the standard primitive a local object would sit on elsewhere, named in the mapping table's words — spoken in the stance's skill and in the mapping table, and in no other Skill</t>
+          <t xml:space="preserve">the mapping table: what this repository has, the responsibility, the same responsibility elsewhere and the move, row by row — the one table that sets a cloud proper noun beside a local object; its third column is the elsewhere column</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`module_skills/README.md`, its hand-written home</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t xml:space="preserve">a seat paragraph in any other Skill; two seats for one object; a seat in an identifier, a key or a path; `target`, `cloud note`, `mapping section`</t>
-        </is>
-      </c>
-      <c r="I416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the image registry (Amazon ECR), the container service (Amazon ECS), the container instance (Amazon EC2), the block volume (Amazon EBS), object storage (Amazon S3), the state machine (AWS Step Functions), the schedule (Amazon EventBridge Scheduler)</t>
+          <t xml:space="preserve">an adapter, a cloud configuration file; a cloud proper noun in an identifier, a key, a path, a make target, a compose service or an environment variable; a path of the elsewhere column read as a proposal for a local directory</t>
         </is>
       </c>
     </row>
@@ -16398,17 +16398,17 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t xml:space="preserve">the resource role: the name a cloud resource would carry, `&lt;project&gt;-&lt;environment&gt;-&lt;resource-role&gt;` — the role a seat's name or the task a row of the mapping table names, lower case with `-` between its words, the project `liora`</t>
-        </is>
-      </c>
-      <c r="C417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`name: liora` and `liora-1m-pipeline` in `docker-compose.yml` — the names of that shape the tree holds, with no environment token</t>
+          <t xml:space="preserve">a seat: the standard primitive a local object would sit on elsewhere, named in the mapping table's words — spoken in the stance's skill and in the mapping table, and in no other Skill</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second list of roles; a role no seat or row names; `dev` or `prod` in a tracked name; a ticker in a resource name; an environment token on the image</t>
+          <t xml:space="preserve">a seat paragraph in any other Skill; two seats for one object; a seat in an identifier, a key or a path; `target`, `cloud note`, `mapping section`</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the image registry (Amazon ECR), the container service (Amazon ECS), the container instance (Amazon EC2), the block volume (Amazon EBS), object storage (Amazon S3), the state machine (AWS Step Functions), the schedule (Amazon EventBridge Scheduler)</t>
         </is>
       </c>
     </row>
@@ -16420,17 +16420,17 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state name: the one-line name a stage would carry as a state of the machine, one per stage, and PublishStores, the copy after a run, which no stage answers to; *Publish* in a state name means write the object where its readers read it</t>
+          <t xml:space="preserve">the resource role: the name a cloud resource would carry, `&lt;project&gt;-&lt;environment&gt;-&lt;resource-role&gt;` — the role a seat's name or the task a row of the mapping table names, lower case with `-` between its words, the project `liora`</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`name: liora` and `liora-1m-pipeline` in `docker-compose.yml` — the names of that shape the tree holds, with no environment token</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state registered one by one; a state name with *and* in it; *publish* as *make public*</t>
-        </is>
-      </c>
-      <c r="I418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a state of AWS Step Functions</t>
+          <t xml:space="preserve">a second list of roles; a role no seat or row names; `dev` or `prod` in a tracked name; a ticker in a resource name; an environment token on the image</t>
         </is>
       </c>
     </row>
@@ -16442,17 +16442,17 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t xml:space="preserve">an instance: one Linux virtual machine elsewhere, the host containers run on — the task host every asset's runs share, with the store volume beside it, and the strategy host</t>
+          <t xml:space="preserve">a state name: the one-line name a stage would carry as a state of the machine, one per stage, and PublishStores, the copy after a run, which no stage answers to; *Publish* in a state name means write the object where its readers read it</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t xml:space="preserve">`instance` or `host` for a container; a host per asset; node</t>
+          <t xml:space="preserve">a state registered one by one; a state name with *and* in it; *publish* as *make public*</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t xml:space="preserve">a container instance (Amazon EC2)</t>
+          <t xml:space="preserve">a state of AWS Step Functions</t>
         </is>
       </c>
     </row>
@@ -16464,22 +16464,17 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store volume: the task host's durable disk — the five stores at `/store/&lt;content&gt;`, each at the path its `STORE_*_DIR` names; the home of state, never the copy</t>
-        </is>
-      </c>
-      <c r="C420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the `./store/&lt;content&gt;` mounts of `docker-compose.yml`, read forward as `&lt;volume&gt;/&lt;content&gt;:/store/&lt;content&gt;`</t>
+          <t xml:space="preserve">an instance: one Linux virtual machine elsewhere, the host containers run on — the task host every asset's runs share, with the store volume beside it, and the strategy host</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset volume; a volume per asset; the volume as the copy; `data_volume`; a shared network filesystem (Amazon EFS)</t>
+          <t xml:space="preserve">`instance` or `host` for a container; a host per asset; node</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t xml:space="preserve">a block volume (Amazon EBS)</t>
+          <t xml:space="preserve">a container instance (Amazon EC2)</t>
         </is>
       </c>
     </row>
@@ -16491,17 +16486,22 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t xml:space="preserve">the copy: the whole files a state after the last stage of a run would copy from the store volume to object storage — never a stage's own write, never mid-run; absent here, described</t>
+          <t xml:space="preserve">the store volume: the task host's durable disk — the five stores at `/store/&lt;content&gt;`, each at the path its `STORE_*_DIR` names; the home of state, never the copy</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the `./store/&lt;content&gt;` mounts of `docker-compose.yml`, read forward as `&lt;volume&gt;/&lt;content&gt;:/store/&lt;content&gt;`</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage writing to object storage; a stage reading the copy; `s3://` in a path constant; an adapter for the copy</t>
+          <t xml:space="preserve">asset volume; a volume per asset; the volume as the copy; `data_volume`; a shared network filesystem (Amazon EFS)</t>
         </is>
       </c>
       <c r="I421" t="inlineStr">
         <is>
-          <t xml:space="preserve">object storage (Amazon S3), written by PublishStores</t>
+          <t xml:space="preserve">a block volume (Amazon EBS)</t>
         </is>
       </c>
     </row>
@@ -16513,12 +16513,17 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t xml:space="preserve">the ladder: the three phases in which the runtime elsewhere would become true, each named for what it changes — *the lift*, *the idiom*, *the image carries the code*; all elsewhere, built nowhere here</t>
+          <t xml:space="preserve">the copy: the whole files a state after the last stage of a run would copy from the store volume to object storage — never a stage's own write, never mid-run; absent here, described</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t xml:space="preserve">a letter or a number for a phase; a phase as a branch or an environment; `dev` / `prod`; a phase built here; rung</t>
+          <t xml:space="preserve">a stage writing to object storage; a stage reading the copy; `s3://` in a path constant; an adapter for the copy</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">object storage (Amazon S3), written by PublishStores</t>
         </is>
       </c>
     </row>
@@ -16530,17 +16535,12 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion threshold: a second concurrent writer of one partition, or a reader that needs one transaction across families — the one condition under which a managed database replaces the table families</t>
+          <t xml:space="preserve">the ladder: the three phases in which the runtime elsewhere would become true, each named for what it changes — *the lift*, *the idiom*, *the image carries the code*; all elsewhere, built nowhere here</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t xml:space="preserve">a database process for one writer; a threshold in rows or bytes</t>
-        </is>
-      </c>
-      <c r="I423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a managed database (Amazon RDS)</t>
+          <t xml:space="preserve">a letter or a number for a phase; a phase as a branch or an environment; `dev` / `prod`; a phase built here; rung</t>
         </is>
       </c>
     </row>
@@ -16552,22 +16552,17 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t xml:space="preserve">the active version: the one version of an asset's artifacts a reader reads, chosen where the reader is; the version is the execution name</t>
-        </is>
-      </c>
-      <c r="C424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`run_id`</t>
+          <t xml:space="preserve">the promotion threshold: a second concurrent writer of one partition, or a reader that needs one transaction across families — the one condition under which a managed database replaces the table families</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t xml:space="preserve">latest, current, prod; a mark inside a file; a version inside an artifact</t>
+          <t xml:space="preserve">a database process for one writer; a threshold in rows or bytes</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">the version prefix `assets_artifacts/&lt;run_id&gt;/` of the copy (Amazon S3)</t>
+          <t xml:space="preserve">a managed database (Amazon RDS)</t>
         </is>
       </c>
     </row>
@@ -16579,22 +16574,22 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t xml:space="preserve">the tunnel: how a reader reaches the page on a host that is not theirs — a local forward onto the loopback port `make on` printed there</t>
+          <t xml:space="preserve">the active version: the one version of an asset's artifacts a reader reads, chosen where the reader is; the version is the execution name</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ssh -N -L` of `README.md` § Quickstart</t>
+          <t xml:space="preserve">`run_id`</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t xml:space="preserve">a public port; a load balancer</t>
+          <t xml:space="preserve">latest, current, prod; a mark inside a file; a version inside an artifact</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t xml:space="preserve">a port-forward, the elsewhere column's word</t>
+          <t xml:space="preserve">the version prefix `assets_artifacts/&lt;run_id&gt;/` of the copy (Amazon S3)</t>
         </is>
       </c>
     </row>
@@ -16606,12 +16601,22 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t xml:space="preserve">read forward: a local object read as the same responsibility elsewhere — the mapping table's third column — with nothing moved</t>
+          <t xml:space="preserve">the tunnel: how a reader reaches the page on a host that is not theirs — a local forward onto the loopback port `make on` printed there</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`ssh -N -L` of `README.md` § Quickstart</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t xml:space="preserve">migrated, ported, deployed, in production</t>
+          <t xml:space="preserve">a public port; a load balancer</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a port-forward, the elsewhere column's word</t>
         </is>
       </c>
     </row>
@@ -16623,12 +16628,12 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t xml:space="preserve">the move: what a local thing's seat elsewhere costs it — a rename, one edit, or absent here, described; the mapping table's fourth column</t>
+          <t xml:space="preserve">read forward: a local object read as the same responsibility elsewhere — the mapping table's third column — with nothing moved</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t xml:space="preserve">migration, deployment, a plan, a roadmap</t>
+          <t xml:space="preserve">migrated, ported, deployed, in production</t>
         </is>
       </c>
     </row>
@@ -16640,44 +16645,34 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t xml:space="preserve">an absent object: a primitive, a state of the machine or a Skill that nothing local answers to and a document describes — a sentence ending, or a verdict reading, *absent here — described*</t>
-        </is>
-      </c>
-      <c r="C428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`AGENTS.md` § Skills absent here, described, for the Skills</t>
+          <t xml:space="preserve">the move: what a local thing's seat elsewhere costs it — a rename, one edit, or absent here, described; the mapping table's fourth column</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t xml:space="preserve">planned, a debt marker, future, ghost, placeholder, missing</t>
+          <t xml:space="preserve">migration, deployment, a plan, a roadmap</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t xml:space="preserve">The page</t>
+          <t xml:space="preserve">Pre-AWS direction</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page: one static page of plain HTML, CSS and JavaScript that reads every datum by a relative path and writes nothing</t>
+          <t xml:space="preserve">an absent object: a primitive, a state of the machine or a Skill that nothing local answers to and a document describes — a sentence ending, or a verdict reading, *absent here — described*</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/index.html`, `style.css` and its scripts `page.js`, `data.js`, `asset.js`, `features.js`, `ml.js`, `run.js`, `scalability.js`</t>
-        </is>
-      </c>
-      <c r="E429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1m crypto research pipeline — status</t>
+          <t xml:space="preserve">`AGENTS.md` § Skills absent here, described, for the Skills</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t xml:space="preserve">a framework or a build step; a second page beside it; a datum computed by the server; an absolute path</t>
+          <t xml:space="preserve">planned, a debt marker, future, ghost, placeholder, missing</t>
         </is>
       </c>
     </row>
@@ -16689,17 +16684,22 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page's reads: where the page takes its data from, by relative path</t>
+          <t xml:space="preserve">the page: one static page of plain HTML, CSS and JavaScript that reads every datum by a relative path and writes nothing</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t xml:space="preserve">`status/data_status.json`, `status/features_status.json`, `status/ml_status.json`, `status/skills_status.json`; `run_records/index.json`, then each record of a run at `run_records/&lt;run_id&gt;/` and the path the index lists</t>
+          <t xml:space="preserve">`module_monitoring/index.html`, `style.css` and its scripts `page.js`, `data.js`, `asset.js`, `features.js`, `ml.js`, `run.js`, `scalability.js`</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1m crypto research pipeline — status</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t xml:space="preserve">an absolute path; a route per snapshot; a directory listing; a store the page reads beside these two</t>
+          <t xml:space="preserve">a framework or a build step; a second page beside it; a datum computed by the server; an absolute path</t>
         </is>
       </c>
     </row>
@@ -16711,22 +16711,17 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three prefixes: what the dashboard's server answers — the page's own files at `/`, the status store under `/status/`, the run-records store under `/run_records/`; every other path 404, and no directory listed</t>
+          <t xml:space="preserve">the page's reads: where the page takes its data from, by relative path</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/serve.py` — `DashboardHandler`, `translate_path()`, `main()`; `STORE_DIR_BY_ROUTE_PREFIX` in `module_monitoring/config.py`, `/status/` onto `STORE_STATUS_DIR` and `/run_records/` onto `STORE_RUN_RECORDS_DIR`; `MODULE_MONITORING_DIR`, `PAGE_FILE_SUFFIXES`, `PAGE_INDEX_FILE_NAME` for the page's own files</t>
+          <t xml:space="preserve">`status/data_status.json`, `status/features_status.json`, `status/ml_status.json`, `status/skills_status.json`; `run_records/index.json`, then each record of a run at `run_records/&lt;run_id&gt;/` and the path the index lists</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t xml:space="preserve">a route per snapshot; a directory listed; a path outside the three prefixes answered; a server that computes, writes or proxies; `dashboard.py`, `proxy.py`, `server.py` beside `serve.py`</t>
-        </is>
-      </c>
-      <c r="I431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`http.server`</t>
+          <t xml:space="preserve">an absolute path; a route per snapshot; a directory listing; a store the page reads beside these two</t>
         </is>
       </c>
     </row>
@@ -16738,17 +16733,22 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t xml:space="preserve">the toolkit the page loads before its own sections</t>
+          <t xml:space="preserve">the three prefixes: what the dashboard's server answers — the page's own files at `/`, the status store under `/status/`, the run-records store under `/run_records/`; every other path 404, and no directory listed</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t xml:space="preserve">`page.js`</t>
+          <t xml:space="preserve">`module_monitoring/serve.py` — `DashboardHandler`, `translate_path()`, `main()`; `STORE_DIR_BY_ROUTE_PREFIX` in `module_monitoring/config.py`, `/status/` onto `STORE_STATUS_DIR` and `/run_records/` onto `STORE_RUN_RECORDS_DIR`; `MODULE_MONITORING_DIR`, `PAGE_FILE_SUFFIXES`, `PAGE_INDEX_FILE_NAME` for the page's own files</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t xml:space="preserve">`utils.js`, `common.js`, `shared.js`, `lib.js`; a page-specific element written from it; a second page beside the status page</t>
+          <t xml:space="preserve">a route per snapshot; a directory listed; a path outside the three prefixes answered; a server that computes, writes or proxies; `dashboard.py`, `proxy.py`, `server.py` beside `serve.py`</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`http.server`</t>
         </is>
       </c>
     </row>
@@ -16760,17 +16760,17 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one selector component of the page — the top tabs, the ML Assets views, the asset rows — each group wired by its `data-key`</t>
+          <t xml:space="preserve">the toolkit the page loads before its own sections</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.pills`, `.pill`, `.pill--active`, `initPills()`, `PILL_HOOKS` in `page.js`; `data-pills` on a group, `data-panel` on its panels</t>
+          <t xml:space="preserve">`page.js`</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second selector component</t>
+          <t xml:space="preserve">`utils.js`, `common.js`, `shared.js`, `lib.js`; a page-specific element written from it; a second page beside the status page</t>
         </is>
       </c>
     </row>
@@ -16782,44 +16782,44 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page's navigation: the seven tabs, the five views of the ML Assets tab, and one row per asset</t>
+          <t xml:space="preserve">the one selector component of the page — the top tabs, the ML Assets views, the asset rows — each group wired by its `data-key`</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t xml:space="preserve">the groups of `data-pills` in `module_monitoring/index.html` — `tab`: `pipeline`, `quality`, `features`, `ml`, `asset`, `scalability`, `lifecycle`; `mlview`: `labels`, `classification`, `strategy`, `search`, `feature-set`; `asset`, filled from the snapshot</t>
-        </is>
-      </c>
-      <c r="E434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pipeline; Data Quality; Features; ML Research; ML Assets; Scalability; Lifecycle — Labels &amp; data; Classification; Strategy; HPO; Feature set</t>
+          <t xml:space="preserve">`.pills`, `.pill`, `.pill--active`, `initPills()`, `PILL_HOOKS` in `page.js`; `data-pills` on a group, `data-panel` on its panels</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t xml:space="preserve">a menu, a sidebar or a second navigation; a tab named for a tool</t>
+          <t xml:space="preserve">a second selector component</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scalability crawler</t>
+          <t xml:space="preserve">The page</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t xml:space="preserve">the crawler: the canon's sub-module that reads each controlled file against the Skills marked for it with the one active vendor, and writes a report per file and its snapshot; it asks nothing, goes on past a failed file and gates nothing</t>
+          <t xml:space="preserve">the page's navigation: the seven tabs, the five views of the ML Assets tab, and one row per asset</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_scalability_crawler`; `make skills-crawl`, after `make skills-sync`; `main()` in `crawl.py`</t>
+          <t xml:space="preserve">the groups of `data-pills` in `module_monitoring/index.html` — `tab`: `pipeline`, `quality`, `features`, `ml`, `asset`, `scalability`, `lifecycle`; `mlview`: `labels`, `classification`, `strategy`, `search`, `feature-set`; `asset`, filled from the snapshot</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pipeline; Data Quality; Features; ML Research; ML Assets; Scalability; Lifecycle — Labels &amp; data; Classification; Strategy; HPO; Feature set</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t xml:space="preserve">a linter, a check, a gate, a CI step; a web crawler, walking sites or services to gather what they hold; conformance, review — names that tell a reader nothing; a TUI of its own, `make skills-terminal` being the canon's terminal</t>
+          <t xml:space="preserve">a menu, a sidebar or a second navigation; a tab named for a tool</t>
         </is>
       </c>
     </row>
@@ -16831,22 +16831,17 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t xml:space="preserve">the files matrix: a row per path — a file or a glob — a column per Skill headed by its stem, an `X` where that Skill is sent with the file; the crawler's whole contract</t>
+          <t xml:space="preserve">the crawler: the canon's sub-module that reads each controlled file against the Skills marked for it with the one active vendor, and writes a report per file and its snapshot; it asks nothing, goes on past a failed file and gates nothing</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t xml:space="preserve">the table of the sheet headed by `FILES_MATRIX_HEADER` in `module_skills/config.py`; `Mark` in `module_skills/sheet.py`</t>
-        </is>
-      </c>
-      <c r="E436" t="inlineStr">
-        <is>
-          <t xml:space="preserve">path; the Skill's stem; `X`</t>
+          <t xml:space="preserve">`sub_module_scalability_crawler`; `make skills-crawl`, after `make skills-sync`; `main()` in `crawl.py`</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column per rule; a mark a crawl writes; a mark derived from `scope`; a generated file, a report or the snapshot as a target; a second row for one path; a precedence between rows; a Markdown table kept beside the crawler</t>
+          <t xml:space="preserve">a linter, a check, a gate, a CI step; a web crawler, walking sites or services to gather what they hold; conformance, review — names that tell a reader nothing; a TUI of its own, `make skills-terminal` being the canon's terminal</t>
         </is>
       </c>
     </row>
@@ -16858,22 +16853,22 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t xml:space="preserve">a mark: `X` under a Skill's column in a row of the files matrix, sending that Skill with every file the row reaches; two rows that reach one file join their marks</t>
+          <t xml:space="preserve">the files matrix: a row per path — a file or a glob — a column per Skill headed by its stem, an `X` where that Skill is sent with the file; the crawler's whole contract</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILL_MARK` in `module_skills/config.py`</t>
+          <t xml:space="preserve">the table of the sheet headed by `FILES_MATRIX_HEADER` in `module_skills/config.py`; `Mark` in `module_skills/sheet.py`</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">`X`; marked; unmarked</t>
+          <t xml:space="preserve">path; the Skill's stem; `X`</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t xml:space="preserve">assign, tag, tick, check, enable; `x`, `✓` or `yes` in a cell; a mark a crawl writes; a mark derived from `scope`; a row that marks no Skill</t>
+          <t xml:space="preserve">a column per rule; a mark a crawl writes; a mark derived from `scope`; a generated file, a report or the snapshot as a target; a second row for one path; a precedence between rows; a Markdown table kept beside the crawler</t>
         </is>
       </c>
     </row>
@@ -16885,22 +16880,22 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t xml:space="preserve">a controlled file: a file a row of the files matrix reaches, read against the Skills marked for it; its key is its path from the root of the tree</t>
+          <t xml:space="preserve">a mark: `X` under a Skill's column in a row of the files matrix, sending that Skill with every file the row reaches; two rows that reach one file join their marks</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ControlledFile`, `build_controlled_files()` in `crawl.py`</t>
+          <t xml:space="preserve">`SKILL_MARK` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">`X`; marked; unmarked</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t xml:space="preserve">listed file; a file the crawler finds by itself; a file read from the working directory; a rendered Skill or the snapshot as a controlled file</t>
+          <t xml:space="preserve">assign, tag, tick, check, enable; `x`, `✓` or `yes` in a cell; a mark a crawl writes; a mark derived from `scope`; a row that marks no Skill</t>
         </is>
       </c>
     </row>
@@ -16912,17 +16907,22 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t xml:space="preserve">the context: the documents sent with a file — the Skills its row of the files matrix marks, each whole as `make skills-sync` rendered it</t>
+          <t xml:space="preserve">a controlled file: a file a row of the files matrix reaches, read against the Skills marked for it; its key is its path from the root of the tree</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_skill_texts()`, `build_message()` in `crawl.py`</t>
+          <t xml:space="preserve">`ControlledFile`, `build_controlled_files()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule filtered out by its `scope` before it is sent; a Skill not marked; the contract; an orientation; a methodology; a list of rules kept per module</t>
+          <t xml:space="preserve">listed file; a file the crawler finds by itself; a file read from the working directory; a rendered Skill or the snapshot as a controlled file</t>
         </is>
       </c>
     </row>
@@ -16934,17 +16934,17 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t xml:space="preserve">a file's message: the Skills marked for it, then the file with every line after its number, then the mission</t>
+          <t xml:space="preserve">the context: the documents sent with a file — the Skills its row of the files matrix marks, each whole as `make skills-sync` rendered it</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_message()` in `crawl.py`; `crawlers_mission.md`</t>
+          <t xml:space="preserve">`load_skill_texts()`, `build_message()` in `crawl.py`</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t xml:space="preserve">a list of unmarked Skills; an orientation; a commit; a measure of the message; a line number the agent has to count</t>
+          <t xml:space="preserve">a rule filtered out by its `scope` before it is sent; a Skill not marked; the contract; an orientation; a methodology; a list of rules kept per module</t>
         </is>
       </c>
     </row>
@@ -16956,17 +16956,17 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mission: what the agent reports of one file, and how — kept by hand</t>
+          <t xml:space="preserve">a file's message: the Skills marked for it, then the file with every line after its number, then the mission</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t xml:space="preserve">`crawlers_mission.md`, `CRAWLERS_MISSION_MD_PATH`</t>
+          <t xml:space="preserve">`build_message()` in `crawl.py`; `crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule restated in it; a work order or a plan</t>
+          <t xml:space="preserve">a list of unmarked Skills; an orientation; a commit; a measure of the message; a line number the agent has to count</t>
         </is>
       </c>
     </row>
@@ -16978,17 +16978,17 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sub-module's folder and the root of the tree: where the crawler's own files are read, and where a controlled file and a Skill lie and the vendor runs</t>
+          <t xml:space="preserve">the mission: what the agent reports of one file, and how — kept by hand</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SUB_MODULE_DIR` in the crawler's `config.py`; `TREE_ROOT_DIR` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`crawlers_mission.md`, `CRAWLERS_MISSION_MD_PATH`</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t xml:space="preserve">a host path; a controlled file read from the working directory</t>
+          <t xml:space="preserve">a rule restated in it; a work order or a plan</t>
         </is>
       </c>
     </row>
@@ -17000,22 +17000,17 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t xml:space="preserve">a vendor: an agent's command line the crawl sends each controlled file to — one table of `vendors_for_crawling.toml`, exactly one `active`, its `argv` the whole command line, run without a shell, the message on its stdin and the answer its stdout</t>
+          <t xml:space="preserve">the sub-module's folder and the root of the tree: where the crawler's own files are read, and where a controlled file and a Skill lie and the vendor runs</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t xml:space="preserve">`vendors_for_crawling.toml` with `active`, `argv`; `VENDORS_FOR_CRAWLING_TOML_PATH`, `load_vendor()`, `AGENT_TIMEOUT_SECONDS`</t>
-        </is>
-      </c>
-      <c r="E443" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vendor</t>
+          <t xml:space="preserve">`SUB_MODULE_DIR` in the crawler's `config.py`; `TREE_ROOT_DIR` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t xml:space="preserve">an API key; a vendor named in the code; a form for its model, effort or permissions; a vendor chosen on a screen; two active vendors; every vendor run in turn</t>
+          <t xml:space="preserve">a host path; a controlled file read from the working directory</t>
         </is>
       </c>
     </row>
@@ -17027,27 +17022,22 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t xml:space="preserve">a report: the one current file per controlled file — the file's key, the vendor and the time, then the answer as it came; reset by every crawl, never tracked</t>
+          <t xml:space="preserve">a vendor: an agent's command line the crawl sends each controlled file to — one table of `vendors_for_crawling.toml`, exactly one `active`, its `argv` the whole command line, run without a shell, the message on its stdin and the answer its stdout</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t xml:space="preserve">`REPORTS_DIR`, `report_path()` in the crawler's `config.py` — `store/status/reports_after_crawled_files/&lt;path&gt;.report.md`; `write_atomically()` in `status.py`</t>
-        </is>
-      </c>
-      <c r="D444" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`report`</t>
+          <t xml:space="preserve">`vendors_for_crawling.toml` with `active`, `argv`; `VENDORS_FOR_CRAWLING_TOML_PATH`, `load_vendor()`, `AGENT_TIMEOUT_SECONDS`</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">vendor</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t xml:space="preserve">a history of entries; an append; a report in the sub-module's folder; a commit in its first line; a report tracked</t>
+          <t xml:space="preserve">an API key; a vendor named in the code; a form for its model, effort or permissions; a vendor chosen on a screen; two active vendors; every vendor run in turn</t>
         </is>
       </c>
     </row>
@@ -17059,17 +17049,27 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t xml:space="preserve">a finding: one line of a report, `rule_id | file:line | problem | correction`; `OK` the answer of a file that departs from nothing</t>
+          <t xml:space="preserve">a report: the one current file per controlled file — the file's key, the vendor and the time, then the answer as it came; reset by every crawl, never tracked</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t xml:space="preserve">`crawlers_mission.md`</t>
+          <t xml:space="preserve">`REPORTS_DIR`, `report_path()` in the crawler's `config.py` — `store/status/reports_after_crawled_files/&lt;path&gt;.report.md`; `write_text()` in `module_skills/sync.py`</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`report`</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">report</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t xml:space="preserve">a finding without a `rule_id`; a rule that was not sent; a table; `conformant` as a line</t>
+          <t xml:space="preserve">a history of entries; an append; a report in the sub-module's folder; a commit in its first line; a report tracked</t>
         </is>
       </c>
     </row>
@@ -17081,27 +17081,17 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t xml:space="preserve">a controlled file's state: where its crawl stands — `pending` before, `running` while the vendor works, `done` once its report is written, `failed` otherwise, `interrupted` where Ctrl-C ended it</t>
+          <t xml:space="preserve">a finding: one line of a report, `rule_id | file:line | problem | correction`; `OK` the answer of a file that departs from nothing</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t xml:space="preserve">`row()` in `status.py`; `main()` in `crawl.py`</t>
-        </is>
-      </c>
-      <c r="D446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`state`</t>
-        </is>
-      </c>
-      <c r="E446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pending; running; done; failed; interrupted</t>
+          <t xml:space="preserve">`crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t xml:space="preserve">`done` read as conformant — it says the report was written; a change of state left out of the snapshot</t>
+          <t xml:space="preserve">a finding without a `rule_id`; a rule that was not sent; a table; `conformant` as a line</t>
         </is>
       </c>
     </row>
@@ -17113,22 +17103,27 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t xml:space="preserve">the crawl's progress: one line per controlled file after its result, then one closing line; the reason a file failed one line on stderr</t>
+          <t xml:space="preserve">a controlled file's state: where its crawl stands — `pending` before, `running` while the vendor works, `done` once its report is written, `failed` otherwise, `interrupted` where Ctrl-C ended it</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t xml:space="preserve">`main()` in `crawl.py`</t>
+          <t xml:space="preserve">`row()` in `status.py`; `main()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`state`</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;current&gt;/&lt;total&gt; | &lt;controlled file&gt; | &lt;vendor&gt; | &lt;state&gt;`; `&lt;processed&gt;/&lt;total&gt; | crawl | &lt;vendor&gt; | done`, `failed` or `interrupted`</t>
+          <t xml:space="preserve">pending; running; done; failed; interrupted</t>
         </is>
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t xml:space="preserve">a spinner, a progress bar, a percentage; an answer summarised on the screen — the report holds it; a results table</t>
+          <t xml:space="preserve">`done` read as conformant — it says the report was written; a change of state left out of the snapshot</t>
         </is>
       </c>
     </row>
@@ -17140,17 +17135,22 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t xml:space="preserve">the refusals and the exits: a state the crawler cannot read ends it in one named line before anything is reset; a file the vendor fails is `failed` and the crawl goes on — 0 every file done, 1 a refusal or a failed file, 130 Ctrl-C</t>
+          <t xml:space="preserve">the crawl's progress: one line per controlled file after its result, then one closing line; the reason a file failed one line on stderr</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SystemExit` in `module_skills/sheet.py`, `module_skills/sync.py` and the crawler's `crawl.py`</t>
+          <t xml:space="preserve">`main()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`&lt;current&gt;/&lt;total&gt; | &lt;controlled file&gt; | &lt;vendor&gt; | &lt;state&gt;`; `&lt;processed&gt;/&lt;total&gt; | crawl | &lt;vendor&gt; | done`, `failed` or `interrupted`</t>
         </is>
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t xml:space="preserve">a traceback for an expected failure; exit 0 after a failure; a crawl that stops at the first failed file</t>
+          <t xml:space="preserve">a spinner, a progress bar, a percentage; an answer summarised on the screen — the report holds it; a results table</t>
         </is>
       </c>
     </row>
@@ -17162,27 +17162,17 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t xml:space="preserve">the snapshot: `skills_status.json`, the current state of every controlled file, sorted by path and rewritten whole at every change; tracked in its neutral state, every controlled file `pending` with no report</t>
+          <t xml:space="preserve">the refusals and the exits: a state the crawler cannot read ends it in one named line before anything is reset; a file the vendor fails is `failed` and the crawl goes on — 0 every file done, 1 a refusal or a failed file, 130 Ctrl-C</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILLS_STATUS_JSON_PATH` in the crawler's `config.py`; `row()`, `write_skills_status()`, `write_atomically()` in `status.py`</t>
-        </is>
-      </c>
-      <c r="D449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`files`, each `path`, `state`, `vendor`, `finished_at_utc`, `report`</t>
-        </is>
-      </c>
-      <c r="E449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">file; state; vendor; finished_at_utc; report</t>
+          <t xml:space="preserve">`SystemExit` in `module_skills/sheet.py`, `module_skills/sync.py` and the crawler's `crawl.py`</t>
         </is>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t xml:space="preserve">a count of crawls; an age; a clock but `finished_at_utc`; a snapshot that reads itself back; a partial file</t>
+          <t xml:space="preserve">a traceback for an expected failure; exit 0 after a failure; a crawl that stops at the first failed file</t>
         </is>
       </c>
     </row>
@@ -17194,104 +17184,136 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
+          <t xml:space="preserve">the snapshot: `skills_status.json`, the current state of every controlled file, sorted by path and rewritten whole at every change; tracked in its neutral state, every controlled file `pending` with no report</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`SKILLS_STATUS_JSON_PATH` in the crawler's `config.py`; `row()`, `write_skills_status()` in `status.py`, through `write_text()` of `module_skills/sync.py`</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`files`, each `path`, `state`, `vendor`, `finished_at_utc`, `report`</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">file; state; vendor; finished_at_utc; report</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a count of crawls; an age; a clock but `finished_at_utc`; a snapshot that reads itself back; a partial file</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scalability crawler</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
           <t xml:space="preserve">the page's view of the reports</t>
         </is>
       </c>
-      <c r="C450" t="inlineStr">
+      <c r="C451" t="inlineStr">
         <is>
           <t xml:space="preserve">`scalability.js` — `SKILLS_STATUS`, `renderCrawlState()`</t>
         </is>
       </c>
-      <c r="E450" t="inlineStr">
+      <c r="E451" t="inlineStr">
         <is>
           <t xml:space="preserve">Scalability — CRAWL STATE</t>
         </is>
       </c>
-      <c r="F450" t="inlineStr">
+      <c r="F451" t="inlineStr">
         <is>
           <t xml:space="preserve">a tab named for a tool; scale for a larger basket, which is `ASSET=&lt;TICKER&gt;`</t>
-        </is>
-      </c>
-    </row>
-    <row r="452">
-      <c r="A452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rule_type_id</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t xml:space="preserve">Architecture</t>
+          <t xml:space="preserve">rule_type_id</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t xml:space="preserve">Naming</t>
+          <t xml:space="preserve">Architecture</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conformities</t>
+          <t xml:space="preserve">Naming</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t xml:space="preserve">Workflow</t>
+          <t xml:space="preserve">Conformities</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t xml:space="preserve">FileLayout</t>
+          <t xml:space="preserve">Workflow</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t xml:space="preserve">UI_TUI</t>
+          <t xml:space="preserve">FileLayout</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scalability</t>
+          <t xml:space="preserve">UI_TUI</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t xml:space="preserve">Complexity</t>
+          <t xml:space="preserve">Scalability</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t xml:space="preserve">Determinism</t>
+          <t xml:space="preserve">Complexity</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t xml:space="preserve">Performance</t>
+          <t xml:space="preserve">Determinism</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
         <is>
           <t xml:space="preserve">Methodology</t>
         </is>

</xml_diff>

<commit_message>
Publish what a reader reads: the page's proposal, a contract and a Y without dead keys
The feature snapshot's proposal carries what the page shows — each fold's growth
and trades, the path's growth, Calmar ratio and profit factor, the threshold —
and its search block drops trial_count_by_loop and champion_trial_index, which
no page reads; the features copy of SELECTION_SCORE_KEY goes with them. The
contract drops the slot no reader of it reads; the snapshot keeps it for the
page. Y drops event_resolution and exit_reference_price: the backtest rescales
the label's barriers and walks its own event, and the ML methodology now says
so. tier and historical_aliases stay published, because the catalogue rule has
features-status fail on a record without its tier.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -935,7 +935,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">One `&lt;TICKER&gt;_catalogue.json` in the asset's folder `ticker=&lt;TICKER&gt;/`, written by `catalogue.write_catalogue()` alone from `catalogue_contract()`: the decision timeframe, the hierarchy with each timeframe's slot and duration, the warm-up, the columns and the default columns per timeframe, and each timeframe's partition as a path under the artifacts store.</t>
+          <t xml:space="preserve">One `&lt;TICKER&gt;_catalogue.json` in the asset's folder `ticker=&lt;TICKER&gt;/`, written by `catalogue.write_catalogue()` alone from `catalogue_contract()`: the decision timeframe, the hierarchy with each timeframe's duration, the warm-up, the columns and the default columns per timeframe, and each timeframe's partition as a path under the artifacts store.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1781,12 +1781,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_features/status.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">At a round's end the ledger's lines by loop, the start's excluded, plus every round's draws less the lines that round's studies left; at a turn's start the draws still to count rebuilt as the recorded count less the lines of the rounds it covers; `status.serpentine_search_block()` copying `trial_count_by_loop`, never recounting it.</t>
+          <t xml:space="preserve">At a round's end the ledger's lines by loop, the start's excluded, plus every round's draws less the lines that round's studies left; at a turn's start the draws still to count rebuilt as the recorded count less the lines of the rounds it covers.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">`label_valid = false` and the ambiguous `event_resolution` on such a row; the `0` its `y` column carries never read as the neutral class, every population and every published class count reading `y` through `sample_valid`.</t>
+          <t xml:space="preserve">`label_valid = false` on such a row, set from the ambiguous `event_resolution` of its walk; the `0` its `y` column carries never read as the neutral class, every population and every published class count reading `y` through `sample_valid`.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -9563,11 +9563,6 @@
           <t xml:space="preserve">`exit_reference_price`</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`exit_reference_price`</t>
-        </is>
-      </c>
       <c r="F158" t="inlineStr">
         <is>
           <t xml:space="preserve">exit_ref</t>
@@ -9592,7 +9587,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t xml:space="preserve">`event_resolution`, `exit_counts.*`</t>
+          <t xml:space="preserve">`exit_counts.*`</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -9664,11 +9659,6 @@
           <t xml:space="preserve">`EVENT_RESOLUTION_{UPPER_BARRIER, LOWER_BARRIER, VERTICAL, AMBIGUOUS}`, named by `EVENT_RESOLUTION_NAMES`</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`event_resolution`</t>
-        </is>
-      </c>
       <c r="F161" t="inlineStr">
         <is>
           <t xml:space="preserve">bare 1 / −1 / 0 / 9</t>
@@ -11392,7 +11382,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t xml:space="preserve">`proposals` in `&lt;TICKER&gt;_serpentine_search.json`, each `proposal`, `trial_index`; `proposals` in the `serpentine_search` block of features_status.json, each `proposal`, `trial_index`, `added_columns_by_timeframe`, `removed_columns_by_timeframe` (against the asset's own set the serpentine search recorded in `inputs`), `mean_relative_logloss_skill`, `validation`, `validation_path`, `entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `selection_score_cagr_validation_path`</t>
+          <t xml:space="preserve">`proposals` in `&lt;TICKER&gt;_serpentine_search.json`, each `proposal`, `trial_index`; `proposals` in the `serpentine_search` block of features_status.json, each `proposal`, `trial_index`, `added_columns_by_timeframe`, `removed_columns_by_timeframe` (against the asset's own set the serpentine search recorded in `inputs`), `mean_relative_logloss_skill`, `validation` (per fold `cagr`, `trade_count`), `validation_path` (`cagr`, `calmar`, `profit_factor`), `entry_edge_threshold`</t>
         </is>
       </c>
       <c r="E219" t="inlineStr">
@@ -12401,7 +12391,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t xml:space="preserve">`features_status.json`: `generated_at_utc`, `catalogue`, `configurables` (the module's records and the serpentine search's, *a CONFIGURABLES record*), `assets` (per asset `ticker`, `row_count_by_timeframe`, `serpentine_search` — `null` while no serpentine search has run; else `trial_count`, `trial_count_by_loop`, `round_count`, `search_converged`, `champion_trial_index`, `inputs_current`, `proposals`)</t>
+          <t xml:space="preserve">`features_status.json`: `generated_at_utc`, `catalogue`, `configurables` (the module's records and the serpentine search's, *a CONFIGURABLES record*), `assets` (per asset `ticker`, `row_count_by_timeframe`, `serpentine_search` — `null` while no serpentine search has run; else `trial_count`, `round_count`, `search_converged`, `inputs_current`, `proposals`)</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
@@ -13458,17 +13448,17 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SELECTION_SCORE_KEY` — identical</t>
+          <t xml:space="preserve">`to_json_safe()` — identical</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/strategy.py`, `module_features/config.py`</t>
+          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t xml:space="preserve">the key a scored state carries its selection score under, chosen by the module that scores it and read by the feature layer's snapshot for every proposal it publishes; neither module imports the other</t>
+          <t xml:space="preserve">numpy canonicalisation is local to the modules that hold numpy values, and the JSON both publish is one form; no module imports another</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13470,17 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t xml:space="preserve">`to_json_safe()` — identical</t>
+          <t xml:space="preserve">`write_json()` — the canonical JSON form, keys sorted and indented</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`</t>
+          <t xml:space="preserve">identical in `module_features/dataset.py` and `module_ml/dataset.py`; equal by value in `module_features/sub_module_terminal/config.py`, which writes plain values without `to_json_safe()`</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t xml:space="preserve">numpy canonicalisation is local to the modules that hold numpy values, and the JSON both publish is one form; no module imports another</t>
+          <t xml:space="preserve">the published JSON is deterministic — the contract, the snapshots, the artifacts and the profile a hand drafts through the features terminal take one form; the terminal holds no numpy value and cannot import a `dataset.py`, which imports duckdb and numpy</t>
         </is>
       </c>
     </row>
@@ -13502,17 +13492,17 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t xml:space="preserve">`write_json()` — the canonical JSON form, keys sorted and indented</t>
+          <t xml:space="preserve">`write_parquet()` — identical</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_features/dataset.py` and `module_ml/dataset.py`; equal by value in `module_features/sub_module_terminal/config.py`, which writes plain values without `to_json_safe()`</t>
+          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t xml:space="preserve">the published JSON is deterministic — the contract, the snapshots, the artifacts and the profile a hand drafts through the features terminal take one form; the terminal holds no numpy value and cannot import a `dataset.py`, which imports duckdb and numpy</t>
+          <t xml:space="preserve">the repr round-trip that makes a Parquet file byte-reproducible; given a homogeneous family it writes that family's `schema.json` from the partition it wrote — `labels` and `oos_predictions`; no module imports another</t>
         </is>
       </c>
     </row>
@@ -13524,17 +13514,17 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t xml:space="preserve">`write_parquet()` — identical</t>
+          <t xml:space="preserve">`load_json()` — identical</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`</t>
+          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t xml:space="preserve">the repr round-trip that makes a Parquet file byte-reproducible; given a homogeneous family it writes that family's `schema.json` from the partition it wrote — `labels` and `oos_predictions`; no module imports another</t>
+          <t xml:space="preserve">the readers of the same JSON files — a stage, and the terminals that read what a stage wrote; a terminal cannot import a `dataset.py`, which imports duckdb and numpy, nor another module's code</t>
         </is>
       </c>
     </row>
@@ -13546,17 +13536,17 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_json()` — identical</t>
+          <t xml:space="preserve">`load_jsonl()` — identical</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`, `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t xml:space="preserve">the readers of the same JSON files — a stage, and the terminals that read what a stage wrote; a terminal cannot import a `dataset.py`, which imports duckdb and numpy, nor another module's code</t>
+          <t xml:space="preserve">a ledger is read back as it was written: HPO's to place a study among the ones before it, the serpentine search's to resume and to answer its own questions, the features terminal's to show the trials the state names</t>
         </is>
       </c>
     </row>
@@ -13568,17 +13558,22 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_jsonl()` — identical</t>
+          <t xml:space="preserve">`recursive_mean()`, `true_range()`, `asof_index()` — identical</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`, `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_features/indicators.py`, `module_ml/labels.py`</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`wilder_smoothing()`, `atr()` — the names these carried before the catalogue named every operation by its word</t>
         </is>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t xml:space="preserve">a ledger is read back as it was written: HPO's to place a study among the ones before it, the serpentine search's to resume and to answer its own questions, the features terminal's to show the trials the state names</t>
+          <t xml:space="preserve">the label defines its own barrier scale and aligns to the last closed bar the way the catalogue does, and the ML module imports no feature code</t>
         </is>
       </c>
     </row>
@@ -13590,22 +13585,17 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t xml:space="preserve">`recursive_mean()`, `true_range()`, `asof_index()` — identical</t>
+          <t xml:space="preserve">`SEED` — equal by value</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/indicators.py`, `module_ml/labels.py`</t>
-        </is>
-      </c>
-      <c r="F303" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`wilder_smoothing()`, `atr()` — the names these carried before the catalogue named every operation by its word</t>
+          <t xml:space="preserve">a CONFIGURABLES record and the constant read from it in `module_ml/config.py`; a constant in `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t xml:space="preserve">the label defines its own barrier scale and aligns to the last closed bar the way the catalogue does, and the ML module imports no feature code</t>
+          <t xml:space="preserve">the seed is one of the values the serpentine search records as the identity of its experiment, and the parameters artifact it reads does not carry it; the sub-module cannot import the ML module</t>
         </is>
       </c>
     </row>
@@ -13617,17 +13607,17 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SEED` — equal by value</t>
+          <t xml:space="preserve">`VALIDATION_FOLD_IDS` — identical</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t xml:space="preserve">a CONFIGURABLES record and the constant read from it in `module_ml/config.py`; a constant in `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t xml:space="preserve">the seed is one of the values the serpentine search records as the identity of its experiment, and the parameters artifact it reads does not carry it; the sub-module cannot import the ML module</t>
+          <t xml:space="preserve">the turn's fold gate reads every fold in the order the selection fixes and the evaluator scores the same ones; which folds select is the method, never the order of the keys a payload happens to carry</t>
         </is>
       </c>
     </row>
@@ -13639,7 +13629,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t xml:space="preserve">`VALIDATION_FOLD_IDS` — identical</t>
+          <t xml:space="preserve">`BARRIER_COORDINATE_CASTS`, `BARRIER_COORDINATE_NAMES` — identical</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -13649,7 +13639,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t xml:space="preserve">the turn's fold gate reads every fold in the order the selection fixes and the evaluator scores the same ones; which folds select is the method, never the order of the keys a payload happens to carry</t>
+          <t xml:space="preserve">the casts are what make an integer and the same number as a float one state, and the order is the order a state is keyed in; a copy differing by one cast turns every cache hit into a miss and the serpentine search pays again for states it already holds</t>
         </is>
       </c>
     </row>
@@ -13661,17 +13651,17 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t xml:space="preserve">`BARRIER_COORDINATE_CASTS`, `BARRIER_COORDINATE_NAMES` — identical</t>
+          <t xml:space="preserve">`START_BY_COORDINATE_DEFAULT` — equal by value</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">a CONFIGURABLES record and the constant read from it in `module_ml/config.py`; constants in `module_features/sub_module_serpentine_search/config.py` and `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t xml:space="preserve">the casts are what make an integer and the same number as a float one state, and the order is the order a state is keyed in; a copy differing by one cast turns every cache hit into a miss and the serpentine search pays again for states it already holds</t>
+          <t xml:space="preserve">the geometry the chain stands at without a promotion, the point the serpentine search pins a coordinate at when the profile does not search it, and the point the features terminal's draft pins it at too; neither side may import the ML module, and the terminal not even its own module's `config.py`</t>
         </is>
       </c>
     </row>
@@ -13683,17 +13673,17 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t xml:space="preserve">`START_BY_COORDINATE_DEFAULT` — equal by value</t>
+          <t xml:space="preserve">`TRADE_EXIT_COORDINATE_NAMES` — identical</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t xml:space="preserve">a CONFIGURABLES record and the constant read from it in `module_ml/config.py`; constants in `module_features/sub_module_serpentine_search/config.py` and `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t xml:space="preserve">the geometry the chain stands at without a promotion, the point the serpentine search pins a coordinate at when the profile does not search it, and the point the features terminal's draft pins it at too; neither side may import the ML module, and the terminal not even its own module's `config.py`</t>
+          <t xml:space="preserve">the serpentine search moves the two as one family and the evaluator leaves them out of a fit identity; a copy that drifts merges states whose fits differ, with wrong numbers and no error</t>
         </is>
       </c>
     </row>
@@ -13705,17 +13695,17 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TRADE_EXIT_COORDINATE_NAMES` — identical</t>
+          <t xml:space="preserve">`SELECTION_FOLD_MEASURE` — identical</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, `module_ml/config.py`</t>
         </is>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t xml:space="preserve">the serpentine search moves the two as one family and the evaluator leaves them out of a fit identity; a copy that drifts merges states whose fits differ, with wrong numbers and no error</t>
+          <t xml:space="preserve">the turn's gate on a move and the gate inside a study ask one question of one set of numbers, so they read one measure</t>
         </is>
       </c>
     </row>
@@ -13727,17 +13717,17 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SELECTION_FOLD_MEASURE` — identical</t>
+          <t xml:space="preserve">`timeframes()` — identical</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, `module_ml/config.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t xml:space="preserve">the turn's gate on a move and the gate inside a study ask one question of one set of numbers, so they read one measure</t>
+          <t xml:space="preserve">both sides read the hierarchy off the asset's contract rather than off their own timeframe register, so a contract an older catalogue wrote reads the same on both</t>
         </is>
       </c>
     </row>
@@ -13749,17 +13739,17 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timeframes()` — identical</t>
+          <t xml:space="preserve">`score_request_json()`, `score_response_json()` — equal by value</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, over its own `artifact_dir()`; `module_features/sub_module_serpentine_search/config.py`, over its module's</t>
         </is>
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t xml:space="preserve">both sides read the hierarchy off the asset's contract rather than off their own timeframe register, so a contract an older catalogue wrote reads the same on both</t>
+          <t xml:space="preserve">one side writes what the other reads: a boundary made of files needs both sides to name the same two, and neither module imports the other</t>
         </is>
       </c>
     </row>
@@ -13771,7 +13761,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_request_json()`, `score_response_json()` — equal by value</t>
+          <t xml:space="preserve">`parameters_json()` — equal by value</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -13781,7 +13771,7 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t xml:space="preserve">one side writes what the other reads: a boundary made of files needs both sides to name the same two, and neither module imports the other</t>
+          <t xml:space="preserve">the ML chain writes the tuned parameters the serpentine search starts from; the writer and the reader of a boundary name one artifact</t>
         </is>
       </c>
     </row>
@@ -13793,17 +13783,17 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t xml:space="preserve">`parameters_json()` — equal by value</t>
+          <t xml:space="preserve">`load_feature_columns()` — equal by value</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, over its own `artifact_dir()`; `module_features/sub_module_serpentine_search/config.py`, over its module's</t>
+          <t xml:space="preserve">`module_ml/dataset.py`; `module_features/sub_module_serpentine_search/serpentine_search.py`</t>
         </is>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t xml:space="preserve">the ML chain writes the tuned parameters the serpentine search starts from; the writer and the reader of a boundary name one artifact</t>
+          <t xml:space="preserve">the asset's feature set — the promoted file's columns in catalogue order, else the default set — is read by the chain that fits it and by the search that starts from it, and neither module imports the other</t>
         </is>
       </c>
     </row>
@@ -13815,17 +13805,17 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_feature_columns()` — equal by value</t>
+          <t xml:space="preserve">`feature_set_json()`, `barriers_json()`, `hyperparameter_point_json()` — equal by value</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/dataset.py`; `module_features/sub_module_serpentine_search/serpentine_search.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`, `module_features/sub_module_terminal/config.py`, each over its own `artifact_dir()` or its module's</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset's feature set — the promoted file's columns in catalogue order, else the default set — is read by the chain that fits it and by the search that starts from it, and neither module imports the other</t>
+          <t xml:space="preserve">the promotion writes the three, the ML chain reads them and the serpentine search the first two, and the features terminal names them on its promotion screen; the writer and the reader of a boundary must name one artifact, and the terminal cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13837,17 +13827,17 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_set_json()`, `barriers_json()`, `hyperparameter_point_json()` — equal by value</t>
+          <t xml:space="preserve">`theta()`, `state_key()` — identical</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`, `module_features/sub_module_terminal/config.py`, each over its own `artifact_dir()` or its module's</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_ml/score.py`</t>
         </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion writes the three, the ML chain reads them and the serpentine search the first two, and the features terminal names them on its promotion screen; the writer and the reader of a boundary must name one artifact, and the terminal cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the serpentine search keys a state to know whether it has scored it, and the module that scores names the parent of a study by the same key: one differing separator and every answer would look like the answer to another question</t>
         </is>
       </c>
     </row>
@@ -13859,7 +13849,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t xml:space="preserve">`theta()`, `state_key()` — identical</t>
+          <t xml:space="preserve">`KIND_SCORE`, `KIND_HYPERPARAMETER` — identical</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -13869,7 +13859,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t xml:space="preserve">the serpentine search keys a state to know whether it has scored it, and the module that scores names the parent of a study by the same key: one differing separator and every answer would look like the answer to another question</t>
+          <t xml:space="preserve">the two kinds of question: one side writes the word into a request and the other branches on it, so one word apart and every question would be answered as the other kind or refused</t>
         </is>
       </c>
     </row>
@@ -13881,17 +13871,17 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t xml:space="preserve">`KIND_SCORE`, `KIND_HYPERPARAMETER` — identical</t>
+          <t xml:space="preserve">`serpentine_search_json()`, `serpentine_search_trials_jsonl()`, `serpentine_search_profile_json()` — equal by value</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_ml/score.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, over its module's `artifact_dir()`; `module_features/sub_module_terminal/config.py`, over its own</t>
         </is>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t xml:space="preserve">the two kinds of question: one side writes the word into a request and the other branches on it, so one word apart and every question would be answered as the other kind or refused</t>
+          <t xml:space="preserve">the features terminal reads the state and the ledger and writes the profile on the host's `python3`, and the sub-module's `config.py` imports the module's, which imports numpy</t>
         </is>
       </c>
     </row>
@@ -13903,17 +13893,17 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t xml:space="preserve">`serpentine_search_json()`, `serpentine_search_trials_jsonl()`, `serpentine_search_profile_json()` — equal by value</t>
+          <t xml:space="preserve">`SERPENTINE_SEARCH_ROUND_LOOPS` — equal by value to the loops of `ROUND_SCHEDULE`</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, over its module's `artifact_dir()`; `module_features/sub_module_terminal/config.py`, over its own</t>
+          <t xml:space="preserve">`module_features/sub_module_terminal/config.py`, written out; `ROUND_SCHEDULE` in `module_features/sub_module_serpentine_search/config.py`, its loops in their order</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal reads the state and the ledger and writes the profile on the host's `python3`, and the sub-module's `config.py` imports the module's, which imports numpy</t>
+          <t xml:space="preserve">the loops a round runs, in its order: the features terminal offers them to a draft, and it cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13925,17 +13915,17 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SERPENTINE_SEARCH_ROUND_LOOPS` — equal by value to the loops of `ROUND_SCHEDULE`</t>
+          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`, `PROMOTE_TARGET` — equal by value</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_terminal/config.py`, written out; `ROUND_SCHEDULE` in `module_features/sub_module_serpentine_search/config.py`, its loops in their order</t>
+          <t xml:space="preserve">CONFIGURABLES records of `module_features/sub_module_serpentine_search/config.py`; constants of `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t xml:space="preserve">the loops a round runs, in its order: the features terminal offers them to a draft, and it cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the features terminal offers the grid to a draft and opens its own screen for the promotion's target on the host's `python3`, and cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13947,17 +13937,17 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`, `PROMOTE_TARGET` — equal by value</t>
+          <t xml:space="preserve">`tui.py`, the whole file — the gum layer of every terminal</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONFIGURABLES records of `module_features/sub_module_serpentine_search/config.py`; constants of `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">identical to the byte in `module_data/sub_module_terminal/tui.py`, `module_features/sub_module_terminal/tui.py`, `module_ml/sub_module_terminal/tui.py`, `module_monitoring/sub_module_terminal/tui.py`, `module_skills/sub_module_terminal/tui.py`</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal offers the grid to a draft and opens its own screen for the promotion's target on the host's `python3`, and cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">one module speaks gum in each, and a package for what the terminals share would make every module import `module_skills` (`AGENTS.md` D02). It holds no sentence about a screen's content — a placeholder, a header and a state's words are the caller's; its own words are the block labels and the line naming the columns a narrow terminal leaves out — so each owner holds the file as its own local adapter</t>
         </is>
       </c>
     </row>
@@ -13969,17 +13959,17 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t xml:space="preserve">`tui.py`, the whole file — the gum layer of every terminal</t>
+          <t xml:space="preserve">`OUTPUT_PLAIN` and the three conditions it reads — `NO_COLOR`, `TERM`, `sys.stdout.isatty()`</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical to the byte in `module_data/sub_module_terminal/tui.py`, `module_features/sub_module_terminal/tui.py`, `module_ml/sub_module_terminal/tui.py`, `module_monitoring/sub_module_terminal/tui.py`, `module_skills/sub_module_terminal/tui.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/config.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`, `module_skills/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t xml:space="preserve">one module speaks gum in each, and a package for what the terminals share would make every module import `module_skills` (`AGENTS.md` D02). It holds no sentence about a screen's content — a placeholder, a header and a state's words are the caller's; its own words are the block labels and the line naming the columns a narrow terminal leaves out — so each owner holds the file as its own local adapter</t>
+          <t xml:space="preserve">plain output follows the environment and is never a flag; each `tui.py` reads its own sub-module's `config.py`, and no module imports another</t>
         </is>
       </c>
     </row>
@@ -13991,17 +13981,17 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OUTPUT_PLAIN` and the three conditions it reads — `NO_COLOR`, `TERM`, `sys.stdout.isatty()`</t>
+          <t xml:space="preserve">the screen helpers `_option_rows()`, `_cancelled_exit_code()`, `_failure_exit_code()`</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/config.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`, `module_skills/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`, `module_monitoring/sub_module_terminal/terminal.py`, `module_skills/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t xml:space="preserve">plain output follows the environment and is never a flag; each `tui.py` reads its own sub-module's `config.py`, and no module imports another</t>
+          <t xml:space="preserve">every terminal uses the same outcome and option conventions, and no terminal imports another module's code; a terminal that asks more than two forms keeps its own step helpers, in its own words</t>
         </is>
       </c>
     </row>
@@ -14013,7 +14003,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t xml:space="preserve">the screen helpers `_option_rows()`, `_cancelled_exit_code()`, `_failure_exit_code()`</t>
+          <t xml:space="preserve">`_make()`</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -14023,7 +14013,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t xml:space="preserve">every terminal uses the same outcome and option conventions, and no terminal imports another module's code; a terminal that asks more than two forms keeps its own step helpers, in its own words</t>
+          <t xml:space="preserve">the one call of make — a terminal starts a target through it and no other way, its lines uncaptured; it takes its arguments open, `_make(*arguments)`, so a target alone and a target with its asset — the promotion's among them — pass through one signature</t>
         </is>
       </c>
     </row>
@@ -14035,7 +14025,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_make()`</t>
+          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()`</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -14045,7 +14035,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one call of make — a terminal starts a target through it and no other way, its lines uncaptured; it takes its arguments open, `_make(*arguments)`, so a target alone and a target with its asset — the promotion's among them — pass through one signature</t>
+          <t xml:space="preserve">the one reading of make — the menu is the Makefile's own targets, read from `make help` and filtered by the terminal's `MENU_TARGET_PATTERN`, so a terminal keeps no second list of them and a target gains its option by carrying a `##`</t>
         </is>
       </c>
     </row>
@@ -14057,7 +14047,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()`</t>
+          <t xml:space="preserve">`_write_target()`</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -14067,7 +14057,7 @@
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one reading of make — the menu is the Makefile's own targets, read from `make help` and filtered by the terminal's `MENU_TARGET_PATTERN`, so a terminal keeps no second list of them and a target gains its option by carrying a `##`</t>
+          <t xml:space="preserve">one plan, one gate and one call for every target a menu offers; each owner holds its own local adapter with the same signature</t>
         </is>
       </c>
     </row>
@@ -14079,17 +14069,17 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_target()`</t>
+          <t xml:space="preserve">`_tickers()`</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`, `module_monitoring/sub_module_terminal/terminal.py`, `module_skills/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t xml:space="preserve">one plan, one gate and one call for every target a menu offers; each owner holds its own local adapter with the same signature</t>
+          <t xml:space="preserve">the three terminals whose module takes an asset read the assets `--tickers` names and ask for them only when a direct run named none; no module defines a basket of its own, and no terminal imports another module's code</t>
         </is>
       </c>
     </row>
@@ -14101,7 +14091,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_tickers()`</t>
+          <t xml:space="preserve">`_present()`</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -14111,29 +14101,34 @@
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three terminals whose module takes an asset read the assets `--tickers` names and ask for them only when a direct run named none; no module defines a basket of its own, and no terminal imports another module's code</t>
+          <t xml:space="preserve">the three terminals whose module keeps an asset's files answer whether one stands in the same word, and a terminal reads another module's files through none of that module's code</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t xml:space="preserve">Twice by extraction</t>
+          <t xml:space="preserve">Terminals</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_present()`</t>
+          <t xml:space="preserve">a module's terminal: the sub-module that shows what the module's stores hold — per asset where the module takes one — and starts one of the module's own targets through `make`; outside an action it creates no domain state, and it gates nothing</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
-        </is>
-      </c>
-      <c r="H327" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the three terminals whose module keeps an asset's files answer whether one stands in the same word, and a terminal reads another module's files through none of that module's code</t>
+          <t xml:space="preserve">`sub_module_terminal` — `module_data/sub_module_terminal/`, `module_features/sub_module_terminal/`, `module_ml/sub_module_terminal/`, `module_monitoring/sub_module_terminal/` and the canon's `module_skills/sub_module_terminal/`, each `terminal.py` with `main()`, `config.py` and `tui.py`</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data terminal; Features terminal; ML terminal; Monitoring terminal; Skills terminal</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a cockpit, a console, a dashboard; a second terminal in one module; a TUI that computes, schedules or gates; `&lt;module&gt;-tui`, `&lt;module&gt;-menu`; the crawler drawing a terminal of its own</t>
         </is>
       </c>
     </row>
@@ -14145,22 +14140,17 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t xml:space="preserve">a module's terminal: the sub-module that shows what the module's stores hold — per asset where the module takes one — and starts one of the module's own targets through `make`; outside an action it creates no domain state, and it gates nothing</t>
+          <t xml:space="preserve">a terminal's entry: the one make target that opens it, run by `python3` on the host and never in a container; it carries no `##`, so it is no option of any menu</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_terminal` — `module_data/sub_module_terminal/`, `module_features/sub_module_terminal/`, `module_ml/sub_module_terminal/`, `module_monitoring/sub_module_terminal/` and the canon's `module_skills/sub_module_terminal/`, each `terminal.py` with `main()`, `config.py` and `tui.py`</t>
-        </is>
-      </c>
-      <c r="E328" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Data terminal; Features terminal; ML terminal; Monitoring terminal; Skills terminal</t>
+          <t xml:space="preserve">`make data-terminal`, `make features-terminal`, `make ml-terminal`, `make monitoring-terminal`, `make skills-terminal`; the three whose module takes an asset given `--tickers` from `ASSET` or `TICKERS_CSV`</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t xml:space="preserve">a cockpit, a console, a dashboard; a second terminal in one module; a TUI that computes, schedules or gates; `&lt;module&gt;-tui`, `&lt;module&gt;-menu`; the crawler drawing a terminal of its own</t>
+          <t xml:space="preserve">a `##` on an entry; a `tmux-` twin of a terminal; `make tui`; a terminal started in a runner</t>
         </is>
       </c>
     </row>
@@ -14172,17 +14162,17 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t xml:space="preserve">a terminal's entry: the one make target that opens it, run by `python3` on the host and never in a container; it carries no `##`, so it is no option of any menu</t>
+          <t xml:space="preserve">a terminal's sources: what a terminal reads</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make data-terminal`, `make features-terminal`, `make ml-terminal`, `make monitoring-terminal`, `make skills-terminal`; the three whose module takes an asset given `--tickers` from `ASSET` or `TICKERS_CSV`</t>
+          <t xml:space="preserve">its own module's `config.py` where that is standard library — the data terminal's, with `lean.py`, and the ML terminal's; the features terminal its own `config.py`'s copies, `module_features/config.py` importing numpy; the monitoring terminal the snapshots through `STORE_STATUS_DIR` and `SNAPSHOT_FILE_NAMES` of its own `config.py`; the skills terminal the canon's `config.py` and, through the crawler's `config.py`, `vendors_for_crawling.toml` and the snapshot; every terminal `make help`</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `##` on an entry; a `tmux-` twin of a terminal; `make tui`; a terminal started in a runner</t>
+          <t xml:space="preserve">a snapshot read for freshness; duckdb; a store literal; another module's code; a third-party package</t>
         </is>
       </c>
     </row>
@@ -14194,17 +14184,22 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t xml:space="preserve">a terminal's sources: what a terminal reads</t>
+          <t xml:space="preserve">the menu: the options a terminal offers — one per target of the one Makefile that carries a `##` and whose name gives it to the terminal's module, then the terminal's own actions, `quit` last</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t xml:space="preserve">its own module's `config.py` where that is standard library — the data terminal's, with `lean.py`, and the ML terminal's; the features terminal its own `config.py`'s copies, `module_features/config.py` importing numpy; the monitoring terminal the snapshots through `STORE_STATUS_DIR` and `SNAPSHOT_FILE_NAMES` of its own `config.py`; the skills terminal the canon's `config.py` and, through the crawler's `config.py`, `vendors_for_crawling.toml` and the snapshot; every terminal `make help`</t>
+          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()` in each `terminal.py`; `MENU_TARGET_PATTERN` in each terminal's `config.py`; `_write_target()`</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t xml:space="preserve">action</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t xml:space="preserve">a snapshot read for freshness; duckdb; a store literal; another module's code; a third-party package</t>
+          <t xml:space="preserve">a second list of the targets in the program that opens the menu; a menu written out by hand; a target offered in a second terminal; the terminal's own entry among its options; `MODULE_TOKEN`, `STAGES`, `WRITES_BY_STAGE`, a target map; a grouping or a sorting of the targets; `run`, `exit`</t>
         </is>
       </c>
     </row>
@@ -14216,22 +14211,22 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t xml:space="preserve">the menu: the options a terminal offers — one per target of the one Makefile that carries a `##` and whose name gives it to the terminal's module, then the terminal's own actions, `quit` last</t>
+          <t xml:space="preserve">the asset choice: the assets a run is about — the ones `--tickers` named, typed only when a direct run named none — then the one asset an action is for, one answered without asking</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()` in each `terminal.py`; `MENU_TARGET_PATTERN` in each terminal's `config.py`; `_write_target()`</t>
+          <t xml:space="preserve">`_tickers()` and its `gum_input` headed `asset`; `gum_choose` headed `asset` over those assets</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t xml:space="preserve">action</t>
+          <t xml:space="preserve">asset</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second list of the targets in the program that opens the menu; a menu written out by hand; a target offered in a second terminal; the terminal's own entry among its options; `MODULE_TOKEN`, `STAGES`, `WRITES_BY_STAGE`, a target map; a grouping or a sorting of the targets; `run`, `exit`</t>
+          <t xml:space="preserve">a ticker typed where the launcher already named the set; a basket the terminal defines; a list of assets read from a store to fill it; a default basket in a module</t>
         </is>
       </c>
     </row>
@@ -14243,22 +14238,22 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset choice: the assets a run is about — the ones `--tickers` named, typed only when a direct run named none — then the one asset an action is for, one answered without asking</t>
+          <t xml:space="preserve">the plan and its gate: the choices, the `command` line verbatim and the target's purpose, then the question that runs or cancels</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_tickers()` and its `gum_input` headed `asset`; `gum_choose` headed `asset` over those assets</t>
+          <t xml:space="preserve">`_write_target()`; the `command` line; `_make()`</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset</t>
+          <t xml:space="preserve">`target`, `purpose` and each variable as `parameter` and `value`; `command make &lt;target&gt; ASSET=&lt;TICKER&gt;`; `&lt;target&gt;?` with the target and `cancel`</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t xml:space="preserve">a ticker typed where the launcher already named the set; a basket the terminal defines; a list of assets read from a store to fill it; a default basket in a module</t>
+          <t xml:space="preserve">a stage run before the gate; a gate that refuses what a hand confirms; `run`</t>
         </is>
       </c>
     </row>
@@ -14270,22 +14265,22 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t xml:space="preserve">the plan and its gate: the choices, the `command` line verbatim and the target's purpose, then the question that runs or cancels</t>
+          <t xml:space="preserve">the features terminal's own actions, the serpentine search's: draft the profile, read the recorded serpentine search, promote the proposal</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_target()`; the `command` line; `_make()`</t>
+          <t xml:space="preserve">`_write_search_profile()`, `_recorded_search_tables()`, `_write_promoted_proposal()` in `module_features/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t xml:space="preserve">`target`, `purpose` and each variable as `parameter` and `value`; `command make &lt;target&gt; ASSET=&lt;TICKER&gt;`; `&lt;target&gt;?` with the target and `cancel`</t>
+          <t xml:space="preserve">draft; recorded search; `features-serpentine-search-promote`</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage run before the gate; a gate that refuses what a hand confirms; `run`</t>
+          <t xml:space="preserve">`status` for the recorded search — the word is a stage's; a start of the serpentine search of its own — the search is the menu's `features-serpentine-search` or its `tmux-` twin; holdout, which the ML chain a promotion is followed by computes; a second menu after the action</t>
         </is>
       </c>
     </row>
@@ -14297,22 +14292,22 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal's own actions, the serpentine search's: draft the profile, read the recorded serpentine search, promote the proposal</t>
+          <t xml:space="preserve">the steps table: the steps of the features terminal's draft in order, above the step it asks — each answered DONE with its choice, the one asked CURRENT, the rest PENDING</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_search_profile()`, `_recorded_search_tables()`, `_write_promoted_proposal()` in `module_features/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">`_step_rows()`, `_step_answer()`, `DRAFT_STEPS` in `module_features/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t xml:space="preserve">draft; recorded search; `features-serpentine-search-promote`</t>
+          <t xml:space="preserve">step; state; choice; select now</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t xml:space="preserve">`status` for the recorded search — the word is a stage's; a start of the serpentine search of its own — the search is the menu's `features-serpentine-search` or its `tmux-` twin; holdout, which the ML chain a promotion is followed by computes; a second menu after the action</t>
+          <t xml:space="preserve">workflow, wizard, stepper; the steps of two actions; a step asked when its one option answers it</t>
         </is>
       </c>
     </row>
@@ -14324,22 +14319,22 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t xml:space="preserve">the steps table: the steps of the features terminal's draft in order, above the step it asks — each answered DONE with its choice, the one asked CURRENT, the rest PENDING</t>
+          <t xml:space="preserve">the one file a terminal writes</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_step_rows()`, `_step_answer()`, `DRAFT_STEPS` in `module_features/sub_module_terminal/terminal.py`</t>
-        </is>
-      </c>
-      <c r="E335" t="inlineStr">
-        <is>
-          <t xml:space="preserve">step; state; choice; select now</t>
+          <t xml:space="preserve">`write_json()`, `serpentine_search_profile_json()` in `module_features/sub_module_terminal/config.py` — the features terminal's draft</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t xml:space="preserve">workflow, wizard, stepper; the steps of two actions; a step asked when its one option answers it</t>
+          <t xml:space="preserve">a second file; a file in the sub-module's own folder</t>
         </is>
       </c>
     </row>
@@ -14351,22 +14346,22 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one file a terminal writes</t>
+          <t xml:space="preserve">the target the features terminal opens its own screen for — the promotion, whose plan shows the one state it promotes</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t xml:space="preserve">`write_json()`, `serpentine_search_profile_json()` in `module_features/sub_module_terminal/config.py` — the features terminal's draft</t>
-        </is>
-      </c>
-      <c r="D336" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
+          <t xml:space="preserve">`PROMOTE_TARGET` in `module_features/sub_module_terminal/config.py`</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the menu's `features-serpentine-search-promote`</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second file; a file in the sub-module's own folder</t>
+          <t xml:space="preserve">a second named target; the module's stages listed beside it; a name for a target that runs bare</t>
         </is>
       </c>
     </row>
@@ -14378,22 +14373,22 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t xml:space="preserve">the target the features terminal opens its own screen for — the promotion, whose plan shows the one state it promotes</t>
+          <t xml:space="preserve">the profile state: where the asset's profile stands against the serpentine search recorded under it — the one comparison the features terminal makes, on parsed objects and not on bytes</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t xml:space="preserve">`PROMOTE_TARGET` in `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`_profile_state()`</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t xml:space="preserve">the menu's `features-serpentine-search-promote`</t>
+          <t xml:space="preserve">`not drafted` / `no search` / `matches the search` / `differs from the search`</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second named target; the module's stages listed beside it; a name for a target that runs bare</t>
+          <t xml:space="preserve">`inputs_current`, which folds the parameters, the catalogue and the asset's own state and stays the page's</t>
         </is>
       </c>
     </row>
@@ -14405,22 +14400,27 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t xml:space="preserve">the profile state: where the asset's profile stands against the serpentine search recorded under it — the one comparison the features terminal makes, on parsed objects and not on bytes</t>
+          <t xml:space="preserve">the coordinate grid: what each coordinate is searched over, one preset, so a grid is a decision of the file and not of a form</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_profile_state()`</t>
+          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`grid_by_coordinate`</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t xml:space="preserve">`not drafted` / `no search` / `matches the search` / `differs from the search`</t>
+          <t xml:space="preserve">grid; points</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs_current`, which folds the parameters, the catalogue and the asset's own state and stays the page's</t>
+          <t xml:space="preserve">a grid typed into a prompt; a point the terminal offers outside the preset</t>
         </is>
       </c>
     </row>
@@ -14432,27 +14432,22 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t xml:space="preserve">the coordinate grid: what each coordinate is searched over, one preset, so a grid is a decision of the file and not of a form</t>
+          <t xml:space="preserve">gum: the terminal instrument the TUI speaks — `gum table --print`, `gum style`, `gum choose`, `gum input`; gum 2, a binary of the host</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`</t>
-        </is>
-      </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`grid_by_coordinate`</t>
-        </is>
-      </c>
-      <c r="E339" t="inlineStr">
-        <is>
-          <t xml:space="preserve">grid; points</t>
+          <t xml:space="preserve">`gum`, over `subprocess` in `tui.py` alone: `gum_table()`, `gum_style()`, `gum_choose()`, `gum_input()`, `_gum()`</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t xml:space="preserve">a grid typed into a prompt; a point the terminal offers outside the preset</t>
+          <t xml:space="preserve">a Python dependency, Rich among them; a chooser, a table or a colour written over curses or escape codes; a gum configuration in the tree; `gum spin`, `gum confirm`; `gum input` for a value the tree already holds, which is a selection and belongs to `gum choose`; gum's own pink and purple</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gum</t>
         </is>
       </c>
     </row>
@@ -14464,22 +14459,22 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t xml:space="preserve">gum: the terminal instrument the TUI speaks — `gum table --print`, `gum style`, `gum choose`, `gum input`; gum 2, a binary of the host</t>
+          <t xml:space="preserve">plain output: the screens without colour, symbol or border, chosen by the environment alone — `NO_COLOR` set and not empty, `TERM=dumb`, or standard output not a terminal</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t xml:space="preserve">`gum`, over `subprocess` in `tui.py` alone: `gum_table()`, `gum_style()`, `gum_choose()`, `gum_input()`, `_gum()`</t>
+          <t xml:space="preserve">`OUTPUT_PLAIN` in each terminal's `config.py`, read by its `tui.py`</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`[&lt;word&gt;]`</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Python dependency, Rich among them; a chooser, a table or a colour written over curses or escape codes; a gum configuration in the tree; `gum spin`, `gum confirm`; `gum input` for a value the tree already holds, which is a selection and belongs to `gum choose`; gum's own pink and purple</t>
-        </is>
-      </c>
-      <c r="I340" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gum</t>
+          <t xml:space="preserve">a flag, `--no-color`, `--simple`, `--a11y`; a theme or a gum configuration in the tree; a meaning a colour alone carries</t>
         </is>
       </c>
     </row>
@@ -14491,22 +14486,22 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t xml:space="preserve">plain output: the screens without colour, symbol or border, chosen by the environment alone — `NO_COLOR` set and not empty, `TERM=dumb`, or standard output not a terminal</t>
+          <t xml:space="preserve">a state word: the closed list of words that say how a step, a file or an action stands — its symbol and colour beside it in normal output, the word in brackets in plain output</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OUTPUT_PLAIN` in each terminal's `config.py`, read by its `tui.py`</t>
+          <t xml:space="preserve">`STATE_SYMBOLS`, `STATE_COLOURS`, `state_label()` in `tui.py`</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t xml:space="preserve">`[&lt;word&gt;]`</t>
+          <t xml:space="preserve">DONE; CURRENT; PENDING; CANCELLED; WARN; ERROR</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t xml:space="preserve">a flag, `--no-color`, `--simple`, `--a11y`; a theme or a gum configuration in the tree; a meaning a colour alone carries</t>
+          <t xml:space="preserve">a colour or a symbol without its word; a coloured row; `ok`, `success` as a state word</t>
         </is>
       </c>
     </row>
@@ -14518,49 +14513,44 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state word: the closed list of words that say how a step, a file or an action stands — its symbol and colour beside it in normal output, the word in brackets in plain output</t>
+          <t xml:space="preserve">the failure block and the exits: a failure on stderr as what failed, where, why and what next, the run's last block — 0 an action done or cancelled, 1 a failure, 2 an unknown argument, 130 Ctrl-C</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STATE_SYMBOLS`, `STATE_COLOURS`, `state_label()` in `tui.py`</t>
+          <t xml:space="preserve">`error_lines()`, `INTERRUPTED_EXIT_CODE` in `tui.py`; `_failure_exit_code()`, `_cancelled_exit_code()` in each `terminal.py`</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t xml:space="preserve">DONE; CURRENT; PENDING; CANCELLED; WARN; ERROR</t>
+          <t xml:space="preserve">where; why; next; `nothing written`</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t xml:space="preserve">a colour or a symbol without its word; a coloured row; `ok`, `success` as a state word</t>
+          <t xml:space="preserve">a traceback for an expected failure; a failure on stdout; exit 0 after a failure</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t xml:space="preserve">Terminals</t>
+          <t xml:space="preserve">Artifacts</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t xml:space="preserve">the failure block and the exits: a failure on stderr as what failed, where, why and what next, the run's last block — 0 an action done or cancelled, 1 a failure, 2 an unknown argument, 130 Ctrl-C</t>
+          <t xml:space="preserve">the family `ohlcv_1m_binance`, `ohlcv_1m_bybit`: one venue's minutes as printed, one partition per asset</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t xml:space="preserve">`error_lines()`, `INTERRUPTED_EXIT_CODE` in `tui.py`; `_failure_exit_code()`, `_cancelled_exit_code()` in each `terminal.py`</t>
-        </is>
-      </c>
-      <c r="E343" t="inlineStr">
-        <is>
-          <t xml:space="preserve">where; why; next; `nothing written`</t>
-        </is>
-      </c>
-      <c r="F343" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a traceback for an expected failure; a failure on stdout; exit 0 after a failure</t>
+          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_&lt;venue&gt;/ticker=&lt;TICKER&gt;/ohlcv_1m_&lt;venue&gt;.parquet` and the family's `schema.json`; `venue_parquet()` in `module_data/config.py`</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume` — the venue's rows, ordered by every column, so a duplicate minute keeps one order; untracked</t>
         </is>
       </c>
     </row>
@@ -14572,17 +14562,17 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `ohlcv_1m_binance`, `ohlcv_1m_bybit`: one venue's minutes as printed, one partition per asset</t>
+          <t xml:space="preserve">the family `ohlcv_1m_canonical`: the canonical 1m series, one partition per asset</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_&lt;venue&gt;/ticker=&lt;TICKER&gt;/ohlcv_1m_&lt;venue&gt;.parquet` and the family's `schema.json`; `venue_parquet()` in `module_data/config.py`</t>
+          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_canonical/ticker=&lt;TICKER&gt;/ohlcv_1m_canonical.parquet` and the family's `schema.json`; `ohlcv_1m_canonical_parquet()`</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume` — the venue's rows, ordered by every column, so a duplicate minute keeps one order; untracked</t>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `source`, `zero_volume`, `binance_valid`, `bybit_valid`, `rel_divergence` — the full grid of the window, ordered by `timestamp_ms`; untracked</t>
         </is>
       </c>
     </row>
@@ -14594,17 +14584,17 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `ohlcv_1m_canonical`: the canonical 1m series, one partition per asset</t>
+          <t xml:space="preserve">the family `bars`: the bars of every timeframe of the timeframe register, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_canonical/ticker=&lt;TICKER&gt;/ohlcv_1m_canonical.parquet` and the family's `schema.json`; `ohlcv_1m_canonical_parquet()`</t>
+          <t xml:space="preserve">`module_features/bars.py` writes `bars/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/bars.parquet` and the family's `schema.json`; `bars_parquet()`</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `source`, `zero_volume`, `binance_valid`, `bybit_valid`, `rel_divergence` — the full grid of the window, ordered by `timestamp_ms`; untracked</t>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `ffill_bars`, `zero_volume_bars` inside the research window, ordered by `timestamp_ms`; untracked</t>
         </is>
       </c>
     </row>
@@ -14616,17 +14606,17 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `bars`: the bars of every timeframe of the timeframe register, one partition per asset and timeframe</t>
+          <t xml:space="preserve">the family `catalogue`: every catalogued column on the decision grid, one partition per asset and timeframe; a partition may omit a column the feature catalogue does not offer on its timeframe, never rename one or change its type</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/bars.py` writes `bars/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/bars.parquet` and the family's `schema.json`; `bars_parquet()`</t>
+          <t xml:space="preserve">`module_features/catalogue.py` writes `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet` and the family's `schema.json` from `catalogue_schema()`, the columns of the union of its partitions in catalogue order; `catalogue_parquet()` — in `module_ml/config.py` the same name over the contract's `parquet_by_timeframe`</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `ffill_bars`, `zero_volume_bars` inside the research window, ordered by `timestamp_ms`; untracked</t>
+          <t xml:space="preserve">`decision_ts` and every definition offered on the partition's timeframe, on the decision grid; untracked</t>
         </is>
       </c>
     </row>
@@ -14638,17 +14628,17 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `catalogue`: every catalogued column on the decision grid, one partition per asset and timeframe; a partition may omit a column the feature catalogue does not offer on its timeframe, never rename one or change its type</t>
+          <t xml:space="preserve">the family `labels`: Y on the decision timeframe, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/catalogue.py` writes `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet` and the family's `schema.json` from `catalogue_schema()`, the columns of the union of its partitions in catalogue order; `catalogue_parquet()` — in `module_ml/config.py` the same name over the contract's `parquet_by_timeframe`</t>
+          <t xml:space="preserve">`module_ml/labels.py` writes `labels/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/labels.parquet` and the family's `schema.json`; `labels_parquet()`</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts` and every definition offered on the partition's timeframe, on the decision grid; untracked</t>
+          <t xml:space="preserve">`decision_ts`, `entry_ts`, `y`, `event_end_ts`, `entry_observable`, `label_valid`, `entry_price`, `upper_barrier`, `lower_barrier`; an ambiguous event carries `y = 0` with `label_valid = false`, so `y` is never read without `label_valid`; untracked</t>
         </is>
       </c>
     </row>
@@ -14660,17 +14650,17 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `labels`: Y on the decision timeframe, one partition per asset and timeframe</t>
+          <t xml:space="preserve">the family `oos_predictions`: the out-of-sample class probabilities, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/labels.py` writes `labels/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/labels.parquet` and the family's `schema.json`; `labels_parquet()`</t>
+          <t xml:space="preserve">`module_ml/train.py` writes `oos_predictions/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/oos_predictions.parquet` and the family's `schema.json`; `oos_predictions_parquet()`</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts`, `entry_ts`, `y`, `event_end_ts`, `entry_observable`, `label_valid`, `event_resolution`, `entry_price`, `upper_barrier`, `lower_barrier`, `exit_reference_price`; an ambiguous event carries `y = 0` with `label_valid = false`, so `y` is never read without `label_valid`; untracked</t>
+          <t xml:space="preserve">`decision_ts`, `oos_fold_id`, `p_short`, `p_neutral`, `p_long` — the full window of every validation fold and of the final holdout; metrics score only the supervised subset; untracked</t>
         </is>
       </c>
     </row>
@@ -14682,17 +14672,17 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `oos_predictions`: the out-of-sample class probabilities, one partition per asset and timeframe</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_README.md`</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/train.py` writes `oos_predictions/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/oos_predictions.parquet` and the family's `schema.json`; `oos_predictions_parquet()`</t>
+          <t xml:space="preserve">`module_ml/status.py` writes it, `asset_readme_md()`; its file list `file_manifest()`, the three files of `HAND_STAGE_FILE_DESCRIPTORS` listed with no size</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts`, `oos_fold_id`, `p_short`, `p_neutral`, `p_long` — the full window of every validation fold and of the final holdout; metrics score only the supervised subset; untracked</t>
+          <t xml:space="preserve">what the folder holds and what came out of it; no timestamp; tracked</t>
         </is>
       </c>
     </row>
@@ -14704,17 +14694,17 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_README.md`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_barriers.json`</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/status.py` writes it, `asset_readme_md()`; its file list `file_manifest()`, the three files of `HAND_STAGE_FILE_DESCRIPTORS` listed with no size</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `barriers_json()`; `load_barriers()` in `module_ml/dataset.py` reads it</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t xml:space="preserve">what the folder holds and what came out of it; no timestamp; tracked</t>
+          <t xml:space="preserve">`label_barrier_true_range_multiplier`, `label_horizon`, `take_profit_true_range_multiplier`, `stop_loss_true_range_multiplier` — the asset's promoted barrier geometry, a hand's choice; absent, `START_BY_COORDINATE_DEFAULT` of `module_ml/config.py` is the asset's; tracked once promoted, like the feature set beside it</t>
         </is>
       </c>
     </row>
@@ -14726,17 +14716,17 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_barriers.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `barriers_json()`; `load_barriers()` in `module_ml/dataset.py` reads it</t>
+          <t xml:space="preserve">`module_features/catalogue.py` writes it from `catalogue_contract()`; `catalogue_json()`</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t xml:space="preserve">`label_barrier_true_range_multiplier`, `label_horizon`, `take_profit_true_range_multiplier`, `stop_loss_true_range_multiplier` — the asset's promoted barrier geometry, a hand's choice; absent, `START_BY_COORDINATE_DEFAULT` of `module_ml/config.py` is the asset's; tracked once promoted, like the feature set beside it</t>
+          <t xml:space="preserve">the feature layer's contract the ML layer reads instead of the feature configuration: `decision_timeframe`, `timeframes` (each `timeframe`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe` — each value a path relative to the artifacts store, `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet`; untracked</t>
         </is>
       </c>
     </row>
@@ -14748,17 +14738,17 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json`</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/catalogue.py` writes it from `catalogue_contract()`; `catalogue_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `feature_set_json()`</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature layer's contract the ML layer reads instead of the feature configuration: `decision_timeframe`, `timeframes` (each `timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe` — each value a path relative to the artifacts store, `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet`; untracked</t>
+          <t xml:space="preserve">`columns_by_timeframe` — the promoted feature set, a hand's choice, and nothing else; absent, the default set is the asset's; tracked once promoted, like the parameters it conditions</t>
         </is>
       </c>
     </row>
@@ -14770,17 +14760,17 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_hyperparameter_point.json`</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `feature_set_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `hyperparameter_point_json()`; `hpo.main()` in `module_ml/hpo.py` reads it</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`columns_by_timeframe` — the promoted feature set, a hand's choice, and nothing else; absent, the default set is the asset's; tracked once promoted, like the parameters it conditions</t>
+          <t xml:space="preserve">`best_params` — the promoted hyper-parameter point, a hand's choice: the first trial of the chain's study, and nothing else; absent, the study draws every point; tracked once promoted, like the feature set and the geometry beside it</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14782,17 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_hyperparameter_point.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_model_evaluation.json`</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `hyperparameter_point_json()`; `hpo.main()` in `module_ml/hpo.py` reads it</t>
+          <t xml:space="preserve">`module_ml/train.py` writes it; `model_evaluation_json()`</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`best_params` — the promoted hyper-parameter point, a hand's choice: the first trial of the chain's study, and nothing else; absent, the study draws every point; tracked once promoted, like the feature set and the geometry beside it</t>
+          <t xml:space="preserve">`validation` — a `fold_&lt;id&gt;` per fold of `VALIDATION_FOLD_IDS` — and `final_holdout`, each `prior_logloss`, `model_logloss`, `relative_logloss_skill`, `scored_row_count`; `validation_importance`, a `fold_&lt;id&gt;` per validation fold, each `gain_importance` and `mean_abs_shap_importance` per column; `feature_columns`; `class_counts`, `labels`, `segments`; untracked</t>
         </is>
       </c>
     </row>
@@ -14814,17 +14804,17 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_model_evaluation.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_parameters.json`</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/train.py` writes it; `model_evaluation_json()`</t>
+          <t xml:space="preserve">`module_ml/hpo.py` writes it; `parameters_json()`</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`validation` — a `fold_&lt;id&gt;` per fold of `VALIDATION_FOLD_IDS` — and `final_holdout`, each `prior_logloss`, `model_logloss`, `relative_logloss_skill`, `scored_row_count`; `validation_importance`, a `fold_&lt;id&gt;` per validation fold, each `gain_importance` and `mean_abs_shap_importance` per column; `feature_columns`; `class_counts`, `labels`, `segments`; untracked</t>
+          <t xml:space="preserve">`hyperparameter_search_result` (`best_params`, `best_cagr_validation_path`, `trial_count`); tracked</t>
         </is>
       </c>
     </row>
@@ -14836,17 +14826,27 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_parameters.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_score_request.json`: the serpentine search's question</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/hpo.py` writes it; `parameters_json()`</t>
+          <t xml:space="preserve">`score_request_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by a turn, `features-serpentine-turn`, read by `module_ml.score`, `ml-score`; the one file the loop of `features-serpentine-search` tests, running `ml-score` and a turn again while it exists</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`kind` (`score` or `hpo`), `round`, `states`</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a key beside these three; a request the evaluator writes; a second file the loop tests</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`hyperparameter_search_result` (`best_params`, `best_cagr_validation_path`, `trial_count`); tracked</t>
+          <t xml:space="preserve">what one family pass asks to be scored: the kind of scoring, the round it runs in, and the states — a state of its own for `score`, a beam parent's scored row for `hpo`; untracked</t>
         </is>
       </c>
     </row>
@@ -14858,27 +14858,27 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_score_request.json`: the serpentine search's question</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_score_response.json`: the serpentine search's answer</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_request_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by a turn, `features-serpentine-turn`, read by `module_ml.score`, `ml-score`; the one file the loop of `features-serpentine-search` tests, running `ml-score` and a turn again while it exists</t>
+          <t xml:space="preserve">`score_response_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by `module_ml.score` alone</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`kind` (`score` or `hpo`), `round`, `states`</t>
+          <t xml:space="preserve">`kind`, `round`, `results`; a `score` result the row of one scored state of the serpentine search, an `hpo` result `state_key`, `trial_count_drawn` and `candidate`</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">a key beside these three; a request the evaluator writes; a second file the loop tests</t>
+          <t xml:space="preserve">a key beside these three; a result out of the order the request named; a response written before every state has one</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t xml:space="preserve">what one family pass asks to be scored: the kind of scoring, the round it runs in, and the states — a state of its own for `score`, a beam parent's scored row for `hpo`; untracked</t>
+          <t xml:space="preserve">what the states of one request are worth, in the order the request named them; `candidate` a scored row or `null`, and `null` is an answer; untracked</t>
         </is>
       </c>
     </row>
@@ -14890,27 +14890,17 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_score_response.json`: the serpentine search's answer</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search.json`</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_response_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by `module_ml.score` alone</t>
-        </is>
-      </c>
-      <c r="D358" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`kind`, `round`, `results`; a `score` result the row of one scored state of the serpentine search, an `hpo` result `state_key`, `trial_count_drawn` and `candidate`</t>
-        </is>
-      </c>
-      <c r="F358" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a key beside these three; a result out of the order the request named; a response written before every state has one</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_json()`</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t xml:space="preserve">what the states of one request are worth, in the order the request named them; `candidate` a scored row or `null`, and `null` is an answer; untracked</t>
+          <t xml:space="preserve">`inputs`, `beam`, `champion_trial_index`, `round_count`, `search_converged`, `path` (each `round`, `loop`, `family`, `trial_index`, `beam`, `move`), `proposals` (each `proposal`, `trial_index`), `trial_count_by_loop` — where the search stands at a round boundary, naming trials by index and carrying none of their columns; tracked once a search has run</t>
         </is>
       </c>
     </row>
@@ -14922,17 +14912,17 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_json()`</t>
+          <t xml:space="preserve">a hand, in the file or through the features terminal's draft; `serpentine_search_profile_json()`</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs`, `beam`, `champion_trial_index`, `round_count`, `search_converged`, `path` (each `round`, `loop`, `family`, `trial_index`, `beam`, `move`), `proposals` (each `proposal`, `trial_index`), `trial_count_by_loop` — where the search stands at a round boundary, naming trials by index and carrying none of their columns; tracked once a search has run</t>
+          <t xml:space="preserve">`columns_admitted_by_timeframe`, `start_columns_by_timeframe` (`null` = the asset's own set), `grid_by_coordinate` (one list per coordinate, in the order it is searched), `loops` (a subset of `SERPENTINE_SEARCH_ROUND_LOOPS`), `path_cagr_noise_standard_deviation` (the asset's noise sigma, `null` on the calibration run) — what a hand asks the serpentine search to look at; drafted, never derived, and tracked</t>
         </is>
       </c>
     </row>
@@ -14944,17 +14934,17 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_trials.jsonl`</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hand, in the file or through the features terminal's draft; `serpentine_search_profile_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_trials_jsonl()`</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`columns_admitted_by_timeframe`, `start_columns_by_timeframe` (`null` = the asset's own set), `grid_by_coordinate` (one list per coordinate, in the order it is searched), `loops` (a subset of `SERPENTINE_SEARCH_ROUND_LOOPS`), `path_cagr_noise_standard_deviation` (the asset's noise sigma, `null` on the calibration run) — what a hand asks the serpentine search to look at; drafted, never derived, and tracked</t>
+          <t xml:space="preserve">one scored state of the serpentine search a line, appended and never rewritten; `trial_index` = the line number, counted from one; tracked once a search has run</t>
         </is>
       </c>
     </row>
@@ -14966,39 +14956,49 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_trials.jsonl`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_strategy_evaluation.json`</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_trials_jsonl()`</t>
+          <t xml:space="preserve">`module_ml/strategy.py` writes it; `strategy_evaluation_json()`</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t xml:space="preserve">one scored state of the serpentine search a line, appended and never rewritten; `trial_index` = the line number, counted from one; tracked once a search has run</t>
+          <t xml:space="preserve">`entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `cleared_point_count`, `median_cagr_over_cleared`, `max_cagr_over_cleared`, `selection_score_cagr_validation_path`, `execution_cost_rate_per_trade_side`; per fold `sharpe`, `cagr`, `max_drawdown`, `calmar`, `profit_factor`, `trade_count`, `hit_rate`, `average_trade_return`, `exposure`, `exit_counts`, `final_equity`; `validation_path` over the validation folds; the final holdout's `equity_curve`; untracked</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artifacts</t>
+          <t xml:space="preserve">Features</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_strategy_evaluation.json`</t>
+          <t xml:space="preserve">a series of one timeframe's bars, with no parameter</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/strategy.py` writes it; `strategy_evaluation_json()`</t>
-        </is>
-      </c>
-      <c r="G362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `cleared_point_count`, `median_cagr_over_cleared`, `max_cagr_over_cleared`, `selection_score_cagr_validation_path`, `execution_cost_rate_per_trade_side`; per fold `sharpe`, `cagr`, `max_drawdown`, `calmar`, `profit_factor`, `trade_count`, `hit_rate`, `average_trade_return`, `exposure`, `exit_counts`, `final_equity`; `validation_path` over the validation folds; the final holdout's `equity_curve`; untracked</t>
+          <t xml:space="preserve">`open`, `high`, `low`, `close`, `volume` — a bar column — and the series with a kernel: `logarithmic_volume`, `true_range`, `cumulative_signed_volume`; `SERIES_KERNELS`, `module_features/indicators.py`</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`inputs` of a term</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the series token</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a series with a parameter; `log_volume`</t>
         </is>
       </c>
     </row>
@@ -15010,27 +15010,32 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t xml:space="preserve">a series of one timeframe's bars, with no parameter</t>
+          <t xml:space="preserve">an indicator — one computation with exactly one integer parameter, named by its token, its invariants one record of the register beside its kernel, the popular names it answers to among them</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`open`, `high`, `low`, `close`, `volume` — a bar column — and the series with a kernel: `logarithmic_volume`, `true_range`, `cumulative_signed_volume`; `SERIES_KERNELS`, `module_features/indicators.py`</t>
+          <t xml:space="preserve">`exponential_smoothing&lt;n&gt;`, `rolling_mean&lt;n&gt;`, `recursive_mean&lt;n&gt;`, `recursive_mean_gain_share&lt;n&gt;`, `rolling_standard_score&lt;n&gt;`, `rolling_range_position&lt;n&gt;`, `rolling_standard_deviation&lt;n&gt;`, `relative_change&lt;n&gt;`, `recursive_mean_upward_movement_share&lt;n&gt;`, `recursive_mean_directional_movement_imbalance&lt;n&gt;`, `rolling_volume_weighted_mean&lt;n&gt;`, `rolling_volume_weighted_close_location&lt;n&gt;`, `rolling_money_flow_gain_share&lt;n&gt;`; `INDICATORS` — `kernel`, `parameter_word`, `warmup_multiple`, `inputs`, `output_range`, `historical_aliases` of a record, `module_features/indicators.py`</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs` of a term</t>
+          <t xml:space="preserve">`indicator`, `parameter_word`, `parameter_bars`, `output_range`, `historical_aliases` of a term</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">the series token</t>
+          <t xml:space="preserve">the token with its parameter, `&lt;PARAMETER_WORD&gt; &lt;n&gt; bars of &lt;inputs&gt;` beside it and `output &lt;low&gt;–&lt;high&gt;` when the indicator is bounded (the catalogue table's terms)</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">a series with a parameter; `log_volume`</t>
+          <t xml:space="preserve">`rsi_14`, `sma_200`, `bb20`; a table of indicator facts in `config.py` beside the register; `kernel` for anything but the function a record computes with; the abbreviations these tokens replaced: `ema`, `sma`, `rsi`, `atr`, `zscore`, `rolling_zscore`, `wilder_smoothing`, `range_position`</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
         </is>
       </c>
     </row>
@@ -15042,32 +15047,27 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t xml:space="preserve">an indicator — one computation with exactly one integer parameter, named by its token, its invariants one record of the register beside its kernel, the popular names it answers to among them</t>
+          <t xml:space="preserve">a term — a series or an indicator inside a feature definition</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t xml:space="preserve">`exponential_smoothing&lt;n&gt;`, `rolling_mean&lt;n&gt;`, `recursive_mean&lt;n&gt;`, `recursive_mean_gain_share&lt;n&gt;`, `rolling_standard_score&lt;n&gt;`, `rolling_range_position&lt;n&gt;`, `rolling_standard_deviation&lt;n&gt;`, `relative_change&lt;n&gt;`, `recursive_mean_upward_movement_share&lt;n&gt;`, `recursive_mean_directional_movement_imbalance&lt;n&gt;`, `rolling_volume_weighted_mean&lt;n&gt;`, `rolling_volume_weighted_close_location&lt;n&gt;`, `rolling_money_flow_gain_share&lt;n&gt;`; `INDICATORS` — `kernel`, `parameter_word`, `warmup_multiple`, `inputs`, `output_range`, `historical_aliases` of a record, `module_features/indicators.py`</t>
+          <t xml:space="preserve">`("&lt;indicator&gt;", &lt;parameter_bars&gt;)` on the default series close, `("&lt;series&gt;", "&lt;indicator&gt;", &lt;parameter_bars&gt;)` on another series, `("&lt;series&gt;",)` a bare series; `term_name()`</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t xml:space="preserve">`indicator`, `parameter_word`, `parameter_bars`, `output_range`, `historical_aliases` of a term</t>
+          <t xml:space="preserve">`terms`</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">the token with its parameter, `&lt;PARAMETER_WORD&gt; &lt;n&gt; bars of &lt;inputs&gt;` beside it and `output &lt;low&gt;–&lt;high&gt;` when the indicator is bounded (the catalogue table's terms)</t>
+          <t xml:space="preserve">terms</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t xml:space="preserve">`rsi_14`, `sma_200`, `bb20`; a table of indicator facts in `config.py` beside the register; `kernel` for anything but the function a record computes with; the abbreviations these tokens replaced: `ema`, `sma`, `rsi`, `atr`, `zscore`, `rolling_zscore`, `wilder_smoothing`, `range_position`</t>
-        </is>
-      </c>
-      <c r="I364" t="inlineStr">
-        <is>
-          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
+          <t xml:space="preserve">atom</t>
         </is>
       </c>
     </row>
@@ -15079,27 +15079,32 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t xml:space="preserve">a term — a series or an indicator inside a feature definition</t>
+          <t xml:space="preserve">a feature definition — terms of one timeframe composed by the operators, with an optional normaliser; the timeframe-less half of a feature, carrying the tier it belongs to and the popular names that denote the whole of it</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t xml:space="preserve">`("&lt;indicator&gt;", &lt;parameter_bars&gt;)` on the default series close, `("&lt;series&gt;", "&lt;indicator&gt;", &lt;parameter_bars&gt;)` on another series, `("&lt;series&gt;",)` a bare series; `term_name()`</t>
+          <t xml:space="preserve">one record of `FEATURE_CATALOGUE`; `feature_definition_name()`; `OPERATORS` = {`minus`, `over`} and `NORMALISERS` = {`centered`}, one record per token beside its kernel in `module_features/catalogue.py`</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t xml:space="preserve">`terms`</t>
+          <t xml:space="preserve">`feature_definition`, `tier` = `CORE` / `EXTENDED` / `COMPOSITE`, `historical_aliases`</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t xml:space="preserve">terms</t>
+          <t xml:space="preserve">definition (the catalogue table)</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t xml:space="preserve">atom</t>
+          <t xml:space="preserve">molecule, family, feature family, indicator (for a composite); `trend`, `momentum`, `volatility`, `structure`, `activity` — a category, not a computation; a popular name as the key, the column or a second name beside the canonical one; a tier written anywhere but the record; `centred` — the normaliser token keeps its American spelling, a column and a key on disk</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
         </is>
       </c>
     </row>
@@ -15111,32 +15116,27 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t xml:space="preserve">a feature definition — terms of one timeframe composed by the operators, with an optional normaliser; the timeframe-less half of a feature, carrying the tier it belongs to and the popular names that denote the whole of it</t>
+          <t xml:space="preserve">a feature — a definition aligned to the decision grid on one timeframe; the column of X and the key of an importance</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t xml:space="preserve">one record of `FEATURE_CATALOGUE`; `feature_definition_name()`; `OPERATORS` = {`minus`, `over`} and `NORMALISERS` = {`centered`}, one record per token beside its kernel in `module_features/catalogue.py`</t>
+          <t xml:space="preserve">`feature_id()` = `&lt;definition&gt;_&lt;timeframe&gt;`</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_definition`, `tier` = `CORE` / `EXTENDED` / `COMPOSITE`, `historical_aliases`</t>
+          <t xml:space="preserve">`feature_columns`, the keys of an importance</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t xml:space="preserve">definition (the catalogue table)</t>
+          <t xml:space="preserve">the feature id — `column &lt;timeframe&gt;` in the FEATURE SET frame</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t xml:space="preserve">molecule, family, feature family, indicator (for a composite); `trend`, `momentum`, `volatility`, `structure`, `activity` — a category, not a computation; a popular name as the key, the column or a second name beside the canonical one; a tier written anywhere but the record; `centred` — the normaliser token keeps its American spelling, a column and a key on disk</t>
-        </is>
-      </c>
-      <c r="I366" t="inlineStr">
-        <is>
-          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
+          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
         </is>
       </c>
     </row>
@@ -15148,27 +15148,27 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t xml:space="preserve">a feature — a definition aligned to the decision grid on one timeframe; the column of X and the key of an importance</t>
+          <t xml:space="preserve">the feature catalogue — every definition the repository can compute, with the timeframes it is offered on; drafted, like the rest of `config.py`</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_id()` = `&lt;definition&gt;_&lt;timeframe&gt;`</t>
+          <t xml:space="preserve">`FEATURE_CATALOGUE`, `catalogue_columns()`, `CATALOGUE_COLUMNS`; the stage `features-catalogue`, `module_features/catalogue.py`</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_columns`, the keys of an importance</t>
+          <t xml:space="preserve">`catalogue` (of `features_status.json`); `&lt;TICKER&gt;_catalogue.json`; the family `catalogue`</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature id — `column &lt;timeframe&gt;` in the FEATURE SET frame</t>
+          <t xml:space="preserve">CATALOGUE</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
+          <t xml:space="preserve">palette, feature list, feature store</t>
         </is>
       </c>
     </row>
@@ -15180,27 +15180,22 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature catalogue — every definition the repository can compute, with the timeframes it is offered on; drafted, like the rest of `config.py`</t>
+          <t xml:space="preserve">the feature layer's contract, per asset — what the ML layer reads instead of this module's configuration</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t xml:space="preserve">`FEATURE_CATALOGUE`, `catalogue_columns()`, `CATALOGUE_COLUMNS`; the stage `features-catalogue`, `module_features/catalogue.py`</t>
+          <t xml:space="preserve">`catalogue_contract()`, `catalogue_json()` in `module_features/config.py`; the descriptor's copy in `module_ml/config.py`; `load_catalogue()` in `module_ml/dataset.py`, `cat`</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue` (of `features_status.json`); `&lt;TICKER&gt;_catalogue.json`; the family `catalogue`</t>
-        </is>
-      </c>
-      <c r="E368" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CATALOGUE</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`: `decision_timeframe`, `timeframes` (`timeframe`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe`</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t xml:space="preserve">palette, feature list, feature store</t>
+          <t xml:space="preserve">an import of `module_features` from `module_ml`; a token or a slot parsed in the ML layer; a second read of the file inside one stage; a path built from the slot grammar outside `module_features`; a parquet named in the contract by anything but its path relative to the artifact store</t>
         </is>
       </c>
     </row>
@@ -15212,22 +15207,27 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature layer's contract, per asset — what the ML layer reads instead of this module's configuration</t>
+          <t xml:space="preserve">the effective history — what a parameter covers on a timeframe, `bars × timeframe`, the quantity the nesting rule compares</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue_contract()`, `catalogue_json()` in `module_features/config.py`; the descriptor's copy in `module_ml/config.py`; `load_catalogue()` in `module_ml/dataset.py`, `cat`</t>
+          <t xml:space="preserve">`definition_effective_history_hours()`</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`: `decision_timeframe`, `timeframes` (`timeframe`, `slot`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe`</t>
+          <t xml:space="preserve">`effective_history_hours_by_timeframe`; `lower_longest_effective_history_hours`, `upper_shortest_effective_history_hours` of `nesting`</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t xml:space="preserve">effective history</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t xml:space="preserve">an import of `module_features` from `module_ml`; a token or a slot parsed in the ML layer; a second read of the file inside one stage; a path built from the slot grammar outside `module_features`; a parquet named in the contract by anything but its path relative to the artifact store</t>
+          <t xml:space="preserve">history (bare — a recursion has no window), span (the parameter word of an exponential smoothing), lookback hours</t>
         </is>
       </c>
     </row>
@@ -15239,27 +15239,22 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t xml:space="preserve">the effective history — what a parameter covers on a timeframe, `bars × timeframe`, the quantity the nesting rule compares</t>
-        </is>
-      </c>
-      <c r="C370" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`definition_effective_history_hours()`</t>
-        </is>
-      </c>
-      <c r="D370" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`effective_history_hours_by_timeframe`; `lower_longest_effective_history_hours`, `upper_shortest_effective_history_hours` of `nesting`</t>
+          <t xml:space="preserve">the Bollinger %b reading — the trade's %b(20, 2σ), `rolling_standard_score20` / 4 + 0.5, an affine map a tree model is invariant to, so no %b column exists</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t xml:space="preserve">effective history</t>
+          <t xml:space="preserve">— (no page shows it; Bollinger %b in the definitions table of `methodology_features.md`)</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t xml:space="preserve">history (bare — a recursion has no window), span (the parameter word of an exponential smoothing), lookback hours</t>
+          <t xml:space="preserve">`bb20`, `%b` as a column, `z / 2 + 0.5`; `zscore20`</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bollinger (technical analysis)</t>
         </is>
       </c>
     </row>
@@ -15271,22 +15266,27 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t xml:space="preserve">the Bollinger %b reading — the trade's %b(20, 2σ), `rolling_standard_score20` / 4 + 0.5, an affine map a tree model is invariant to, so no %b column exists</t>
+          <t xml:space="preserve">the definitions an asset's model sees until a promotion — the frozen experiment's default definitions on every timeframe of the register, in the order it stacks them</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME`; `definition_in_default_set` of a record</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`definition_in_default_set`; `default_columns_by_timeframe` of the contract</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t xml:space="preserve">— (no page shows it; Bollinger %b in the definitions table of `methodology_features.md`)</t>
+          <t xml:space="preserve">default set</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t xml:space="preserve">`bb20`, `%b` as a column, `z / 2 + 0.5`; `zscore20`</t>
-        </is>
-      </c>
-      <c r="I371" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bollinger (technical analysis)</t>
+          <t xml:space="preserve">the frozen fifteen (as a name)</t>
         </is>
       </c>
     </row>
@@ -15298,59 +15298,49 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t xml:space="preserve">the definitions an asset's model sees until a promotion — the frozen experiment's default definitions on every timeframe of the register, in the order it stacks them</t>
+          <t xml:space="preserve">the definition the strategy hierarchy reads on every timeframe, set or no set</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME`; `definition_in_default_set` of a record</t>
+          <t xml:space="preserve">`TREND_GATE_FEATURE_DEFINITION` in `module_ml/config.py` — the name of the catalogue's first definition, owned by the strategy that reads it; the gate's timeframe is the top of the contract's hierarchy, `trend_gate_timeframe(cat)`</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t xml:space="preserve">`definition_in_default_set`; `default_columns_by_timeframe` of the contract</t>
+          <t xml:space="preserve">`trend_gate_feature`</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t xml:space="preserve">default set</t>
+          <t xml:space="preserve">gate (the asset's STRATEGY frame)</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t xml:space="preserve">the frozen fifteen (as a name)</t>
+          <t xml:space="preserve">`TREND_FAMILY`; a column literal in `asset.js`; a second copy of the name in the feature layer, which reads nothing of it</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t xml:space="preserve">Features</t>
+          <t xml:space="preserve">Asset containers</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t xml:space="preserve">the definition the strategy hierarchy reads on every timeframe, set or no set</t>
+          <t xml:space="preserve">an asset container: a runner's one-off for one asset, exiting with its stage</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TREND_GATE_FEATURE_DEFINITION` in `module_ml/config.py` — the name of the catalogue's first definition, owned by the strategy that reads it; the gate's timeframe is the top of the contract's hierarchy, `trend_gate_timeframe(cat)`</t>
-        </is>
-      </c>
-      <c r="D373" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`trend_gate_feature`</t>
-        </is>
-      </c>
-      <c r="E373" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gate (the asset's STRATEGY frame)</t>
+          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TREND_FAMILY`; a column literal in `asset.js`; a second copy of the name in the feature layer, which reads nothing of it</t>
+          <t xml:space="preserve">a compose service per asset; a resident per asset; a `restart:` policy; a published port</t>
         </is>
       </c>
     </row>
@@ -15362,17 +15352,17 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t xml:space="preserve">an asset container: a runner's one-off for one asset, exiting with its stage</t>
+          <t xml:space="preserve">a runner: a compose service that is a role and a one-off — no command of its own; the run supplies one and the container exits with the stage</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
+          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t xml:space="preserve">a compose service per asset; a resident per asset; a `restart:` policy; a published port</t>
+          <t xml:space="preserve">`pipeline`, one runner for every module; a stage run by `exec` inside a resident; a runner with a `command:`</t>
         </is>
       </c>
     </row>
@@ -15384,17 +15374,17 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t xml:space="preserve">a runner: a compose service that is a role and a one-off — no command of its own; the run supplies one and the container exits with the stage</t>
+          <t xml:space="preserve">a service's mounts: the tree at `/app` and the stores it touches at `/store/&lt;content&gt;`, read-only where it only reads</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
+          <t xml:space="preserve">`.:/app` and `./store/&lt;content&gt;:/store/&lt;content&gt;` in each service's `volumes:` of `docker-compose.yml`, respelled whole because a service's key replaces the anchor's</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t xml:space="preserve">`pipeline`, one runner for every module; a stage run by `exec` inside a resident; a runner with a `command:`</t>
+          <t xml:space="preserve">`/app/store/&lt;content&gt;` as an address; a mount of a store the service does not touch; a named volume</t>
         </is>
       </c>
     </row>
@@ -15406,17 +15396,17 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t xml:space="preserve">a service's mounts: the tree at `/app` and the stores it touches at `/store/&lt;content&gt;`, read-only where it only reads</t>
+          <t xml:space="preserve">the memory ceiling of the one runner that needs it — HPO and XGBoost allocate above `DUCKDB_MEMORY_LIMIT`</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.:/app` and `./store/&lt;content&gt;:/store/&lt;content&gt;` in each service's `volumes:` of `docker-compose.yml`, respelled whole because a service's key replaces the anchor's</t>
+          <t xml:space="preserve">`deploy.resources.limits.memory` of the `ml` runner alone</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t xml:space="preserve">`/app/store/&lt;content&gt;` as an address; a mount of a store the service does not touch; a named volume</t>
+          <t xml:space="preserve">`mem_limit` beside it, a CPU quota, a reservation; a ceiling on the anchor, so on the dashboard too</t>
         </is>
       </c>
     </row>
@@ -15428,17 +15418,17 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t xml:space="preserve">the memory ceiling of the one runner that needs it — HPO and XGBoost allocate above `DUCKDB_MEMORY_LIMIT`</t>
+          <t xml:space="preserve">the thread cap: every computation's threads pinned to one — OpenMP's by the compose anchor's environment, beside the store contract, DuckDB's and XGBoost's in the code</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t xml:space="preserve">`deploy.resources.limits.memory` of the `ml` runner alone</t>
+          <t xml:space="preserve">`OMP_NUM_THREADS` in the `x-store-environment` anchor of `docker-compose.yml`; `SET threads=1` on every DuckDB connection; `nthread` of the booster's parameters in `module_ml/config.py`</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t xml:space="preserve">`mem_limit` beside it, a CPU quota, a reservation; a ceiling on the anchor, so on the dashboard too</t>
+          <t xml:space="preserve">a thread count read from a stage's command line; a cap set per service</t>
         </is>
       </c>
     </row>
@@ -15450,17 +15440,17 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t xml:space="preserve">the thread cap: every computation's threads pinned to one — OpenMP's by the compose anchor's environment, beside the store contract, DuckDB's and XGBoost's in the code</t>
+          <t xml:space="preserve">the dashboard's command: the server, on the container's internal port</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OMP_NUM_THREADS` in the `x-store-environment` anchor of `docker-compose.yml`; `SET threads=1` on every DuckDB connection; `nthread` of the booster's parameters in `module_ml/config.py`</t>
+          <t xml:space="preserve">`command: python -m module_monitoring.serve` of `dashboard`; `CONTAINER_PORT` and `BIND_ADDRESS` in `module_monitoring/config.py`</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t xml:space="preserve">a thread count read from a stage's command line; a cap set per service</t>
+          <t xml:space="preserve">a port or a bind address read from the environment or the command line; `PORT` inside a container</t>
         </is>
       </c>
     </row>
@@ -15472,17 +15462,22 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t xml:space="preserve">the dashboard's command: the server, on the container's internal port</t>
+          <t xml:space="preserve">the host port: the host side of the dashboard's mapping, measured at invocation and never written down — and the page's address, the one `make on` prints</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command: python -m module_monitoring.serve` of `dashboard`; `CONTAINER_PORT` and `BIND_ADDRESS` in `module_monitoring/config.py`</t>
+          <t xml:space="preserve">`PORT` of the `Makefile` — the port the dashboard already publishes, else the first free one upward from the internal port's number; `PORT=n` overrides; the `ports:` of `dashboard`, published on `127.0.0.1`</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`dashboard at http://127.0.0.1:&lt;port&gt;/`</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t xml:space="preserve">a port or a bind address read from the environment or the command line; `PORT` inside a container</t>
+          <t xml:space="preserve">the internal port's number as the page's address in a document, a command or a comment; a second variable for it; `PORT` inside a container; a measurement outside the `Makefile`</t>
         </is>
       </c>
     </row>
@@ -15494,22 +15489,17 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t xml:space="preserve">the host port: the host side of the dashboard's mapping, measured at invocation and never written down — and the page's address, the one `make on` prints</t>
+          <t xml:space="preserve">the compose project: the one fixed name every container, network and volume of this project carries on every host</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t xml:space="preserve">`PORT` of the `Makefile` — the port the dashboard already publishes, else the first free one upward from the internal port's number; `PORT=n` overrides; the `ports:` of `dashboard`, published on `127.0.0.1`</t>
-        </is>
-      </c>
-      <c r="E380" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`dashboard at http://127.0.0.1:&lt;port&gt;/`</t>
+          <t xml:space="preserve">`name: liora` in `docker-compose.yml` — the resident `liora-dashboard-1`</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t xml:space="preserve">the internal port's number as the page's address in a document, a command or a comment; a second variable for it; `PORT` inside a container; a measurement outside the `Makefile`</t>
+          <t xml:space="preserve">a name derived from the checkout's directory; a project per ticker; two checkouts of the project up at once on one host — they share the name: run one, or set `COMPOSE_PROJECT_NAME`</t>
         </is>
       </c>
     </row>
@@ -15521,17 +15511,17 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t xml:space="preserve">the compose project: the one fixed name every container, network and volume of this project carries on every host</t>
+          <t xml:space="preserve">how long a container lives: one-off — a `run --rm` process that exits with its stage — or resident — a server that stays up</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t xml:space="preserve">`name: liora` in `docker-compose.yml` — the resident `liora-dashboard-1`</t>
+          <t xml:space="preserve">`run --rm -T`, the `run` macro of the `Makefile`, for a one-off; `up -d dashboard` of `make on` for the one resident</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t xml:space="preserve">a name derived from the checkout's directory; a project per ticker; two checkouts of the project up at once on one host — they share the name: run one, or set `COMPOSE_PROJECT_NAME`</t>
+          <t xml:space="preserve">one-shot, ephemeral, daemon, long-running; `task` or `job` for the one-off; a stage run in a resident</t>
         </is>
       </c>
     </row>
@@ -15543,39 +15533,49 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t xml:space="preserve">how long a container lives: one-off — a `run --rm` process that exits with its stage — or resident — a server that stays up</t>
+          <t xml:space="preserve">the presentation switch: the dashboard up with the page's address printed and opened, or every container of this project down, in one word</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run --rm -T`, the `run` macro of the `Makefile`, for a one-off; `up -d dashboard` of `make on` for the one resident</t>
+          <t xml:space="preserve">`make on`, `make off` — the two bare lifecycle targets a presenter types</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t xml:space="preserve">one-shot, ephemeral, daemon, long-running; `task` or `job` for the one-off; a stage run in a resident</t>
+          <t xml:space="preserve">`start` / `stop`, bare `up` / `down` (compose's), `run`, a second switch pair; a switch that runs a stage</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset containers</t>
+          <t xml:space="preserve">Run record</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t xml:space="preserve">the presentation switch: the dashboard up with the page's address printed and opened, or every container of this project down, in one word</t>
+          <t xml:space="preserve">one recorded run of the chain — the execution name, read forward</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make on`, `make off` — the two bare lifecycle targets a presenter types</t>
+          <t xml:space="preserve">`run_id`; `RUN_ID` of the `Makefile`, `&lt;YYYYMMDDTHHMMSS&gt;Z_&lt;short commit&gt;` — the UTC time, then git's short commit — so it sorts by time and names the code that ran</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`run_id`</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">run</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t xml:space="preserve">`start` / `stop`, bare `up` / `down` (compose's), `run`, a second switch pair; a switch that runs a stage</t>
+          <t xml:space="preserve">build, job, a content hash; a generated run id bound to no project name; a run id inside an artifact or a ledger</t>
         </is>
       </c>
     </row>
@@ -15587,27 +15587,27 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t xml:space="preserve">one recorded run of the chain — the execution name, read forward</t>
+          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run_id`; `RUN_ID` of the `Makefile`, `&lt;YYYYMMDDTHHMMSS&gt;Z_&lt;short commit&gt;` — the UTC time, then git's short commit — so it sorts by time and names the code that ran</t>
+          <t xml:space="preserve">the target name; `RECORDED_STAGES` in the `Makefile` — `DATA_STAGES`, `FEATURES_STAGES`, `ML_STAGES` in order; `make all-record`</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run_id`</t>
+          <t xml:space="preserve">`stage` — the file name `&lt;stage&gt;.json`</t>
         </is>
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t xml:space="preserve">run</t>
+          <t xml:space="preserve">stage</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t xml:space="preserve">build, job, a content hash; a generated run id bound to no project name; a run id inside an artifact or a ledger</t>
+          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
         </is>
       </c>
     </row>
@@ -15619,27 +15619,22 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
+          <t xml:space="preserve">the command the recorder ran</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t xml:space="preserve">the target name; `RECORDED_STAGES` in the `Makefile` — `DATA_STAGES`, `FEATURES_STAGES`, `ML_STAGES` in order; `make all-record`</t>
+          <t xml:space="preserve">`command` — the make command line, joined by spaces</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t xml:space="preserve">`stage` — the file name `&lt;stage&gt;.json`</t>
-        </is>
-      </c>
-      <c r="E385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">stage</t>
+          <t xml:space="preserve">`command`</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
+          <t xml:space="preserve">a stage's own command line; anything a stage says about itself</t>
         </is>
       </c>
     </row>
@@ -15651,22 +15646,27 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t xml:space="preserve">the command the recorder ran</t>
+          <t xml:space="preserve">the exit code: how the stage ended; `all-record` stops at the first stage that exits non-zero and keeps its record</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command` — the make command line, joined by spaces</t>
+          <t xml:space="preserve">the command's exit code, `record.py`'s own</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command`</t>
+          <t xml:space="preserve">`exit_code`</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">exit</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage's own command line; anything a stage says about itself</t>
+          <t xml:space="preserve">status, ok</t>
         </is>
       </c>
     </row>
@@ -15678,27 +15678,27 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t xml:space="preserve">the exit code: how the stage ended; `all-record` stops at the first stage that exits non-zero and keeps its record</t>
+          <t xml:space="preserve">the stage timing: when the stage ran, and for how long</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t xml:space="preserve">the command's exit code, `record.py`'s own</t>
+          <t xml:space="preserve">`main()` in `record.py` — the UTC clock before and after the command, the monotonic clock for the duration</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t xml:space="preserve">`exit_code`</t>
+          <t xml:space="preserve">`started_at_utc`, `ended_at_utc`, `duration_seconds`</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t xml:space="preserve">exit</t>
+          <t xml:space="preserve">start; time; start / end and total time in the run's header</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t xml:space="preserve">status, ok</t>
+          <t xml:space="preserve">wall, elapsed</t>
         </is>
       </c>
     </row>
@@ -15710,27 +15710,27 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stage timing: when the stage ran, and for how long</t>
+          <t xml:space="preserve">the store diff: what the stage did to the stores — every file added, changed (size or mtime moved) or removed, by store and path</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t xml:space="preserve">`main()` in `record.py` — the UTC clock before and after the command, the monotonic clock for the duration</t>
+          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the four stores of `STORES` — every store but the trials store</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t xml:space="preserve">`started_at_utc`, `ended_at_utc`, `duration_seconds`</t>
+          <t xml:space="preserve">`store_diff` with `added`, `changed` — each `store`, `path`, `size_bytes`, `mtime_ns` — and `removed` — each `store`, `path`</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t xml:space="preserve">start; time; start / end and total time in the run's header</t>
+          <t xml:space="preserve">added / changed / removed; bytes written; the STORES frame</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t xml:space="preserve">wall, elapsed</t>
+          <t xml:space="preserve">output, artifacts, a stage → artifact map; a trial ledger read by the recorder</t>
         </is>
       </c>
     </row>
@@ -15742,27 +15742,17 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store diff: what the stage did to the stores — every file added, changed (size or mtime moved) or removed, by store and path</t>
+          <t xml:space="preserve">the basket one run covered — not in the record: the recorder knows no basket</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the four stores of `STORES` — every store but the trials store</t>
-        </is>
-      </c>
-      <c r="D389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`store_diff` with `added`, `changed` — each `store`, `path`, `size_bytes`, `mtime_ns` — and `removed` — each `store`, `path`</t>
-        </is>
-      </c>
-      <c r="E389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">added / changed / removed; bytes written; the STORES frame</t>
+          <t xml:space="preserve">the launcher's `TICKERS`, which the make target the recorder wraps carries into every stage command</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t xml:space="preserve">output, artifacts, a stage → artifact map; a trial ledger read by the recorder</t>
+          <t xml:space="preserve">`ticker`, the first of the basket standing for it; one record per asset</t>
         </is>
       </c>
     </row>
@@ -15774,17 +15764,27 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t xml:space="preserve">the basket one run covered — not in the record: the recorder knows no basket</t>
+          <t xml:space="preserve">the run index: every run with a record, newest first, each with its records — the one file the page reads to find a run</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t xml:space="preserve">the launcher's `TICKERS`, which the make target the recorder wraps carries into every stage command</t>
+          <t xml:space="preserve">`build_run_index()` in `record.py`, written again after every record from the store's listing, as `store/run_records/index.json`</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`generated_at_utc`; `runs[]`, each `run_id` and `records` — the record files, relative to the run's directory, in path order</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`&lt;n&gt; recorded run(s) · showing &lt;run_id&gt; · &lt;n&gt; records`</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ticker`, the first of the basket standing for it; one record per asset</t>
+          <t xml:space="preserve">a run list per asset; a listing by the page; a route that lists the store; an index written by a stage</t>
         </is>
       </c>
     </row>
@@ -15796,27 +15796,22 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run index: every run with a record, newest first, each with its records — the one file the page reads to find a run</t>
+          <t xml:space="preserve">the stage records of one run, in the order the stages started — each read by the page at the relative path the index lists</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_run_index()` in `record.py`, written again after every record from the store's listing, as `store/run_records/index.json`</t>
-        </is>
-      </c>
-      <c r="D391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`generated_at_utc`; `runs[]`, each `run_id` and `records` — the record files, relative to the run's directory, in path order</t>
+          <t xml:space="preserve">`runs[].records` of the index; `fetchRunRecord()` in `module_monitoring/run.js`, which sorts them by `started_at_utc`</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;n&gt; recorded run(s) · showing &lt;run_id&gt; · &lt;n&gt; records`</t>
+          <t xml:space="preserve">STAGES — stage, asset, start, time, exit, added, changed, removed, bytes written</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t xml:space="preserve">a run list per asset; a listing by the page; a route that lists the store; an index written by a stage</t>
+          <t xml:space="preserve">a record per asset of a basket stage; an envelope built by a server</t>
         </is>
       </c>
     </row>
@@ -15828,44 +15823,39 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stage records of one run, in the order the stages started — each read by the page at the relative path the index lists</t>
+          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, written whole after the stage's second listing so it never appears in its own difference; untracked</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t xml:space="preserve">`runs[].records` of the index; `fetchRunRecord()` in `module_monitoring/run.js`, which sorts them by `started_at_utc`</t>
-        </is>
-      </c>
-      <c r="E392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STAGES — stage, asset, start, time, exit, added, changed, removed, bytes written</t>
+          <t xml:space="preserve">`STORE_RUN_RECORDS_DIR`, `store/run_records/&lt;run_id&gt;/&lt;stage&gt;.json`; `write_json()` in `record.py`, beside its place, then moved onto it</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">a record per asset of a basket stage; an envelope built by a server</t>
+          <t xml:space="preserve">a `runtime/` folder under an asset; one run record per asset; a run record tracked</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run record</t>
+          <t xml:space="preserve">Documentation ownership</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, written whole after the stage's second listing so it never appears in its own difference; untracked</t>
+          <t xml:space="preserve">a generated document: one the sync renders from the sheet and a hand never edits, its first line the marker, its rules cited by `rule_id`</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STORE_RUN_RECORDS_DIR`, `store/run_records/&lt;run_id&gt;/&lt;stage&gt;.json`; `write_json()` in `record.py`, beside its place, then moved onto it</t>
+          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `runtime/` folder under an asset; one run record per asset; a run record tracked</t>
+          <t xml:space="preserve">a Skill edited in its file; a Skill cited by a numbered or titled section — a rule is cited by its `rule_id`; a hand-written `skill_*.md`</t>
         </is>
       </c>
     </row>
@@ -15877,17 +15867,17 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generated document: one the sync renders from the sheet and a hand never edits, its first line the marker, its rules cited by `rule_id`</t>
+          <t xml:space="preserve">a hand-written document: one a hand keeps and the sync never touches, no marker on its first line</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
+          <t xml:space="preserve">`AGENTS.md`, `CLAUDE.md`, `README.md`, `module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`, `module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`, every `README_sub_module_&lt;subject&gt;.md`, `module_skills/README.md`, `module_skills/sub_module_scalability_crawler/crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Skill edited in its file; a Skill cited by a numbered or titled section — a rule is cited by its `rule_id`; a hand-written `skill_*.md`</t>
+          <t xml:space="preserve">a rule kept only there; a second copy of a rule</t>
         </is>
       </c>
     </row>
@@ -15899,17 +15889,17 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hand-written document: one a hand keeps and the sync never touches, no marker on its first line</t>
+          <t xml:space="preserve">a normative document describing one module's own responsibility</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md`, `CLAUDE.md`, `README.md`, `module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`, `module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`, every `README_sub_module_&lt;subject&gt;.md`, `module_skills/README.md`, `module_skills/sub_module_scalability_crawler/crawlers_mission.md`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_&lt;domain&gt;`</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule kept only there; a second copy of a rule</t>
+          <t xml:space="preserve">a module's rule kept in `module_skills/`; a per-module `docs/` or `doc/` folder</t>
         </is>
       </c>
     </row>
@@ -15921,17 +15911,17 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t xml:space="preserve">a normative document describing one module's own responsibility</t>
+          <t xml:space="preserve">a normative document that crosses modules or governs the project — the canon's</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_&lt;domain&gt;`</t>
+          <t xml:space="preserve">`module_skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_skills`</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t xml:space="preserve">a module's rule kept in `module_skills/`; a per-module `docs/` or `doc/` folder</t>
+          <t xml:space="preserve">a cross-cutting rule filed under one module; an edit to a copy</t>
         </is>
       </c>
     </row>
@@ -15943,17 +15933,17 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t xml:space="preserve">a normative document that crosses modules or governs the project — the canon's</t>
+          <t xml:space="preserve">a sub-module skill: the normative document about one sub-module alone, kept beside its code as `skill_&lt;subject&gt;.md` — the serpentine search's and the crawler's; a terminal has none of its own, `module_skills/skill_tui_designer.md` holding what the terminals share</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_skills`</t>
+          <t xml:space="preserve">`sub_module_&lt;subject&gt;/skill_&lt;subject&gt;.md`, rendered from its owner's tab</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t xml:space="preserve">a cross-cutting rule filed under one module; an edit to a copy</t>
+          <t xml:space="preserve">a sub-module's own rule among `module_skills/skill_*.md` or in its module's `skills/`; a rule two sub-modules obey kept beside one of them; a `skill_&lt;module&gt;_terminal.md`; a `skills/` folder for one document</t>
         </is>
       </c>
     </row>
@@ -15965,17 +15955,17 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module skill: the normative document about one sub-module alone, kept beside its code as `skill_&lt;subject&gt;.md` — the serpentine search's and the crawler's; a terminal has none of its own, `module_skills/skill_tui_designer.md` holding what the terminals share</t>
+          <t xml:space="preserve">the directory holding one module's own documents: its Skills and its methodology</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_&lt;subject&gt;/skill_&lt;subject&gt;.md`, rendered from its owner's tab</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/`</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module's own rule among `module_skills/skill_*.md` or in its module's `skills/`; a rule two sub-modules obey kept beside one of them; a `skill_&lt;module&gt;_terminal.md`; a `skills/` folder for one document</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skill/`, `module_&lt;domain&gt;/documentation/`</t>
         </is>
       </c>
     </row>
@@ -15987,17 +15977,17 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t xml:space="preserve">the directory holding one module's own documents: its Skills and its methodology</t>
+          <t xml:space="preserve">the name register: one concept, one name, in code, artifacts and interface, and the copies no module may import across — rendered from the glossary table of the sheet with the register's own rules</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/`</t>
+          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skill/`, `module_&lt;domain&gt;/documentation/`</t>
+          <t xml:space="preserve">a register edited by hand; a second register; a name entering the tree in a commit that does not add its row</t>
         </is>
       </c>
     </row>
@@ -16009,17 +15999,17 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t xml:space="preserve">the name register: one concept, one name, in code, artifacts and interface, and the copies no module may import across — rendered from the glossary table of the sheet with the register's own rules</t>
+          <t xml:space="preserve">the sheet: the one source of every Skill and of the register — a tab per owner, each with its rule table; the glossary and the `rule_type_id` list; the skill register and the files matrix</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
+          <t xml:space="preserve">`module_skills/skills_sheet.xlsx`, `SKILLS_SHEET_PATH`; `load_sheet()` in `module_skills/sheet.py`; `RULE_HEADER`, `SKILL_REGISTER_HEADER`, `GLOSSARY_HEADER`, `RULE_TYPE_ID_HEADER`, `FILES_MATRIX_HEADER` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t xml:space="preserve">a register edited by hand; a second register; a name entering the tree in a commit that does not add its row</t>
+          <t xml:space="preserve">a Skill edited in its file; a second workbook; a CSV or JSON beside it; a sheet written by code</t>
         </is>
       </c>
     </row>
@@ -16031,17 +16021,17 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sheet: the one source of every Skill and of the register — a tab per owner, each with its rule table; the glossary and the `rule_type_id` list; the skill register and the files matrix</t>
+          <t xml:space="preserve">the skill register: a row per generated Skill — the tab that holds its rules, its `skill_path` and its summary</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skills_sheet.xlsx`, `SKILLS_SHEET_PATH`; `load_sheet()` in `module_skills/sheet.py`; `RULE_HEADER`, `SKILL_REGISTER_HEADER`, `GLOSSARY_HEADER`, `RULE_TYPE_ID_HEADER`, `FILES_MATRIX_HEADER` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`SKILL_REGISTER_HEADER` in `module_skills/config.py`; `Skill` in `module_skills/sheet.py`</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Skill edited in its file; a second workbook; a CSV or JSON beside it; a sheet written by code</t>
+          <t xml:space="preserve">document register, `DOCUMENT_REGISTER_HEADER`; a Skill without a register row; a summary in a rule row; an owner read off the files matrix</t>
         </is>
       </c>
     </row>
@@ -16053,17 +16043,17 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t xml:space="preserve">the skill register: a row per generated Skill — the tab that holds its rules, its `skill_path` and its summary</t>
+          <t xml:space="preserve">the sync: every Skill and the register rendered from the sheet beside what each governs, and every generated file the sheet no longer names deleted</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILL_REGISTER_HEADER` in `module_skills/config.py`; `Skill` in `module_skills/sheet.py`</t>
+          <t xml:space="preserve">`make skills-sync`; `main()`, `to_markdown()`, `build_documents()`, `write_text()`, `delete_stale()` in `module_skills/sync.py`; `GENERATED_MARKER`</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t xml:space="preserve">document register, `DOCUMENT_REGISTER_HEADER`; a Skill without a register row; a summary in a rule row; an owner read off the files matrix</t>
+          <t xml:space="preserve">distribute, generate, export; a stamp; a comparison of copies; a Markdown edited by hand; a sync that reads the sheet twice; a document without the marker deleted</t>
         </is>
       </c>
     </row>
@@ -16075,17 +16065,17 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sync: every Skill and the register rendered from the sheet beside what each governs, and every generated file the sheet no longer names deleted</t>
+          <t xml:space="preserve">the table of every configurable: every CONFIGURABLES record of the controlled `config.py` files, read as literals, on stdout</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make skills-sync`; `main()`, `to_markdown()`, `build_documents()`, `write_text()`, `delete_stale()` in `module_skills/sync.py`; `GENERATED_MARKER`</t>
+          <t xml:space="preserve">`make skills-configurables`; `main()`, `load_records()`, `to_cell()` in `module_skills/configurables.py`</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">distribute, generate, export; a stamp; a comparison of copies; a Markdown edited by hand; a sync that reads the sheet twice; a document without the marker deleted</t>
+          <t xml:space="preserve">a file the table is written into; an import of the module whose records it reads; a record the table carries and no `config.py` holds</t>
         </is>
       </c>
     </row>
@@ -16097,17 +16087,17 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t xml:space="preserve">the table of every configurable: every CONFIGURABLES record of the controlled `config.py` files, read as literals, on stdout</t>
+          <t xml:space="preserve">the contract: what every change answers to, read in full before a session's first edit</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make skills-configurables`; `main()`, `load_records()`, `to_cell()` in `module_skills/configurables.py`</t>
+          <t xml:space="preserve">`AGENTS.md` at the root</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">a file the table is written into; an import of the module whose records it reads; a record the table carries and no `config.py` holds</t>
+          <t xml:space="preserve">a second contract; a per-module `AGENTS.md`</t>
         </is>
       </c>
     </row>
@@ -16119,17 +16109,17 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t xml:space="preserve">the contract: what every change answers to, read in full before a session's first edit</t>
+          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md` at the root</t>
+          <t xml:space="preserve">`CLAUDE.md` at the root</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second contract; a per-module `AGENTS.md`</t>
+          <t xml:space="preserve">a rule written in it; a per-module `CLAUDE.md`; `CLAUDE.local.md` or `.claude/` inside the tree</t>
         </is>
       </c>
     </row>
@@ -16141,17 +16131,17 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
+          <t xml:space="preserve">the project's front door: what the project is, how to run it and where its Skills are</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t xml:space="preserve">`CLAUDE.md` at the root</t>
+          <t xml:space="preserve">`README.md` at the root</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule written in it; a per-module `CLAUDE.md`; `CLAUDE.local.md` or `.claude/` inside the tree</t>
+          <t xml:space="preserve">a rule restated in it; a front door that restates a Skill or a decision table</t>
         </is>
       </c>
     </row>
@@ -16163,17 +16153,17 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t xml:space="preserve">the project's front door: what the project is, how to run it and where its Skills are</t>
+          <t xml:space="preserve">one module's reader-facing front door, its orientation</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README.md` at the root</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule restated in it; a front door that restates a Skill or a decision table</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/README.md`; an orientation that restates a Skill or a decision table</t>
         </is>
       </c>
     </row>
@@ -16185,17 +16175,17 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t xml:space="preserve">one module's reader-facing front door, its orientation</t>
+          <t xml:space="preserve">a sub-module's orientation, beside its code</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/README.md`; an orientation that restates a Skill or a decision table</t>
+          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
         </is>
       </c>
     </row>
@@ -16207,17 +16197,17 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module's orientation, beside its code</t>
+          <t xml:space="preserve">the design rationale: the section of a module's orientation that says, per object, analogous pair or the module's documents, why here, why beside these, why this boundary and which mapping row it answers to — the fourth the test of the first three</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
+          <t xml:space="preserve">`## Design rationale` of each `README_module_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
+          <t xml:space="preserve">a decision table; a rule restated; an object with no row or two; ADR, decision record, decision log, `docs/`</t>
         </is>
       </c>
     </row>
@@ -16229,17 +16219,17 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t xml:space="preserve">the design rationale: the section of a module's orientation that says, per object, analogous pair or the module's documents, why here, why beside these, why this boundary and which mapping row it answers to — the fourth the test of the first three</t>
+          <t xml:space="preserve">a methodology document: reference material for a human — the equations, the derivations and the citations of one module</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t xml:space="preserve">`## Design rationale` of each `README_module_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t xml:space="preserve">a decision table; a rule restated; an object with no row or two; ADR, decision record, decision log, `docs/`</t>
+          <t xml:space="preserve">a row of the files matrix; a document the crawler sends; a rule stated only there</t>
         </is>
       </c>
     </row>
@@ -16251,39 +16241,44 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t xml:space="preserve">a methodology document: reference material for a human — the equations, the derivations and the citations of one module</t>
+          <t xml:space="preserve">the canon's index: every Skill by its path, and the canon's prose that is no rule, the mapping table among it</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`module_skills/README.md`</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t xml:space="preserve">a row of the files matrix; a document the crawler sends; a rule stated only there</t>
+          <t xml:space="preserve">a collection of copies; an index that restates a rule it links to</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentation ownership</t>
+          <t xml:space="preserve">Pre-AWS direction</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t xml:space="preserve">the canon's index: every Skill by its path, and the canon's prose that is no rule, the mapping table among it</t>
+          <t xml:space="preserve">the stance: a local academic architecture whose boundaries would survive a move onto standard cloud primitives, with no cloud used and none planned</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/README.md`</t>
+          <t xml:space="preserve">`module_skills/skill_pre_aws_solution.md` — `pre_aws` its stem, the one tracked name that carries the word; no identifier</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t xml:space="preserve">a collection of copies; an index that restates a rule it links to</t>
+          <t xml:space="preserve">cloud-ready, AWS-ready, cloud-native; a migration plan, a deployment guide; `pre-aws` or `PreAWS` in prose</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pre-AWS — before Amazon Web Services (AWS), the cloud the mapping reads forward to</t>
         </is>
       </c>
     </row>
@@ -16295,22 +16290,22 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stance: a local academic architecture whose boundaries would survive a move onto standard cloud primitives, with no cloud used and none planned</t>
+          <t xml:space="preserve">compute: a process that reads a store, writes a store and exits, owning no asset state between invocations</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_pre_aws_solution.md` — `pre_aws` its stem, the one tracked name that carries the word; no identifier</t>
+          <t xml:space="preserve">every stage's `main()`, `python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;`; the one-off container that runs it</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t xml:space="preserve">cloud-ready, AWS-ready, cloud-native; a migration plan, a deployment guide; `pre-aws` or `PreAWS` in prose</t>
+          <t xml:space="preserve">a container as the home of an asset's state; a resident as a requirement of a stage; an in-process cache between stages; `worker`, `processor`</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-AWS — before Amazon Web Services (AWS), the cloud the mapping reads forward to</t>
+          <t xml:space="preserve">a task — one run of the one task definition on the container instance every asset's runs share (Amazon ECS on Amazon EC2)</t>
         </is>
       </c>
     </row>
@@ -16322,22 +16317,22 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t xml:space="preserve">compute: a process that reads a store, writes a store and exits, owning no asset state between invocations</t>
+          <t xml:space="preserve">the rebuild condition: whether an asset's artifacts must be rebuilt from its canonical series, answered without launching anything; its freshness half is unwritten, its names reserved — `has_new_market_data()`, `requires_canonical_rebuild()`, `requires_feature_rebuild()`, `requires_model_rebuild()`</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t xml:space="preserve">every stage's `main()`, `python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;`; the one-off container that runs it</t>
+          <t xml:space="preserve">`is_artifact_set_complete()` in `module_ml/config.py`, its completeness half; the rerun table of `module_ml/skills/methodology_ml.md`, read by a human</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t xml:space="preserve">a container as the home of an asset's state; a resident as a requirement of a stage; an in-process cache between stages; `worker`, `processor`</t>
+          <t xml:space="preserve">a scheduler, a watcher, an event bus; a function that both detects new data and trains; `should_run()`, `check_update()`, `trigger()`</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">a task — one run of the one task definition on the container instance every asset's runs share (Amazon ECS on Amazon EC2)</t>
+          <t xml:space="preserve">a choice state between two states of the machine (AWS Step Functions)</t>
         </is>
       </c>
     </row>
@@ -16349,22 +16344,17 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t xml:space="preserve">the rebuild condition: whether an asset's artifacts must be rebuilt from its canonical series, answered without launching anything; its freshness half is unwritten, its names reserved — `has_new_market_data()`, `requires_canonical_rebuild()`, `requires_feature_rebuild()`, `requires_model_rebuild()`</t>
+          <t xml:space="preserve">the mapping table: what this repository has, the responsibility, the same responsibility elsewhere and the move, row by row — the one table that sets a cloud proper noun beside a local object; its third column is the elsewhere column</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t xml:space="preserve">`is_artifact_set_complete()` in `module_ml/config.py`, its completeness half; the rerun table of `module_ml/skills/methodology_ml.md`, read by a human</t>
+          <t xml:space="preserve">`module_skills/README.md`, its hand-written home</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t xml:space="preserve">a scheduler, a watcher, an event bus; a function that both detects new data and trains; `should_run()`, `check_update()`, `trigger()`</t>
-        </is>
-      </c>
-      <c r="I415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a choice state between two states of the machine (AWS Step Functions)</t>
+          <t xml:space="preserve">an adapter, a cloud configuration file; a cloud proper noun in an identifier, a key, a path, a make target, a compose service or an environment variable; a path of the elsewhere column read as a proposal for a local directory</t>
         </is>
       </c>
     </row>
@@ -16376,17 +16366,17 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mapping table: what this repository has, the responsibility, the same responsibility elsewhere and the move, row by row — the one table that sets a cloud proper noun beside a local object; its third column is the elsewhere column</t>
-        </is>
-      </c>
-      <c r="C416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`module_skills/README.md`, its hand-written home</t>
+          <t xml:space="preserve">a seat: the standard primitive a local object would sit on elsewhere, named in the mapping table's words — spoken in the stance's skill and in the mapping table, and in no other Skill</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t xml:space="preserve">an adapter, a cloud configuration file; a cloud proper noun in an identifier, a key, a path, a make target, a compose service or an environment variable; a path of the elsewhere column read as a proposal for a local directory</t>
+          <t xml:space="preserve">a seat paragraph in any other Skill; two seats for one object; a seat in an identifier, a key or a path; `target`, `cloud note`, `mapping section`</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the image registry (Amazon ECR), the container service (Amazon ECS), the container instance (Amazon EC2), the block volume (Amazon EBS), object storage (Amazon S3), the state machine (AWS Step Functions), the schedule (Amazon EventBridge Scheduler)</t>
         </is>
       </c>
     </row>
@@ -16398,17 +16388,17 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t xml:space="preserve">a seat: the standard primitive a local object would sit on elsewhere, named in the mapping table's words — spoken in the stance's skill and in the mapping table, and in no other Skill</t>
+          <t xml:space="preserve">the resource role: the name a cloud resource would carry, `&lt;project&gt;-&lt;environment&gt;-&lt;resource-role&gt;` — the role a seat's name or the task a row of the mapping table names, lower case with `-` between its words, the project `liora`</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`name: liora` and `liora-1m-pipeline` in `docker-compose.yml` — the names of that shape the tree holds, with no environment token</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t xml:space="preserve">a seat paragraph in any other Skill; two seats for one object; a seat in an identifier, a key or a path; `target`, `cloud note`, `mapping section`</t>
-        </is>
-      </c>
-      <c r="I417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the image registry (Amazon ECR), the container service (Amazon ECS), the container instance (Amazon EC2), the block volume (Amazon EBS), object storage (Amazon S3), the state machine (AWS Step Functions), the schedule (Amazon EventBridge Scheduler)</t>
+          <t xml:space="preserve">a second list of roles; a role no seat or row names; `dev` or `prod` in a tracked name; a ticker in a resource name; an environment token on the image</t>
         </is>
       </c>
     </row>
@@ -16420,17 +16410,17 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t xml:space="preserve">the resource role: the name a cloud resource would carry, `&lt;project&gt;-&lt;environment&gt;-&lt;resource-role&gt;` — the role a seat's name or the task a row of the mapping table names, lower case with `-` between its words, the project `liora`</t>
-        </is>
-      </c>
-      <c r="C418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`name: liora` and `liora-1m-pipeline` in `docker-compose.yml` — the names of that shape the tree holds, with no environment token</t>
+          <t xml:space="preserve">a state name: the one-line name a stage would carry as a state of the machine, one per stage, and PublishStores, the copy after a run, which no stage answers to; *Publish* in a state name means write the object where its readers read it</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second list of roles; a role no seat or row names; `dev` or `prod` in a tracked name; a ticker in a resource name; an environment token on the image</t>
+          <t xml:space="preserve">a state registered one by one; a state name with *and* in it; *publish* as *make public*</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a state of AWS Step Functions</t>
         </is>
       </c>
     </row>
@@ -16442,17 +16432,17 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state name: the one-line name a stage would carry as a state of the machine, one per stage, and PublishStores, the copy after a run, which no stage answers to; *Publish* in a state name means write the object where its readers read it</t>
+          <t xml:space="preserve">an instance: one Linux virtual machine elsewhere, the host containers run on — the task host every asset's runs share, with the store volume beside it, and the strategy host</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state registered one by one; a state name with *and* in it; *publish* as *make public*</t>
+          <t xml:space="preserve">`instance` or `host` for a container; a host per asset; node</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state of AWS Step Functions</t>
+          <t xml:space="preserve">a container instance (Amazon EC2)</t>
         </is>
       </c>
     </row>
@@ -16464,17 +16454,22 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t xml:space="preserve">an instance: one Linux virtual machine elsewhere, the host containers run on — the task host every asset's runs share, with the store volume beside it, and the strategy host</t>
+          <t xml:space="preserve">the store volume: the task host's durable disk — the five stores at `/store/&lt;content&gt;`, each at the path its `STORE_*_DIR` names; the home of state, never the copy</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the `./store/&lt;content&gt;` mounts of `docker-compose.yml`, read forward as `&lt;volume&gt;/&lt;content&gt;:/store/&lt;content&gt;`</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t xml:space="preserve">`instance` or `host` for a container; a host per asset; node</t>
+          <t xml:space="preserve">asset volume; a volume per asset; the volume as the copy; `data_volume`; a shared network filesystem (Amazon EFS)</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t xml:space="preserve">a container instance (Amazon EC2)</t>
+          <t xml:space="preserve">a block volume (Amazon EBS)</t>
         </is>
       </c>
     </row>
@@ -16486,22 +16481,17 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store volume: the task host's durable disk — the five stores at `/store/&lt;content&gt;`, each at the path its `STORE_*_DIR` names; the home of state, never the copy</t>
-        </is>
-      </c>
-      <c r="C421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the `./store/&lt;content&gt;` mounts of `docker-compose.yml`, read forward as `&lt;volume&gt;/&lt;content&gt;:/store/&lt;content&gt;`</t>
+          <t xml:space="preserve">the copy: the whole files a state after the last stage of a run would copy from the store volume to object storage — never a stage's own write, never mid-run; absent here, described</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset volume; a volume per asset; the volume as the copy; `data_volume`; a shared network filesystem (Amazon EFS)</t>
+          <t xml:space="preserve">a stage writing to object storage; a stage reading the copy; `s3://` in a path constant; an adapter for the copy</t>
         </is>
       </c>
       <c r="I421" t="inlineStr">
         <is>
-          <t xml:space="preserve">a block volume (Amazon EBS)</t>
+          <t xml:space="preserve">object storage (Amazon S3), written by PublishStores</t>
         </is>
       </c>
     </row>
@@ -16513,17 +16503,12 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t xml:space="preserve">the copy: the whole files a state after the last stage of a run would copy from the store volume to object storage — never a stage's own write, never mid-run; absent here, described</t>
+          <t xml:space="preserve">the ladder: the three phases in which the runtime elsewhere would become true, each named for what it changes — *the lift*, *the idiom*, *the image carries the code*; all elsewhere, built nowhere here</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage writing to object storage; a stage reading the copy; `s3://` in a path constant; an adapter for the copy</t>
-        </is>
-      </c>
-      <c r="I422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">object storage (Amazon S3), written by PublishStores</t>
+          <t xml:space="preserve">a letter or a number for a phase; a phase as a branch or an environment; `dev` / `prod`; a phase built here; rung</t>
         </is>
       </c>
     </row>
@@ -16535,12 +16520,17 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t xml:space="preserve">the ladder: the three phases in which the runtime elsewhere would become true, each named for what it changes — *the lift*, *the idiom*, *the image carries the code*; all elsewhere, built nowhere here</t>
+          <t xml:space="preserve">the promotion threshold: a second concurrent writer of one partition, or a reader that needs one transaction across families — the one condition under which a managed database replaces the table families</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t xml:space="preserve">a letter or a number for a phase; a phase as a branch or an environment; `dev` / `prod`; a phase built here; rung</t>
+          <t xml:space="preserve">a database process for one writer; a threshold in rows or bytes</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a managed database (Amazon RDS)</t>
         </is>
       </c>
     </row>
@@ -16552,17 +16542,22 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion threshold: a second concurrent writer of one partition, or a reader that needs one transaction across families — the one condition under which a managed database replaces the table families</t>
+          <t xml:space="preserve">the active version: the one version of an asset's artifacts a reader reads, chosen where the reader is; the version is the execution name</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`run_id`</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t xml:space="preserve">a database process for one writer; a threshold in rows or bytes</t>
+          <t xml:space="preserve">latest, current, prod; a mark inside a file; a version inside an artifact</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">a managed database (Amazon RDS)</t>
+          <t xml:space="preserve">the version prefix `assets_artifacts/&lt;run_id&gt;/` of the copy (Amazon S3)</t>
         </is>
       </c>
     </row>
@@ -16574,22 +16569,22 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t xml:space="preserve">the active version: the one version of an asset's artifacts a reader reads, chosen where the reader is; the version is the execution name</t>
+          <t xml:space="preserve">the tunnel: how a reader reaches the page on a host that is not theirs — a local forward onto the loopback port `make on` printed there</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run_id`</t>
+          <t xml:space="preserve">`ssh -N -L` of `README.md` § Quickstart</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t xml:space="preserve">latest, current, prod; a mark inside a file; a version inside an artifact</t>
+          <t xml:space="preserve">a public port; a load balancer</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t xml:space="preserve">the version prefix `assets_artifacts/&lt;run_id&gt;/` of the copy (Amazon S3)</t>
+          <t xml:space="preserve">a port-forward, the elsewhere column's word</t>
         </is>
       </c>
     </row>
@@ -16601,22 +16596,12 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t xml:space="preserve">the tunnel: how a reader reaches the page on a host that is not theirs — a local forward onto the loopback port `make on` printed there</t>
-        </is>
-      </c>
-      <c r="C426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`ssh -N -L` of `README.md` § Quickstart</t>
+          <t xml:space="preserve">read forward: a local object read as the same responsibility elsewhere — the mapping table's third column — with nothing moved</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t xml:space="preserve">a public port; a load balancer</t>
-        </is>
-      </c>
-      <c r="I426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a port-forward, the elsewhere column's word</t>
+          <t xml:space="preserve">migrated, ported, deployed, in production</t>
         </is>
       </c>
     </row>
@@ -16628,12 +16613,12 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t xml:space="preserve">read forward: a local object read as the same responsibility elsewhere — the mapping table's third column — with nothing moved</t>
+          <t xml:space="preserve">the move: what a local thing's seat elsewhere costs it — a rename, one edit, or absent here, described; the mapping table's fourth column</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t xml:space="preserve">migrated, ported, deployed, in production</t>
+          <t xml:space="preserve">migration, deployment, a plan, a roadmap</t>
         </is>
       </c>
     </row>
@@ -16645,34 +16630,44 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t xml:space="preserve">the move: what a local thing's seat elsewhere costs it — a rename, one edit, or absent here, described; the mapping table's fourth column</t>
+          <t xml:space="preserve">an absent object: a primitive, a state of the machine or a Skill that nothing local answers to and a document describes — a sentence ending, or a verdict reading, *absent here — described*</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`AGENTS.md` § Skills absent here, described, for the Skills</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t xml:space="preserve">migration, deployment, a plan, a roadmap</t>
+          <t xml:space="preserve">planned, a debt marker, future, ghost, placeholder, missing</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-AWS direction</t>
+          <t xml:space="preserve">The page</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t xml:space="preserve">an absent object: a primitive, a state of the machine or a Skill that nothing local answers to and a document describes — a sentence ending, or a verdict reading, *absent here — described*</t>
+          <t xml:space="preserve">the page: one static page of plain HTML, CSS and JavaScript that reads every datum by a relative path and writes nothing</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md` § Skills absent here, described, for the Skills</t>
+          <t xml:space="preserve">`module_monitoring/index.html`, `style.css` and its scripts `page.js`, `data.js`, `asset.js`, `features.js`, `ml.js`, `run.js`, `scalability.js`</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1m crypto research pipeline — status</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t xml:space="preserve">planned, a debt marker, future, ghost, placeholder, missing</t>
+          <t xml:space="preserve">a framework or a build step; a second page beside it; a datum computed by the server; an absolute path</t>
         </is>
       </c>
     </row>
@@ -16684,22 +16679,17 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page: one static page of plain HTML, CSS and JavaScript that reads every datum by a relative path and writes nothing</t>
+          <t xml:space="preserve">the page's reads: where the page takes its data from, by relative path</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/index.html`, `style.css` and its scripts `page.js`, `data.js`, `asset.js`, `features.js`, `ml.js`, `run.js`, `scalability.js`</t>
-        </is>
-      </c>
-      <c r="E430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1m crypto research pipeline — status</t>
+          <t xml:space="preserve">`status/data_status.json`, `status/features_status.json`, `status/ml_status.json`, `status/skills_status.json`; `run_records/index.json`, then each record of a run at `run_records/&lt;run_id&gt;/` and the path the index lists</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t xml:space="preserve">a framework or a build step; a second page beside it; a datum computed by the server; an absolute path</t>
+          <t xml:space="preserve">an absolute path; a route per snapshot; a directory listing; a store the page reads beside these two</t>
         </is>
       </c>
     </row>
@@ -16711,17 +16701,22 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page's reads: where the page takes its data from, by relative path</t>
+          <t xml:space="preserve">the three prefixes: what the dashboard's server answers — the page's own files at `/`, the status store under `/status/`, the run-records store under `/run_records/`; every other path 404, and no directory listed</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t xml:space="preserve">`status/data_status.json`, `status/features_status.json`, `status/ml_status.json`, `status/skills_status.json`; `run_records/index.json`, then each record of a run at `run_records/&lt;run_id&gt;/` and the path the index lists</t>
+          <t xml:space="preserve">`module_monitoring/serve.py` — `DashboardHandler`, `translate_path()`, `main()`; `STORE_DIR_BY_ROUTE_PREFIX` in `module_monitoring/config.py`, `/status/` onto `STORE_STATUS_DIR` and `/run_records/` onto `STORE_RUN_RECORDS_DIR`; `MODULE_MONITORING_DIR`, `PAGE_FILE_SUFFIXES`, `PAGE_INDEX_FILE_NAME` for the page's own files</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t xml:space="preserve">an absolute path; a route per snapshot; a directory listing; a store the page reads beside these two</t>
+          <t xml:space="preserve">a route per snapshot; a directory listed; a path outside the three prefixes answered; a server that computes, writes or proxies; `dashboard.py`, `proxy.py`, `server.py` beside `serve.py`</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`http.server`</t>
         </is>
       </c>
     </row>
@@ -16733,22 +16728,17 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three prefixes: what the dashboard's server answers — the page's own files at `/`, the status store under `/status/`, the run-records store under `/run_records/`; every other path 404, and no directory listed</t>
+          <t xml:space="preserve">the toolkit the page loads before its own sections</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/serve.py` — `DashboardHandler`, `translate_path()`, `main()`; `STORE_DIR_BY_ROUTE_PREFIX` in `module_monitoring/config.py`, `/status/` onto `STORE_STATUS_DIR` and `/run_records/` onto `STORE_RUN_RECORDS_DIR`; `MODULE_MONITORING_DIR`, `PAGE_FILE_SUFFIXES`, `PAGE_INDEX_FILE_NAME` for the page's own files</t>
+          <t xml:space="preserve">`page.js`</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t xml:space="preserve">a route per snapshot; a directory listed; a path outside the three prefixes answered; a server that computes, writes or proxies; `dashboard.py`, `proxy.py`, `server.py` beside `serve.py`</t>
-        </is>
-      </c>
-      <c r="I432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`http.server`</t>
+          <t xml:space="preserve">`utils.js`, `common.js`, `shared.js`, `lib.js`; a page-specific element written from it; a second page beside the status page</t>
         </is>
       </c>
     </row>
@@ -16760,17 +16750,17 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t xml:space="preserve">the toolkit the page loads before its own sections</t>
+          <t xml:space="preserve">the one selector component of the page — the top tabs, the ML Assets views, the asset rows — each group wired by its `data-key`</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t xml:space="preserve">`page.js`</t>
+          <t xml:space="preserve">`.pills`, `.pill`, `.pill--active`, `initPills()`, `PILL_HOOKS` in `page.js`; `data-pills` on a group, `data-panel` on its panels</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t xml:space="preserve">`utils.js`, `common.js`, `shared.js`, `lib.js`; a page-specific element written from it; a second page beside the status page</t>
+          <t xml:space="preserve">a second selector component</t>
         </is>
       </c>
     </row>
@@ -16782,44 +16772,44 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one selector component of the page — the top tabs, the ML Assets views, the asset rows — each group wired by its `data-key`</t>
+          <t xml:space="preserve">the page's navigation: the seven tabs, the five views of the ML Assets tab, and one row per asset</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.pills`, `.pill`, `.pill--active`, `initPills()`, `PILL_HOOKS` in `page.js`; `data-pills` on a group, `data-panel` on its panels</t>
+          <t xml:space="preserve">the groups of `data-pills` in `module_monitoring/index.html` — `tab`: `pipeline`, `quality`, `features`, `ml`, `asset`, `scalability`, `lifecycle`; `mlview`: `labels`, `classification`, `strategy`, `search`, `feature-set`; `asset`, filled from the snapshot</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pipeline; Data Quality; Features; ML Research; ML Assets; Scalability; Lifecycle — Labels &amp; data; Classification; Strategy; HPO; Feature set</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second selector component</t>
+          <t xml:space="preserve">a menu, a sidebar or a second navigation; a tab named for a tool</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t xml:space="preserve">The page</t>
+          <t xml:space="preserve">Scalability crawler</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page's navigation: the seven tabs, the five views of the ML Assets tab, and one row per asset</t>
+          <t xml:space="preserve">the crawler: the canon's sub-module that reads each controlled file against the Skills marked for it with the one active vendor, and writes a report per file and its snapshot; it asks nothing, goes on past a failed file and gates nothing</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t xml:space="preserve">the groups of `data-pills` in `module_monitoring/index.html` — `tab`: `pipeline`, `quality`, `features`, `ml`, `asset`, `scalability`, `lifecycle`; `mlview`: `labels`, `classification`, `strategy`, `search`, `feature-set`; `asset`, filled from the snapshot</t>
-        </is>
-      </c>
-      <c r="E435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pipeline; Data Quality; Features; ML Research; ML Assets; Scalability; Lifecycle — Labels &amp; data; Classification; Strategy; HPO; Feature set</t>
+          <t xml:space="preserve">`sub_module_scalability_crawler`; `make skills-crawl`, after `make skills-sync`; `main()` in `crawl.py`</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t xml:space="preserve">a menu, a sidebar or a second navigation; a tab named for a tool</t>
+          <t xml:space="preserve">a linter, a check, a gate, a CI step; a web crawler, walking sites or services to gather what they hold; conformance, review — names that tell a reader nothing; a TUI of its own, `make skills-terminal` being the canon's terminal</t>
         </is>
       </c>
     </row>
@@ -16831,17 +16821,22 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t xml:space="preserve">the crawler: the canon's sub-module that reads each controlled file against the Skills marked for it with the one active vendor, and writes a report per file and its snapshot; it asks nothing, goes on past a failed file and gates nothing</t>
+          <t xml:space="preserve">the files matrix: a row per path — a file or a glob — a column per Skill headed by its stem, an `X` where that Skill is sent with the file; the crawler's whole contract</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_scalability_crawler`; `make skills-crawl`, after `make skills-sync`; `main()` in `crawl.py`</t>
+          <t xml:space="preserve">the table of the sheet headed by `FILES_MATRIX_HEADER` in `module_skills/config.py`; `Mark` in `module_skills/sheet.py`</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">path; the Skill's stem; `X`</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t xml:space="preserve">a linter, a check, a gate, a CI step; a web crawler, walking sites or services to gather what they hold; conformance, review — names that tell a reader nothing; a TUI of its own, `make skills-terminal` being the canon's terminal</t>
+          <t xml:space="preserve">a column per rule; a mark a crawl writes; a mark derived from `scope`; a generated file, a report or the snapshot as a target; a second row for one path; a precedence between rows; a Markdown table kept beside the crawler</t>
         </is>
       </c>
     </row>
@@ -16853,22 +16848,22 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t xml:space="preserve">the files matrix: a row per path — a file or a glob — a column per Skill headed by its stem, an `X` where that Skill is sent with the file; the crawler's whole contract</t>
+          <t xml:space="preserve">a mark: `X` under a Skill's column in a row of the files matrix, sending that Skill with every file the row reaches; two rows that reach one file join their marks</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t xml:space="preserve">the table of the sheet headed by `FILES_MATRIX_HEADER` in `module_skills/config.py`; `Mark` in `module_skills/sheet.py`</t>
+          <t xml:space="preserve">`SKILL_MARK` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">path; the Skill's stem; `X`</t>
+          <t xml:space="preserve">`X`; marked; unmarked</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column per rule; a mark a crawl writes; a mark derived from `scope`; a generated file, a report or the snapshot as a target; a second row for one path; a precedence between rows; a Markdown table kept beside the crawler</t>
+          <t xml:space="preserve">assign, tag, tick, check, enable; `x`, `✓` or `yes` in a cell; a mark a crawl writes; a mark derived from `scope`; a row that marks no Skill</t>
         </is>
       </c>
     </row>
@@ -16880,22 +16875,22 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t xml:space="preserve">a mark: `X` under a Skill's column in a row of the files matrix, sending that Skill with every file the row reaches; two rows that reach one file join their marks</t>
+          <t xml:space="preserve">a controlled file: a file a row of the files matrix reaches, read against the Skills marked for it; its key is its path from the root of the tree</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILL_MARK` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`ControlledFile`, `build_controlled_files()` in `crawl.py`</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t xml:space="preserve">`X`; marked; unmarked</t>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t xml:space="preserve">assign, tag, tick, check, enable; `x`, `✓` or `yes` in a cell; a mark a crawl writes; a mark derived from `scope`; a row that marks no Skill</t>
+          <t xml:space="preserve">listed file; a file the crawler finds by itself; a file read from the working directory; a rendered Skill or the snapshot as a controlled file</t>
         </is>
       </c>
     </row>
@@ -16907,22 +16902,17 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t xml:space="preserve">a controlled file: a file a row of the files matrix reaches, read against the Skills marked for it; its key is its path from the root of the tree</t>
+          <t xml:space="preserve">the context: the documents sent with a file — the Skills its row of the files matrix marks, each whole as `make skills-sync` rendered it</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ControlledFile`, `build_controlled_files()` in `crawl.py`</t>
-        </is>
-      </c>
-      <c r="E439" t="inlineStr">
-        <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">`load_skill_texts()`, `build_message()` in `crawl.py`</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t xml:space="preserve">listed file; a file the crawler finds by itself; a file read from the working directory; a rendered Skill or the snapshot as a controlled file</t>
+          <t xml:space="preserve">a rule filtered out by its `scope` before it is sent; a Skill not marked; the contract; an orientation; a methodology; a list of rules kept per module</t>
         </is>
       </c>
     </row>
@@ -16934,17 +16924,17 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t xml:space="preserve">the context: the documents sent with a file — the Skills its row of the files matrix marks, each whole as `make skills-sync` rendered it</t>
+          <t xml:space="preserve">a file's message: the Skills marked for it, then the file with every line after its number, then the mission</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_skill_texts()`, `build_message()` in `crawl.py`</t>
+          <t xml:space="preserve">`build_message()` in `crawl.py`; `crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule filtered out by its `scope` before it is sent; a Skill not marked; the contract; an orientation; a methodology; a list of rules kept per module</t>
+          <t xml:space="preserve">a list of unmarked Skills; an orientation; a commit; a measure of the message; a line number the agent has to count</t>
         </is>
       </c>
     </row>
@@ -16956,17 +16946,17 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t xml:space="preserve">a file's message: the Skills marked for it, then the file with every line after its number, then the mission</t>
+          <t xml:space="preserve">the mission: what the agent reports of one file, and how — kept by hand</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_message()` in `crawl.py`; `crawlers_mission.md`</t>
+          <t xml:space="preserve">`crawlers_mission.md`, `CRAWLERS_MISSION_MD_PATH`</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t xml:space="preserve">a list of unmarked Skills; an orientation; a commit; a measure of the message; a line number the agent has to count</t>
+          <t xml:space="preserve">a rule restated in it; a work order or a plan</t>
         </is>
       </c>
     </row>
@@ -16978,17 +16968,17 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mission: what the agent reports of one file, and how — kept by hand</t>
+          <t xml:space="preserve">the sub-module's folder and the root of the tree: where the crawler's own files are read, and where a controlled file and a Skill lie and the vendor runs</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t xml:space="preserve">`crawlers_mission.md`, `CRAWLERS_MISSION_MD_PATH`</t>
+          <t xml:space="preserve">`SUB_MODULE_DIR` in the crawler's `config.py`; `TREE_ROOT_DIR` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule restated in it; a work order or a plan</t>
+          <t xml:space="preserve">a host path; a controlled file read from the working directory</t>
         </is>
       </c>
     </row>
@@ -17000,17 +16990,22 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sub-module's folder and the root of the tree: where the crawler's own files are read, and where a controlled file and a Skill lie and the vendor runs</t>
+          <t xml:space="preserve">a vendor: an agent's command line the crawl sends each controlled file to — one table of `vendors_for_crawling.toml`, exactly one `active`, its `argv` the whole command line, run without a shell, the message on its stdin and the answer its stdout</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SUB_MODULE_DIR` in the crawler's `config.py`; `TREE_ROOT_DIR` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`vendors_for_crawling.toml` with `active`, `argv`; `VENDORS_FOR_CRAWLING_TOML_PATH`, `load_vendor()`, `AGENT_TIMEOUT_SECONDS`</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vendor</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t xml:space="preserve">a host path; a controlled file read from the working directory</t>
+          <t xml:space="preserve">an API key; a vendor named in the code; a form for its model, effort or permissions; a vendor chosen on a screen; two active vendors; every vendor run in turn</t>
         </is>
       </c>
     </row>
@@ -17022,22 +17017,27 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t xml:space="preserve">a vendor: an agent's command line the crawl sends each controlled file to — one table of `vendors_for_crawling.toml`, exactly one `active`, its `argv` the whole command line, run without a shell, the message on its stdin and the answer its stdout</t>
+          <t xml:space="preserve">a report: the one current file per controlled file — the file's key, the vendor and the time, then the answer as it came; reset by every crawl, never tracked</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t xml:space="preserve">`vendors_for_crawling.toml` with `active`, `argv`; `VENDORS_FOR_CRAWLING_TOML_PATH`, `load_vendor()`, `AGENT_TIMEOUT_SECONDS`</t>
+          <t xml:space="preserve">`REPORTS_DIR`, `report_path()` in the crawler's `config.py` — `store/status/reports_after_crawled_files/&lt;path&gt;.report.md`; `write_text()` in `module_skills/sync.py`</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`report`</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t xml:space="preserve">vendor</t>
+          <t xml:space="preserve">report</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t xml:space="preserve">an API key; a vendor named in the code; a form for its model, effort or permissions; a vendor chosen on a screen; two active vendors; every vendor run in turn</t>
+          <t xml:space="preserve">a history of entries; an append; a report in the sub-module's folder; a commit in its first line; a report tracked</t>
         </is>
       </c>
     </row>
@@ -17049,27 +17049,17 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t xml:space="preserve">a report: the one current file per controlled file — the file's key, the vendor and the time, then the answer as it came; reset by every crawl, never tracked</t>
+          <t xml:space="preserve">a finding: one line of a report, `rule_id | file:line | problem | correction`; `OK` the answer of a file that departs from nothing</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t xml:space="preserve">`REPORTS_DIR`, `report_path()` in the crawler's `config.py` — `store/status/reports_after_crawled_files/&lt;path&gt;.report.md`; `write_text()` in `module_skills/sync.py`</t>
-        </is>
-      </c>
-      <c r="D445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`report`</t>
-        </is>
-      </c>
-      <c r="E445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">`crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t xml:space="preserve">a history of entries; an append; a report in the sub-module's folder; a commit in its first line; a report tracked</t>
+          <t xml:space="preserve">a finding without a `rule_id`; a rule that was not sent; a table; `conformant` as a line</t>
         </is>
       </c>
     </row>
@@ -17081,17 +17071,27 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t xml:space="preserve">a finding: one line of a report, `rule_id | file:line | problem | correction`; `OK` the answer of a file that departs from nothing</t>
+          <t xml:space="preserve">a controlled file's state: where its crawl stands — `pending` before, `running` while the vendor works, `done` once its report is written, `failed` otherwise, `interrupted` where Ctrl-C ended it</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t xml:space="preserve">`crawlers_mission.md`</t>
+          <t xml:space="preserve">`row()` in `status.py`; `main()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`state`</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pending; running; done; failed; interrupted</t>
         </is>
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t xml:space="preserve">a finding without a `rule_id`; a rule that was not sent; a table; `conformant` as a line</t>
+          <t xml:space="preserve">`done` read as conformant — it says the report was written; a change of state left out of the snapshot</t>
         </is>
       </c>
     </row>
@@ -17103,27 +17103,22 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t xml:space="preserve">a controlled file's state: where its crawl stands — `pending` before, `running` while the vendor works, `done` once its report is written, `failed` otherwise, `interrupted` where Ctrl-C ended it</t>
+          <t xml:space="preserve">the crawl's progress: one line per controlled file after its result, then one closing line; the reason a file failed one line on stderr</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t xml:space="preserve">`row()` in `status.py`; `main()` in `crawl.py`</t>
-        </is>
-      </c>
-      <c r="D447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`state`</t>
+          <t xml:space="preserve">`main()` in `crawl.py`</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t xml:space="preserve">pending; running; done; failed; interrupted</t>
+          <t xml:space="preserve">`&lt;current&gt;/&lt;total&gt; | &lt;controlled file&gt; | &lt;vendor&gt; | &lt;state&gt;`; `&lt;processed&gt;/&lt;total&gt; | crawl | &lt;vendor&gt; | done`, `failed` or `interrupted`</t>
         </is>
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t xml:space="preserve">`done` read as conformant — it says the report was written; a change of state left out of the snapshot</t>
+          <t xml:space="preserve">a spinner, a progress bar, a percentage; an answer summarised on the screen — the report holds it; a results table</t>
         </is>
       </c>
     </row>
@@ -17135,22 +17130,17 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t xml:space="preserve">the crawl's progress: one line per controlled file after its result, then one closing line; the reason a file failed one line on stderr</t>
+          <t xml:space="preserve">the refusals and the exits: a state the crawler cannot read ends it in one named line before anything is reset; a file the vendor fails is `failed` and the crawl goes on — 0 every file done, 1 a refusal or a failed file, 130 Ctrl-C</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t xml:space="preserve">`main()` in `crawl.py`</t>
-        </is>
-      </c>
-      <c r="E448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`&lt;current&gt;/&lt;total&gt; | &lt;controlled file&gt; | &lt;vendor&gt; | &lt;state&gt;`; `&lt;processed&gt;/&lt;total&gt; | crawl | &lt;vendor&gt; | done`, `failed` or `interrupted`</t>
+          <t xml:space="preserve">`SystemExit` in `module_skills/sheet.py`, `module_skills/sync.py` and the crawler's `crawl.py`</t>
         </is>
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t xml:space="preserve">a spinner, a progress bar, a percentage; an answer summarised on the screen — the report holds it; a results table</t>
+          <t xml:space="preserve">a traceback for an expected failure; exit 0 after a failure; a crawl that stops at the first failed file</t>
         </is>
       </c>
     </row>
@@ -17162,17 +17152,27 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t xml:space="preserve">the refusals and the exits: a state the crawler cannot read ends it in one named line before anything is reset; a file the vendor fails is `failed` and the crawl goes on — 0 every file done, 1 a refusal or a failed file, 130 Ctrl-C</t>
+          <t xml:space="preserve">the snapshot: `skills_status.json`, the current state of every controlled file, sorted by path and rewritten whole at every change; tracked in its neutral state, every controlled file `pending` with no report</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SystemExit` in `module_skills/sheet.py`, `module_skills/sync.py` and the crawler's `crawl.py`</t>
+          <t xml:space="preserve">`SKILLS_STATUS_JSON_PATH` in the crawler's `config.py`; `row()`, `write_skills_status()` in `status.py`, through `write_text()` of `module_skills/sync.py`</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`files`, each `path`, `state`, `vendor`, `finished_at_utc`, `report`</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">file; state; vendor; finished_at_utc; report</t>
         </is>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t xml:space="preserve">a traceback for an expected failure; exit 0 after a failure; a crawl that stops at the first failed file</t>
+          <t xml:space="preserve">a count of crawls; an age; a clock but `finished_at_utc`; a snapshot that reads itself back; a partial file</t>
         </is>
       </c>
     </row>
@@ -17184,136 +17184,104 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t xml:space="preserve">the snapshot: `skills_status.json`, the current state of every controlled file, sorted by path and rewritten whole at every change; tracked in its neutral state, every controlled file `pending` with no report</t>
+          <t xml:space="preserve">the page's view of the reports</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILLS_STATUS_JSON_PATH` in the crawler's `config.py`; `row()`, `write_skills_status()` in `status.py`, through `write_text()` of `module_skills/sync.py`</t>
-        </is>
-      </c>
-      <c r="D450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`files`, each `path`, `state`, `vendor`, `finished_at_utc`, `report`</t>
+          <t xml:space="preserve">`scalability.js` — `SKILLS_STATUS`, `renderCrawlState()`</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t xml:space="preserve">file; state; vendor; finished_at_utc; report</t>
+          <t xml:space="preserve">Scalability — CRAWL STATE</t>
         </is>
       </c>
       <c r="F450" t="inlineStr">
         <is>
-          <t xml:space="preserve">a count of crawls; an age; a clock but `finished_at_utc`; a snapshot that reads itself back; a partial file</t>
-        </is>
-      </c>
-    </row>
-    <row r="451">
-      <c r="A451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Scalability crawler</t>
-        </is>
-      </c>
-      <c r="B451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the page's view of the reports</t>
-        </is>
-      </c>
-      <c r="C451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`scalability.js` — `SKILLS_STATUS`, `renderCrawlState()`</t>
-        </is>
-      </c>
-      <c r="E451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Scalability — CRAWL STATE</t>
-        </is>
-      </c>
-      <c r="F451" t="inlineStr">
-        <is>
           <t xml:space="preserve">a tab named for a tool; scale for a larger basket, which is `ASSET=&lt;TICKER&gt;`</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rule_type_id</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t xml:space="preserve">rule_type_id</t>
+          <t xml:space="preserve">Architecture</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t xml:space="preserve">Architecture</t>
+          <t xml:space="preserve">Naming</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t xml:space="preserve">Naming</t>
+          <t xml:space="preserve">Conformities</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conformities</t>
+          <t xml:space="preserve">Workflow</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t xml:space="preserve">Workflow</t>
+          <t xml:space="preserve">FileLayout</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t xml:space="preserve">FileLayout</t>
+          <t xml:space="preserve">UI_TUI</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t xml:space="preserve">UI_TUI</t>
+          <t xml:space="preserve">Scalability</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scalability</t>
+          <t xml:space="preserve">Complexity</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t xml:space="preserve">Complexity</t>
+          <t xml:space="preserve">Determinism</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t xml:space="preserve">Determinism</t>
+          <t xml:space="preserve">Performance</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Performance</t>
-        </is>
-      </c>
-    </row>
-    <row r="464">
-      <c r="A464" t="inlineStr">
         <is>
           <t xml:space="preserve">Methodology</t>
         </is>

</xml_diff>

<commit_message>
Measure the three stores a stage writes, and drop the branches no state reaches
record.py lists raw_1m, assets_artifacts and status: the run records are where
it writes, after its second listing, so their diff was always empty; the
absent-store return, the usage check and the start failure a make command never
has go with it, and the page's Lifecycle tab loses the asset column no record
fills. Gone too: the ids no script or rule reads, SKILLS_STATUS, the null checks
no snapshot can trip, Bybit's silent empty list for a malformed answer, the
IF NOT EXISTS and missing_ok ingest never needs, the zero share of an empty
series, the ML status's contract and size fallbacks, the answer's .get() and
the sheet's path guard. The refusals the rules ask for stay one line: the
crawler's and the sheet's reading of what a hand edits.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -15715,7 +15715,7 @@
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the four stores of `STORES` — every store but the trials store</t>
+          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the three stores of `STORES` — every store but the trials store and the run records it writes</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
@@ -15806,7 +15806,7 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAGES — stage, asset, start, time, exit, added, changed, removed, bytes written</t>
+          <t xml:space="preserve">STAGES — stage, start, time, exit, added, changed, removed, bytes written</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
@@ -15823,7 +15823,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, written whole after the stage's second listing so it never appears in its own difference; untracked</t>
+          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, in a store the recorder does not list; untracked</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">

</xml_diff>

<commit_message>
Drop the lines the pinned interpreter never needs and the reads made twice
Python 3.12 is pinned and no annotation refers forward, so the 52 files lose
`from __future__ import annotations`; every module still imports where it runs,
on the host and in its runner. A parameter only ever given its default becomes
the value it stands for: the venues' REQUEST_ATTEMPT_COUNT, the sheet's path.
The features terminal reads the contract once — its state table takes the parsed
file, so its copy of `_present()` goes; hpo keeps the admissible flag it already
holds; STORE_RUN_RECORDS_DIR is marked and registered like every store read, and
two gaps of three blank lines close to two.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -13167,7 +13167,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STORE_ASSETS_ARTIFACTS_DIR` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`; `STORE_STATUS_DIR` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_monitoring/config.py`, `module_monitoring/sub_module_terminal/config.py`, and resolved in `module_skills/sub_module_scalability_crawler/config.py`; `STORE_RAW_1M_DIR` in `module_data/config.py`; `STORE_TRIALS_DIR` in `module_ml/config.py`</t>
+          <t xml:space="preserve">`STORE_ASSETS_ARTIFACTS_DIR` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`; `STORE_STATUS_DIR` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_monitoring/config.py`, `module_monitoring/sub_module_terminal/config.py`, and resolved in `module_skills/sub_module_scalability_crawler/config.py`; `STORE_RAW_1M_DIR` in `module_data/config.py`; `STORE_TRIALS_DIR` in `module_ml/config.py`; `STORE_RUN_RECORDS_DIR` in `module_monitoring/config.py`</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
@@ -14096,12 +14096,12 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three terminals whose module keeps an asset's files answer whether one stands in the same word, and a terminal reads another module's files through none of that module's code</t>
+          <t xml:space="preserve">the data and ML terminals answer whether an asset's file stands in the same word, and a terminal reads another module's files through none of that module's code</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Name the spool and the folds' whole selection, and let the register's sections be cited
The register gains the spool that write_venue_spool() and write_parquet() fill
and DuckDB reads once, so the naming rule's "registered domain noun" holds. The
validation folds select the barrier geometry too once a state is promoted — the
register row, the ML config comment and every asset README now say so.
RULE-TABLES-A-RULE-IS-CITED-BY-ITS-ID names the register's sections as its one
citable part of a generated document. Six skill summaries lose the tagline, two
register rows their history, the features README its section that never
existed, and the documents their relative code-span paths.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -6585,7 +6585,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t xml:space="preserve">A row of the contract, cited by its number in `AGENTS.md`.</t>
+          <t xml:space="preserve">A section of the register, `module_skills/skill_glossary.md` § &lt;section&gt;, titled by the register's own `section` column; a row of the contract, cited by its number in `AGENTS.md`.</t>
         </is>
       </c>
     </row>
@@ -8775,7 +8775,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">the validation folds — the folds used for the data-driven selection of model hyper-parameters, the entry edge threshold and, once a set is promoted, the feature set; every state the serpentine search compares is scored on them</t>
+          <t xml:space="preserve">the validation folds — the folds used for the data-driven selection of model hyper-parameters, the entry edge threshold and, once a state is promoted, the feature set and the barrier geometry; every state the serpentine search compares is scored on them</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -12780,22 +12780,17 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t xml:space="preserve">a partition: one asset's rows of a family, and one timeframe's where the family has one</t>
+          <t xml:space="preserve">a spool: a CSV file a writer fills with rows and DuckDB reads once into a table or a Parquet file — in the system's temporary directory, deleted by the writer that made it</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ticker=&lt;TICKER&gt;/`, `timeframe=&lt;timeframe&gt;/` — Hive's `key=value`, the value the ticker in capitals and the compact timeframe token; `partition_dir()`</t>
+          <t xml:space="preserve">`write_venue_spool()` in `module_data/ingest.py`; the spool of `write_parquet()` in `module_features/dataset.py` and `module_ml/dataset.py`</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;/` without its key; a lower-case ticker as a partition value; a slot as a partition value; a column inside the partition repeating its key</t>
-        </is>
-      </c>
-      <c r="I268" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hive</t>
+          <t xml:space="preserve">a spool in a store; a spool left behind; a spool read twice</t>
         </is>
       </c>
     </row>
@@ -12807,17 +12802,22 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t xml:space="preserve">the schema of a family: its columns and types as data, written by the family's one writer beside its partitions — the columns of the union of the partitions, the partition keys absent</t>
+          <t xml:space="preserve">a partition: one asset's rows of a family, and one timeframe's where the family has one</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;store&gt;/&lt;family&gt;/schema.json`, `schema_json()` in every writer's `config.py` — a list of `column` and `type` in the writer's order, in DuckDB's type spelling; from `load_partition_schema()`, the writer's `DESCRIBE` of the partition it wrote, for a homogeneous family; from `catalogue_schema()` in `module_features/config.py` for `catalogue`; from `TRIAL_COLUMNS` in `module_ml/hpo.py` for `hpo_trials` and `score_trials`</t>
+          <t xml:space="preserve">`ticker=&lt;TICKER&gt;/`, `timeframe=&lt;timeframe&gt;/` — Hive's `key=value`, the value the ticker in capitals and the compact timeframe token; `partition_dir()`</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t xml:space="preserve">a schema written by hand; a schema read off one partition of a family whose partitions differ; a partition that renames a column or changes its type; a second type spelling</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;/` without its key; a lower-case ticker as a partition value; a slot as a partition value; a column inside the partition repeating its key</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hive</t>
         </is>
       </c>
     </row>
@@ -12829,22 +12829,17 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset's folder: its non-tabular files, one file per artifact responsibility, named `&lt;TICKER&gt;_&lt;artifact&gt;.&lt;ext&gt;`, at the segment `ticker=&lt;TICKER&gt;/` of the artifacts store</t>
+          <t xml:space="preserve">the schema of a family: its columns and types as data, written by the family's one writer beside its partitions — the columns of the union of the partitions, the partition keys absent</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t xml:space="preserve">`store/assets_artifacts/ticker=&lt;TICKER&gt;/`; `artifact_dir()` in `module_features/config.py`, `module_ml/config.py` and `module_features/sub_module_terminal/config.py`; one descriptor per file in the `config.py` of the module that writes it</t>
+          <t xml:space="preserve">`&lt;store&gt;/&lt;family&gt;/schema.json`, `schema_json()` in every writer's `config.py` — a list of `column` and `type` in the writer's order, in DuckDB's type spelling; from `load_partition_schema()`, the writer's `DESCRIBE` of the partition it wrote, for a homogeneous family; from `catalogue_schema()` in `module_features/config.py` for `catalogue`; from `TRIAL_COLUMNS` in `module_ml/hpo.py` for `hpo_trials` and `score_trials`</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Parquet file in the asset's folder; a file without the `&lt;TICKER&gt;_` prefix; `&lt;TICKER&gt;/` without its key; a path assembled at the point of use</t>
-        </is>
-      </c>
-      <c r="G270" t="inlineStr">
-        <is>
-          <t xml:space="preserve">its tracked remnant: `&lt;TICKER&gt;_README.md`, `&lt;TICKER&gt;_parameters.json` and, once written, `&lt;TICKER&gt;_serpentine_search_profile.json`, `&lt;TICKER&gt;_serpentine_search.json`, `&lt;TICKER&gt;_serpentine_search_trials.jsonl`, `&lt;TICKER&gt;_feature_set.json`, `&lt;TICKER&gt;_barriers.json`, `&lt;TICKER&gt;_hyperparameter_point.json`; every other file the chain rebuilds</t>
+          <t xml:space="preserve">a schema written by hand; a schema read off one partition of a family whose partitions differ; a partition that renames a column or changes its type; a second type spelling</t>
         </is>
       </c>
     </row>
@@ -12856,17 +12851,22 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset: the one a per-asset process is run for, and the namespace every partition and every per-asset file is selected by</t>
+          <t xml:space="preserve">the asset's folder: its non-tabular files, one file per artifact responsibility, named `&lt;TICKER&gt;_&lt;artifact&gt;.&lt;ext&gt;`, at the segment `ticker=&lt;TICKER&gt;/` of the artifacts store</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ticker` — in code, in a key, and as the partition value `ticker=&lt;TICKER&gt;`; `--tickers` of a stage's command line, `build_ticker_parser()` with no default; `ASSET=&lt;TICKER&gt;` on the make line narrowing `TICKER_LIST`, read by no stage</t>
+          <t xml:space="preserve">`store/assets_artifacts/ticker=&lt;TICKER&gt;/`; `artifact_dir()` in `module_features/config.py`, `module_ml/config.py` and `module_features/sub_module_terminal/config.py`; one descriptor per file in the `config.py` of the module that writes it</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TICKER`, `SYMBOL`, `ASSET_TICKER` as its name; a per-asset `.env`; a module, a file, a function, a compose service or an image named for a ticker; `ASSET` read by a stage</t>
+          <t xml:space="preserve">a Parquet file in the asset's folder; a file without the `&lt;TICKER&gt;_` prefix; `&lt;TICKER&gt;/` without its key; a path assembled at the point of use</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its tracked remnant: `&lt;TICKER&gt;_README.md`, `&lt;TICKER&gt;_parameters.json` and, once written, `&lt;TICKER&gt;_serpentine_search_profile.json`, `&lt;TICKER&gt;_serpentine_search.json`, `&lt;TICKER&gt;_serpentine_search_trials.jsonl`, `&lt;TICKER&gt;_feature_set.json`, `&lt;TICKER&gt;_barriers.json`, `&lt;TICKER&gt;_hyperparameter_point.json`; every other file the chain rebuilds</t>
         </is>
       </c>
     </row>
@@ -12878,39 +12878,39 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t xml:space="preserve">the basket, as the launcher defines it</t>
+          <t xml:space="preserve">the asset: the one a per-asset process is run for, and the namespace every partition and every per-asset file is selected by</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TICKERS` in the `Makefile`, the basket's one list; `TICKER_LIST`, the list the `each` macro goes over, which `ASSET` narrows; `one_asset`, the one ticker of `TICKERS` a hand's action on the serpentine search names; `TICKERS_CSV`, the basket as one `--tickers` argument of a basket-wide stage, which `ASSET` never narrows</t>
+          <t xml:space="preserve">`ticker` — in code, in a key, and as the partition value `ticker=&lt;TICKER&gt;`; `--tickers` of a stage's command line, `build_ticker_parser()` with no default; `ASSET=&lt;TICKER&gt;` on the make line narrowing `TICKER_LIST`, read by no stage</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t xml:space="preserve">a basket in a module's `config.py`; a second list in `docker-compose.yml`; a stage that defaults to it; a basket a terminal defines or reads from a store</t>
+          <t xml:space="preserve">`TICKER`, `SYMBOL`, `ASSET_TICKER` as its name; a per-asset `.env`; a module, a file, a function, a compose service or an image named for a ticker; `ASSET` read by a stage</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t xml:space="preserve">The tree</t>
+          <t xml:space="preserve">Stores</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t xml:space="preserve">a module: its package, its orientation, its own skills and its sub-modules under one directory</t>
+          <t xml:space="preserve">the basket, as the launcher defines it</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/` holding `&lt;file&gt;.py`, `README_module_&lt;domain&gt;.md`, `skills/` and each `sub_module_&lt;subject&gt;/`</t>
+          <t xml:space="preserve">`TICKERS` in the `Makefile`, the basket's one list; `TICKER_LIST`, the list the `each` macro goes over, which `ASSET` narrows; `one_asset`, the one ticker of `TICKERS` a hand's action on the serpentine search names; `TICKERS_CSV`, the basket as one `--tickers` argument of a basket-wide stage, which `ASSET` never narrows</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t xml:space="preserve">a numbered directory; a package split across two places; a module's rule filed outside it; a repository per module</t>
+          <t xml:space="preserve">a basket in a module's `config.py`; a second list in `docker-compose.yml`; a stage that defaults to it; a basket a terminal defines or reads from a store</t>
         </is>
       </c>
     </row>
@@ -12922,17 +12922,17 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t xml:space="preserve">the canon: the module of the rules that cross modules or govern the project — the sheet, what the sync renders from it, the index, and its two sub-modules; it takes no part in the chain's dataflow and no module imports it</t>
+          <t xml:space="preserve">a module: its package, its orientation, its own skills and its sub-modules under one directory</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/` — `module_skills/config.py`, `module_skills/sheet.py`, `module_skills/sync.py`, `module_skills/configurables.py`, `module_skills/sub_module_scalability_crawler/`, `module_skills/sub_module_terminal/`; `SKILLS_SHEET_PATH`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/` holding `&lt;file&gt;.py`, `README_module_&lt;domain&gt;.md`, `skills/` and each `sub_module_&lt;subject&gt;/`</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage of the chain; a runtime import of it by a module; a cross-cutting rule filed under one module; a third-party package</t>
+          <t xml:space="preserve">a numbered directory; a package split across two places; a module's rule filed outside it; a repository per module</t>
         </is>
       </c>
     </row>
@@ -12944,17 +12944,17 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module: a nesting inside the module, or the canon, that owns it — its own `config.py`, an action module with `main()` for each action of a hand, `tui.py` where it draws a terminal, its orientation `README_sub_module_&lt;subject&gt;.md` beside it; no part in the chain's dataflow, a hand's research outside the chain at most, whose promotion writes files the chain reads</t>
+          <t xml:space="preserve">the canon: the module of the rules that cross modules or govern the project — the sheet, what the sync renders from it, the index, and its two sub-modules; it takes no part in the chain's dataflow and no module imports it</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_&lt;subject&gt;/` — `module_data/sub_module_terminal/`, `module_features/sub_module_terminal/`, `module_ml/sub_module_terminal/`, `module_monitoring/sub_module_terminal/`, `module_features/sub_module_serpentine_search/`, `module_skills/sub_module_scalability_crawler/`, `module_skills/sub_module_terminal/`</t>
+          <t xml:space="preserve">`module_skills/` — `module_skills/config.py`, `module_skills/sheet.py`, `module_skills/sync.py`, `module_skills/configurables.py`, `module_skills/sub_module_scalability_crawler/`, `module_skills/sub_module_terminal/`; `SKILLS_SHEET_PATH`</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module at the root; a sub-module of a sub-module; the domain repeated in the folder, `sub_module_ml_terminal`; a sub-module that imports another module</t>
+          <t xml:space="preserve">a stage of the chain; a runtime import of it by a module; a cross-cutting rule filed under one module; a third-party package</t>
         </is>
       </c>
     </row>
@@ -12966,17 +12966,17 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t xml:space="preserve">the project's one image</t>
+          <t xml:space="preserve">a sub-module: a nesting inside the module, or the canon, that owns it — its own `config.py`, an action module with `main()` for each action of a hand, `tui.py` where it draws a terminal, its orientation `README_sub_module_&lt;subject&gt;.md` beside it; no part in the chain's dataflow, a hand's research outside the chain at most, whose promotion writes files the chain reads</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t xml:space="preserve">`liora-1m-pipeline` — `image:` on the `x-service` anchor of `docker-compose.yml`, built by `make build` from the root `Dockerfile` onto `python:3.12-slim`: the pins of `requirements.txt` and no code</t>
+          <t xml:space="preserve">`sub_module_&lt;subject&gt;/` — `module_data/sub_module_terminal/`, `module_features/sub_module_terminal/`, `module_ml/sub_module_terminal/`, `module_monitoring/sub_module_terminal/`, `module_features/sub_module_serpentine_search/`, `module_skills/sub_module_scalability_crawler/`, `module_skills/sub_module_terminal/`</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t xml:space="preserve">an image per module, per service or per asset; a `Dockerfile` in a module; compose's `&lt;project&gt;-&lt;service&gt;` default</t>
+          <t xml:space="preserve">a sub-module at the root; a sub-module of a sub-module; the domain repeated in the folder, `sub_module_ml_terminal`; a sub-module that imports another module</t>
         </is>
       </c>
     </row>
@@ -12988,17 +12988,17 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t xml:space="preserve">a path written `module_&lt;domain&gt;/…` in the contract or a Skill</t>
+          <t xml:space="preserve">the project's one image</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t xml:space="preserve">the package as it lies at the root of the tree</t>
+          <t xml:space="preserve">`liora-1m-pipeline` — `image:` on the `x-service` anchor of `docker-compose.yml`, built by `make build` from the root `Dockerfile` onto `python:3.12-slim`: the pins of `requirements.txt` and no code</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `../module_&lt;x&gt;` relative path; a path built at the point of use</t>
+          <t xml:space="preserve">an image per module, per service or per asset; a `Dockerfile` in a module; compose's `&lt;project&gt;-&lt;service&gt;` default</t>
         </is>
       </c>
     </row>
@@ -13010,22 +13010,17 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t xml:space="preserve">a comment that explains a Python module-level constant, placed by what it explains</t>
+          <t xml:space="preserve">a path written `module_&lt;domain&gt;/…` in the contract or a Skill</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t xml:space="preserve">inline comment — PEP 8's word for a comment on its statement's own line; block comment — PEP 8's word for the comment lines directly above the code they apply to</t>
+          <t xml:space="preserve">the package as it lies at the root of the tree</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t xml:space="preserve">trailing comment, end-of-line comment, side comment</t>
-        </is>
-      </c>
-      <c r="I278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PEP 8</t>
+          <t xml:space="preserve">a `../module_&lt;x&gt;` relative path; a path built at the point of use</t>
         </is>
       </c>
     </row>
@@ -13037,27 +13032,22 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t xml:space="preserve">a CONFIGURABLES record: one value an operator may set in a module, its value written nowhere else, beside its class, unit and meaning, whether a terminal reads it, whether it is part of the experiment's identity, what changing it reruns and what it risks</t>
+          <t xml:space="preserve">a comment that explains a Python module-level constant, placed by what it explains</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t xml:space="preserve">`CONFIGURABLES`, `VALUE_BY_CONFIGURABLE` in `module_features/config.py`, `module_features/sub_module_serpentine_search/config.py` and `module_ml/config.py`; `CONFIGURABLES_NAME`, `CONFIGURABLE_FIELDS` in `module_skills/config.py`; `make skills-configurables`</t>
-        </is>
-      </c>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`configurables` in `features_status.json` and in `ml_status.json`, each record `name`, `class`, `value`, `unit`, `meaning`, `tui`, `experiment_identity`, `requires_rerun`, `risk`</t>
-        </is>
-      </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CONFIGURABLES — a frame on the Features tab and on the ML Research tab</t>
+          <t xml:space="preserve">inline comment — PEP 8's word for a comment on its statement's own line; block comment — PEP 8's word for the comment lines directly above the code they apply to</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t xml:space="preserve">a value an operator may set written outside its record; the feature catalogue, a derived value or a constant of the method as a record; a copy of a record without the marker; a record's value restated in a document</t>
+          <t xml:space="preserve">trailing comment, end-of-line comment, side comment</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PEP 8</t>
         </is>
       </c>
     </row>
@@ -13069,44 +13059,54 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t xml:space="preserve">the class of a configurable: `DEFAULT` a starting point of the experiment, `SPECTRUM` the legal values of one knob, `OVERRIDE` an operator's explicit override, `WIRING` a technical setting of a run; a value derived from records and a constant of the method stand below the block, derived and fixed</t>
+          <t xml:space="preserve">a CONFIGURABLES record: one value an operator may set in a module, its value written nowhere else, beside its class, unit and meaning, whether a terminal reads it, whether it is part of the experiment's identity, what changing it reruns and what it risks</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t xml:space="preserve">the `class` of a record in a `CONFIGURABLES` block</t>
+          <t xml:space="preserve">`CONFIGURABLES`, `VALUE_BY_CONFIGURABLE` in `module_features/config.py`, `module_features/sub_module_serpentine_search/config.py` and `module_ml/config.py`; `CONFIGURABLES_NAME`, `CONFIGURABLE_FIELDS` in `module_skills/config.py`; `make skills-configurables`</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t xml:space="preserve">`class`</t>
+          <t xml:space="preserve">`configurables` in `features_status.json` and in `ml_status.json`, each record `name`, `class`, `value`, `unit`, `meaning`, `tui`, `experiment_identity`, `requires_rerun`, `risk`</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONFIGURABLES — a frame on the Features tab and on the ML Research tab</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t xml:space="preserve">a record classed derived or fixed; a class that hides a second default; a feature set as a spectrum</t>
+          <t xml:space="preserve">a value an operator may set written outside its record; the feature catalogue, a derived value or a constant of the method as a record; a copy of a record without the marker; a record's value restated in a document</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t xml:space="preserve">Twice by extraction</t>
+          <t xml:space="preserve">The tree</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t xml:space="preserve">the unit constants — equal by value, each holder keeping the ones it uses</t>
+          <t xml:space="preserve">the class of a configurable: `DEFAULT` a starting point of the experiment, `SPECTRUM` the legal values of one knob, `OVERRIDE` an operator's explicit override, `WIRING` a technical setting of a run; a value derived from records and a constant of the method stand below the block, derived and fixed</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t xml:space="preserve">`MILLISECONDS_PER_SECOND` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_monitoring/page.js`; `MILLISECONDS_PER_MINUTE` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`; `MILLISECONDS_PER_DAY` in `module_data/config.py`, `module_features/config.py`; `MINUTES_PER_HOUR` in `module_features/config.py`, `module_monitoring/data.js`; `HOURS_PER_DAY` in `module_monitoring/data.js`; `SECONDS_PER_MINUTE` in `module_monitoring/page.js`</t>
-        </is>
-      </c>
-      <c r="H281" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a unit is a unit: importing one across a boundary would drag the module behind it (`AGENTS.md` D02), and the page's scripts import no Python</t>
+          <t xml:space="preserve">the `class` of a record in a `CONFIGURABLES` block</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`class`</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a record classed derived or fixed; a class that hides a second default; a feature set as a spectrum</t>
         </is>
       </c>
     </row>
@@ -13118,17 +13118,17 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t xml:space="preserve">`BYTES_PER_KIBIBYTE` — equal by value</t>
+          <t xml:space="preserve">the unit constants — equal by value, each holder keeping the ones it uses</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`; the browser's own in `module_monitoring/page.js`</t>
+          <t xml:space="preserve">`MILLISECONDS_PER_SECOND` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_monitoring/page.js`; `MILLISECONDS_PER_MINUTE` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`; `MILLISECONDS_PER_DAY` in `module_data/config.py`, `module_features/config.py`; `MINUTES_PER_HOUR` in `module_features/config.py`, `module_monitoring/data.js`; `HOURS_PER_DAY` in `module_monitoring/data.js`; `SECONDS_PER_MINUTE` in `module_monitoring/page.js`</t>
         </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t xml:space="preserve">a unit, like the unit constants: the ML module and the page each size a file, and neither imports the other</t>
+          <t xml:space="preserve">a unit is a unit: importing one across a boundary would drag the module behind it (`AGENTS.md` D02), and the page's scripts import no Python</t>
         </is>
       </c>
     </row>
@@ -13140,17 +13140,17 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t xml:space="preserve">`DUCKDB_MEMORY_LIMIT` — equal by value</t>
+          <t xml:space="preserve">`BYTES_PER_KIBIBYTE` — equal by value</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t xml:space="preserve">a constant in `module_data/config.py`; a CONFIGURABLES record and the constant read from it in `module_features/config.py` and `module_ml/config.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`; the browser's own in `module_monitoring/page.js`</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t xml:space="preserve">every DuckDB connection of every module pins the same ceiling beside `threads=1`, and no module imports another</t>
+          <t xml:space="preserve">a unit, like the unit constants: the ML module and the page each size a file, and neither imports the other</t>
         </is>
       </c>
     </row>
@@ -13162,17 +13162,17 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store reads — each holder reading the stores it touches, identical but where the row says</t>
+          <t xml:space="preserve">`DUCKDB_MEMORY_LIMIT` — equal by value</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STORE_ASSETS_ARTIFACTS_DIR` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`; `STORE_STATUS_DIR` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_monitoring/config.py`, `module_monitoring/sub_module_terminal/config.py`, and resolved in `module_skills/sub_module_scalability_crawler/config.py`; `STORE_RAW_1M_DIR` in `module_data/config.py`; `STORE_TRIALS_DIR` in `module_ml/config.py`; `STORE_RUN_RECORDS_DIR` in `module_monitoring/config.py`</t>
+          <t xml:space="preserve">a constant in `module_data/config.py`; a CONFIGURABLES record and the constant read from it in `module_features/config.py` and `module_ml/config.py`</t>
         </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store contract is read as `Path(os.environ[...])` where it is used, and no module imports another: the artifacts and status stores every module of the chain touches, the status store the dashboard's server and the monitoring terminal each read for themselves, the snapshot the crawler writes — resolved there because the crawl compares it with the resolved paths the files matrix reaches — the raw store the data module alone touches, the trials store the ML module alone writes</t>
+          <t xml:space="preserve">every DuckDB connection of every module pins the same ceiling beside `threads=1`, and no module imports another</t>
         </is>
       </c>
     </row>
@@ -13184,17 +13184,17 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t xml:space="preserve">`artifact_dir()` — identical</t>
+          <t xml:space="preserve">the store reads — each holder reading the stores it touches, identical but where the row says</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`STORE_ASSETS_ARTIFACTS_DIR` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`; `STORE_STATUS_DIR` in `module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_monitoring/config.py`, `module_monitoring/sub_module_terminal/config.py`, and resolved in `module_skills/sub_module_scalability_crawler/config.py`; `STORE_RAW_1M_DIR` in `module_data/config.py`; `STORE_TRIALS_DIR` in `module_ml/config.py`; `STORE_RUN_RECORDS_DIR` in `module_monitoring/config.py`</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset's folder is where every per-asset file of the chain lies, its path grammar one and spelled once per owner; the features terminal runs on the host's `python3` and cannot import `module_features/config.py`, which imports numpy through `.indicators`</t>
+          <t xml:space="preserve">the store contract is read as `Path(os.environ[...])` where it is used, and no module imports another: the artifacts and status stores every module of the chain touches, the status store the dashboard's server and the monitoring terminal each read for themselves, the snapshot the crawler writes — resolved there because the crawl compares it with the resolved paths the files matrix reaches — the raw store the data module alone touches, the trials store the ML module alone writes</t>
         </is>
       </c>
     </row>
@@ -13206,17 +13206,17 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t xml:space="preserve">`partition_dir()` — identical</t>
+          <t xml:space="preserve">`artifact_dir()` — identical</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H286" t="inlineStr">
         <is>
-          <t xml:space="preserve">every writer and reader of a table family builds its partition by one grammar, and no module imports another; the features terminal counts an asset's partitions of `bars` and `catalogue` without its module's `config.py`</t>
+          <t xml:space="preserve">the asset's folder is where every per-asset file of the chain lies, its path grammar one and spelled once per owner; the features terminal runs on the host's `python3` and cannot import `module_features/config.py`, which imports numpy through `.indicators`</t>
         </is>
       </c>
     </row>
@@ -13228,17 +13228,17 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t xml:space="preserve">`schema_json()` — identical</t>
+          <t xml:space="preserve">`partition_dir()` — identical</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/config.py`, `module_features/config.py`, `module_ml/config.py`</t>
+          <t xml:space="preserve">`module_data/config.py`, `module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t xml:space="preserve">every module that writes a family writes its schema beside the partitions at one path, and no module imports another</t>
+          <t xml:space="preserve">every writer and reader of a table family builds its partition by one grammar, and no module imports another; the features terminal counts an asset's partitions of `bars` and `catalogue` without its module's `config.py`</t>
         </is>
       </c>
     </row>
@@ -13250,7 +13250,7 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ohlcv_1m_canonical_parquet()` — identical</t>
+          <t xml:space="preserve">`schema_json()` — identical</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -13260,7 +13260,7 @@
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t xml:space="preserve">the data module writes the canonical family, the feature module aggregates it into bars and the ML module walks its minutes for the labels; no module imports another</t>
+          <t xml:space="preserve">every module that writes a family writes its schema beside the partitions at one path, and no module imports another</t>
         </is>
       </c>
     </row>
@@ -13272,17 +13272,17 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t xml:space="preserve">`bars_parquet()` — identical</t>
+          <t xml:space="preserve">`ohlcv_1m_canonical_parquet()` — identical</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/config.py`, `module_ml/config.py`</t>
+          <t xml:space="preserve">`module_data/config.py`, `module_features/config.py`, `module_ml/config.py`</t>
         </is>
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature module writes the bars and the ML module reads them for a label's barrier scale and its decision grid; no module imports another</t>
+          <t xml:space="preserve">the data module writes the canonical family, the feature module aggregates it into bars and the ML module walks its minutes for the labels; no module imports another</t>
         </is>
       </c>
     </row>
@@ -13294,17 +13294,17 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_partition_schema()` — identical</t>
+          <t xml:space="preserve">`bars_parquet()` — identical</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/ingest.py`, `module_features/dataset.py`, `module_ml/dataset.py`; `DESCRIBE SELECT * FROM read_parquet(&lt;partition&gt;, hive_partitioning=false)` — read as a Hive tree, a single `ticker=&lt;TICKER&gt;/` file would grow a `ticker` column</t>
+          <t xml:space="preserve">`module_features/config.py`, `module_ml/config.py`</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t xml:space="preserve">every writer of a homogeneous family writes its `schema.json` from the partition it just wrote, and no module imports another</t>
+          <t xml:space="preserve">the feature module writes the bars and the ML module reads them for a label's barrier scale and its decision grid; no module imports another</t>
         </is>
       </c>
     </row>
@@ -13316,17 +13316,17 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t xml:space="preserve">`to_utc_ms()` — identical</t>
+          <t xml:space="preserve">`load_partition_schema()` — identical</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/config.py`, `module_features/config.py`, `module_ml/config.py`</t>
+          <t xml:space="preserve">`module_data/ingest.py`, `module_features/dataset.py`, `module_ml/dataset.py`; `DESCRIBE SELECT * FROM read_parquet(&lt;partition&gt;, hive_partitioning=false)` — read as a Hive tree, a single `ticker=&lt;TICKER&gt;/` file would grow a `ticker` column</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t xml:space="preserve">the day literals of the three modules are turned into milliseconds by the same function, and no module imports another</t>
+          <t xml:space="preserve">every writer of a homogeneous family writes its `schema.json` from the partition it just wrote, and no module imports another</t>
         </is>
       </c>
     </row>
@@ -13338,7 +13338,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_ticker_parser()`, `parse_tickers()` — identical</t>
+          <t xml:space="preserve">`to_utc_ms()` — identical</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -13348,7 +13348,7 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one command line every stage shares, `--tickers` with no default, and no module imports another; `module_monitoring` runs no stage and parses no ticker argument</t>
+          <t xml:space="preserve">the day literals of the three modules are turned into milliseconds by the same function, and no module imports another</t>
         </is>
       </c>
     </row>
@@ -13360,7 +13360,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t xml:space="preserve">`rounded()` — identical</t>
+          <t xml:space="preserve">`build_ticker_parser()`, `parse_tickers()` — identical</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -13370,7 +13370,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three snapshots round the same way, and no module imports another</t>
+          <t xml:space="preserve">the one command line every stage shares, `--tickers` with no default, and no module imports another; `module_monitoring` runs no stage and parses no ticker argument</t>
         </is>
       </c>
     </row>
@@ -13382,17 +13382,17 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t xml:space="preserve">`RESEARCH_START_UTC`, `RESEARCH_END_UTC`, `RESEARCH_START_MS`, `RESEARCH_END_MS` — equal by value</t>
+          <t xml:space="preserve">`rounded()` — identical</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/config.py`, the two dates its CONFIGURABLES records hold; `module_ml/config.py`, the first and the last of `FOLD_BOUNDS_UTC`</t>
+          <t xml:space="preserve">`module_data/config.py`, `module_features/config.py`, `module_ml/config.py`</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t xml:space="preserve">the frozen window is the experiment's: the feature layer bounds the bars and the catalogue by it, the ML layer the labels and the folds, each owning its literal, and neither imports the other</t>
+          <t xml:space="preserve">the three snapshots round the same way, and no module imports another</t>
         </is>
       </c>
     </row>
@@ -13404,17 +13404,17 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue_json()` — identical</t>
+          <t xml:space="preserve">`RESEARCH_START_UTC`, `RESEARCH_END_UTC`, `RESEARCH_START_MS`, `RESEARCH_END_MS` — equal by value</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_features/config.py`, the two dates its CONFIGURABLES records hold; `module_ml/config.py`, the first and the last of `FOLD_BOUNDS_UTC`</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t xml:space="preserve">the writer names the contract it writes, the reader the contract it reads, and the features terminal the contract it shows a hand — without its module's `config.py`, which imports numpy</t>
+          <t xml:space="preserve">the frozen window is the experiment's: the feature layer bounds the bars and the catalogue by it, the ML layer the labels and the folds, each owning its literal, and neither imports the other</t>
         </is>
       </c>
     </row>
@@ -13426,17 +13426,17 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_id()` — identical</t>
+          <t xml:space="preserve">`catalogue_json()` — identical</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/config.py`, `module_ml/config.py`</t>
+          <t xml:space="preserve">`module_features/config.py`, `module_ml/config.py`, `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t xml:space="preserve">the id grammar `module_features` owns, composed where the columns of X are named — the one copy downstream, the ML module importing no feature code</t>
+          <t xml:space="preserve">the writer names the contract it writes, the reader the contract it reads, and the features terminal the contract it shows a hand — without its module's `config.py`, which imports numpy</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t xml:space="preserve">`to_json_safe()` — identical</t>
+          <t xml:space="preserve">`feature_id()` — identical</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`</t>
+          <t xml:space="preserve">`module_features/config.py`, `module_ml/config.py`</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t xml:space="preserve">numpy canonicalisation is local to the modules that hold numpy values, and the JSON both publish is one form; no module imports another</t>
+          <t xml:space="preserve">the id grammar `module_features` owns, composed where the columns of X are named — the one copy downstream, the ML module importing no feature code</t>
         </is>
       </c>
     </row>
@@ -13470,17 +13470,17 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t xml:space="preserve">`write_json()` — the canonical JSON form, keys sorted and indented</t>
+          <t xml:space="preserve">`to_json_safe()` — identical</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_features/dataset.py` and `module_ml/dataset.py`; equal by value in `module_features/sub_module_terminal/config.py`, which writes plain values without `to_json_safe()`</t>
+          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t xml:space="preserve">the published JSON is deterministic — the contract, the snapshots, the artifacts and the profile a hand drafts through the features terminal take one form; the terminal holds no numpy value and cannot import a `dataset.py`, which imports duckdb and numpy</t>
+          <t xml:space="preserve">numpy canonicalisation is local to the modules that hold numpy values, and the JSON both publish is one form; no module imports another</t>
         </is>
       </c>
     </row>
@@ -13492,17 +13492,17 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t xml:space="preserve">`write_parquet()` — identical</t>
+          <t xml:space="preserve">`write_json()` — the canonical JSON form, keys sorted and indented</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`</t>
+          <t xml:space="preserve">identical in `module_features/dataset.py` and `module_ml/dataset.py`; equal by value in `module_features/sub_module_terminal/config.py`, which writes plain values without `to_json_safe()`</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t xml:space="preserve">the repr round-trip that makes a Parquet file byte-reproducible; given a homogeneous family it writes that family's `schema.json` from the partition it wrote — `labels` and `oos_predictions`; no module imports another</t>
+          <t xml:space="preserve">the published JSON is deterministic — the contract, the snapshots, the artifacts and the profile a hand drafts through the features terminal take one form; the terminal holds no numpy value and cannot import a `dataset.py`, which imports duckdb and numpy</t>
         </is>
       </c>
     </row>
@@ -13514,17 +13514,17 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_json()` — identical</t>
+          <t xml:space="preserve">`write_parquet()` — identical</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`</t>
         </is>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t xml:space="preserve">the readers of the same JSON files — a stage, and the terminals that read what a stage wrote; a terminal cannot import a `dataset.py`, which imports duckdb and numpy, nor another module's code</t>
+          <t xml:space="preserve">the repr round-trip that makes a Parquet file byte-reproducible; given a homogeneous family it writes that family's `schema.json` from the partition it wrote — `labels` and `oos_predictions`; no module imports another</t>
         </is>
       </c>
     </row>
@@ -13536,17 +13536,17 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_jsonl()` — identical</t>
+          <t xml:space="preserve">`load_json()` — identical</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`, `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t xml:space="preserve">a ledger is read back as it was written: HPO's to place a study among the ones before it, the serpentine search's to resume and to answer its own questions, the features terminal's to show the trials the state names</t>
+          <t xml:space="preserve">the readers of the same JSON files — a stage, and the terminals that read what a stage wrote; a terminal cannot import a `dataset.py`, which imports duckdb and numpy, nor another module's code</t>
         </is>
       </c>
     </row>
@@ -13558,22 +13558,17 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t xml:space="preserve">`recursive_mean()`, `true_range()`, `asof_index()` — identical</t>
+          <t xml:space="preserve">`load_jsonl()` — identical</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/indicators.py`, `module_ml/labels.py`</t>
-        </is>
-      </c>
-      <c r="F302" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`wilder_smoothing()`, `atr()` — the names these carried before the catalogue named every operation by its word</t>
+          <t xml:space="preserve">`module_features/dataset.py`, `module_ml/dataset.py`, `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t xml:space="preserve">the label defines its own barrier scale and aligns to the last closed bar the way the catalogue does, and the ML module imports no feature code</t>
+          <t xml:space="preserve">a ledger is read back as it was written: HPO's to place a study among the ones before it, the serpentine search's to resume and to answer its own questions, the features terminal's to show the trials the state names</t>
         </is>
       </c>
     </row>
@@ -13585,17 +13580,22 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SEED` — equal by value</t>
+          <t xml:space="preserve">`recursive_mean()`, `true_range()`, `asof_index()` — identical</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t xml:space="preserve">a CONFIGURABLES record and the constant read from it in `module_ml/config.py`; a constant in `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">`module_features/indicators.py`, `module_ml/labels.py`</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`wilder_smoothing()`, `atr()` — an abbreviation or a popular name where the catalogue names an operation by its word</t>
         </is>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t xml:space="preserve">the seed is one of the values the serpentine search records as the identity of its experiment, and the parameters artifact it reads does not carry it; the sub-module cannot import the ML module</t>
+          <t xml:space="preserve">the label defines its own barrier scale and aligns to the last closed bar the way the catalogue does, and the ML module imports no feature code</t>
         </is>
       </c>
     </row>
@@ -13607,17 +13607,17 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t xml:space="preserve">`VALIDATION_FOLD_IDS` — identical</t>
+          <t xml:space="preserve">`SEED` — equal by value</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">a CONFIGURABLES record and the constant read from it in `module_ml/config.py`; a constant in `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t xml:space="preserve">the turn's fold gate reads every fold in the order the selection fixes and the evaluator scores the same ones; which folds select is the method, never the order of the keys a payload happens to carry</t>
+          <t xml:space="preserve">the seed is one of the values the serpentine search records as the identity of its experiment, and the parameters artifact it reads does not carry it; the sub-module cannot import the ML module</t>
         </is>
       </c>
     </row>
@@ -13629,7 +13629,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t xml:space="preserve">`BARRIER_COORDINATE_CASTS`, `BARRIER_COORDINATE_NAMES` — identical</t>
+          <t xml:space="preserve">`VALIDATION_FOLD_IDS` — identical</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -13639,7 +13639,7 @@
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t xml:space="preserve">the casts are what make an integer and the same number as a float one state, and the order is the order a state is keyed in; a copy differing by one cast turns every cache hit into a miss and the serpentine search pays again for states it already holds</t>
+          <t xml:space="preserve">the turn's fold gate reads every fold in the order the selection fixes and the evaluator scores the same ones; which folds select is the method, never the order of the keys a payload happens to carry</t>
         </is>
       </c>
     </row>
@@ -13651,17 +13651,17 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t xml:space="preserve">`START_BY_COORDINATE_DEFAULT` — equal by value</t>
+          <t xml:space="preserve">`BARRIER_COORDINATE_CASTS`, `BARRIER_COORDINATE_NAMES` — identical</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t xml:space="preserve">a CONFIGURABLES record and the constant read from it in `module_ml/config.py`; constants in `module_features/sub_module_serpentine_search/config.py` and `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t xml:space="preserve">the geometry the chain stands at without a promotion — where the serpentine search starts, and where the features terminal's draft pins a coordinate it does not search; neither side may import the ML module, and the terminal not even its own module's `config.py`</t>
+          <t xml:space="preserve">the casts are what make an integer and the same number as a float one state, and the order is the order a state is keyed in; a copy differing by one cast turns every cache hit into a miss and the serpentine search pays again for states it already holds</t>
         </is>
       </c>
     </row>
@@ -13673,17 +13673,17 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TRADE_EXIT_COORDINATE_NAMES` — identical</t>
+          <t xml:space="preserve">`START_BY_COORDINATE_DEFAULT` — equal by value</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">a CONFIGURABLES record and the constant read from it in `module_ml/config.py`; constants in `module_features/sub_module_serpentine_search/config.py` and `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t xml:space="preserve">the serpentine search moves the two as one family and the evaluator leaves them out of a fit identity; a copy that drifts merges states whose fits differ, with wrong numbers and no error</t>
+          <t xml:space="preserve">the geometry the chain stands at without a promotion — where the serpentine search starts, and where the features terminal's draft pins a coordinate it does not search; neither side may import the ML module, and the terminal not even its own module's `config.py`</t>
         </is>
       </c>
     </row>
@@ -13695,17 +13695,17 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SELECTION_FOLD_MEASURE` — identical</t>
+          <t xml:space="preserve">`TRADE_EXIT_COORDINATE_NAMES` — identical</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, `module_ml/config.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t xml:space="preserve">the turn's gate on a move and the gate inside a study ask one question of one set of numbers, so they read one measure</t>
+          <t xml:space="preserve">the serpentine search moves the two as one family and the evaluator leaves them out of a fit identity; a copy that drifts merges states whose fits differ, with wrong numbers and no error</t>
         </is>
       </c>
     </row>
@@ -13717,17 +13717,17 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timeframes()` — identical</t>
+          <t xml:space="preserve">`SELECTION_FOLD_MEASURE` — identical</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, `module_ml/config.py`</t>
         </is>
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t xml:space="preserve">both sides read the hierarchy off the asset's contract rather than off their own timeframe register, so a contract an older catalogue wrote reads the same on both</t>
+          <t xml:space="preserve">the turn's gate on a move and the gate inside a study ask one question of one set of numbers, so they read one measure</t>
         </is>
       </c>
     </row>
@@ -13739,17 +13739,17 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_request_json()`, `score_response_json()` — equal by value</t>
+          <t xml:space="preserve">`timeframes()` — identical</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, over its own `artifact_dir()`; `module_features/sub_module_serpentine_search/config.py`, over its module's</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`</t>
         </is>
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t xml:space="preserve">one side writes what the other reads: a boundary made of files needs both sides to name the same two, and neither module imports the other</t>
+          <t xml:space="preserve">both sides read the hierarchy off the asset's contract rather than off their own timeframe register, so a contract an older catalogue wrote reads the same on both</t>
         </is>
       </c>
     </row>
@@ -13761,7 +13761,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t xml:space="preserve">`parameters_json()` — equal by value</t>
+          <t xml:space="preserve">`score_request_json()`, `score_response_json()` — equal by value</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -13771,7 +13771,7 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t xml:space="preserve">the ML chain writes the tuned parameters the serpentine search starts from; the writer and the reader of a boundary name one artifact</t>
+          <t xml:space="preserve">one side writes what the other reads: a boundary made of files needs both sides to name the same two, and neither module imports the other</t>
         </is>
       </c>
     </row>
@@ -13783,17 +13783,17 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_feature_columns()` — equal by value</t>
+          <t xml:space="preserve">`parameters_json()` — equal by value</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/dataset.py`; `module_features/sub_module_serpentine_search/serpentine_search.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, over its own `artifact_dir()`; `module_features/sub_module_serpentine_search/config.py`, over its module's</t>
         </is>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset's feature set — the promoted file's columns in catalogue order, else the default set — is read by the chain that fits it and by the search that starts from it, and neither module imports the other</t>
+          <t xml:space="preserve">the ML chain writes the tuned parameters the serpentine search starts from; the writer and the reader of a boundary name one artifact</t>
         </is>
       </c>
     </row>
@@ -13805,17 +13805,17 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_set_json()`, `barriers_json()`, `hyperparameter_point_json()` — equal by value</t>
+          <t xml:space="preserve">`load_feature_columns()` — equal by value</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`, `module_features/sub_module_terminal/config.py`, each over its own `artifact_dir()` or its module's</t>
+          <t xml:space="preserve">`module_ml/dataset.py`; `module_features/sub_module_serpentine_search/serpentine_search.py`</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion writes the three, the ML chain reads them and the serpentine search the first two, and the features terminal names them on its promotion screen; the writer and the reader of a boundary must name one artifact, and the terminal cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the asset's feature set — the promoted file's columns in catalogue order, else the default set — is read by the chain that fits it and by the search that starts from it, and neither module imports the other</t>
         </is>
       </c>
     </row>
@@ -13827,17 +13827,17 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t xml:space="preserve">`theta()`, `state_key()` — identical</t>
+          <t xml:space="preserve">`feature_set_json()`, `barriers_json()`, `hyperparameter_point_json()` — equal by value</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_ml/score.py`</t>
+          <t xml:space="preserve">`module_ml/config.py`, `module_features/sub_module_serpentine_search/config.py`, `module_features/sub_module_terminal/config.py`, each over its own `artifact_dir()` or its module's</t>
         </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t xml:space="preserve">the serpentine search keys a state to know whether it has scored it, and the module that scores names the parent of a study by the same key: one differing separator and every answer would look like the answer to another question</t>
+          <t xml:space="preserve">the promotion writes the three, the ML chain reads them and the serpentine search the first two, and the features terminal names them on its promotion screen; the writer and the reader of a boundary must name one artifact, and the terminal cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13849,7 +13849,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t xml:space="preserve">`KIND_SCORE`, `KIND_HYPERPARAMETER` — identical</t>
+          <t xml:space="preserve">`theta()`, `state_key()` — identical</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -13859,7 +13859,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t xml:space="preserve">the two kinds of question: one side writes the word into a request and the other branches on it, so one word apart and every question would be answered as the other kind or refused</t>
+          <t xml:space="preserve">the serpentine search keys a state to know whether it has scored it, and the module that scores names the parent of a study by the same key: one differing separator and every answer would look like the answer to another question</t>
         </is>
       </c>
     </row>
@@ -13871,17 +13871,17 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t xml:space="preserve">`serpentine_search_json()`, `serpentine_search_trials_jsonl()`, `serpentine_search_profile_json()` — equal by value</t>
+          <t xml:space="preserve">`KIND_SCORE`, `KIND_HYPERPARAMETER` — identical</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, over its module's `artifact_dir()`; `module_features/sub_module_terminal/config.py`, over its own</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py`, `module_ml/score.py`</t>
         </is>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal reads the state and the ledger and writes the profile on the host's `python3`, and the sub-module's `config.py` imports the module's, which imports numpy</t>
+          <t xml:space="preserve">the two kinds of question: one side writes the word into a request and the other branches on it, so one word apart and every question would be answered as the other kind or refused</t>
         </is>
       </c>
     </row>
@@ -13893,17 +13893,17 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SERPENTINE_SEARCH_ROUND_LOOPS` — equal by value to the loops of `ROUND_SCHEDULE`</t>
+          <t xml:space="preserve">`serpentine_search_json()`, `serpentine_search_trials_jsonl()`, `serpentine_search_profile_json()` — equal by value</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_terminal/config.py`, written out; `ROUND_SCHEDULE` in `module_features/sub_module_serpentine_search/config.py`, its loops in their order</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/config.py`, over its module's `artifact_dir()`; `module_features/sub_module_terminal/config.py`, over its own</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t xml:space="preserve">the loops a round runs, in its order: the features terminal offers them to a draft, and it cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the features terminal reads the state and the ledger and writes the profile on the host's `python3`, and the sub-module's `config.py` imports the module's, which imports numpy</t>
         </is>
       </c>
     </row>
@@ -13915,17 +13915,17 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`, `PROMOTE_TARGET` — equal by value</t>
+          <t xml:space="preserve">`SERPENTINE_SEARCH_ROUND_LOOPS` — equal by value to the loops of `ROUND_SCHEDULE`</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONFIGURABLES records of `module_features/sub_module_serpentine_search/config.py`; constants of `module_features/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">`module_features/sub_module_terminal/config.py`, written out; `ROUND_SCHEDULE` in `module_features/sub_module_serpentine_search/config.py`, its loops in their order</t>
         </is>
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal offers the grid to a draft and opens its own screen for the promotion's target on the host's `python3`, and cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
+          <t xml:space="preserve">the loops a round runs, in its order: the features terminal offers them to a draft, and it cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13937,17 +13937,17 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t xml:space="preserve">`tui.py`, the whole file — the gum layer of every terminal</t>
+          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`, `PROMOTE_TARGET` — equal by value</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical to the byte in `module_data/sub_module_terminal/tui.py`, `module_features/sub_module_terminal/tui.py`, `module_ml/sub_module_terminal/tui.py`, `module_monitoring/sub_module_terminal/tui.py`, `module_skills/sub_module_terminal/tui.py`</t>
+          <t xml:space="preserve">CONFIGURABLES records of `module_features/sub_module_serpentine_search/config.py`; constants of `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t xml:space="preserve">one module speaks gum in each, and a package for what the terminals share would make every module import `module_skills` (`AGENTS.md` D02). It holds no sentence about a screen's content — a placeholder, a header and a state's words are the caller's; its own words are the block labels and the line naming the columns a narrow terminal leaves out — so each owner holds the file as its own local adapter</t>
+          <t xml:space="preserve">the features terminal offers the grid to a draft and opens its own screen for the promotion's target on the host's `python3`, and cannot import the sub-module's `config.py`, which imports numpy through the module's</t>
         </is>
       </c>
     </row>
@@ -13959,17 +13959,17 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OUTPUT_PLAIN` and the three conditions it reads — `NO_COLOR`, `TERM`, `sys.stdout.isatty()`</t>
+          <t xml:space="preserve">`tui.py`, the whole file — the gum layer of every terminal</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/config.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`, `module_skills/sub_module_terminal/config.py`</t>
+          <t xml:space="preserve">identical to the byte in `module_data/sub_module_terminal/tui.py`, `module_features/sub_module_terminal/tui.py`, `module_ml/sub_module_terminal/tui.py`, `module_monitoring/sub_module_terminal/tui.py`, `module_skills/sub_module_terminal/tui.py`</t>
         </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t xml:space="preserve">plain output follows the environment and is never a flag; each `tui.py` reads its own sub-module's `config.py`, and no module imports another</t>
+          <t xml:space="preserve">one module speaks gum in each, and a package for what the terminals share would make every module import `module_skills` (`AGENTS.md` D02). It holds no sentence about a screen's content — a placeholder, a header and a state's words are the caller's; its own words are the block labels and the line naming the columns a narrow terminal leaves out — so each owner holds the file as its own local adapter</t>
         </is>
       </c>
     </row>
@@ -13981,17 +13981,17 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t xml:space="preserve">the screen helpers `_option_rows()`, `_cancelled_exit_code()`, `_failure_exit_code()`</t>
+          <t xml:space="preserve">`OUTPUT_PLAIN` and the three conditions it reads — `NO_COLOR`, `TERM`, `sys.stdout.isatty()`</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`, `module_monitoring/sub_module_terminal/terminal.py`, `module_skills/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/config.py`, `module_features/sub_module_terminal/config.py`, `module_ml/sub_module_terminal/config.py`, `module_monitoring/sub_module_terminal/config.py`, `module_skills/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t xml:space="preserve">every terminal uses the same outcome and option conventions, and no terminal imports another module's code; a terminal that asks more than two forms keeps its own step helpers, in its own words</t>
+          <t xml:space="preserve">plain output follows the environment and is never a flag; each `tui.py` reads its own sub-module's `config.py`, and no module imports another</t>
         </is>
       </c>
     </row>
@@ -14003,7 +14003,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_make()`</t>
+          <t xml:space="preserve">the screen helpers `_option_rows()`, `_cancelled_exit_code()`, `_failure_exit_code()`</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -14013,7 +14013,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one call of make — a terminal starts a target through it and no other way, its lines uncaptured; it takes its arguments open, `_make(*arguments)`, so a target alone and a target with its asset — the promotion's among them — pass through one signature</t>
+          <t xml:space="preserve">every terminal uses the same outcome and option conventions, and no terminal imports another module's code; a terminal that asks more than two forms keeps its own step helpers, in its own words</t>
         </is>
       </c>
     </row>
@@ -14025,7 +14025,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()`</t>
+          <t xml:space="preserve">`_make()`</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -14035,7 +14035,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one reading of make — the menu is the Makefile's own targets, read from `make help` and filtered by the terminal's `MENU_TARGET_PATTERN`, so a terminal keeps no second list of them and a target gains its option by carrying a `##`</t>
+          <t xml:space="preserve">the one call of make — a terminal starts a target through it and no other way, its lines uncaptured; it takes its arguments open, `_make(*arguments)`, so a target alone and a target with its asset — the promotion's among them — pass through one signature</t>
         </is>
       </c>
     </row>
@@ -14047,7 +14047,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_target()`</t>
+          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()`</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -14057,7 +14057,7 @@
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t xml:space="preserve">one plan, one gate and one call for every target a menu offers; each owner holds its own local adapter with the same signature</t>
+          <t xml:space="preserve">the one reading of make — the menu is the Makefile's own targets, read from `make help` and filtered by the terminal's `MENU_TARGET_PATTERN`, so a terminal keeps no second list of them and a target gains its option by carrying a `##`</t>
         </is>
       </c>
     </row>
@@ -14069,17 +14069,17 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_tickers()`</t>
+          <t xml:space="preserve">`_write_target()`</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`, `module_monitoring/sub_module_terminal/terminal.py`, `module_skills/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three terminals whose module takes an asset read the assets `--tickers` names and ask for them only when a direct run named none; no module defines a basket of its own, and no terminal imports another module's code</t>
+          <t xml:space="preserve">one plan, one gate and one call for every target a menu offers; each owner holds its own local adapter with the same signature</t>
         </is>
       </c>
     </row>
@@ -14091,44 +14091,39 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_present()`</t>
+          <t xml:space="preserve">`_tickers()`</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_features/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t xml:space="preserve">the data and ML terminals answer whether an asset's file stands in the same word, and a terminal reads another module's files through none of that module's code</t>
+          <t xml:space="preserve">the three terminals whose module takes an asset read the assets `--tickers` names and ask for them only when a direct run named none; no module defines a basket of its own, and no terminal imports another module's code</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t xml:space="preserve">Terminals</t>
+          <t xml:space="preserve">Twice by extraction</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t xml:space="preserve">a module's terminal: the sub-module that shows what the module's stores hold — per asset where the module takes one — and starts one of the module's own targets through `make`; outside an action it creates no domain state, and it gates nothing</t>
+          <t xml:space="preserve">`_present()`</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_terminal` — `module_data/sub_module_terminal/`, `module_features/sub_module_terminal/`, `module_ml/sub_module_terminal/`, `module_monitoring/sub_module_terminal/` and the canon's `module_skills/sub_module_terminal/`, each `terminal.py` with `main()`, `config.py` and `tui.py`</t>
-        </is>
-      </c>
-      <c r="E327" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Data terminal; Features terminal; ML terminal; Monitoring terminal; Skills terminal</t>
-        </is>
-      </c>
-      <c r="F327" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a cockpit, a console, a dashboard; a second terminal in one module; a TUI that computes, schedules or gates; `&lt;module&gt;-tui`, `&lt;module&gt;-menu`; the crawler drawing a terminal of its own</t>
+          <t xml:space="preserve">identical in `module_data/sub_module_terminal/terminal.py`, `module_ml/sub_module_terminal/terminal.py`</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the data and ML terminals answer whether an asset's file stands in the same word, and a terminal reads another module's files through none of that module's code</t>
         </is>
       </c>
     </row>
@@ -14140,17 +14135,22 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t xml:space="preserve">a terminal's entry: the one make target that opens it, run by `python3` on the host and never in a container; it carries no `##`, so it is no option of any menu</t>
+          <t xml:space="preserve">a module's terminal: the sub-module that shows what the module's stores hold — per asset where the module takes one — and starts one of the module's own targets through `make`; outside an action it creates no domain state, and it gates nothing</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make data-terminal`, `make features-terminal`, `make ml-terminal`, `make monitoring-terminal`, `make skills-terminal`; the three whose module takes an asset given `--tickers` from `ASSET` or `TICKERS_CSV`</t>
+          <t xml:space="preserve">`sub_module_terminal` — `module_data/sub_module_terminal/`, `module_features/sub_module_terminal/`, `module_ml/sub_module_terminal/`, `module_monitoring/sub_module_terminal/` and the canon's `module_skills/sub_module_terminal/`, each `terminal.py` with `main()`, `config.py` and `tui.py`</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data terminal; Features terminal; ML terminal; Monitoring terminal; Skills terminal</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `##` on an entry; a `tmux-` twin of a terminal; `make tui`; a terminal started in a runner</t>
+          <t xml:space="preserve">a cockpit, a console, a dashboard; a second terminal in one module; a TUI that computes, schedules or gates; `&lt;module&gt;-tui`, `&lt;module&gt;-menu`; the crawler drawing a terminal of its own</t>
         </is>
       </c>
     </row>
@@ -14162,17 +14162,17 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t xml:space="preserve">a terminal's sources: what a terminal reads</t>
+          <t xml:space="preserve">a terminal's entry: the one make target that opens it, run by `python3` on the host and never in a container; it carries no `##`, so it is no option of any menu</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t xml:space="preserve">its own module's `config.py` where that is standard library — the data terminal's, with `lean.py`, and the ML terminal's; the features terminal its own `config.py`'s copies, `module_features/config.py` importing numpy; the monitoring terminal the snapshots through `STORE_STATUS_DIR` and `SNAPSHOT_FILE_NAMES` of its own `config.py`; the skills terminal the canon's `config.py` and, through the crawler's `config.py`, `vendors_for_crawling.toml` and the snapshot; every terminal `make help`</t>
+          <t xml:space="preserve">`make data-terminal`, `make features-terminal`, `make ml-terminal`, `make monitoring-terminal`, `make skills-terminal`; the three whose module takes an asset given `--tickers` from `ASSET` or `TICKERS_CSV`</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t xml:space="preserve">a snapshot read for freshness; duckdb; a store literal; another module's code; a third-party package</t>
+          <t xml:space="preserve">a `##` on an entry; a `tmux-` twin of a terminal; `make tui`; a terminal started in a runner</t>
         </is>
       </c>
     </row>
@@ -14184,22 +14184,17 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t xml:space="preserve">the menu: the options a terminal offers — one per target of the one Makefile that carries a `##` and whose name gives it to the terminal's module, then the terminal's own actions, `quit` last</t>
+          <t xml:space="preserve">a terminal's sources: what a terminal reads</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()` in each `terminal.py`; `MENU_TARGET_PATTERN` in each terminal's `config.py`; `_write_target()`</t>
-        </is>
-      </c>
-      <c r="E330" t="inlineStr">
-        <is>
-          <t xml:space="preserve">action</t>
+          <t xml:space="preserve">its own module's `config.py` where that is standard library — the data terminal's, with `lean.py`, and the ML terminal's; the features terminal its own `config.py`'s copies, `module_features/config.py` importing numpy; the monitoring terminal the snapshots through `STORE_STATUS_DIR` and `SNAPSHOT_FILE_NAMES` of its own `config.py`; the skills terminal the canon's `config.py` and, through the crawler's `config.py`, `vendors_for_crawling.toml` and the snapshot; every terminal `make help`</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second list of the targets in the program that opens the menu; a menu written out by hand; a target offered in a second terminal; the terminal's own entry among its options; `MODULE_TOKEN`, `STAGES`, `WRITES_BY_STAGE`, a target map; a grouping or a sorting of the targets; `run`, `exit`</t>
+          <t xml:space="preserve">a snapshot read for freshness; duckdb; a store literal; another module's code; a third-party package</t>
         </is>
       </c>
     </row>
@@ -14211,22 +14206,22 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset choice: the assets a run is about — the ones `--tickers` named, typed only when a direct run named none — then the one asset an action is for, one answered without asking</t>
+          <t xml:space="preserve">the menu: the options a terminal offers — one per target of the one Makefile that carries a `##` and whose name gives it to the terminal's module, then the terminal's own actions, `quit` last</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_tickers()` and its `gum_input` headed `asset`; `gum_choose` headed `asset` over those assets</t>
+          <t xml:space="preserve">`HELP_LINE_PATTERN`, `_target_rows()` in each `terminal.py`; `MENU_TARGET_PATTERN` in each terminal's `config.py`; `_write_target()`</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset</t>
+          <t xml:space="preserve">action</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t xml:space="preserve">a ticker typed where the launcher already named the set; a basket the terminal defines; a list of assets read from a store to fill it; a default basket in a module</t>
+          <t xml:space="preserve">a second list of the targets in the program that opens the menu; a menu written out by hand; a target offered in a second terminal; the terminal's own entry among its options; `MODULE_TOKEN`, `STAGES`, `WRITES_BY_STAGE`, a target map; a grouping or a sorting of the targets; `run`, `exit`</t>
         </is>
       </c>
     </row>
@@ -14238,22 +14233,22 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t xml:space="preserve">the plan and its gate: the choices, the `command` line verbatim and the target's purpose, then the question that runs or cancels</t>
+          <t xml:space="preserve">the asset choice: the assets a run is about — the ones `--tickers` named, typed only when a direct run named none — then the one asset an action is for, one answered without asking</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_target()`; the `command` line; `_make()`</t>
+          <t xml:space="preserve">`_tickers()` and its `gum_input` headed `asset`; `gum_choose` headed `asset` over those assets</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t xml:space="preserve">`target`, `purpose` and each variable as `parameter` and `value`; `command make &lt;target&gt; ASSET=&lt;TICKER&gt;`; `&lt;target&gt;?` with the target and `cancel`</t>
+          <t xml:space="preserve">asset</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage run before the gate; a gate that refuses what a hand confirms; `run`</t>
+          <t xml:space="preserve">a ticker typed where the launcher already named the set; a basket the terminal defines; a list of assets read from a store to fill it; a default basket in a module</t>
         </is>
       </c>
     </row>
@@ -14265,22 +14260,22 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t xml:space="preserve">the features terminal's own actions, the serpentine search's: draft the profile, read the recorded serpentine search, promote the proposal</t>
+          <t xml:space="preserve">the plan and its gate: the choices, the `command` line verbatim and the target's purpose, then the question that runs or cancels</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_write_search_profile()`, `_recorded_search_tables()`, `_write_promoted_proposal()` in `module_features/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">`_write_target()`; the `command` line; `_make()`</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t xml:space="preserve">draft; recorded search; `features-serpentine-search-promote`</t>
+          <t xml:space="preserve">`target`, `purpose` and each variable as `parameter` and `value`; `command make &lt;target&gt; ASSET=&lt;TICKER&gt;`; `&lt;target&gt;?` with the target and `cancel`</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t xml:space="preserve">`status` for the recorded search — the word is a stage's; a start of the serpentine search of its own — the search is the menu's `features-serpentine-search` or its `tmux-` twin; holdout, which the ML chain a promotion is followed by computes; a second menu after the action</t>
+          <t xml:space="preserve">a stage run before the gate; a gate that refuses what a hand confirms; `run`</t>
         </is>
       </c>
     </row>
@@ -14292,22 +14287,22 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t xml:space="preserve">the steps table: the steps of the features terminal's draft in order, above the step it asks — each answered DONE with its choice, the one asked CURRENT, the rest PENDING</t>
+          <t xml:space="preserve">the features terminal's own actions, the serpentine search's: draft the profile, read the recorded serpentine search, promote the proposal</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_step_rows()`, `_step_answer()`, `DRAFT_STEPS` in `module_features/sub_module_terminal/terminal.py`</t>
+          <t xml:space="preserve">`_write_search_profile()`, `_recorded_search_tables()`, `_write_promoted_proposal()` in `module_features/sub_module_terminal/terminal.py`</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t xml:space="preserve">step; state; choice; select now</t>
+          <t xml:space="preserve">draft; recorded search; `features-serpentine-search-promote`</t>
         </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t xml:space="preserve">workflow, wizard, stepper; the steps of two actions; a step asked when its one option answers it</t>
+          <t xml:space="preserve">`status` for the recorded search — the word is a stage's; a start of the serpentine search of its own — the search is the menu's `features-serpentine-search` or its `tmux-` twin; holdout, which the ML chain a promotion is followed by computes; a second menu after the action</t>
         </is>
       </c>
     </row>
@@ -14319,22 +14314,22 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one file a terminal writes</t>
+          <t xml:space="preserve">the steps table: the steps of the features terminal's draft in order, above the step it asks — each answered DONE with its choice, the one asked CURRENT, the rest PENDING</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t xml:space="preserve">`write_json()`, `serpentine_search_profile_json()` in `module_features/sub_module_terminal/config.py` — the features terminal's draft</t>
-        </is>
-      </c>
-      <c r="D335" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
+          <t xml:space="preserve">`_step_rows()`, `_step_answer()`, `DRAFT_STEPS` in `module_features/sub_module_terminal/terminal.py`</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t xml:space="preserve">step; state; choice; select now</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second file; a file in the sub-module's own folder</t>
+          <t xml:space="preserve">workflow, wizard, stepper; the steps of two actions; a step asked when its one option answers it</t>
         </is>
       </c>
     </row>
@@ -14346,22 +14341,22 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t xml:space="preserve">the target the features terminal opens its own screen for — the promotion, whose plan shows the one state it promotes</t>
+          <t xml:space="preserve">the one file a terminal writes</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t xml:space="preserve">`PROMOTE_TARGET` in `module_features/sub_module_terminal/config.py`</t>
-        </is>
-      </c>
-      <c r="E336" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the menu's `features-serpentine-search-promote`</t>
+          <t xml:space="preserve">`write_json()`, `serpentine_search_profile_json()` in `module_features/sub_module_terminal/config.py` — the features terminal's draft</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second named target; the module's stages listed beside it; a name for a target that runs bare</t>
+          <t xml:space="preserve">a second file; a file in the sub-module's own folder</t>
         </is>
       </c>
     </row>
@@ -14373,22 +14368,22 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t xml:space="preserve">the profile state: where the asset's profile stands against the serpentine search recorded under it — the one comparison the features terminal makes, on parsed objects and not on bytes</t>
+          <t xml:space="preserve">the target the features terminal opens its own screen for — the promotion, whose plan shows the one state it promotes</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t xml:space="preserve">`_profile_state()`</t>
+          <t xml:space="preserve">`PROMOTE_TARGET` in `module_features/sub_module_terminal/config.py`</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t xml:space="preserve">`not drafted` / `no search` / `matches the search` / `differs from the search`</t>
+          <t xml:space="preserve">the menu's `features-serpentine-search-promote`</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs_current`, which folds the parameters, the catalogue and the asset's own state and stays the page's</t>
+          <t xml:space="preserve">a second named target; the module's stages listed beside it; a name for a target that runs bare</t>
         </is>
       </c>
     </row>
@@ -14400,27 +14395,22 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t xml:space="preserve">the coordinate grid: what each coordinate is searched over, one preset, so a grid is a decision of the file and not of a form</t>
+          <t xml:space="preserve">the profile state: where the asset's profile stands against the serpentine search recorded under it — the one comparison the features terminal makes, on parsed objects and not on bytes</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`</t>
-        </is>
-      </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`grid_by_coordinate`</t>
+          <t xml:space="preserve">`_profile_state()`</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t xml:space="preserve">grid; points</t>
+          <t xml:space="preserve">`not drafted` / `no search` / `matches the search` / `differs from the search`</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t xml:space="preserve">a grid typed into a prompt; a point the terminal offers outside the preset</t>
+          <t xml:space="preserve">`inputs_current`, which folds the parameters, the catalogue and the asset's own state and stays the page's</t>
         </is>
       </c>
     </row>
@@ -14432,22 +14422,27 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t xml:space="preserve">gum: the terminal instrument the TUI speaks — `gum table --print`, `gum style`, `gum choose`, `gum input`; gum 2, a binary of the host</t>
+          <t xml:space="preserve">the coordinate grid: what each coordinate is searched over, one preset, so a grid is a decision of the file and not of a form</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t xml:space="preserve">`gum`, over `subprocess` in `tui.py` alone: `gum_table()`, `gum_style()`, `gum_choose()`, `gum_input()`, `_gum()`</t>
+          <t xml:space="preserve">`GRID_BY_COORDINATE_DEFAULT`</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`grid_by_coordinate`</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t xml:space="preserve">grid; points</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Python dependency, Rich among them; a chooser, a table or a colour written over curses or escape codes; a gum configuration in the tree; `gum spin`, `gum confirm`; `gum input` for a value the tree already holds, which is a selection and belongs to `gum choose`; gum's own pink and purple</t>
-        </is>
-      </c>
-      <c r="I339" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gum</t>
+          <t xml:space="preserve">a grid typed into a prompt; a point the terminal offers outside the preset</t>
         </is>
       </c>
     </row>
@@ -14459,22 +14454,22 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t xml:space="preserve">plain output: the screens without colour, symbol or border, chosen by the environment alone — `NO_COLOR` set and not empty, `TERM=dumb`, or standard output not a terminal</t>
+          <t xml:space="preserve">gum: the terminal instrument the TUI speaks — `gum table --print`, `gum style`, `gum choose`, `gum input`; gum 2, a binary of the host</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OUTPUT_PLAIN` in each terminal's `config.py`, read by its `tui.py`</t>
-        </is>
-      </c>
-      <c r="E340" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`[&lt;word&gt;]`</t>
+          <t xml:space="preserve">`gum`, over `subprocess` in `tui.py` alone: `gum_table()`, `gum_style()`, `gum_choose()`, `gum_input()`, `_gum()`</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t xml:space="preserve">a flag, `--no-color`, `--simple`, `--a11y`; a theme or a gum configuration in the tree; a meaning a colour alone carries</t>
+          <t xml:space="preserve">a Python dependency, Rich among them; a chooser, a table or a colour written over curses or escape codes; a gum configuration in the tree; `gum spin`, `gum confirm`; `gum input` for a value the tree already holds, which is a selection and belongs to `gum choose`; gum's own pink and purple</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gum</t>
         </is>
       </c>
     </row>
@@ -14486,22 +14481,22 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state word: the closed list of words that say how a step, a file or an action stands — its symbol and colour beside it in normal output, the word in brackets in plain output</t>
+          <t xml:space="preserve">plain output: the screens without colour, symbol or border, chosen by the environment alone — `NO_COLOR` set and not empty, `TERM=dumb`, or standard output not a terminal</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STATE_SYMBOLS`, `STATE_COLOURS`, `state_label()` in `tui.py`</t>
+          <t xml:space="preserve">`OUTPUT_PLAIN` in each terminal's `config.py`, read by its `tui.py`</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t xml:space="preserve">DONE; CURRENT; PENDING; CANCELLED; WARN; ERROR</t>
+          <t xml:space="preserve">`[&lt;word&gt;]`</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t xml:space="preserve">a colour or a symbol without its word; a coloured row; `ok`, `success` as a state word</t>
+          <t xml:space="preserve">a flag, `--no-color`, `--simple`, `--a11y`; a theme or a gum configuration in the tree; a meaning a colour alone carries</t>
         </is>
       </c>
     </row>
@@ -14513,44 +14508,49 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t xml:space="preserve">the failure block and the exits: a failure on stderr as what failed, where, why and what next, the run's last block — 0 an action done or cancelled, 1 a failure, 2 an unknown argument, 130 Ctrl-C</t>
+          <t xml:space="preserve">a state word: the closed list of words that say how a step, a file or an action stands — its symbol and colour beside it in normal output, the word in brackets in plain output</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t xml:space="preserve">`error_lines()`, `INTERRUPTED_EXIT_CODE` in `tui.py`; `_failure_exit_code()`, `_cancelled_exit_code()` in each `terminal.py`</t>
+          <t xml:space="preserve">`STATE_SYMBOLS`, `STATE_COLOURS`, `state_label()` in `tui.py`</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t xml:space="preserve">where; why; next; `nothing written`</t>
+          <t xml:space="preserve">DONE; CURRENT; PENDING; CANCELLED; WARN; ERROR</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t xml:space="preserve">a traceback for an expected failure; a failure on stdout; exit 0 after a failure</t>
+          <t xml:space="preserve">a colour or a symbol without its word; a coloured row; `ok`, `success` as a state word</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t xml:space="preserve">Artifacts</t>
+          <t xml:space="preserve">Terminals</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `ohlcv_1m_binance`, `ohlcv_1m_bybit`: one venue's minutes as printed, one partition per asset</t>
+          <t xml:space="preserve">the failure block and the exits: a failure on stderr as what failed, where, why and what next, the run's last block — 0 an action done or cancelled, 1 a failure, 2 an unknown argument, 130 Ctrl-C</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_&lt;venue&gt;/ticker=&lt;TICKER&gt;/ohlcv_1m_&lt;venue&gt;.parquet` and the family's `schema.json`; `venue_parquet()` in `module_data/config.py`</t>
-        </is>
-      </c>
-      <c r="G343" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume` — the venue's rows, ordered by every column, so a duplicate minute keeps one order; untracked</t>
+          <t xml:space="preserve">`error_lines()`, `INTERRUPTED_EXIT_CODE` in `tui.py`; `_failure_exit_code()`, `_cancelled_exit_code()` in each `terminal.py`</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t xml:space="preserve">where; why; next; `nothing written`</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a traceback for an expected failure; a failure on stdout; exit 0 after a failure</t>
         </is>
       </c>
     </row>
@@ -14562,17 +14562,17 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `ohlcv_1m_canonical`: the canonical 1m series, one partition per asset</t>
+          <t xml:space="preserve">the family `ohlcv_1m_binance`, `ohlcv_1m_bybit`: one venue's minutes as printed, one partition per asset</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_canonical/ticker=&lt;TICKER&gt;/ohlcv_1m_canonical.parquet` and the family's `schema.json`; `ohlcv_1m_canonical_parquet()`</t>
+          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_&lt;venue&gt;/ticker=&lt;TICKER&gt;/ohlcv_1m_&lt;venue&gt;.parquet` and the family's `schema.json`; `venue_parquet()` in `module_data/config.py`</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `source`, `zero_volume`, `binance_valid`, `bybit_valid`, `rel_divergence` — the full grid of the window, ordered by `timestamp_ms`; untracked</t>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume` — the venue's rows, ordered by every column, so a duplicate minute keeps one order; untracked</t>
         </is>
       </c>
     </row>
@@ -14584,17 +14584,17 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `bars`: the bars of every timeframe of the timeframe register, one partition per asset and timeframe</t>
+          <t xml:space="preserve">the family `ohlcv_1m_canonical`: the canonical 1m series, one partition per asset</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/bars.py` writes `bars/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/bars.parquet` and the family's `schema.json`; `bars_parquet()`</t>
+          <t xml:space="preserve">`module_data/ingest.py` writes `ohlcv_1m_canonical/ticker=&lt;TICKER&gt;/ohlcv_1m_canonical.parquet` and the family's `schema.json`; `ohlcv_1m_canonical_parquet()`</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `ffill_bars`, `zero_volume_bars` inside the research window, ordered by `timestamp_ms`; untracked</t>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `source`, `zero_volume`, `binance_valid`, `bybit_valid`, `rel_divergence` — the full grid of the window, ordered by `timestamp_ms`; untracked</t>
         </is>
       </c>
     </row>
@@ -14606,17 +14606,17 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `catalogue`: every catalogued column on the decision grid, one partition per asset and timeframe; a partition may omit a column the feature catalogue does not offer on its timeframe, never rename one or change its type</t>
+          <t xml:space="preserve">the family `bars`: the bars of every timeframe of the timeframe register, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/catalogue.py` writes `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet` and the family's `schema.json` from `catalogue_schema()`, the columns of the union of its partitions in catalogue order; `catalogue_parquet()` — in `module_ml/config.py` the same name over the contract's `parquet_by_timeframe`</t>
+          <t xml:space="preserve">`module_features/bars.py` writes `bars/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/bars.parquet` and the family's `schema.json`; `bars_parquet()`</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts` and every definition offered on the partition's timeframe, on the decision grid; untracked</t>
+          <t xml:space="preserve">`timestamp_ms`, `open`, `high`, `low`, `close`, `volume`, `ffill_bars`, `zero_volume_bars` inside the research window, ordered by `timestamp_ms`; untracked</t>
         </is>
       </c>
     </row>
@@ -14628,17 +14628,17 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `labels`: Y on the decision timeframe, one partition per asset and timeframe</t>
+          <t xml:space="preserve">the family `catalogue`: every catalogued column on the decision grid, one partition per asset and timeframe; a partition may omit a column the feature catalogue does not offer on its timeframe, never rename one or change its type</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/labels.py` writes `labels/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/labels.parquet` and the family's `schema.json`; `labels_parquet()`</t>
+          <t xml:space="preserve">`module_features/catalogue.py` writes `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet` and the family's `schema.json` from `catalogue_schema()`, the columns of the union of its partitions in catalogue order; `catalogue_parquet()` — in `module_ml/config.py` the same name over the contract's `parquet_by_timeframe`</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts`, `entry_ts`, `y`, `event_end_ts`, `entry_observable`, `label_valid`, `entry_price`, `upper_barrier`, `lower_barrier`; an ambiguous event carries `y = 0` with `label_valid = false`, so `y` is never read without `label_valid`; untracked</t>
+          <t xml:space="preserve">`decision_ts` and every definition offered on the partition's timeframe, on the decision grid; untracked</t>
         </is>
       </c>
     </row>
@@ -14650,17 +14650,17 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t xml:space="preserve">the family `oos_predictions`: the out-of-sample class probabilities, one partition per asset and timeframe</t>
+          <t xml:space="preserve">the family `labels`: Y on the decision timeframe, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/train.py` writes `oos_predictions/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/oos_predictions.parquet` and the family's `schema.json`; `oos_predictions_parquet()`</t>
+          <t xml:space="preserve">`module_ml/labels.py` writes `labels/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/labels.parquet` and the family's `schema.json`; `labels_parquet()`</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t xml:space="preserve">`decision_ts`, `oos_fold_id`, `p_short`, `p_neutral`, `p_long` — the full window of every validation fold and of the final holdout; metrics score only the supervised subset; untracked</t>
+          <t xml:space="preserve">`decision_ts`, `entry_ts`, `y`, `event_end_ts`, `entry_observable`, `label_valid`, `entry_price`, `upper_barrier`, `lower_barrier`; an ambiguous event carries `y = 0` with `label_valid = false`, so `y` is never read without `label_valid`; untracked</t>
         </is>
       </c>
     </row>
@@ -14672,17 +14672,17 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_README.md`</t>
+          <t xml:space="preserve">the family `oos_predictions`: the out-of-sample class probabilities, one partition per asset and timeframe</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/status.py` writes it, `asset_readme_md()`; its file list `file_manifest()`, the three files of `HAND_STAGE_FILE_DESCRIPTORS` listed with no size</t>
+          <t xml:space="preserve">`module_ml/train.py` writes `oos_predictions/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/oos_predictions.parquet` and the family's `schema.json`; `oos_predictions_parquet()`</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t xml:space="preserve">what the folder holds and what came out of it; no timestamp; tracked</t>
+          <t xml:space="preserve">`decision_ts`, `oos_fold_id`, `p_short`, `p_neutral`, `p_long` — the full window of every validation fold and of the final holdout; metrics score only the supervised subset; untracked</t>
         </is>
       </c>
     </row>
@@ -14694,17 +14694,17 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_barriers.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_README.md`</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `barriers_json()`; `load_barriers()` in `module_ml/dataset.py` reads it</t>
+          <t xml:space="preserve">`module_ml/status.py` writes it, `asset_readme_md()`; its file list `file_manifest()`, the three files of `HAND_STAGE_FILE_DESCRIPTORS` listed with no size</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t xml:space="preserve">`label_barrier_true_range_multiplier`, `label_horizon`, `take_profit_true_range_multiplier`, `stop_loss_true_range_multiplier` — the asset's promoted barrier geometry, a hand's choice; absent, `START_BY_COORDINATE_DEFAULT` of `module_ml/config.py` is the asset's; tracked once promoted, like the feature set beside it</t>
+          <t xml:space="preserve">what the folder holds and what came out of it; no timestamp; tracked</t>
         </is>
       </c>
     </row>
@@ -14716,17 +14716,17 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_barriers.json`</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/catalogue.py` writes it from `catalogue_contract()`; `catalogue_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `barriers_json()`; `load_barriers()` in `module_ml/dataset.py` reads it</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature layer's contract the ML layer reads instead of the feature configuration: `decision_timeframe`, `timeframes` (each `timeframe`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe` — each value a path relative to the artifacts store, `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet`; untracked</t>
+          <t xml:space="preserve">`label_barrier_true_range_multiplier`, `label_horizon`, `take_profit_true_range_multiplier`, `stop_loss_true_range_multiplier` — the asset's promoted barrier geometry, a hand's choice; absent, `START_BY_COORDINATE_DEFAULT` of `module_ml/config.py` is the asset's; tracked once promoted, like the feature set beside it</t>
         </is>
       </c>
     </row>
@@ -14738,17 +14738,17 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `feature_set_json()`</t>
+          <t xml:space="preserve">`module_features/catalogue.py` writes it from `catalogue_contract()`; `catalogue_json()`</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t xml:space="preserve">`columns_by_timeframe` — the promoted feature set, a hand's choice, and nothing else; absent, the default set is the asset's; tracked once promoted, like the parameters it conditions</t>
+          <t xml:space="preserve">the feature layer's contract the ML layer reads instead of the feature configuration: `decision_timeframe`, `timeframes` (each `timeframe`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe` — each value a path relative to the artifacts store, `catalogue/ticker=&lt;TICKER&gt;/timeframe=&lt;timeframe&gt;/catalogue.parquet`; untracked</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_hyperparameter_point.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_feature_set.json`</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `hyperparameter_point_json()`; `hpo.main()` in `module_ml/hpo.py` reads it</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `feature_set_json()`</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t xml:space="preserve">`best_params` — the promoted hyper-parameter point, a hand's choice: the first trial of the chain's study, and nothing else; absent, the study draws every point; tracked once promoted, like the feature set and the geometry beside it</t>
+          <t xml:space="preserve">`columns_by_timeframe` — the promoted feature set, a hand's choice, and nothing else; absent, the default set is the asset's; tracked once promoted, like the parameters it conditions</t>
         </is>
       </c>
     </row>
@@ -14782,17 +14782,17 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_model_evaluation.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_hyperparameter_point.json`</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/train.py` writes it; `model_evaluation_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/promote.py` writes it; `hyperparameter_point_json()`; `hpo.main()` in `module_ml/hpo.py` reads it</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t xml:space="preserve">`validation` — a `fold_&lt;id&gt;` per fold of `VALIDATION_FOLD_IDS` — and `final_holdout`, each `prior_logloss`, `model_logloss`, `relative_logloss_skill`, `scored_row_count`; `validation_importance`, a `fold_&lt;id&gt;` per validation fold, each `gain_importance` and `mean_abs_shap_importance` per column; `feature_columns`; `class_counts`, `labels`, `segments`; untracked</t>
+          <t xml:space="preserve">`best_params` — the promoted hyper-parameter point, a hand's choice: the first trial of the chain's study, and nothing else; absent, the study draws every point; tracked once promoted, like the feature set and the geometry beside it</t>
         </is>
       </c>
     </row>
@@ -14804,17 +14804,17 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_parameters.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_model_evaluation.json`</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/hpo.py` writes it; `parameters_json()`</t>
+          <t xml:space="preserve">`module_ml/train.py` writes it; `model_evaluation_json()`</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t xml:space="preserve">`hyperparameter_search_result` (`best_params`, `best_cagr_validation_path`, `trial_count`); tracked</t>
+          <t xml:space="preserve">`validation` — a `fold_&lt;id&gt;` per fold of `VALIDATION_FOLD_IDS` — and `final_holdout`, each `prior_logloss`, `model_logloss`, `relative_logloss_skill`, `scored_row_count`; `validation_importance`, a `fold_&lt;id&gt;` per validation fold, each `gain_importance` and `mean_abs_shap_importance` per column; `feature_columns`; `class_counts`, `labels`, `segments`; untracked</t>
         </is>
       </c>
     </row>
@@ -14826,27 +14826,17 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_score_request.json`: the serpentine search's question</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_parameters.json`</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_request_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by a turn, `features-serpentine-turn`, read by `module_ml.score`, `ml-score`; the one file the loop of `features-serpentine-search` tests, running `ml-score` and a turn again while it exists</t>
-        </is>
-      </c>
-      <c r="D356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`kind` (`score` or `hpo`), `round`, `states`</t>
-        </is>
-      </c>
-      <c r="F356" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a key beside these three; a request the evaluator writes; a second file the loop tests</t>
+          <t xml:space="preserve">`module_ml/hpo.py` writes it; `parameters_json()`</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t xml:space="preserve">what one family pass asks to be scored: the kind of scoring, the round it runs in, and the states — a state of its own for `score`, a beam parent's scored row for `hpo`; untracked</t>
+          <t xml:space="preserve">`hyperparameter_search_result` (`best_params`, `best_cagr_validation_path`, `trial_count`); tracked</t>
         </is>
       </c>
     </row>
@@ -14858,27 +14848,27 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_score_response.json`: the serpentine search's answer</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_score_request.json`: the serpentine search's question</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`score_response_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by `module_ml.score` alone</t>
+          <t xml:space="preserve">`score_request_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by a turn, `features-serpentine-turn`, read by `module_ml.score`, `ml-score`; the one file the loop of `features-serpentine-search` tests, running `ml-score` and a turn again while it exists</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t xml:space="preserve">`kind`, `round`, `results`; a `score` result the row of one scored state of the serpentine search, an `hpo` result `state_key`, `trial_count_drawn` and `candidate`</t>
+          <t xml:space="preserve">`kind` (`score` or `hpo`), `round`, `states`</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">a key beside these three; a result out of the order the request named; a response written before every state has one</t>
+          <t xml:space="preserve">a key beside these three; a request the evaluator writes; a second file the loop tests</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t xml:space="preserve">what the states of one request are worth, in the order the request named them; `candidate` a scored row or `null`, and `null` is an answer; untracked</t>
+          <t xml:space="preserve">what one family pass asks to be scored: the kind of scoring, the round it runs in, and the states — a state of its own for `score`, a beam parent's scored row for `hpo`; untracked</t>
         </is>
       </c>
     </row>
@@ -14890,17 +14880,27 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_score_response.json`: the serpentine search's answer</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_json()`</t>
+          <t xml:space="preserve">`score_response_json()` in `module_ml/config.py` and `module_features/sub_module_serpentine_search/config.py`; written by `module_ml.score` alone</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`kind`, `round`, `results`; a `score` result the row of one scored state of the serpentine search, an `hpo` result `state_key`, `trial_count_drawn` and `candidate`</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a key beside these three; a result out of the order the request named; a response written before every state has one</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs`, `beam`, `champion_trial_index`, `round_count`, `search_converged`, `path` (each `round`, `loop`, `family`, `trial_index`, `beam`, `move`), `proposals` (each `proposal`, `trial_index`), `trial_count_by_loop` — where the search stands at a round boundary, naming trials by index and carrying none of their columns; tracked once a search has run</t>
+          <t xml:space="preserve">what the states of one request are worth, in the order the request named them; `candidate` a scored row or `null`, and `null` is an answer; untracked</t>
         </is>
       </c>
     </row>
@@ -14912,17 +14912,17 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search.json`</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hand, in the file or through the features terminal's draft; `serpentine_search_profile_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_json()`</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t xml:space="preserve">`columns_admitted_by_timeframe`, `start_columns_by_timeframe` (`null` = the asset's own set), `grid_by_coordinate` (one list per coordinate, in the order it is searched), `loops` (a subset of `SERPENTINE_SEARCH_ROUND_LOOPS`), `path_cagr_noise_standard_deviation` (the asset's noise sigma, `null` on the calibration run) — what a hand asks the serpentine search to look at; drafted, never derived, and tracked</t>
+          <t xml:space="preserve">`inputs`, `beam`, `champion_trial_index`, `round_count`, `search_converged`, `path` (each `round`, `loop`, `family`, `trial_index`, `beam`, `move`), `proposals` (each `proposal`, `trial_index`), `trial_count_by_loop` — where the search stands at a round boundary, naming trials by index and carrying none of their columns; tracked once a search has run</t>
         </is>
       </c>
     </row>
@@ -14934,17 +14934,17 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_trials.jsonl`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_profile.json`</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_trials_jsonl()`</t>
+          <t xml:space="preserve">a hand, in the file or through the features terminal's draft; `serpentine_search_profile_json()`</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t xml:space="preserve">one scored state of the serpentine search a line, appended and never rewritten; `trial_index` = the line number, counted from one; tracked once a search has run</t>
+          <t xml:space="preserve">`columns_admitted_by_timeframe`, `start_columns_by_timeframe` (`null` = the asset's own set), `grid_by_coordinate` (one list per coordinate, in the order it is searched), `loops` (a subset of `SERPENTINE_SEARCH_ROUND_LOOPS`), `path_cagr_noise_standard_deviation` (the asset's noise sigma, `null` on the calibration run) — what a hand asks the serpentine search to look at; drafted, never derived, and tracked</t>
         </is>
       </c>
     </row>
@@ -14956,49 +14956,39 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_strategy_evaluation.json`</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_serpentine_search_trials.jsonl`</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_ml/strategy.py` writes it; `strategy_evaluation_json()`</t>
+          <t xml:space="preserve">`module_features/sub_module_serpentine_search/serpentine_search.py` writes it; `serpentine_search_trials_jsonl()`</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t xml:space="preserve">`entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `cleared_point_count`, `median_cagr_over_cleared`, `max_cagr_over_cleared`, `selection_score_cagr_validation_path`, `execution_cost_rate_per_trade_side`; per fold `sharpe`, `cagr`, `max_drawdown`, `calmar`, `profit_factor`, `trade_count`, `hit_rate`, `average_trade_return`, `exposure`, `exit_counts`, `final_equity`; `validation_path` over the validation folds; the final holdout's `equity_curve`; untracked</t>
+          <t xml:space="preserve">one scored state of the serpentine search a line, appended and never rewritten; `trial_index` = the line number, counted from one; tracked once a search has run</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Features</t>
+          <t xml:space="preserve">Artifacts</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t xml:space="preserve">a series of one timeframe's bars, with no parameter</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_strategy_evaluation.json`</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t xml:space="preserve">`open`, `high`, `low`, `close`, `volume` — a bar column — and the series with a kernel: `logarithmic_volume`, `true_range`, `cumulative_signed_volume`; `SERIES_KERNELS`, `module_features/indicators.py`</t>
-        </is>
-      </c>
-      <c r="D362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`inputs` of a term</t>
-        </is>
-      </c>
-      <c r="E362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the series token</t>
-        </is>
-      </c>
-      <c r="F362" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a series with a parameter; `log_volume`</t>
+          <t xml:space="preserve">`module_ml/strategy.py` writes it; `strategy_evaluation_json()`</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`entry_edge_threshold`, `entry_edge_threshold_constraint_met`, `cleared_point_count`, `median_cagr_over_cleared`, `max_cagr_over_cleared`, `selection_score_cagr_validation_path`, `execution_cost_rate_per_trade_side`; per fold `sharpe`, `cagr`, `max_drawdown`, `calmar`, `profit_factor`, `trade_count`, `hit_rate`, `average_trade_return`, `exposure`, `exit_counts`, `final_equity`; `validation_path` over the validation folds; the final holdout's `equity_curve`; untracked</t>
         </is>
       </c>
     </row>
@@ -15010,32 +15000,27 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t xml:space="preserve">an indicator — one computation with exactly one integer parameter, named by its token, its invariants one record of the register beside its kernel, the popular names it answers to among them</t>
+          <t xml:space="preserve">a series of one timeframe's bars, with no parameter</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`exponential_smoothing&lt;n&gt;`, `rolling_mean&lt;n&gt;`, `recursive_mean&lt;n&gt;`, `recursive_mean_gain_share&lt;n&gt;`, `rolling_standard_score&lt;n&gt;`, `rolling_range_position&lt;n&gt;`, `rolling_standard_deviation&lt;n&gt;`, `relative_change&lt;n&gt;`, `recursive_mean_upward_movement_share&lt;n&gt;`, `recursive_mean_directional_movement_imbalance&lt;n&gt;`, `rolling_volume_weighted_mean&lt;n&gt;`, `rolling_volume_weighted_close_location&lt;n&gt;`, `rolling_money_flow_gain_share&lt;n&gt;`; `INDICATORS` — `kernel`, `parameter_word`, `warmup_multiple`, `inputs`, `output_range`, `historical_aliases` of a record, `module_features/indicators.py`</t>
+          <t xml:space="preserve">`open`, `high`, `low`, `close`, `volume` — a bar column — and the series with a kernel: `logarithmic_volume`, `true_range`, `cumulative_signed_volume`; `SERIES_KERNELS`, `module_features/indicators.py`</t>
         </is>
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`indicator`, `parameter_word`, `parameter_bars`, `output_range`, `historical_aliases` of a term</t>
+          <t xml:space="preserve">`inputs` of a term</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t xml:space="preserve">the token with its parameter, `&lt;PARAMETER_WORD&gt; &lt;n&gt; bars of &lt;inputs&gt;` beside it and `output &lt;low&gt;–&lt;high&gt;` when the indicator is bounded (the catalogue table's terms)</t>
+          <t xml:space="preserve">the series token</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">`rsi_14`, `sma_200`, `bb20`; a table of indicator facts in `config.py` beside the register; `kernel` for anything but the function a record computes with; the abbreviations these tokens replaced: `ema`, `sma`, `rsi`, `atr`, `zscore`, `rolling_zscore`, `wilder_smoothing`, `range_position`</t>
-        </is>
-      </c>
-      <c r="I363" t="inlineStr">
-        <is>
-          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
+          <t xml:space="preserve">a series with a parameter; `log_volume`</t>
         </is>
       </c>
     </row>
@@ -15047,27 +15032,32 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t xml:space="preserve">a term — a series or an indicator inside a feature definition</t>
+          <t xml:space="preserve">an indicator — one computation with exactly one integer parameter, named by its token, its invariants one record of the register beside its kernel, the popular names it answers to among them</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t xml:space="preserve">`("&lt;indicator&gt;", &lt;parameter_bars&gt;)` on the default series close, `("&lt;series&gt;", "&lt;indicator&gt;", &lt;parameter_bars&gt;)` on another series, `("&lt;series&gt;",)` a bare series; `term_name()`</t>
+          <t xml:space="preserve">`exponential_smoothing&lt;n&gt;`, `rolling_mean&lt;n&gt;`, `recursive_mean&lt;n&gt;`, `recursive_mean_gain_share&lt;n&gt;`, `rolling_standard_score&lt;n&gt;`, `rolling_range_position&lt;n&gt;`, `rolling_standard_deviation&lt;n&gt;`, `relative_change&lt;n&gt;`, `recursive_mean_upward_movement_share&lt;n&gt;`, `recursive_mean_directional_movement_imbalance&lt;n&gt;`, `rolling_volume_weighted_mean&lt;n&gt;`, `rolling_volume_weighted_close_location&lt;n&gt;`, `rolling_money_flow_gain_share&lt;n&gt;`; `INDICATORS` — `kernel`, `parameter_word`, `warmup_multiple`, `inputs`, `output_range`, `historical_aliases` of a record, `module_features/indicators.py`</t>
         </is>
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t xml:space="preserve">`terms`</t>
+          <t xml:space="preserve">`indicator`, `parameter_word`, `parameter_bars`, `output_range`, `historical_aliases` of a term</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t xml:space="preserve">terms</t>
+          <t xml:space="preserve">the token with its parameter, `&lt;PARAMETER_WORD&gt; &lt;n&gt; bars of &lt;inputs&gt;` beside it and `output &lt;low&gt;–&lt;high&gt;` when the indicator is bounded (the catalogue table's terms)</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t xml:space="preserve">atom</t>
+          <t xml:space="preserve">`rsi_14`, `sma_200`, `bb20`; a table of indicator facts in `config.py` beside the register; `kernel` for anything but the function a record computes with; an abbreviation for a token: `ema`, `sma`, `rsi`, `atr`, `zscore`, `rolling_zscore`, `wilder_smoothing`, `range_position`</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
         </is>
       </c>
     </row>
@@ -15079,32 +15069,27 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t xml:space="preserve">a feature definition — terms of one timeframe composed by the operators, with an optional normaliser; the timeframe-less half of a feature, carrying the tier it belongs to and the popular names that denote the whole of it</t>
+          <t xml:space="preserve">a term — a series or an indicator inside a feature definition</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t xml:space="preserve">one record of `FEATURE_CATALOGUE`; `feature_definition_name()`; `OPERATORS` = {`minus`, `over`} and `NORMALISERS` = {`centered`}, one record per token beside its kernel in `module_features/catalogue.py`</t>
+          <t xml:space="preserve">`("&lt;indicator&gt;", &lt;parameter_bars&gt;)` on the default series close, `("&lt;series&gt;", "&lt;indicator&gt;", &lt;parameter_bars&gt;)` on another series, `("&lt;series&gt;",)` a bare series; `term_name()`</t>
         </is>
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_definition`, `tier` = `CORE` / `EXTENDED` / `COMPOSITE`, `historical_aliases`</t>
+          <t xml:space="preserve">`terms`</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t xml:space="preserve">definition (the catalogue table)</t>
+          <t xml:space="preserve">terms</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t xml:space="preserve">molecule, family, feature family, indicator (for a composite); `trend`, `momentum`, `volatility`, `structure`, `activity` — a category, not a computation; a popular name as the key, the column or a second name beside the canonical one; a tier written anywhere but the record; `centred` — the normaliser token keeps its American spelling, a column and a key on disk</t>
-        </is>
-      </c>
-      <c r="I365" t="inlineStr">
-        <is>
-          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
+          <t xml:space="preserve">atom</t>
         </is>
       </c>
     </row>
@@ -15116,27 +15101,32 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t xml:space="preserve">a feature — a definition aligned to the decision grid on one timeframe; the column of X and the key of an importance</t>
+          <t xml:space="preserve">a feature definition — terms of one timeframe composed by the operators, with an optional normaliser; the timeframe-less half of a feature, carrying the tier it belongs to and the popular names that denote the whole of it</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_id()` = `&lt;definition&gt;_&lt;timeframe&gt;`</t>
+          <t xml:space="preserve">one record of `FEATURE_CATALOGUE`; `feature_definition_name()`; `OPERATORS` = {`minus`, `over`} and `NORMALISERS` = {`centered`}, one record per token beside its kernel in `module_features/catalogue.py`</t>
         </is>
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t xml:space="preserve">`feature_columns`, the keys of an importance</t>
+          <t xml:space="preserve">`feature_definition`, `tier` = `CORE` / `EXTENDED` / `COMPOSITE`, `historical_aliases`</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature id — `column &lt;timeframe&gt;` in the FEATURE SET frame</t>
+          <t xml:space="preserve">definition (the catalogue table)</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
+          <t xml:space="preserve">molecule, family, feature family, indicator (for a composite); `trend`, `momentum`, `volatility`, `structure`, `activity` — a category, not a computation; a popular name as the key, the column or a second name beside the canonical one; a tier written anywhere but the record; `centred` — the normaliser token keeps its American spelling, a column and a key on disk</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t xml:space="preserve">technical analysis — the popular names, in `historical_aliases` alone</t>
         </is>
       </c>
     </row>
@@ -15148,27 +15138,27 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature catalogue — every definition the repository can compute, with the timeframes it is offered on; drafted, like the rest of `config.py`</t>
+          <t xml:space="preserve">a feature — a definition aligned to the decision grid on one timeframe; the column of X and the key of an importance</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t xml:space="preserve">`FEATURE_CATALOGUE`, `catalogue_columns()`, `CATALOGUE_COLUMNS`; the stage `features-catalogue`, `module_features/catalogue.py`</t>
+          <t xml:space="preserve">`feature_id()` = `&lt;definition&gt;_&lt;timeframe&gt;`</t>
         </is>
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue` (of `features_status.json`); `&lt;TICKER&gt;_catalogue.json`; the family `catalogue`</t>
+          <t xml:space="preserve">`feature_columns`, the keys of an importance</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t xml:space="preserve">CATALOGUE</t>
+          <t xml:space="preserve">the feature id — `column &lt;timeframe&gt;` in the FEATURE SET frame</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t xml:space="preserve">palette, feature list, feature store</t>
+          <t xml:space="preserve">a column literal in a page script; a parquet column with a timeframe (the partition `timeframe=&lt;timeframe&gt;/` carries it)</t>
         </is>
       </c>
     </row>
@@ -15180,22 +15170,27 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t xml:space="preserve">the feature layer's contract, per asset — what the ML layer reads instead of this module's configuration</t>
+          <t xml:space="preserve">the feature catalogue — every definition the repository can compute, with the timeframes it is offered on; drafted, like the rest of `config.py`</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t xml:space="preserve">`catalogue_contract()`, `catalogue_json()` in `module_features/config.py`; the descriptor's copy in `module_ml/config.py`; `load_catalogue()` in `module_ml/dataset.py`, `cat`</t>
+          <t xml:space="preserve">`FEATURE_CATALOGUE`, `catalogue_columns()`, `CATALOGUE_COLUMNS`; the stage `features-catalogue`, `module_features/catalogue.py`</t>
         </is>
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`: `decision_timeframe`, `timeframes` (`timeframe`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe`</t>
+          <t xml:space="preserve">`catalogue` (of `features_status.json`); `&lt;TICKER&gt;_catalogue.json`; the family `catalogue`</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CATALOGUE</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t xml:space="preserve">an import of `module_features` from `module_ml`; a token or a slot parsed in the ML layer; a second read of the file inside one stage; a path built from the slot grammar outside `module_features`; a parquet named in the contract by anything but its path relative to the artifact store</t>
+          <t xml:space="preserve">palette, feature list, feature store</t>
         </is>
       </c>
     </row>
@@ -15207,27 +15202,22 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t xml:space="preserve">the effective history — what a parameter covers on a timeframe, `bars × timeframe`, the quantity the nesting rule compares</t>
+          <t xml:space="preserve">the feature layer's contract, per asset — what the ML layer reads instead of this module's configuration</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t xml:space="preserve">`definition_effective_history_hours()`</t>
+          <t xml:space="preserve">`catalogue_contract()`, `catalogue_json()` in `module_features/config.py`; the descriptor's copy in `module_ml/config.py`; `load_catalogue()` in `module_ml/dataset.py`, `cat`</t>
         </is>
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t xml:space="preserve">`effective_history_hours_by_timeframe`; `lower_longest_effective_history_hours`, `upper_shortest_effective_history_hours` of `nesting`</t>
-        </is>
-      </c>
-      <c r="E369" t="inlineStr">
-        <is>
-          <t xml:space="preserve">effective history</t>
+          <t xml:space="preserve">`&lt;TICKER&gt;_catalogue.json`: `decision_timeframe`, `timeframes` (`timeframe`, `duration_ms`), `warmup_top_timeframe_bars`, `warmup_end_ms`, `columns_by_timeframe`, `default_columns_by_timeframe`, `parquet_by_timeframe`</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t xml:space="preserve">history (bare — a recursion has no window), span (the parameter word of an exponential smoothing), lookback hours</t>
+          <t xml:space="preserve">an import of `module_features` from `module_ml`; a token or a slot parsed in the ML layer; a second read of the file inside one stage; a path built from the slot grammar outside `module_features`; a parquet named in the contract by anything but its path relative to the artifact store</t>
         </is>
       </c>
     </row>
@@ -15239,22 +15229,27 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t xml:space="preserve">the Bollinger %b reading — the trade's %b(20, 2σ), `rolling_standard_score20` / 4 + 0.5, an affine map a tree model is invariant to, so no %b column exists</t>
+          <t xml:space="preserve">the effective history — what a parameter covers on a timeframe, `bars × timeframe`, the quantity the nesting rule compares</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`definition_effective_history_hours()`</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`effective_history_hours_by_timeframe`; `lower_longest_effective_history_hours`, `upper_shortest_effective_history_hours` of `nesting`</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t xml:space="preserve">— (no page shows it; Bollinger %b in the definitions table of `methodology_features.md`)</t>
+          <t xml:space="preserve">effective history</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t xml:space="preserve">`bb20`, `%b` as a column, `z / 2 + 0.5`; `zscore20`</t>
-        </is>
-      </c>
-      <c r="I370" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bollinger (technical analysis)</t>
+          <t xml:space="preserve">history (bare — a recursion has no window), span (the parameter word of an exponential smoothing), lookback hours</t>
         </is>
       </c>
     </row>
@@ -15266,27 +15261,22 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t xml:space="preserve">the definitions an asset's model sees until a promotion — the frozen experiment's default definitions on every timeframe of the register, in the order it stacks them</t>
-        </is>
-      </c>
-      <c r="C371" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME`; `definition_in_default_set` of a record</t>
-        </is>
-      </c>
-      <c r="D371" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`definition_in_default_set`; `default_columns_by_timeframe` of the contract</t>
+          <t xml:space="preserve">the Bollinger %b reading — the trade's %b(20, 2σ), `rolling_standard_score20` / 4 + 0.5, an affine map a tree model is invariant to, so no %b column exists</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t xml:space="preserve">default set</t>
+          <t xml:space="preserve">— (no page shows it; Bollinger %b in the definitions table of `methodology_features.md`)</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t xml:space="preserve">the frozen fifteen (as a name)</t>
+          <t xml:space="preserve">`bb20`, `%b` as a column, `z / 2 + 0.5`; `zscore20`</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bollinger (technical analysis)</t>
         </is>
       </c>
     </row>
@@ -15298,49 +15288,59 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t xml:space="preserve">the definition the strategy hierarchy reads on every timeframe, set or no set</t>
+          <t xml:space="preserve">the definitions an asset's model sees until a promotion — the frozen experiment's default definitions on every timeframe of the register, in the order it stacks them</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TREND_GATE_FEATURE_DEFINITION` in `module_ml/config.py` — the name of the catalogue's first definition, owned by the strategy that reads it; the gate's timeframe is the top of the contract's hierarchy, `trend_gate_timeframe(cat)`</t>
+          <t xml:space="preserve">`DEFAULT_FEATURE_COLUMNS_BY_TIMEFRAME`; `definition_in_default_set` of a record</t>
         </is>
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t xml:space="preserve">`trend_gate_feature`</t>
+          <t xml:space="preserve">`definition_in_default_set`; `default_columns_by_timeframe` of the contract</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t xml:space="preserve">gate (the asset's STRATEGY frame)</t>
+          <t xml:space="preserve">default set</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t xml:space="preserve">`TREND_FAMILY`; a column literal in `asset.js`; a second copy of the name in the feature layer, which reads nothing of it</t>
+          <t xml:space="preserve">the frozen fifteen (as a name)</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t xml:space="preserve">Asset containers</t>
+          <t xml:space="preserve">Features</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t xml:space="preserve">an asset container: a runner's one-off for one asset, exiting with its stage</t>
+          <t xml:space="preserve">the definition the strategy hierarchy reads on every timeframe, set or no set</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
+          <t xml:space="preserve">`TREND_GATE_FEATURE_DEFINITION` in `module_ml/config.py` — the name of the catalogue's first definition, owned by the strategy that reads it; the gate's timeframe is the top of the contract's hierarchy, `trend_gate_timeframe(cat)`</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`trend_gate_feature`</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gate (the asset's STRATEGY frame)</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t xml:space="preserve">a compose service per asset; a resident per asset; a `restart:` policy; a published port</t>
+          <t xml:space="preserve">`TREND_FAMILY`; a column literal in `asset.js`; a second copy of the name in the feature layer, which reads nothing of it</t>
         </is>
       </c>
     </row>
@@ -15352,17 +15352,17 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t xml:space="preserve">a runner: a compose service that is a role and a one-off — no command of its own; the run supplies one and the container exits with the stage</t>
+          <t xml:space="preserve">an asset container: a runner's one-off for one asset, exiting with its stage</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
+          <t xml:space="preserve">the `stage` macro of the `Makefile` — `docker compose run --rm -T &lt;runner&gt; python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;` — once per ticker of `TICKER_LIST` through `each` and `fanout`, `JOBS` at a time</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t xml:space="preserve">`pipeline`, one runner for every module; a stage run by `exec` inside a resident; a runner with a `command:`</t>
+          <t xml:space="preserve">a compose service per asset; a resident per asset; a `restart:` policy; a published port</t>
         </is>
       </c>
     </row>
@@ -15374,17 +15374,17 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t xml:space="preserve">a service's mounts: the tree at `/app` and the stores it touches at `/store/&lt;content&gt;`, read-only where it only reads</t>
+          <t xml:space="preserve">a runner: a compose service that is a role and a one-off — no command of its own; the run supplies one and the container exits with the stage</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.:/app` and `./store/&lt;content&gt;:/store/&lt;content&gt;` in each service's `volumes:` of `docker-compose.yml`, respelled whole because a service's key replaces the anchor's</t>
+          <t xml:space="preserve">`data`, `features`, `ml` — each the `x-service` anchor, which carries the one `build:` and `image:`, with its `volumes:` respelled; the `run`, `stage`, `each`, `fanout` and `basket` macros of the `Makefile`</t>
         </is>
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t xml:space="preserve">`/app/store/&lt;content&gt;` as an address; a mount of a store the service does not touch; a named volume</t>
+          <t xml:space="preserve">`pipeline`, one runner for every module; a stage run by `exec` inside a resident; a runner with a `command:`</t>
         </is>
       </c>
     </row>
@@ -15396,17 +15396,17 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t xml:space="preserve">the memory ceiling of the one runner that needs it — HPO and XGBoost allocate above `DUCKDB_MEMORY_LIMIT`</t>
+          <t xml:space="preserve">a service's mounts: the tree at `/app` and the stores it touches at `/store/&lt;content&gt;`, read-only where it only reads</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t xml:space="preserve">`deploy.resources.limits.memory` of the `ml` runner alone</t>
+          <t xml:space="preserve">`.:/app` and `./store/&lt;content&gt;:/store/&lt;content&gt;` in each service's `volumes:` of `docker-compose.yml`, respelled whole because a service's key replaces the anchor's</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t xml:space="preserve">`mem_limit` beside it, a CPU quota, a reservation; a ceiling on the anchor, so on the dashboard too</t>
+          <t xml:space="preserve">`/app/store/&lt;content&gt;` as an address; a mount of a store the service does not touch; a named volume</t>
         </is>
       </c>
     </row>
@@ -15418,17 +15418,17 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t xml:space="preserve">the thread cap: every computation's threads pinned to one — OpenMP's by the compose anchor's environment, beside the store contract, DuckDB's and XGBoost's in the code</t>
+          <t xml:space="preserve">the memory ceiling of the one runner that needs it — HPO and XGBoost allocate above `DUCKDB_MEMORY_LIMIT`</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t xml:space="preserve">`OMP_NUM_THREADS` in the `x-store-environment` anchor of `docker-compose.yml`; `SET threads=1` on every DuckDB connection; `nthread` of the booster's parameters in `module_ml/config.py`</t>
+          <t xml:space="preserve">`deploy.resources.limits.memory` of the `ml` runner alone</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t xml:space="preserve">a thread count read from a stage's command line; a cap set per service</t>
+          <t xml:space="preserve">`mem_limit` beside it, a CPU quota, a reservation; a ceiling on the anchor, so on the dashboard too</t>
         </is>
       </c>
     </row>
@@ -15440,17 +15440,17 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t xml:space="preserve">the dashboard's command: the server, on the container's internal port</t>
+          <t xml:space="preserve">the thread cap: every computation's threads pinned to one — OpenMP's by the compose anchor's environment, beside the store contract, DuckDB's and XGBoost's in the code</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command: python -m module_monitoring.serve` of `dashboard`; `CONTAINER_PORT` and `BIND_ADDRESS` in `module_monitoring/config.py`</t>
+          <t xml:space="preserve">`OMP_NUM_THREADS` in the `x-store-environment` anchor of `docker-compose.yml`; `SET threads=1` on every DuckDB connection; `nthread` of the booster's parameters in `module_ml/config.py`</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t xml:space="preserve">a port or a bind address read from the environment or the command line; `PORT` inside a container</t>
+          <t xml:space="preserve">a thread count read from a stage's command line; a cap set per service</t>
         </is>
       </c>
     </row>
@@ -15462,22 +15462,17 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t xml:space="preserve">the host port: the host side of the dashboard's mapping, measured at invocation and never written down — and the page's address, the one `make on` prints</t>
+          <t xml:space="preserve">the dashboard's command: the server, on the container's internal port</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t xml:space="preserve">`PORT` of the `Makefile` — the port the dashboard already publishes, else the first free one upward from the internal port's number; `PORT=n` overrides; the `ports:` of `dashboard`, published on `127.0.0.1`</t>
-        </is>
-      </c>
-      <c r="E379" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`dashboard at http://127.0.0.1:&lt;port&gt;/`</t>
+          <t xml:space="preserve">`command: python -m module_monitoring.serve` of `dashboard`; `CONTAINER_PORT` and `BIND_ADDRESS` in `module_monitoring/config.py`</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t xml:space="preserve">the internal port's number as the page's address in a document, a command or a comment; a second variable for it; `PORT` inside a container; a measurement outside the `Makefile`</t>
+          <t xml:space="preserve">a port or a bind address read from the environment or the command line; `PORT` inside a container</t>
         </is>
       </c>
     </row>
@@ -15489,17 +15484,22 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t xml:space="preserve">the compose project: the one fixed name every container, network and volume of this project carries on every host</t>
+          <t xml:space="preserve">the host port: the host side of the dashboard's mapping, measured at invocation and never written down — and the page's address, the one `make on` prints</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t xml:space="preserve">`name: liora` in `docker-compose.yml` — the resident `liora-dashboard-1`</t>
+          <t xml:space="preserve">`PORT` of the `Makefile` — the port the dashboard already publishes, else the first free one upward from the internal port's number; `PORT=n` overrides; the `ports:` of `dashboard`, published on `127.0.0.1`</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`dashboard at http://127.0.0.1:&lt;port&gt;/`</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t xml:space="preserve">a name derived from the checkout's directory; a project per ticker; two checkouts of the project up at once on one host — they share the name: run one, or set `COMPOSE_PROJECT_NAME`</t>
+          <t xml:space="preserve">the internal port's number as the page's address in a document, a command or a comment; a second variable for it; `PORT` inside a container; a measurement outside the `Makefile`</t>
         </is>
       </c>
     </row>
@@ -15511,17 +15511,17 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t xml:space="preserve">how long a container lives: one-off — a `run --rm` process that exits with its stage — or resident — a server that stays up</t>
+          <t xml:space="preserve">the compose project: the one fixed name every container, network and volume of this project carries on every host</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run --rm -T`, the `run` macro of the `Makefile`, for a one-off; `up -d dashboard` of `make on` for the one resident</t>
+          <t xml:space="preserve">`name: liora` in `docker-compose.yml` — the resident `liora-dashboard-1`</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t xml:space="preserve">one-shot, ephemeral, daemon, long-running; `task` or `job` for the one-off; a stage run in a resident</t>
+          <t xml:space="preserve">a name derived from the checkout's directory; a project per ticker; two checkouts of the project up at once on one host — they share the name: run one, or set `COMPOSE_PROJECT_NAME`</t>
         </is>
       </c>
     </row>
@@ -15533,49 +15533,39 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t xml:space="preserve">the presentation switch: the dashboard up with the page's address printed and opened, or every container of this project down, in one word</t>
+          <t xml:space="preserve">how long a container lives: one-off — a `run --rm` process that exits with its stage — or resident — a server that stays up</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make on`, `make off` — the two bare lifecycle targets a presenter types</t>
+          <t xml:space="preserve">`run --rm -T`, the `run` macro of the `Makefile`, for a one-off; `up -d dashboard` of `make on` for the one resident</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t xml:space="preserve">`start` / `stop`, bare `up` / `down` (compose's), `run`, a second switch pair; a switch that runs a stage</t>
+          <t xml:space="preserve">one-shot, ephemeral, daemon, long-running; `task` or `job` for the one-off; a stage run in a resident</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run record</t>
+          <t xml:space="preserve">Asset containers</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t xml:space="preserve">one recorded run of the chain — the execution name, read forward</t>
+          <t xml:space="preserve">the presentation switch: the dashboard up with the page's address printed and opened, or every container of this project down, in one word</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t xml:space="preserve">`run_id`; `RUN_ID` of the `Makefile`, `&lt;YYYYMMDDTHHMMSS&gt;Z_&lt;short commit&gt;` — the UTC time, then git's short commit — so it sorts by time and names the code that ran</t>
-        </is>
-      </c>
-      <c r="D383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`run_id`</t>
-        </is>
-      </c>
-      <c r="E383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">run</t>
+          <t xml:space="preserve">`make on`, `make off` — the two bare lifecycle targets a presenter types</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t xml:space="preserve">build, job, a content hash; a generated run id bound to no project name; a run id inside an artifact or a ledger</t>
+          <t xml:space="preserve">`start` / `stop`, bare `up` / `down` (compose's), `run`, a second switch pair; a switch that runs a stage</t>
         </is>
       </c>
     </row>
@@ -15587,27 +15577,27 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
+          <t xml:space="preserve">one recorded run of the chain — the execution name, read forward</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t xml:space="preserve">the target name; `RECORDED_STAGES` in the `Makefile` — `DATA_STAGES`, `FEATURES_STAGES`, `ML_STAGES` in order; `make all-record`</t>
+          <t xml:space="preserve">`run_id`; `RUN_ID` of the `Makefile`, `&lt;YYYYMMDDTHHMMSS&gt;Z_&lt;short commit&gt;` — the UTC time, then git's short commit — so it sorts by time and names the code that ran</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t xml:space="preserve">`stage` — the file name `&lt;stage&gt;.json`</t>
+          <t xml:space="preserve">`run_id`</t>
         </is>
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t xml:space="preserve">stage</t>
+          <t xml:space="preserve">run</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
+          <t xml:space="preserve">build, job, a content hash; a generated run id bound to no project name; a run id inside an artifact or a ledger</t>
         </is>
       </c>
     </row>
@@ -15619,22 +15609,27 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t xml:space="preserve">the command the recorder ran</t>
+          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command` — the make command line, joined by spaces</t>
+          <t xml:space="preserve">the target name; `RECORDED_STAGES` in the `Makefile` — `DATA_STAGES`, `FEATURES_STAGES`, `ML_STAGES` in order; `make all-record`</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t xml:space="preserve">`command`</t>
+          <t xml:space="preserve">`stage` — the file name `&lt;stage&gt;.json`</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stage</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage's own command line; anything a stage says about itself</t>
+          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
         </is>
       </c>
     </row>
@@ -15646,27 +15641,22 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t xml:space="preserve">the exit code: how the stage ended; `all-record` stops at the first stage that exits non-zero and keeps its record</t>
+          <t xml:space="preserve">the command the recorder ran</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t xml:space="preserve">the command's exit code, `record.py`'s own</t>
+          <t xml:space="preserve">`command` — the make command line, joined by spaces</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t xml:space="preserve">`exit_code`</t>
-        </is>
-      </c>
-      <c r="E386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">exit</t>
+          <t xml:space="preserve">`command`</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t xml:space="preserve">status, ok</t>
+          <t xml:space="preserve">a stage's own command line; anything a stage says about itself</t>
         </is>
       </c>
     </row>
@@ -15678,27 +15668,27 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stage timing: when the stage ran, and for how long</t>
+          <t xml:space="preserve">the exit code: how the stage ended; `all-record` stops at the first stage that exits non-zero and keeps its record</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t xml:space="preserve">`main()` in `record.py` — the UTC clock before and after the command, the monotonic clock for the duration</t>
+          <t xml:space="preserve">the command's exit code, `record.py`'s own</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t xml:space="preserve">`started_at_utc`, `ended_at_utc`, `duration_seconds`</t>
+          <t xml:space="preserve">`exit_code`</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t xml:space="preserve">start; time; start / end and total time in the run's header</t>
+          <t xml:space="preserve">exit</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t xml:space="preserve">wall, elapsed</t>
+          <t xml:space="preserve">status, ok</t>
         </is>
       </c>
     </row>
@@ -15710,27 +15700,27 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store diff: what the stage did to the stores — every file added, changed (size or mtime moved) or removed, by store and path</t>
+          <t xml:space="preserve">the stage timing: when the stage ran, and for how long</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the three stores of `STORES` — every store but the trials store and the run records it writes</t>
+          <t xml:space="preserve">`main()` in `record.py` — the UTC clock before and after the command, the monotonic clock for the duration</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t xml:space="preserve">`store_diff` with `added`, `changed` — each `store`, `path`, `size_bytes`, `mtime_ns` — and `removed` — each `store`, `path`</t>
+          <t xml:space="preserve">`started_at_utc`, `ended_at_utc`, `duration_seconds`</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t xml:space="preserve">added / changed / removed; bytes written; the STORES frame</t>
+          <t xml:space="preserve">start; time; start / end and total time in the run's header</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t xml:space="preserve">output, artifacts, a stage → artifact map; a trial ledger read by the recorder</t>
+          <t xml:space="preserve">wall, elapsed</t>
         </is>
       </c>
     </row>
@@ -15742,17 +15732,27 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t xml:space="preserve">the basket one run covered — not in the record: the recorder knows no basket</t>
+          <t xml:space="preserve">the store diff: what the stage did to the stores — every file added, changed (size or mtime moved) or removed, by store and path</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t xml:space="preserve">the launcher's `TICKERS`, which the make target the recorder wraps carries into every stage command</t>
+          <t xml:space="preserve">`listing()`, `store_diff()` in `record.py`, over the three stores of `STORES` — every store but the trials store and the run records it writes</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`store_diff` with `added`, `changed` — each `store`, `path`, `size_bytes`, `mtime_ns` — and `removed` — each `store`, `path`</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">added / changed / removed; bytes written; the STORES frame</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ticker`, the first of the basket standing for it; one record per asset</t>
+          <t xml:space="preserve">output, artifacts, a stage → artifact map; a trial ledger read by the recorder</t>
         </is>
       </c>
     </row>
@@ -15764,27 +15764,17 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run index: every run with a record, newest first, each with its records — the one file the page reads to find a run</t>
+          <t xml:space="preserve">the basket one run covered — not in the record: the recorder knows no basket</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_run_index()` in `record.py`, written again after every record from the store's listing, as `store/run_records/index.json`</t>
-        </is>
-      </c>
-      <c r="D390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`generated_at_utc`; `runs[]`, each `run_id` and `records` — the record files, relative to the run's directory, in path order</t>
-        </is>
-      </c>
-      <c r="E390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`&lt;n&gt; recorded run(s) · showing &lt;run_id&gt; · &lt;n&gt; records`</t>
+          <t xml:space="preserve">the launcher's `TICKERS`, which the make target the recorder wraps carries into every stage command</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t xml:space="preserve">a run list per asset; a listing by the page; a route that lists the store; an index written by a stage</t>
+          <t xml:space="preserve">`ticker`, the first of the basket standing for it; one record per asset</t>
         </is>
       </c>
     </row>
@@ -15796,22 +15786,27 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stage records of one run, in the order the stages started — each read by the page at the relative path the index lists</t>
+          <t xml:space="preserve">the run index: every run with a record, newest first, each with its records — the one file the page reads to find a run</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t xml:space="preserve">`runs[].records` of the index; `fetchRunRecord()` in `module_monitoring/run.js`, which sorts them by `started_at_utc`</t>
+          <t xml:space="preserve">`build_run_index()` in `record.py`, written again after every record from the store's listing, as `store/run_records/index.json`</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`generated_at_utc`; `runs[]`, each `run_id` and `records` — the record files, relative to the run's directory, in path order</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">STAGES — stage, start, time, exit, added, changed, removed, bytes written</t>
+          <t xml:space="preserve">`&lt;n&gt; recorded run(s) · showing &lt;run_id&gt; · &lt;n&gt; records`</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t xml:space="preserve">a record per asset of a basket stage; an envelope built by a server</t>
+          <t xml:space="preserve">a run list per asset; a listing by the page; a route that lists the store; an index written by a stage</t>
         </is>
       </c>
     </row>
@@ -15823,39 +15818,44 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, in a store the recorder does not list; untracked</t>
+          <t xml:space="preserve">the stage records of one run, in the order the stages started — each read by the page at the relative path the index lists</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t xml:space="preserve">`STORE_RUN_RECORDS_DIR`, `store/run_records/&lt;run_id&gt;/&lt;stage&gt;.json`; `write_json()` in `record.py`, beside its place, then moved onto it</t>
+          <t xml:space="preserve">`runs[].records` of the index; `fetchRunRecord()` in `module_monitoring/run.js`, which sorts them by `started_at_utc`</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">STAGES — stage, start, time, exit, added, changed, removed, bytes written</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `runtime/` folder under an asset; one run record per asset; a run record tracked</t>
+          <t xml:space="preserve">a record per asset of a basket stage; an envelope built by a server</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documentation ownership</t>
+          <t xml:space="preserve">Run record</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generated document: one the sync renders from the sheet and a hand never edits, its first line the marker, its rules cited by `rule_id`</t>
+          <t xml:space="preserve">the run directory: where a run's records live — one file per stage, in a store the recorder does not list; untracked</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
+          <t xml:space="preserve">`STORE_RUN_RECORDS_DIR`, `store/run_records/&lt;run_id&gt;/&lt;stage&gt;.json`; `write_json()` in `record.py`, beside its place, then moved onto it</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Skill edited in its file; a Skill cited by a numbered or titled section — a rule is cited by its `rule_id`; a hand-written `skill_*.md`</t>
+          <t xml:space="preserve">a `runtime/` folder under an asset; one run record per asset; a run record tracked</t>
         </is>
       </c>
     </row>
@@ -15867,17 +15867,17 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t xml:space="preserve">a hand-written document: one a hand keeps and the sync never touches, no marker on its first line</t>
+          <t xml:space="preserve">a generated document: one the sync renders from the sheet and a hand never edits, its first line the marker, its rules cited by `rule_id`</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md`, `CLAUDE.md`, `README.md`, `module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`, `module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`, every `README_sub_module_&lt;subject&gt;.md`, `module_skills/README.md`, `module_skills/sub_module_scalability_crawler/crawlers_mission.md`</t>
+          <t xml:space="preserve">every `skill_*.md` and `module_skills/skill_glossary.md`; `skill_places()`, `GENERATED_MARKER` in `module_skills/config.py`; `make skills-sync`</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule kept only there; a second copy of a rule</t>
+          <t xml:space="preserve">a Skill edited in its file; a Skill cited by a numbered or titled section — a rule is cited by its `rule_id`; a hand-written `skill_*.md`</t>
         </is>
       </c>
     </row>
@@ -15889,17 +15889,17 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t xml:space="preserve">a normative document describing one module's own responsibility</t>
+          <t xml:space="preserve">a hand-written document: one a hand keeps and the sync never touches, no marker on its first line</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_&lt;domain&gt;`</t>
+          <t xml:space="preserve">`AGENTS.md`, `CLAUDE.md`, `README.md`, `module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`, `module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`, every `README_sub_module_&lt;subject&gt;.md`, `module_skills/README.md`, `module_skills/sub_module_scalability_crawler/crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t xml:space="preserve">a module's rule kept in `module_skills/`; a per-module `docs/` or `doc/` folder</t>
+          <t xml:space="preserve">a rule kept only there; a second copy of a rule</t>
         </is>
       </c>
     </row>
@@ -15911,17 +15911,17 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t xml:space="preserve">a normative document that crosses modules or governs the project — the canon's</t>
+          <t xml:space="preserve">a normative document describing one module's own responsibility</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_skills`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_&lt;domain&gt;`</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t xml:space="preserve">a cross-cutting rule filed under one module; an edit to a copy</t>
+          <t xml:space="preserve">a module's rule kept in `module_skills/`; a per-module `docs/` or `doc/` folder</t>
         </is>
       </c>
     </row>
@@ -15933,17 +15933,17 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module skill: the normative document about one sub-module alone, kept beside its code as `skill_&lt;subject&gt;.md` — the serpentine search's and the crawler's; a terminal has none of its own, `module_skills/skill_tui_designer.md` holding what the terminals share</t>
+          <t xml:space="preserve">a normative document that crosses modules or governs the project — the canon's</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_&lt;subject&gt;/skill_&lt;subject&gt;.md`, rendered from its owner's tab</t>
+          <t xml:space="preserve">`module_skills/skill_&lt;subject&gt;.md`, its rules on the sheet's tab `module_skills`</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module's own rule among `module_skills/skill_*.md` or in its module's `skills/`; a rule two sub-modules obey kept beside one of them; a `skill_&lt;module&gt;_terminal.md`; a `skills/` folder for one document</t>
+          <t xml:space="preserve">a cross-cutting rule filed under one module; an edit to a copy</t>
         </is>
       </c>
     </row>
@@ -15955,17 +15955,17 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t xml:space="preserve">the directory holding one module's own documents: its Skills and its methodology</t>
+          <t xml:space="preserve">a sub-module skill: the normative document about one sub-module alone, kept beside its code as `skill_&lt;subject&gt;.md` — the serpentine search's and the crawler's; a terminal has none of its own, `module_skills/skill_tui_designer.md` holding what the terminals share</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/`</t>
+          <t xml:space="preserve">`sub_module_&lt;subject&gt;/skill_&lt;subject&gt;.md`, rendered from its owner's tab</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skill/`, `module_&lt;domain&gt;/documentation/`</t>
+          <t xml:space="preserve">a sub-module's own rule among `module_skills/skill_*.md` or in its module's `skills/`; a rule two sub-modules obey kept beside one of them; a `skill_&lt;module&gt;_terminal.md`; a `skills/` folder for one document</t>
         </is>
       </c>
     </row>
@@ -15977,17 +15977,17 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t xml:space="preserve">the name register: one concept, one name, in code, artifacts and interface, and the copies no module may import across — rendered from the glossary table of the sheet with the register's own rules</t>
+          <t xml:space="preserve">the directory holding one module's own documents: its Skills and its methodology</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/`</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t xml:space="preserve">a register edited by hand; a second register; a name entering the tree in a commit that does not add its row</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skill/`, `module_&lt;domain&gt;/documentation/`</t>
         </is>
       </c>
     </row>
@@ -15999,17 +15999,17 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sheet: the one source of every Skill and of the register — a tab per owner, each with its rule table; the glossary and the `rule_type_id` list; the skill register and the files matrix</t>
+          <t xml:space="preserve">the name register: one concept, one name, in code, artifacts and interface, and the copies no module may import across — rendered from the glossary table of the sheet with the register's own rules</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skills_sheet.xlsx`, `SKILLS_SHEET_PATH`; `load_sheet()` in `module_skills/sheet.py`; `RULE_HEADER`, `SKILL_REGISTER_HEADER`, `GLOSSARY_HEADER`, `RULE_TYPE_ID_HEADER`, `FILES_MATRIX_HEADER` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`module_skills/skill_glossary.md`; `GLOSSARY_SKILL_PATH`, `GLOSSARY_HEADER` in `module_skills/config.py`; `to_markdown()` in `module_skills/sync.py`</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t xml:space="preserve">a Skill edited in its file; a second workbook; a CSV or JSON beside it; a sheet written by code</t>
+          <t xml:space="preserve">a register edited by hand; a second register; a name entering the tree in a commit that does not add its row</t>
         </is>
       </c>
     </row>
@@ -16021,17 +16021,17 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t xml:space="preserve">the skill register: a row per generated Skill — the tab that holds its rules, its `skill_path` and its summary</t>
+          <t xml:space="preserve">the sheet: the one source of every Skill and of the register — a tab per owner, each with its rule table; the glossary and the `rule_type_id` list; the skill register and the files matrix</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILL_REGISTER_HEADER` in `module_skills/config.py`; `Skill` in `module_skills/sheet.py`</t>
+          <t xml:space="preserve">`module_skills/skills_sheet.xlsx`, `SKILLS_SHEET_PATH`; `load_sheet()` in `module_skills/sheet.py`; `RULE_HEADER`, `SKILL_REGISTER_HEADER`, `GLOSSARY_HEADER`, `RULE_TYPE_ID_HEADER`, `FILES_MATRIX_HEADER` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t xml:space="preserve">document register, `DOCUMENT_REGISTER_HEADER`; a Skill without a register row; a summary in a rule row; an owner read off the files matrix</t>
+          <t xml:space="preserve">a Skill edited in its file; a second workbook; a CSV or JSON beside it; a sheet written by code</t>
         </is>
       </c>
     </row>
@@ -16043,17 +16043,17 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sync: every Skill and the register rendered from the sheet beside what each governs, and every generated file the sheet no longer names deleted</t>
+          <t xml:space="preserve">the skill register: a row per generated Skill — the tab that holds its rules, its `skill_path` and its summary</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make skills-sync`; `main()`, `to_markdown()`, `build_documents()`, `write_text()`, `delete_stale()` in `module_skills/sync.py`; `GENERATED_MARKER`</t>
+          <t xml:space="preserve">`SKILL_REGISTER_HEADER` in `module_skills/config.py`; `Skill` in `module_skills/sheet.py`</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t xml:space="preserve">distribute, generate, export; a stamp; a comparison of copies; a Markdown edited by hand; a sync that reads the sheet twice; a document without the marker deleted</t>
+          <t xml:space="preserve">document register, `DOCUMENT_REGISTER_HEADER`; a Skill without a register row; a summary in a rule row; an owner read off the files matrix</t>
         </is>
       </c>
     </row>
@@ -16065,17 +16065,17 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t xml:space="preserve">the table of every configurable: every CONFIGURABLES record of the controlled `config.py` files, read as literals, on stdout</t>
+          <t xml:space="preserve">the sync: every Skill and the register rendered from the sheet beside what each governs, and every generated file the sheet no longer names deleted</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t xml:space="preserve">`make skills-configurables`; `main()`, `load_records()`, `to_cell()` in `module_skills/configurables.py`</t>
+          <t xml:space="preserve">`make skills-sync`; `main()`, `to_markdown()`, `build_documents()`, `write_text()`, `delete_stale()` in `module_skills/sync.py`; `GENERATED_MARKER`</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">a file the table is written into; an import of the module whose records it reads; a record the table carries and no `config.py` holds</t>
+          <t xml:space="preserve">distribute, generate, export; a stamp; a comparison of copies; a Markdown edited by hand; a sync that reads the sheet twice; a document without the marker deleted</t>
         </is>
       </c>
     </row>
@@ -16087,17 +16087,17 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t xml:space="preserve">the contract: what every change answers to, read in full before a session's first edit</t>
+          <t xml:space="preserve">the table of every configurable: every CONFIGURABLES record of the controlled `config.py` files, read as literals, on stdout</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t xml:space="preserve">`AGENTS.md` at the root</t>
+          <t xml:space="preserve">`make skills-configurables`; `main()`, `load_records()`, `to_cell()` in `module_skills/configurables.py`</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second contract; a per-module `AGENTS.md`</t>
+          <t xml:space="preserve">a file the table is written into; an import of the module whose records it reads; a record the table carries and no `config.py` holds</t>
         </is>
       </c>
     </row>
@@ -16109,17 +16109,17 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
+          <t xml:space="preserve">the contract: what every change answers to, read in full before a session's first edit</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t xml:space="preserve">`CLAUDE.md` at the root</t>
+          <t xml:space="preserve">`AGENTS.md` at the root</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule written in it; a per-module `CLAUDE.md`; `CLAUDE.local.md` or `.claude/` inside the tree</t>
+          <t xml:space="preserve">a second contract; a per-module `AGENTS.md`</t>
         </is>
       </c>
     </row>
@@ -16131,17 +16131,17 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t xml:space="preserve">the project's front door: what the project is, how to run it and where its Skills are</t>
+          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README.md` at the root</t>
+          <t xml:space="preserve">`CLAUDE.md` at the root</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule restated in it; a front door that restates a Skill or a decision table</t>
+          <t xml:space="preserve">a rule written in it; a per-module `CLAUDE.md`; `CLAUDE.local.md` or `.claude/` inside the tree</t>
         </is>
       </c>
     </row>
@@ -16153,17 +16153,17 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t xml:space="preserve">one module's reader-facing front door, its orientation</t>
+          <t xml:space="preserve">the project's front door: what the project is, how to run it and where its Skills are</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`README.md` at the root</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/README.md`; an orientation that restates a Skill or a decision table</t>
+          <t xml:space="preserve">a rule restated in it; a front door that restates a Skill or a decision table</t>
         </is>
       </c>
     </row>
@@ -16175,17 +16175,17 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t xml:space="preserve">a sub-module's orientation, beside its code</t>
+          <t xml:space="preserve">one module's reader-facing front door, its orientation</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/README_module_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/README.md`; an orientation that restates a Skill or a decision table</t>
         </is>
       </c>
     </row>
@@ -16197,17 +16197,17 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t xml:space="preserve">the design rationale: the section of a module's orientation that says, per object, analogous pair or the module's documents, why here, why beside these, why this boundary and which mapping row it answers to — the fourth the test of the first three</t>
+          <t xml:space="preserve">a sub-module's orientation, beside its code</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t xml:space="preserve">`## Design rationale` of each `README_module_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`README_sub_module_&lt;subject&gt;.md` — each `sub_module_terminal/README_sub_module_terminal.md`, `module_skills/sub_module_scalability_crawler/README_sub_module_scalability_crawler.md`, `module_features/sub_module_serpentine_search/README_sub_module_serpentine_search.md`</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t xml:space="preserve">a decision table; a rule restated; an object with no row or two; ADR, decision record, decision log, `docs/`</t>
+          <t xml:space="preserve">a `README.md` inside a package; an orientation that restates a Skill; a section of its module's orientation in its place</t>
         </is>
       </c>
     </row>
@@ -16219,17 +16219,17 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t xml:space="preserve">a methodology document: reference material for a human — the equations, the derivations and the citations of one module</t>
+          <t xml:space="preserve">the design rationale: the section of a module's orientation that says, per object, analogous pair or the module's documents, why here, why beside these, why this boundary and which mapping row it answers to — the fourth the test of the first three</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`</t>
+          <t xml:space="preserve">`## Design rationale` of each `README_module_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t xml:space="preserve">a row of the files matrix; a document the crawler sends; a rule stated only there</t>
+          <t xml:space="preserve">a decision table; a rule restated; an object with no row or two; ADR, decision record, decision log, `docs/`</t>
         </is>
       </c>
     </row>
@@ -16241,44 +16241,39 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t xml:space="preserve">the canon's index: every Skill by its path, and the canon's prose that is no rule, the mapping table among it</t>
+          <t xml:space="preserve">a methodology document: reference material for a human — the equations, the derivations and the citations of one module</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/README.md`</t>
+          <t xml:space="preserve">`module_&lt;domain&gt;/skills/methodology_&lt;domain&gt;.md`</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t xml:space="preserve">a collection of copies; an index that restates a rule it links to</t>
+          <t xml:space="preserve">a row of the files matrix; a document the crawler sends; a rule stated only there</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pre-AWS direction</t>
+          <t xml:space="preserve">Documentation ownership</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t xml:space="preserve">the stance: a local academic architecture whose boundaries would survive a move onto standard cloud primitives, with no cloud used and none planned</t>
+          <t xml:space="preserve">the canon's index: every Skill by its path, and the canon's prose that is no rule, the mapping table among it</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skill_pre_aws_solution.md` — `pre_aws` its stem, the one tracked name that carries the word; no identifier</t>
+          <t xml:space="preserve">`module_skills/README.md`</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t xml:space="preserve">cloud-ready, AWS-ready, cloud-native; a migration plan, a deployment guide; `pre-aws` or `PreAWS` in prose</t>
-        </is>
-      </c>
-      <c r="I412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pre-AWS — before Amazon Web Services (AWS), the cloud the mapping reads forward to</t>
+          <t xml:space="preserve">a collection of copies; an index that restates a rule it links to</t>
         </is>
       </c>
     </row>
@@ -16290,22 +16285,22 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t xml:space="preserve">compute: a process that reads a store, writes a store and exits, owning no asset state between invocations</t>
+          <t xml:space="preserve">the stance: a local academic architecture whose boundaries would survive a move onto standard cloud primitives, with no cloud used and none planned</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t xml:space="preserve">every stage's `main()`, `python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;`; the one-off container that runs it</t>
+          <t xml:space="preserve">`module_skills/skill_pre_aws_solution.md` — `pre_aws` its stem, the one tracked name that carries the word; no identifier</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t xml:space="preserve">a container as the home of an asset's state; a resident as a requirement of a stage; an in-process cache between stages; `worker`, `processor`</t>
+          <t xml:space="preserve">cloud-ready, AWS-ready, cloud-native; a migration plan, a deployment guide; `pre-aws` or `PreAWS` in prose</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t xml:space="preserve">a task — one run of the one task definition on the container instance every asset's runs share (Amazon ECS on Amazon EC2)</t>
+          <t xml:space="preserve">Pre-AWS — before Amazon Web Services (AWS), the cloud the mapping reads forward to</t>
         </is>
       </c>
     </row>
@@ -16317,22 +16312,22 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t xml:space="preserve">the rebuild condition: whether an asset's artifacts must be rebuilt from its canonical series, answered without launching anything; its freshness half is unwritten, its names reserved — `has_new_market_data()`, `requires_canonical_rebuild()`, `requires_feature_rebuild()`, `requires_model_rebuild()`</t>
+          <t xml:space="preserve">compute: a process that reads a store, writes a store and exits, owning no asset state between invocations</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t xml:space="preserve">`is_artifact_set_complete()` in `module_ml/config.py`, its completeness half; the rerun table of `module_ml/skills/methodology_ml.md`, read by a human</t>
+          <t xml:space="preserve">every stage's `main()`, `python -m &lt;module&gt;.&lt;stage&gt; --tickers &lt;TICKER&gt;`; the one-off container that runs it</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t xml:space="preserve">a scheduler, a watcher, an event bus; a function that both detects new data and trains; `should_run()`, `check_update()`, `trigger()`</t>
+          <t xml:space="preserve">a container as the home of an asset's state; a resident as a requirement of a stage; an in-process cache between stages; `worker`, `processor`</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">a choice state between two states of the machine (AWS Step Functions)</t>
+          <t xml:space="preserve">a task — one run of the one task definition on the container instance every asset's runs share (Amazon ECS on Amazon EC2)</t>
         </is>
       </c>
     </row>
@@ -16344,17 +16339,22 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mapping table: what this repository has, the responsibility, the same responsibility elsewhere and the move, row by row — the one table that sets a cloud proper noun beside a local object; its third column is the elsewhere column</t>
+          <t xml:space="preserve">the rebuild condition: whether an asset's artifacts must be rebuilt from its canonical series, answered without launching anything; its freshness half is unwritten, its names reserved — `has_new_market_data()`, `requires_canonical_rebuild()`, `requires_feature_rebuild()`, `requires_model_rebuild()`</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/README.md`, its hand-written home</t>
+          <t xml:space="preserve">`is_artifact_set_complete()` in `module_ml/config.py`, its completeness half; the rerun table of `module_ml/skills/methodology_ml.md`, read by a human</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t xml:space="preserve">an adapter, a cloud configuration file; a cloud proper noun in an identifier, a key, a path, a make target, a compose service or an environment variable; a path of the elsewhere column read as a proposal for a local directory</t>
+          <t xml:space="preserve">a scheduler, a watcher, an event bus; a function that both detects new data and trains; `should_run()`, `check_update()`, `trigger()`</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a choice state between two states of the machine (AWS Step Functions)</t>
         </is>
       </c>
     </row>
@@ -16366,17 +16366,17 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t xml:space="preserve">a seat: the standard primitive a local object would sit on elsewhere, named in the mapping table's words — spoken in the stance's skill and in the mapping table, and in no other Skill</t>
+          <t xml:space="preserve">the mapping table: what this repository has, the responsibility, the same responsibility elsewhere and the move, row by row — the one table that sets a cloud proper noun beside a local object; its third column is the elsewhere column</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`module_skills/README.md`, its hand-written home</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t xml:space="preserve">a seat paragraph in any other Skill; two seats for one object; a seat in an identifier, a key or a path; `target`, `cloud note`, `mapping section`</t>
-        </is>
-      </c>
-      <c r="I416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the image registry (Amazon ECR), the container service (Amazon ECS), the container instance (Amazon EC2), the block volume (Amazon EBS), object storage (Amazon S3), the state machine (AWS Step Functions), the schedule (Amazon EventBridge Scheduler)</t>
+          <t xml:space="preserve">an adapter, a cloud configuration file; a cloud proper noun in an identifier, a key, a path, a make target, a compose service or an environment variable; a path of the elsewhere column read as a proposal for a local directory</t>
         </is>
       </c>
     </row>
@@ -16388,17 +16388,17 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t xml:space="preserve">the resource role: the name a cloud resource would carry, `&lt;project&gt;-&lt;environment&gt;-&lt;resource-role&gt;` — the role a seat's name or the task a row of the mapping table names, lower case with `-` between its words, the project `liora`</t>
-        </is>
-      </c>
-      <c r="C417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`name: liora` and `liora-1m-pipeline` in `docker-compose.yml` — the names of that shape the tree holds, with no environment token</t>
+          <t xml:space="preserve">a seat: the standard primitive a local object would sit on elsewhere, named in the mapping table's words — spoken in the stance's skill and in the mapping table, and in no other Skill</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second list of roles; a role no seat or row names; `dev` or `prod` in a tracked name; a ticker in a resource name; an environment token on the image</t>
+          <t xml:space="preserve">a seat paragraph in any other Skill; two seats for one object; a seat in an identifier, a key or a path; `target`, `cloud note`, `mapping section`</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the image registry (Amazon ECR), the container service (Amazon ECS), the container instance (Amazon EC2), the block volume (Amazon EBS), object storage (Amazon S3), the state machine (AWS Step Functions), the schedule (Amazon EventBridge Scheduler)</t>
         </is>
       </c>
     </row>
@@ -16410,17 +16410,17 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state name: the one-line name a stage would carry as a state of the machine, one per stage, and PublishStores, the copy after a run, which no stage answers to; *Publish* in a state name means write the object where its readers read it</t>
+          <t xml:space="preserve">the resource role: the name a cloud resource would carry, `&lt;project&gt;-&lt;environment&gt;-&lt;resource-role&gt;` — the role a seat's name or the task a row of the mapping table names, lower case with `-` between its words, the project `liora`</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`name: liora` and `liora-1m-pipeline` in `docker-compose.yml` — the names of that shape the tree holds, with no environment token</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t xml:space="preserve">a state registered one by one; a state name with *and* in it; *publish* as *make public*</t>
-        </is>
-      </c>
-      <c r="I418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a state of AWS Step Functions</t>
+          <t xml:space="preserve">a second list of roles; a role no seat or row names; `dev` or `prod` in a tracked name; a ticker in a resource name; an environment token on the image</t>
         </is>
       </c>
     </row>
@@ -16432,17 +16432,17 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t xml:space="preserve">an instance: one Linux virtual machine elsewhere, the host containers run on — the task host every asset's runs share, with the store volume beside it, and the strategy host</t>
+          <t xml:space="preserve">a state name: the one-line name a stage would carry as a state of the machine, one per stage, and PublishStores, the copy after a run, which no stage answers to; *Publish* in a state name means write the object where its readers read it</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t xml:space="preserve">`instance` or `host` for a container; a host per asset; node</t>
+          <t xml:space="preserve">a state registered one by one; a state name with *and* in it; *publish* as *make public*</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t xml:space="preserve">a container instance (Amazon EC2)</t>
+          <t xml:space="preserve">a state of AWS Step Functions</t>
         </is>
       </c>
     </row>
@@ -16454,22 +16454,17 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t xml:space="preserve">the store volume: the task host's durable disk — the five stores at `/store/&lt;content&gt;`, each at the path its `STORE_*_DIR` names; the home of state, never the copy</t>
-        </is>
-      </c>
-      <c r="C420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the `./store/&lt;content&gt;` mounts of `docker-compose.yml`, read forward as `&lt;volume&gt;/&lt;content&gt;:/store/&lt;content&gt;`</t>
+          <t xml:space="preserve">an instance: one Linux virtual machine elsewhere, the host containers run on — the task host every asset's runs share, with the store volume beside it, and the strategy host</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset volume; a volume per asset; the volume as the copy; `data_volume`; a shared network filesystem (Amazon EFS)</t>
+          <t xml:space="preserve">`instance` or `host` for a container; a host per asset; node</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t xml:space="preserve">a block volume (Amazon EBS)</t>
+          <t xml:space="preserve">a container instance (Amazon EC2)</t>
         </is>
       </c>
     </row>
@@ -16481,17 +16476,22 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t xml:space="preserve">the copy: the whole files a state after the last stage of a run would copy from the store volume to object storage — never a stage's own write, never mid-run; absent here, described</t>
+          <t xml:space="preserve">the store volume: the task host's durable disk — the five stores at `/store/&lt;content&gt;`, each at the path its `STORE_*_DIR` names; the home of state, never the copy</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the `./store/&lt;content&gt;` mounts of `docker-compose.yml`, read forward as `&lt;volume&gt;/&lt;content&gt;:/store/&lt;content&gt;`</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage writing to object storage; a stage reading the copy; `s3://` in a path constant; an adapter for the copy</t>
+          <t xml:space="preserve">asset volume; a volume per asset; the volume as the copy; `data_volume`; a shared network filesystem (Amazon EFS)</t>
         </is>
       </c>
       <c r="I421" t="inlineStr">
         <is>
-          <t xml:space="preserve">object storage (Amazon S3), written by PublishStores</t>
+          <t xml:space="preserve">a block volume (Amazon EBS)</t>
         </is>
       </c>
     </row>
@@ -16503,12 +16503,17 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t xml:space="preserve">the ladder: the three phases in which the runtime elsewhere would become true, each named for what it changes — *the lift*, *the idiom*, *the image carries the code*; all elsewhere, built nowhere here</t>
+          <t xml:space="preserve">the copy: the whole files a state after the last stage of a run would copy from the store volume to object storage — never a stage's own write, never mid-run; absent here, described</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t xml:space="preserve">a letter or a number for a phase; a phase as a branch or an environment; `dev` / `prod`; a phase built here; rung</t>
+          <t xml:space="preserve">a stage writing to object storage; a stage reading the copy; `s3://` in a path constant; an adapter for the copy</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">object storage (Amazon S3), written by PublishStores</t>
         </is>
       </c>
     </row>
@@ -16520,17 +16525,12 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t xml:space="preserve">the promotion threshold: a second concurrent writer of one partition, or a reader that needs one transaction across families — the one condition under which a managed database replaces the table families</t>
+          <t xml:space="preserve">the ladder: the three phases in which the runtime elsewhere would become true, each named for what it changes — *the lift*, *the idiom*, *the image carries the code*; all elsewhere, built nowhere here</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t xml:space="preserve">a database process for one writer; a threshold in rows or bytes</t>
-        </is>
-      </c>
-      <c r="I423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a managed database (Amazon RDS)</t>
+          <t xml:space="preserve">a letter or a number for a phase; a phase as a branch or an environment; `dev` / `prod`; a phase built here; rung</t>
         </is>
       </c>
     </row>
@@ -16542,22 +16542,17 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t xml:space="preserve">the active version: the one version of an asset's artifacts a reader reads, chosen where the reader is; the version is the execution name</t>
-        </is>
-      </c>
-      <c r="C424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`run_id`</t>
+          <t xml:space="preserve">the promotion threshold: a second concurrent writer of one partition, or a reader that needs one transaction across families — the one condition under which a managed database replaces the table families</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t xml:space="preserve">latest, current, prod; a mark inside a file; a version inside an artifact</t>
+          <t xml:space="preserve">a database process for one writer; a threshold in rows or bytes</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">the version prefix `assets_artifacts/&lt;run_id&gt;/` of the copy (Amazon S3)</t>
+          <t xml:space="preserve">a managed database (Amazon RDS)</t>
         </is>
       </c>
     </row>
@@ -16569,22 +16564,22 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t xml:space="preserve">the tunnel: how a reader reaches the page on a host that is not theirs — a local forward onto the loopback port `make on` printed there</t>
+          <t xml:space="preserve">the active version: the one version of an asset's artifacts a reader reads, chosen where the reader is; the version is the execution name</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ssh -N -L` of `README.md` § Quickstart</t>
+          <t xml:space="preserve">`run_id`</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t xml:space="preserve">a public port; a load balancer</t>
+          <t xml:space="preserve">latest, current, prod; a mark inside a file; a version inside an artifact</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t xml:space="preserve">a port-forward, the elsewhere column's word</t>
+          <t xml:space="preserve">the version prefix `assets_artifacts/&lt;run_id&gt;/` of the copy (Amazon S3)</t>
         </is>
       </c>
     </row>
@@ -16596,12 +16591,22 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t xml:space="preserve">read forward: a local object read as the same responsibility elsewhere — the mapping table's third column — with nothing moved</t>
+          <t xml:space="preserve">the tunnel: how a reader reaches the page on a host that is not theirs — a local forward onto the loopback port `make on` printed there</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`ssh -N -L` of `README.md` § Quickstart</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t xml:space="preserve">migrated, ported, deployed, in production</t>
+          <t xml:space="preserve">a public port; a load balancer</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a port-forward, the elsewhere column's word</t>
         </is>
       </c>
     </row>
@@ -16613,12 +16618,12 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t xml:space="preserve">the move: what a local thing's seat elsewhere costs it — a rename, one edit, or absent here, described; the mapping table's fourth column</t>
+          <t xml:space="preserve">read forward: a local object read as the same responsibility elsewhere — the mapping table's third column — with nothing moved</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t xml:space="preserve">migration, deployment, a plan, a roadmap</t>
+          <t xml:space="preserve">migrated, ported, deployed, in production</t>
         </is>
       </c>
     </row>
@@ -16630,44 +16635,34 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t xml:space="preserve">an absent object: a primitive, a state of the machine or a Skill that nothing local answers to and a document describes — a sentence ending, or a verdict reading, *absent here — described*</t>
-        </is>
-      </c>
-      <c r="C428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`AGENTS.md` § Skills absent here, described, for the Skills</t>
+          <t xml:space="preserve">the move: what a local thing's seat elsewhere costs it — a rename, one edit, or absent here, described; the mapping table's fourth column</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t xml:space="preserve">planned, a debt marker, future, ghost, placeholder, missing</t>
+          <t xml:space="preserve">migration, deployment, a plan, a roadmap</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t xml:space="preserve">The page</t>
+          <t xml:space="preserve">Pre-AWS direction</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page: one static page of plain HTML, CSS and JavaScript that reads every datum by a relative path and writes nothing</t>
+          <t xml:space="preserve">an absent object: a primitive, a state of the machine or a Skill that nothing local answers to and a document describes — a sentence ending, or a verdict reading, *absent here — described*</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/index.html`, `style.css` and its scripts `page.js`, `data.js`, `asset.js`, `features.js`, `ml.js`, `run.js`, `scalability.js`</t>
-        </is>
-      </c>
-      <c r="E429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1m crypto research pipeline — status</t>
+          <t xml:space="preserve">`AGENTS.md` § Skills absent here, described, for the Skills</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t xml:space="preserve">a framework or a build step; a second page beside it; a datum computed by the server; an absolute path</t>
+          <t xml:space="preserve">planned, a debt marker, future, ghost, placeholder, missing</t>
         </is>
       </c>
     </row>
@@ -16679,17 +16674,22 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page's reads: where the page takes its data from, by relative path</t>
+          <t xml:space="preserve">the page: one static page of plain HTML, CSS and JavaScript that reads every datum by a relative path and writes nothing</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t xml:space="preserve">`status/data_status.json`, `status/features_status.json`, `status/ml_status.json`, `status/skills_status.json`; `run_records/index.json`, then each record of a run at `run_records/&lt;run_id&gt;/` and the path the index lists</t>
+          <t xml:space="preserve">`module_monitoring/index.html`, `style.css` and its scripts `page.js`, `data.js`, `asset.js`, `features.js`, `ml.js`, `run.js`, `scalability.js`</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1m crypto research pipeline — status</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t xml:space="preserve">an absolute path; a route per snapshot; a directory listing; a store the page reads beside these two</t>
+          <t xml:space="preserve">a framework or a build step; a second page beside it; a datum computed by the server; an absolute path</t>
         </is>
       </c>
     </row>
@@ -16701,22 +16701,17 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t xml:space="preserve">the three prefixes: what the dashboard's server answers — the page's own files at `/`, the status store under `/status/`, the run-records store under `/run_records/`; every other path 404, and no directory listed</t>
+          <t xml:space="preserve">the page's reads: where the page takes its data from, by relative path</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_monitoring/serve.py` — `DashboardHandler`, `translate_path()`, `main()`; `STORE_DIR_BY_ROUTE_PREFIX` in `module_monitoring/config.py`, `/status/` onto `STORE_STATUS_DIR` and `/run_records/` onto `STORE_RUN_RECORDS_DIR`; `MODULE_MONITORING_DIR`, `PAGE_FILE_SUFFIXES`, `PAGE_INDEX_FILE_NAME` for the page's own files</t>
+          <t xml:space="preserve">`status/data_status.json`, `status/features_status.json`, `status/ml_status.json`, `status/skills_status.json`; `run_records/index.json`, then each record of a run at `run_records/&lt;run_id&gt;/` and the path the index lists</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t xml:space="preserve">a route per snapshot; a directory listed; a path outside the three prefixes answered; a server that computes, writes or proxies; `dashboard.py`, `proxy.py`, `server.py` beside `serve.py`</t>
-        </is>
-      </c>
-      <c r="I431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`http.server`</t>
+          <t xml:space="preserve">an absolute path; a route per snapshot; a directory listing; a store the page reads beside these two</t>
         </is>
       </c>
     </row>
@@ -16728,17 +16723,22 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t xml:space="preserve">the toolkit the page loads before its own sections</t>
+          <t xml:space="preserve">the three prefixes: what the dashboard's server answers — the page's own files at `/`, the status store under `/status/`, the run-records store under `/run_records/`; every other path 404, and no directory listed</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t xml:space="preserve">`page.js`</t>
+          <t xml:space="preserve">`module_monitoring/serve.py` — `DashboardHandler`, `translate_path()`, `main()`; `STORE_DIR_BY_ROUTE_PREFIX` in `module_monitoring/config.py`, `/status/` onto `STORE_STATUS_DIR` and `/run_records/` onto `STORE_RUN_RECORDS_DIR`; `MODULE_MONITORING_DIR`, `PAGE_FILE_SUFFIXES`, `PAGE_INDEX_FILE_NAME` for the page's own files</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t xml:space="preserve">`utils.js`, `common.js`, `shared.js`, `lib.js`; a page-specific element written from it; a second page beside the status page</t>
+          <t xml:space="preserve">a route per snapshot; a directory listed; a path outside the three prefixes answered; a server that computes, writes or proxies; `dashboard.py`, `proxy.py`, `server.py` beside `serve.py`</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`http.server`</t>
         </is>
       </c>
     </row>
@@ -16750,17 +16750,17 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one selector component of the page — the top tabs, the ML Assets views, the asset rows — each group wired by its `data-key`</t>
+          <t xml:space="preserve">the toolkit the page loads before its own sections</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t xml:space="preserve">`.pills`, `.pill`, `.pill--active`, `initPills()`, `PILL_HOOKS` in `page.js`; `data-pills` on a group, `data-panel` on its panels</t>
+          <t xml:space="preserve">`page.js`</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t xml:space="preserve">a second selector component</t>
+          <t xml:space="preserve">`utils.js`, `common.js`, `shared.js`, `lib.js`; a page-specific element written from it; a second page beside the status page</t>
         </is>
       </c>
     </row>
@@ -16772,44 +16772,44 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t xml:space="preserve">the page's navigation: the seven tabs, the five views of the ML Assets tab, and one row per asset</t>
+          <t xml:space="preserve">the one selector component of the page — the top tabs, the ML Assets views, the asset rows — each group wired by its `data-key`</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t xml:space="preserve">the groups of `data-pills` in `module_monitoring/index.html` — `tab`: `pipeline`, `quality`, `features`, `ml`, `asset`, `scalability`, `lifecycle`; `mlview`: `labels`, `classification`, `strategy`, `search`, `feature-set`; `asset`, filled from the snapshot</t>
-        </is>
-      </c>
-      <c r="E434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pipeline; Data Quality; Features; ML Research; ML Assets; Scalability; Lifecycle — Labels &amp; data; Classification; Strategy; HPO; Feature set</t>
+          <t xml:space="preserve">`.pills`, `.pill`, `.pill--active`, `initPills()`, `PILL_HOOKS` in `page.js`; `data-pills` on a group, `data-panel` on its panels</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t xml:space="preserve">a menu, a sidebar or a second navigation; a tab named for a tool</t>
+          <t xml:space="preserve">a second selector component</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scalability crawler</t>
+          <t xml:space="preserve">The page</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t xml:space="preserve">the crawler: the canon's sub-module that reads each controlled file against the Skills marked for it with the one active vendor, and writes a report per file and its snapshot; it asks nothing, goes on past a failed file and gates nothing</t>
+          <t xml:space="preserve">the page's navigation: the seven tabs, the five views of the ML Assets tab, and one row per asset</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sub_module_scalability_crawler`; `make skills-crawl`, after `make skills-sync`; `main()` in `crawl.py`</t>
+          <t xml:space="preserve">the groups of `data-pills` in `module_monitoring/index.html` — `tab`: `pipeline`, `quality`, `features`, `ml`, `asset`, `scalability`, `lifecycle`; `mlview`: `labels`, `classification`, `strategy`, `search`, `feature-set`; `asset`, filled from the snapshot</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pipeline; Data Quality; Features; ML Research; ML Assets; Scalability; Lifecycle — Labels &amp; data; Classification; Strategy; HPO; Feature set</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t xml:space="preserve">a linter, a check, a gate, a CI step; a web crawler, walking sites or services to gather what they hold; conformance, review — names that tell a reader nothing; a TUI of its own, `make skills-terminal` being the canon's terminal</t>
+          <t xml:space="preserve">a menu, a sidebar or a second navigation; a tab named for a tool</t>
         </is>
       </c>
     </row>
@@ -16821,22 +16821,17 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t xml:space="preserve">the files matrix: a row per path — a file or a glob — a column per Skill headed by its stem, an `X` where that Skill is sent with the file; the crawler's whole contract</t>
+          <t xml:space="preserve">the crawler: the canon's sub-module that reads each controlled file against the Skills marked for it with the one active vendor, and writes a report per file and its snapshot; it asks nothing, goes on past a failed file and gates nothing</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t xml:space="preserve">the table of the sheet headed by `FILES_MATRIX_HEADER` in `module_skills/config.py`; `Mark` in `module_skills/sheet.py`</t>
-        </is>
-      </c>
-      <c r="E436" t="inlineStr">
-        <is>
-          <t xml:space="preserve">path; the Skill's stem; `X`</t>
+          <t xml:space="preserve">`sub_module_scalability_crawler`; `make skills-crawl`, after `make skills-sync`; `main()` in `crawl.py`</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t xml:space="preserve">a column per rule; a mark a crawl writes; a mark derived from `scope`; a generated file, a report or the snapshot as a target; a second row for one path; a precedence between rows; a Markdown table kept beside the crawler</t>
+          <t xml:space="preserve">a linter, a check, a gate, a CI step; a web crawler, walking sites or services to gather what they hold; conformance, review — names that tell a reader nothing; a TUI of its own, `make skills-terminal` being the canon's terminal</t>
         </is>
       </c>
     </row>
@@ -16848,22 +16843,22 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t xml:space="preserve">a mark: `X` under a Skill's column in a row of the files matrix, sending that Skill with every file the row reaches; two rows that reach one file join their marks</t>
+          <t xml:space="preserve">the files matrix: a row per path — a file or a glob — a column per Skill headed by its stem, an `X` where that Skill is sent with the file; the crawler's whole contract</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILL_MARK` in `module_skills/config.py`</t>
+          <t xml:space="preserve">the table of the sheet headed by `FILES_MATRIX_HEADER` in `module_skills/config.py`; `Mark` in `module_skills/sheet.py`</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">`X`; marked; unmarked</t>
+          <t xml:space="preserve">path; the Skill's stem; `X`</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t xml:space="preserve">assign, tag, tick, check, enable; `x`, `✓` or `yes` in a cell; a mark a crawl writes; a mark derived from `scope`; a row that marks no Skill</t>
+          <t xml:space="preserve">a column per rule; a mark a crawl writes; a mark derived from `scope`; a generated file, a report or the snapshot as a target; a second row for one path; a precedence between rows; a Markdown table kept beside the crawler</t>
         </is>
       </c>
     </row>
@@ -16875,22 +16870,22 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t xml:space="preserve">a controlled file: a file a row of the files matrix reaches, read against the Skills marked for it; its key is its path from the root of the tree</t>
+          <t xml:space="preserve">a mark: `X` under a Skill's column in a row of the files matrix, sending that Skill with every file the row reaches; two rows that reach one file join their marks</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t xml:space="preserve">`ControlledFile`, `build_controlled_files()` in `crawl.py`</t>
+          <t xml:space="preserve">`SKILL_MARK` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t xml:space="preserve">file</t>
+          <t xml:space="preserve">`X`; marked; unmarked</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t xml:space="preserve">listed file; a file the crawler finds by itself; a file read from the working directory; a rendered Skill or the snapshot as a controlled file</t>
+          <t xml:space="preserve">assign, tag, tick, check, enable; `x`, `✓` or `yes` in a cell; a mark a crawl writes; a mark derived from `scope`; a row that marks no Skill</t>
         </is>
       </c>
     </row>
@@ -16902,17 +16897,22 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t xml:space="preserve">the context: the documents sent with a file — the Skills its row of the files matrix marks, each whole as `make skills-sync` rendered it</t>
+          <t xml:space="preserve">a controlled file: a file a row of the files matrix reaches, read against the Skills marked for it; its key is its path from the root of the tree</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t xml:space="preserve">`load_skill_texts()`, `build_message()` in `crawl.py`</t>
+          <t xml:space="preserve">`ControlledFile`, `build_controlled_files()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">file</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule filtered out by its `scope` before it is sent; a Skill not marked; the contract; an orientation; a methodology; a list of rules kept per module</t>
+          <t xml:space="preserve">listed file; a file the crawler finds by itself; a file read from the working directory; a rendered Skill or the snapshot as a controlled file</t>
         </is>
       </c>
     </row>
@@ -16924,17 +16924,17 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t xml:space="preserve">a file's message: the Skills marked for it, then the file with every line after its number, then the mission</t>
+          <t xml:space="preserve">the context: the documents sent with a file — the Skills its row of the files matrix marks, each whole as `make skills-sync` rendered it</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_message()` in `crawl.py`; `crawlers_mission.md`</t>
+          <t xml:space="preserve">`load_skill_texts()`, `build_message()` in `crawl.py`</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t xml:space="preserve">a list of unmarked Skills; an orientation; a commit; a measure of the message; a line number the agent has to count</t>
+          <t xml:space="preserve">a rule filtered out by its `scope` before it is sent; a Skill not marked; the contract; an orientation; a methodology; a list of rules kept per module</t>
         </is>
       </c>
     </row>
@@ -16946,17 +16946,17 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mission: what the agent reports of one file, and how — kept by hand</t>
+          <t xml:space="preserve">a file's message: the Skills marked for it, then the file with every line after its number, then the mission</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t xml:space="preserve">`crawlers_mission.md`, `CRAWLERS_MISSION_MD_PATH`</t>
+          <t xml:space="preserve">`build_message()` in `crawl.py`; `crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t xml:space="preserve">a rule restated in it; a work order or a plan</t>
+          <t xml:space="preserve">a list of unmarked Skills; an orientation; a commit; a measure of the message; a line number the agent has to count</t>
         </is>
       </c>
     </row>
@@ -16968,17 +16968,17 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t xml:space="preserve">the sub-module's folder and the root of the tree: where the crawler's own files are read, and where a controlled file and a Skill lie and the vendor runs</t>
+          <t xml:space="preserve">the mission: what the agent reports of one file, and how — kept by hand</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SUB_MODULE_DIR` in the crawler's `config.py`; `TREE_ROOT_DIR` in `module_skills/config.py`</t>
+          <t xml:space="preserve">`crawlers_mission.md`, `CRAWLERS_MISSION_MD_PATH`</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t xml:space="preserve">a host path; a controlled file read from the working directory</t>
+          <t xml:space="preserve">a rule restated in it; a work order or a plan</t>
         </is>
       </c>
     </row>
@@ -16990,22 +16990,17 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t xml:space="preserve">a vendor: an agent's command line the crawl sends each controlled file to — one table of `vendors_for_crawling.toml`, exactly one `active`, its `argv` the whole command line, run without a shell, the message on its stdin and the answer its stdout</t>
+          <t xml:space="preserve">the sub-module's folder and the root of the tree: where the crawler's own files are read, and where a controlled file and a Skill lie and the vendor runs</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t xml:space="preserve">`vendors_for_crawling.toml` with `active`, `argv`; `VENDORS_FOR_CRAWLING_TOML_PATH`, `load_vendor()`, `AGENT_TIMEOUT_SECONDS`</t>
-        </is>
-      </c>
-      <c r="E443" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vendor</t>
+          <t xml:space="preserve">`SUB_MODULE_DIR` in the crawler's `config.py`; `TREE_ROOT_DIR` in `module_skills/config.py`</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t xml:space="preserve">an API key; a vendor named in the code; a form for its model, effort or permissions; a vendor chosen on a screen; two active vendors; every vendor run in turn</t>
+          <t xml:space="preserve">a host path; a controlled file read from the working directory</t>
         </is>
       </c>
     </row>
@@ -17017,27 +17012,22 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t xml:space="preserve">a report: the one current file per controlled file — the file's key, the vendor and the time, then the answer as it came; reset by every crawl, never tracked</t>
+          <t xml:space="preserve">a vendor: an agent's command line the crawl sends each controlled file to — one table of `vendors_for_crawling.toml`, exactly one `active`, its `argv` the whole command line, run without a shell, the message on its stdin and the answer its stdout</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t xml:space="preserve">`REPORTS_DIR`, `report_path()` in the crawler's `config.py` — `store/status/reports_after_crawled_files/&lt;path&gt;.report.md`; `write_text()` in `module_skills/sync.py`</t>
-        </is>
-      </c>
-      <c r="D444" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`report`</t>
+          <t xml:space="preserve">`vendors_for_crawling.toml` with `active`, `argv`; `VENDORS_FOR_CRAWLING_TOML_PATH`, `load_vendor()`, `AGENT_TIMEOUT_SECONDS`</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t xml:space="preserve">report</t>
+          <t xml:space="preserve">vendor</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t xml:space="preserve">a history of entries; an append; a report in the sub-module's folder; a commit in its first line; a report tracked</t>
+          <t xml:space="preserve">an API key; a vendor named in the code; a form for its model, effort or permissions; a vendor chosen on a screen; two active vendors; every vendor run in turn</t>
         </is>
       </c>
     </row>
@@ -17049,17 +17039,27 @@
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t xml:space="preserve">a finding: one line of a report, `rule_id | file:line | problem | correction`; `OK` the answer of a file that departs from nothing</t>
+          <t xml:space="preserve">a report: the one current file per controlled file — the file's key, the vendor and the time, then the answer as it came; reset by every crawl, never tracked</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t xml:space="preserve">`crawlers_mission.md`</t>
+          <t xml:space="preserve">`REPORTS_DIR`, `report_path()` in the crawler's `config.py` — `store/status/reports_after_crawled_files/&lt;path&gt;.report.md`; `write_text()` in `module_skills/sync.py`</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`report`</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">report</t>
         </is>
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t xml:space="preserve">a finding without a `rule_id`; a rule that was not sent; a table; `conformant` as a line</t>
+          <t xml:space="preserve">a history of entries; an append; a report in the sub-module's folder; a commit in its first line; a report tracked</t>
         </is>
       </c>
     </row>
@@ -17071,27 +17071,17 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t xml:space="preserve">a controlled file's state: where its crawl stands — `pending` before, `running` while the vendor works, `done` once its report is written, `failed` otherwise, `interrupted` where Ctrl-C ended it</t>
+          <t xml:space="preserve">a finding: one line of a report, `rule_id | file:line | problem | correction`; `OK` the answer of a file that departs from nothing</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t xml:space="preserve">`row()` in `status.py`; `main()` in `crawl.py`</t>
-        </is>
-      </c>
-      <c r="D446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`state`</t>
-        </is>
-      </c>
-      <c r="E446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pending; running; done; failed; interrupted</t>
+          <t xml:space="preserve">`crawlers_mission.md`</t>
         </is>
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t xml:space="preserve">`done` read as conformant — it says the report was written; a change of state left out of the snapshot</t>
+          <t xml:space="preserve">a finding without a `rule_id`; a rule that was not sent; a table; `conformant` as a line</t>
         </is>
       </c>
     </row>
@@ -17103,22 +17093,27 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t xml:space="preserve">the crawl's progress: one line per controlled file after its result, then one closing line; the reason a file failed one line on stderr</t>
+          <t xml:space="preserve">a controlled file's state: where its crawl stands — `pending` before, `running` while the vendor works, `done` once its report is written, `failed` otherwise, `interrupted` where Ctrl-C ended it</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t xml:space="preserve">`main()` in `crawl.py`</t>
+          <t xml:space="preserve">`row()` in `status.py`; `main()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`state`</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t xml:space="preserve">`&lt;current&gt;/&lt;total&gt; | &lt;controlled file&gt; | &lt;vendor&gt; | &lt;state&gt;`; `&lt;processed&gt;/&lt;total&gt; | crawl | &lt;vendor&gt; | done`, `failed` or `interrupted`</t>
+          <t xml:space="preserve">pending; running; done; failed; interrupted</t>
         </is>
       </c>
       <c r="F447" t="inlineStr">
         <is>
-          <t xml:space="preserve">a spinner, a progress bar, a percentage; an answer summarised on the screen — the report holds it; a results table</t>
+          <t xml:space="preserve">`done` read as conformant — it says the report was written; a change of state left out of the snapshot</t>
         </is>
       </c>
     </row>
@@ -17130,17 +17125,22 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t xml:space="preserve">the refusals and the exits: a state the crawler cannot read ends it in one named line before anything is reset; a file the vendor fails is `failed` and the crawl goes on — 0 every file done, 1 a refusal or a failed file, 130 Ctrl-C</t>
+          <t xml:space="preserve">the crawl's progress: one line per controlled file after its result, then one closing line; the reason a file failed one line on stderr</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SystemExit` in `module_skills/sheet.py`, `module_skills/sync.py` and the crawler's `crawl.py`</t>
+          <t xml:space="preserve">`main()` in `crawl.py`</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`&lt;current&gt;/&lt;total&gt; | &lt;controlled file&gt; | &lt;vendor&gt; | &lt;state&gt;`; `&lt;processed&gt;/&lt;total&gt; | crawl | &lt;vendor&gt; | done`, `failed` or `interrupted`</t>
         </is>
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t xml:space="preserve">a traceback for an expected failure; exit 0 after a failure; a crawl that stops at the first failed file</t>
+          <t xml:space="preserve">a spinner, a progress bar, a percentage; an answer summarised on the screen — the report holds it; a results table</t>
         </is>
       </c>
     </row>
@@ -17152,27 +17152,17 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t xml:space="preserve">the snapshot: `skills_status.json`, the current state of every controlled file, sorted by path and rewritten whole at every change; tracked in its neutral state, every controlled file `pending` with no report</t>
+          <t xml:space="preserve">the refusals and the exits: a state the crawler cannot read ends it in one named line before anything is reset; a file the vendor fails is `failed` and the crawl goes on — 0 every file done, 1 a refusal or a failed file, 130 Ctrl-C</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t xml:space="preserve">`SKILLS_STATUS_JSON_PATH` in the crawler's `config.py`; `row()`, `write_skills_status()` in `status.py`, through `write_text()` of `module_skills/sync.py`</t>
-        </is>
-      </c>
-      <c r="D449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">`files`, each `path`, `state`, `vendor`, `finished_at_utc`, `report`</t>
-        </is>
-      </c>
-      <c r="E449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">file; state; vendor; finished_at_utc; report</t>
+          <t xml:space="preserve">`SystemExit` in `module_skills/sheet.py`, `module_skills/sync.py` and the crawler's `crawl.py`</t>
         </is>
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t xml:space="preserve">a count of crawls; an age; a clock but `finished_at_utc`; a snapshot that reads itself back; a partial file</t>
+          <t xml:space="preserve">a traceback for an expected failure; exit 0 after a failure; a crawl that stops at the first failed file</t>
         </is>
       </c>
     </row>
@@ -17184,104 +17174,136 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
+          <t xml:space="preserve">the snapshot: `skills_status.json`, the current state of every controlled file, sorted by path and rewritten whole at every change; tracked in its neutral state, every controlled file `pending` with no report</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`SKILLS_STATUS_JSON_PATH` in the crawler's `config.py`; `row()`, `write_skills_status()` in `status.py`, through `write_text()` of `module_skills/sync.py`</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">`files`, each `path`, `state`, `vendor`, `finished_at_utc`, `report`</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">file; state; vendor; finished_at_utc; report</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a count of crawls; an age; a clock but `finished_at_utc`; a snapshot that reads itself back; a partial file</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Scalability crawler</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
           <t xml:space="preserve">the page's view of the reports</t>
         </is>
       </c>
-      <c r="C450" t="inlineStr">
+      <c r="C451" t="inlineStr">
         <is>
           <t xml:space="preserve">`scalability.js` — `SKILLS_STATUS`, `renderCrawlState()`</t>
         </is>
       </c>
-      <c r="E450" t="inlineStr">
+      <c r="E451" t="inlineStr">
         <is>
           <t xml:space="preserve">Scalability — CRAWL STATE</t>
         </is>
       </c>
-      <c r="F450" t="inlineStr">
+      <c r="F451" t="inlineStr">
         <is>
           <t xml:space="preserve">a tab named for a tool; scale for a larger basket, which is `ASSET=&lt;TICKER&gt;`</t>
-        </is>
-      </c>
-    </row>
-    <row r="452">
-      <c r="A452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rule_type_id</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t xml:space="preserve">Architecture</t>
+          <t xml:space="preserve">rule_type_id</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t xml:space="preserve">Naming</t>
+          <t xml:space="preserve">Architecture</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conformities</t>
+          <t xml:space="preserve">Naming</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t xml:space="preserve">Workflow</t>
+          <t xml:space="preserve">Conformities</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t xml:space="preserve">FileLayout</t>
+          <t xml:space="preserve">Workflow</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t xml:space="preserve">UI_TUI</t>
+          <t xml:space="preserve">FileLayout</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scalability</t>
+          <t xml:space="preserve">UI_TUI</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t xml:space="preserve">Complexity</t>
+          <t xml:space="preserve">Scalability</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t xml:space="preserve">Determinism</t>
+          <t xml:space="preserve">Complexity</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t xml:space="preserve">Performance</t>
+          <t xml:space="preserve">Determinism</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
         <is>
           <t xml:space="preserve">Methodology</t>
         </is>
@@ -17324,7 +17346,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">How an agent works on this repository: extend the module that owns a responsibility, register a new name in the commit that brings it, prove a change by running what it affects, and add a module only for a responsibility of its own. *The repository shows the destination, not the road* — subtract, don't add; the values the contract states in `AGENTS.md` § Values are not restated here.</t>
+          <t xml:space="preserve">How an agent works on this repository: extend the module that owns a responsibility, register a new name in the commit that brings it, prove a change by running what it affects, and add a module only for a responsibility of its own. Subtract, don't add; the values the contract states in `AGENTS.md` § Values are not restated here.</t>
         </is>
       </c>
     </row>
@@ -17358,7 +17380,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two runs of the same experiment give the same bits — for the same code, the same frozen input window and the same execution environment, never a byte-identical rebuild of that environment at an arbitrary future date: thread caps at one, fixed seeds, pinned orders and a sort before every write, and speed only from processes side by side. *The repository shows the destination, not the road*: bit parity is the proof, and no test suite stands in for it.</t>
+          <t xml:space="preserve">Two runs of the same experiment give the same bits — for the same code, the same frozen input window and the same execution environment, never a byte-identical rebuild of that environment at an arbitrary future date: thread caps at one, fixed seeds, pinned orders and a sort before every write, and speed only from processes side by side. Bit parity is the proof, and no test suite stands in for it.</t>
         </is>
       </c>
     </row>
@@ -17392,7 +17414,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">The one register of this project's names — a register, not an encyclopaedia: it confirms what a name already says and is never needed to decode it; the rules a name obeys are Skills, and the derivations a human reads are a methodology's. *The repository shows the destination, not the road*: the crawler reads a file against the register where the files matrix marks it, and gates nothing.</t>
+          <t xml:space="preserve">The one register of this project's names — a register, not an encyclopaedia: it confirms what a name already says and is never needed to decode it; the rules a name obeys are Skills, and the derivations a human reads are a methodology's. The crawler reads a file against the register where the files matrix marks it, and gates nothing.</t>
         </is>
       </c>
     </row>
@@ -17443,7 +17465,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Every name in this repository — a variable, a parameter, a function, a key, a directory — explains itself, so an agent never has to guess: a name is measured by the thoughts a reader needs to use it correctly, not by the characters it saves. *The repository shows the destination, not the road*: the names carry the discipline, no check gates them, and the crawler's reports say where they drift.</t>
+          <t xml:space="preserve">Every name in this repository — a variable, a parameter, a function, a key, a directory — explains itself, so an agent never has to guess: a name is measured by the thoughts a reader needs to use it correctly, not by the characters it saves. The names carry the discipline, no check gates them, and the crawler's reports say where they drift.</t>
         </is>
       </c>
     </row>
@@ -17460,7 +17482,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">A directory listing is read by eye before any parser reads it, and every machine sorts it lexicographically — so a name is designed for the order it will land in, on any server, under any locale. *The repository shows the destination, not the road*: the order is designed; the crawler reads against it every controlled file whose row marks it, and gates nothing.</t>
+          <t xml:space="preserve">A directory listing is read by eye before any parser reads it, and every machine sorts it lexicographically — so a name is designed for the order it will land in, on any server, under any locale. The order is designed; the crawler reads against it every controlled file whose row marks it, and gates nothing.</t>
         </is>
       </c>
     </row>
@@ -17494,7 +17516,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/sub_module_scalability_crawler/` reads each controlled file of the files matrix against the Skills a hand marks for it, writes one report per file a hand reads, and its snapshot. A hand starts it with `make skills-crawl`, which runs `make skills-sync` first, and nothing schedules it; it gates nothing, writes nothing but its reports and its snapshot, and commits nothing (`AGENTS.md` § Values). *The repository shows the destination, not the road*: the rules draw the destination, and a report says where one file stands from it.</t>
+          <t xml:space="preserve">`module_skills/sub_module_scalability_crawler/` reads each controlled file of the files matrix against the Skills a hand marks for it, writes one report per file a hand reads, and its snapshot. A hand starts it with `make skills-crawl`, which runs `make skills-sync` first, and nothing schedules it; it gates nothing, writes nothing but its reports and its snapshot, and commits nothing (`AGENTS.md` § Values); the rules draw the destination, and a report says where one file stands from it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Name the page's two state globals and its tab nav by what the page still holds
The crawl snapshot is rendered as it arrives and held nowhere, so the page keeps
two state globals, ML_STATUS and FEATURES_STATUS: the rule that counted three
becomes DASHBOARD-CONVENTIONS-TWO-STATE-GLOBALS, and the register's crawl view
names renderCrawlState() alone. The tab list is the data-pills="tab" nav, the
anchor the page's code selects by, in the tab rule and in the monitoring README.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -3339,12 +3339,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DASHBOARD-CONVENTIONS-THREE-STATE-GLOBALS</t>
+          <t xml:space="preserve">DASHBOARD-CONVENTIONS-TWO-STATE-GLOBALS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The page keeps three state globals — `ML_STATUS` and `FEATURES_STATUS` in `ml.js`, `SKILLS_STATUS` in `scalability.js` — the snapshots it holds after their fetch; the data snapshot and the run records are rendered as they arrive and held nowhere.</t>
+          <t xml:space="preserve">The page keeps two state globals — `ML_STATUS` and `FEATURES_STATUS` in `ml.js` — the snapshots it holds after their fetch because more than one tab renders from them; the data snapshot, the crawl snapshot and the run records are rendered as they arrive and held nowhere.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">A file-scope `let` for those three alone and a `const` for every other file-scope binding; `PILL_HOOKS`, the pill-hook registry of `page.js`, a registry and not state; a new state global entering this rule in the commit that adds it.</t>
+          <t xml:space="preserve">A file-scope `let` for those two alone and a `const` for every other file-scope binding; `PILL_HOOKS`, the pill-hook registry of `page.js`, a registry and not state; a new state global entering this rule in the commit that adds it.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">The tabs of `#tabs` in `index.html`, in their order and by their labels, named alike by `README.md` (its quickstart and its Dashboard section), by the tab's row in `module_monitoring/README_module_monitoring.md` and by the register wherever it lists them.</t>
+          <t xml:space="preserve">The tabs of the `data-pills="tab"` nav of `index.html`, in their order and by their labels, named alike by `README.md` (its quickstart and its Dashboard section), by the tab's row in `module_monitoring/README_module_monitoring.md` and by the register wherever it lists them.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -17211,7 +17211,7 @@
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t xml:space="preserve">`scalability.js` — `SKILLS_STATUS`, `renderCrawlState()`</t>
+          <t xml:space="preserve">`scalability.js` — `renderCrawlState()`</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">

</xml_diff>

<commit_message>
Hold the values and the shape in AGENTS.md, and cite the rows for the rest
AGENTS.md keeps its sections and its D rows and says what the sheet does not:
the values, the modules and their boundary, the stance of the Pre-AWS
direction, the vocabulary's principles, grammar and boundaries, the rejected
words, the default choice and the conditions of every commit. What a row of the
sheet already rules is cited by its rule_id instead of restated, and what told
a history or answered an objection nobody raised is gone: 568 lines become 315.
The stale parts go with it — run_dir() and run_payload(), a § The topology that
never existed, the second "a second compose file", the sub-module "three times"
(three kinds), and the crawler that "edits no tracked file" (it rewrites its
snapshot). The path exceptions AGENTS.md alone listed move into
PRE-AWS-SOLUTION-A-PATH-IS-BUILT-BY-ONE-DESCRIPTOR, and CLAUDE.md is the door
alone: @AGENTS.md and the line that it adds no rule.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -5697,7 +5697,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_data/lean.py`, which builds the QuantConnect Lean tree's own file names inside the folder `raw_symbol_dir()` builds.</t>
+          <t xml:space="preserve">`module_data/lean.py`, which builds the QuantConnect Lean tree's own file names inside the folder `raw_symbol_dir()` builds; `record.py`, which lists the three pipeline stores by their variables; the Makefile's serpentine search targets, which name the files they test and remove — the loop `&lt;TICKER&gt;_score_request.json`, the reset what the turn and `ml-score` write for one asset; and the page, which has no `config.py` and reads by relative path (`DASHBOARD-CONVENTIONS-THE-PAGE-READS-BY-RELATIVE-PATH`).</t>
         </is>
       </c>
     </row>
@@ -16131,7 +16131,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md` and names the working path; it points and holds no rule</t>
+          <t xml:space="preserve">the door a session opens before the contract: it loads the contract with `@AGENTS.md`, points and holds no rule</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">

</xml_diff>

<commit_message>
Tell a run from a turn and a stage, and let a comment explain
An experiment is a frozen comparison contract, a run one execution of an
experiment, a turn one resumable step of a serpentine search and a stage one
pipeline stage. RESEARCH-SEMANTICS-AN-EXPERIMENT-IS-FROZEN-AND-A-RUN-EXECUTES-IT
called the turns of a search runs and the register counted a make invocation
as one; a run is now a recorded run of the chain or a search carried from its
start to its outcome, and a turn, a stage or a make invocation as such is never
a run.

RESEARCH-SEMANTICS-ONE-CONCEPT-HAS-ONE-DEFINITION forbade every explanation in
a docstring or a comment. A docstring or a comment may describe a local
consequence or an invariant of a concept; it never gives it a second meaning or
a second canonical name, and neither does a README. Both ids stay.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -6607,7 +6607,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">An experiment is the frozen context a comparison is made in, and a run is one execution of it, resumable from what its files say; a calibration search is an experiment of its own, and a streak of minutes is never a run.</t>
+          <t xml:space="preserve">An experiment is a frozen comparison contract, a run is one execution of an experiment, resumable from what its files say, a turn is one resumable step of a serpentine search and a stage is one pipeline stage; a turn, a stage and a make invocation as such are never a run, a calibration search is an experiment of its own, and a streak of minutes is never a run.</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6617,7 +6617,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">The chain's CONFIGURABLES records at a commit and a serpentine search's `inputs` as experiments; `run_id` and the turns of one search as runs; a calibration search; `longest_flat_streak_minutes`; no calibration run.</t>
+          <t xml:space="preserve">The chain's CONFIGURABLES records at a commit and a serpentine search's `inputs` as experiments; a recorded run of the chain (`run_id`) and a serpentine search carried from its start to its outcome, however many invocations it takes, as runs; `turn()` as a turn; a target of `RECORDED_STAGES` as a stage; a calibration search; `longest_flat_streak_minutes`; no calibration run.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve">A rule of meaning here, a row of `module_skills/skill_glossary.md`, a value in `methodology_features.md` or `methodology_ml.md` citing the rule, a name in code; no second definition in a README, a docstring or a comment.</t>
+          <t xml:space="preserve">A rule of meaning here, a row of `module_skills/skill_glossary.md`, a value in `methodology_features.md` or `methodology_ml.md` citing the rule, a name in code; a docstring or a comment may describe a local consequence or an invariant of a concept but never gives it a second meaning or a second canonical name, and neither does a README.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -11893,7 +11893,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t xml:space="preserve">a turn — one call of the serpentine search: it reads where the serpentine search stands, carries it as far as the answers on disk allow, and leaves the next question or an ended search</t>
+          <t xml:space="preserve">a turn — one resumable step of a serpentine search: it reads where the serpentine search stands, carries it as far as the answers on disk allow, and leaves the next question or an ended search</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -11908,7 +11908,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t xml:space="preserve">a step, an iteration, a tick; a turn that asks two questions; a cursor, a journal or a lock recording where a turn stopped — the ledger and the search's progress are the record</t>
+          <t xml:space="preserve">a run; an iteration, a tick; a turn that asks two questions; a cursor, a journal or a lock recording where a turn stopped — the ledger and the search's progress are the record</t>
         </is>
       </c>
     </row>
@@ -16915,12 +16915,12 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t xml:space="preserve">a run — one execution of an experiment, resumable from what its files say: a recorded run of the chain, one make invocation, the turns of one serpentine search</t>
+          <t xml:space="preserve">a run — one execution of an experiment, resumable from what its files say: a recorded run of the chain, or a serpentine search carried from its start to its outcome, however many invocations it takes</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t xml:space="preserve">`RUN_ID` of the `Makefile`; a turn's resume from the ledger and the search's progress</t>
+          <t xml:space="preserve">`RUN_ID` of the `Makefile`; a search's resume from its ledger and its progress</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
@@ -16935,7 +16935,7 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t xml:space="preserve">an experiment; a streak of minutes; the methodology</t>
+          <t xml:space="preserve">an experiment; a turn; a stage; a make invocation as such; a streak of minutes; the methodology</t>
         </is>
       </c>
     </row>
@@ -16947,7 +16947,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t xml:space="preserve">a stage of a run: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
+          <t xml:space="preserve">a stage — one pipeline stage: one make target of `RECORDED_STAGES`, wrapped by `record.py` from outside every container; one seam, `data-download`, runs the two download commands in one target</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -16967,7 +16967,7 @@
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t xml:space="preserve">step, task; a stage naming itself in its record</t>
+          <t xml:space="preserve">step, task; a run; a stage naming itself in its record</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Return no noise sigma where too few pairs measure one
path_cagr_noise_standard_deviation() took the median of whatever pairs a
ledger held: none crashed it, and one gave a median absolute deviation of
zero, a sigma of no noise at all. It now returns None, not measurable, with
fewer than two fit-changing pairs; a calibration search prints that its
ledger measured none, the profile keeps null, and the missing sigma already
keeps the search from proposing anything. BTC's ledger still measures
0.01617443644117703.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -1823,7 +1823,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">`path_cagr_noise_standard_deviation` in `&lt;TICKER&gt;_serpentine_search_profile.json`, `null` or a number, read by the turn and carried unchanged by the features terminal's draft; a calibration search's last turn printing the estimate of its own ledger — the median absolute deviation of the path-CAGR differences between each line and its parent, both meeting the threshold constraint and the child fitted on its own, times `NOISE_MEDIAN_ABSOLUTE_DEVIATION_SCALE` over the square root of two.</t>
+          <t xml:space="preserve">`path_cagr_noise_standard_deviation` in `&lt;TICKER&gt;_serpentine_search_profile.json`, `null` or a number, read by the turn and carried unchanged by the features terminal's draft; a calibration search's last turn printing the estimate of its own ledger — the median absolute deviation of the path-CAGR differences between each line and its parent, both meeting the threshold constraint and the child fitted on its own, times `NOISE_MEDIAN_ABSOLUTE_DEVIATION_SCALE` over the square root of two; `None`, not measurable, where fewer than two such pairs qualify, the profile then keeping `null` and the search proposing nothing.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -12562,7 +12562,7 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t xml:space="preserve">the asset's noise sigma — the standard deviation of one evaluation's path CAGR, measured once off the ledgers of the asset's calibration searches and drafted into its profile by a decision; absent on the calibration search that measures it</t>
+          <t xml:space="preserve">the asset's noise sigma — the standard deviation of one evaluation's path CAGR, measured once off the ledgers of the asset's calibration searches and drafted into its profile by a decision; absent on the calibration search that measures it, and not measurable — `None` — on ledgers with fewer than two fit-changing pairs</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">

</xml_diff>

<commit_message>
Name the snapshot's boolean for what it compares, the search inputs
inputs_current of the feature snapshot says whether a recorded serpentine
search's inputs are the ones a turn would build now, and its docstring spoke
of "the contract", which read as the evaluation contract. It is renamed
search_inputs_current and means that comparison alone: the evaluation
contract is no part of it, since this module cannot know the one the next
answer will carry, and the next turn's probe compares it. The docstring names
the catalogue contract it reads; the page, the features terminal's README,
the rule texts and the register move with the key, and the tracked snapshot
is written again by features-status.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -1453,7 +1453,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">`build_search_inputs()` — the research window, the seed and the warm-up, `best_params`, the catalogue's columns, the asset's active columns and barriers, the profile, the beam width and the round budget — recorded in the search's progress and compared by equality at every turn: equal resumes at the round boundary, different removes the ledger, the request and the response before the first question; `evaluation_contract` of every response — `score.evaluation_contract()`, the module's records whose `experiment_identity` is true and the maximum label horizon `dataset.load_maximum_label_horizon_minutes()` derives — recorded from the first and compared with every answer read at a turn's start, a different one restarting the search as different inputs do; `serpentine_search_block()` publishing `inputs_current` as a boolean, raising nothing on a missing profile and publishing no proposal while it is false; `features-serpentine-search-reset`, `ASSET=` one ticker of `TICKERS`, removing `&lt;TICKER&gt;_serpentine_search.json`, `&lt;TICKER&gt;_serpentine_search_state_evaluations.jsonl`, `&lt;TICKER&gt;_score_request.json`, `&lt;TICKER&gt;_score_response.json` and the asset's partition `score_trials/ticker=&lt;TICKER&gt;/` of the trials store, keeping the profile, the promoted search state, the chain's files and `hpo_trials`, and running no stage.</t>
+          <t xml:space="preserve">`build_search_inputs()` — the research window, the seed and the warm-up, `best_params`, the catalogue's columns, the asset's active columns and barriers, the profile, the beam width and the round budget — recorded in the search's progress and compared by equality at every turn: equal resumes at the round boundary, different removes the ledger, the request and the response before the first question; `evaluation_contract` of every response — `score.evaluation_contract()`, the module's records whose `experiment_identity` is true and the maximum label horizon `dataset.load_maximum_label_horizon_minutes()` derives — recorded from the first and compared with every answer read at a turn's start, a different one restarting the search as different inputs do; `serpentine_search_block()` publishing `search_inputs_current` as a boolean, raising nothing on a missing profile and publishing no proposal while it is false; `features-serpentine-search-reset`, `ASSET=` one ticker of `TICKERS`, removing `&lt;TICKER&gt;_serpentine_search.json`, `&lt;TICKER&gt;_serpentine_search_state_evaluations.jsonl`, `&lt;TICKER&gt;_score_request.json`, `&lt;TICKER&gt;_score_response.json` and the asset's partition `score_trials/ticker=&lt;TICKER&gt;/` of the trials store, keeping the profile, the promoted search state, the chain's files and `hpo_trials`, and running no stage.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">`proposals_block()` at every round boundary returning the champion as proposal 1 when `search_outcome` is set, `champion_state_evaluation_index` is not 1 and its gain clears `proposal_threshold_multiple()` of N times the sigma, an empty list otherwise and always without a noise sigma; the snapshot publishing the proposals only while `inputs_current` holds.</t>
+          <t xml:space="preserve">`proposals_block()` at every round boundary returning the champion as proposal 1 when `search_outcome` is set, `champion_state_evaluation_index` is not 1 and its gain clears `proposal_threshold_multiple()` of N times the sigma, an empty list otherwise and always without a noise sigma; the snapshot publishing the proposals only while `search_inputs_current` holds.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -12712,7 +12712,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t xml:space="preserve">current inputs — a recorded serpentine search's inputs that are still the asset's own</t>
+          <t xml:space="preserve">the current search inputs — whether a recorded serpentine search's inputs are the ones a turn would build now, and nothing else: the evaluation contract is no part of it, the next turn's probe comparing that</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -12722,7 +12722,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs_current`</t>
+          <t xml:space="preserve">`search_inputs_current`</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t xml:space="preserve">stale, dirty, outdated; a guard that refuses the promotion</t>
+          <t xml:space="preserve">stale, dirty, outdated; a guard that refuses the promotion; `inputs_current`; an evaluation contract rebuilt in `module_features`</t>
         </is>
       </c>
     </row>
@@ -13650,7 +13650,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t xml:space="preserve">`features_status.json`: `generated_at_utc`, `catalogue`, `configurables` (the module's records and the serpentine search's, *a CONFIGURABLES record*), `assets` (per asset `ticker`, `row_count_by_timeframe`, `serpentine_search` — `null` while no serpentine search has run; else `state_evaluation_count`, `selection_hypothesis_count`, `round_count`, `beam_changed`, `search_outcome`, `inputs_current`, `proposals`)</t>
+          <t xml:space="preserve">`features_status.json`: `generated_at_utc`, `catalogue`, `configurables` (the module's records and the serpentine search's, *a CONFIGURABLES record*), `assets` (per asset `ticker`, `row_count_by_timeframe`, `serpentine_search` — `null` while no serpentine search has run; else `state_evaluation_count`, `selection_hypothesis_count`, `round_count`, `beam_changed`, `search_outcome`, `search_inputs_current`, `proposals`)</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -15706,7 +15706,7 @@
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t xml:space="preserve">`inputs_current`, which folds the parameters, the catalogue and the asset's own search state and stays the page's</t>
+          <t xml:space="preserve">`search_inputs_current`, which folds the parameters, the catalogue and the asset's own search state and stays the page's</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Name the ML layer's locals, writers and barrier walk, as the crawl asked
The crawl's findings on the ML layer, each checked against its rule; no
number moves. The barrier walk names what it holds: entry_minute_rows,
upper_barrier_hit and lower_barrier_hit, their offsets in minutes and the
resolution_offset_minutes it returns, which strategy.py and event_end_ts()
read under that name, and the open and the volume of the 1m path by their
quantities. HPO's study writer takes the closed verb, write_trials(), and
its locals say what they hold (sweeps_by_fold, cleared_thresholds,
floor_clearing_thresholds, parent_admissible_thresholds,
hyperparameter_point_json, parameters_json); X and Y align on
y_decision_rows, and the gain importance reads total_gain_by_column. The
docstrings name the recursive mean of the true range and
LABEL_BARRIER_TRUE_RANGE_TIMEFRAME rather than ATR14 of a 1h bar, the
package names search states, and the ML README spells HPO out once.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -12749,7 +12749,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t xml:space="preserve">`sweep_selection()`, the return of `objective()` inside `build_objective()` in `module_ml/hpo.py`, logged per trial by `log_trials()` under `TRIAL_METRIC_KEY`</t>
+          <t xml:space="preserve">`sweep_selection()`, the return of `objective()` inside `build_objective()` in `module_ml/hpo.py`, logged per trial by `write_trials()` under `TRIAL_METRIC_KEY`</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -13961,7 +13961,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t xml:space="preserve">`store/trials/`, `STORE_TRIALS_DIR`, mounted into the `ml` runner alone; `hpo_trials_jsonl()`, `score_trials_jsonl()` in `module_ml/config.py` — `&lt;family&gt;/ticker=&lt;TICKER&gt;/&lt;family&gt;.jsonl`, the family's `schema.json` beside its partitions; `log_trials()` in `module_ml/hpo.py` the one appender, `study_index` counted off the writer's own partition</t>
+          <t xml:space="preserve">`store/trials/`, `STORE_TRIALS_DIR`, mounted into the `ml` runner alone; `hpo_trials_jsonl()`, `score_trials_jsonl()` in `module_ml/config.py` — `&lt;family&gt;/ticker=&lt;TICKER&gt;/&lt;family&gt;.jsonl`, the family's `schema.json` beside its partitions; `write_trials()` in `module_ml/hpo.py` the one appender, `study_index` counted off the writer's own partition</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -14010,7 +14010,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t xml:space="preserve">`log_trials()`, `trial_row()` in `module_ml/hpo.py`; `origin` `hpo` from `ml-hpo`, `serpentine_search` from `ml-score`</t>
+          <t xml:space="preserve">`write_trials()`, `trial_row()` in `module_ml/hpo.py`; `origin` `hpo` from `ml-hpo`, `serpentine_search` from `ml-score`</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">

</xml_diff>

<commit_message>
Call the rendered name register the register, as the crawl asked
The glossary is the sheet's table; what the sync renders from it into
module_skills/skill_glossary.md is the register, as the register's own
rows for the sheet and the name register say. The canon module's
docstring, its config.py, the sync's docstring and the Makefile's comment
called the rendered document the glossary; so did two rules of the files
and folders Skill, FILES-AND-FOLDERS-SHEET-IS-THE-SOURCE and
FILES-AND-FOLDERS-SKILL-IS-RENDERED, whose ids stay with their meaning.
Where the word names the table, as in the refusal of a concept
registered twice, it stays.
</commit_message>
<xml_diff>
--- a/module_skills/skills_sheet.xlsx
+++ b/module_skills/skills_sheet.xlsx
@@ -5275,7 +5275,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">`module_skills/skills_sheet.xlsx` is the one source of every Skill and of the glossary, and its files matrix is the crawler's whole contract: `X` chooses the context, the row names the controlled file.</t>
+          <t xml:space="preserve">`module_skills/skills_sheet.xlsx` is the one source of every Skill and of the register, and its files matrix is the crawler's whole contract: `X` chooses the context, the row names the controlled file.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">One workbook; every Skill and the glossary rendered from it; a row of the files matrix per controlled file or glob; no total of Skills, rules, documents or controlled files written in a tracked file.</t>
+          <t xml:space="preserve">One workbook; every Skill and the register rendered from it; a row of the files matrix per controlled file or glob; no total of Skills, rules, documents or controlled files written in a tracked file.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">`GENERATED_MARKER` of `module_skills/config.py` on line 1, the stem of `skill_path` as its heading, the summary, one list per `rule_type_id` and, in the glossary, the register after them; a change made on the sheet and synced; a generated document the sheet no longer names deleted by the sync; each Skill in `module_skills/`, in a module's `skills/` or beside the sub-module it governs.</t>
+          <t xml:space="preserve">`GENERATED_MARKER` of `module_skills/config.py` on line 1, the stem of `skill_path` as its heading, the summary, one list per `rule_type_id` and, in `module_skills/skill_glossary.md`, the register after them; a change made on the sheet and synced; a generated document the sheet no longer names deleted by the sync; each Skill in `module_skills/`, in a module's `skills/` or beside the sub-module it governs.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">

</xml_diff>